<commit_message>
v1.17: proyección base G/P Total real, tasa promedio, días naturales, marcha G/P acum
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E49"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -1226,9 +1226,26 @@
         <v>Implementacion</v>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>01/03/2026</v>
+      </c>
+      <c r="B49" t="str">
+        <v>09:30</v>
+      </c>
+      <c r="C49" t="str">
+        <v>Proyección Int. caución: base Total real y marcha</v>
+      </c>
+      <c r="D49" t="str">
+        <v>Punto de partida = G/P Total real (totalIngresos - totalEgresos) + interés acumulado; tasa = promedio del último mes real; días naturales (31 ene, 28 feb, etc.); Int T-1 día 1 = interés acumulado real; modal marcha proyectado: desglose G/P acum Total real + Int. acum = Base partida; columna G/P acum solo G/P (Día 1 = Total real).</v>
+      </c>
+      <c r="E49" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E48"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E49"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1590,7 +1607,7 @@
         <v>Int. por caución proyectado</v>
       </c>
       <c r="B44" t="str">
-        <v>Para cada mes proyectado: punto de partida = G/P + interés del período anterior (último real para mes 1; proyectado 1 para mes 2; proyectado 2 para mes 3). Se aplica la última tasa conocida en cadena. Sin salto respecto al último valor real.</v>
+        <v>Punto de partida = G/P Total real (Total de la tabla) + interés acumulado; tasa = promedio del último mes real; días naturales del mes (31 ene, 28/29 feb, etc.); Int T-1 día 1 = interés acumulado real. Modal marcha: desglose G/P acum Total real + Int. acum = Base partida; columna G/P acum muestra solo G/P (Día 1 = Total real).</v>
       </c>
     </row>
     <row r="45">
@@ -1697,7 +1714,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C19"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1902,16 +1919,27 @@
         <v>Proyección 3 meses: config (mediana/promedio, meses historia), ventana rodante; Int. por caución proyectado con punto de partida = último real (G/P+interés) y última tasa en cadena; disclaimer bajo proyección. Despliegue a producción.</v>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>1.17</v>
+      </c>
+      <c r="B19" t="str">
+        <v>01/03/2026</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Proyección: punto de partida = G/P Total real (no último mes); tasa = promedio último mes real; días naturales por mes; Int T-1 día 1 = interés acumulado real; modal marcha proyectado con desglose (G/P acum Total real + Int. acum) y columna G/P acum solo G/P (Día 1 = Total real). Despliegue a producción.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C19"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="90.83203125" customWidth="1"/>
@@ -1986,51 +2014,62 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Listado y edición completa de transacciones</v>
+        <v>Proyección de flujo (próximos 3 meses)</v>
       </c>
       <c r="B7" t="str">
-        <v>Solapa Todas las transacciones con listado completo, filtros por mes y categoría, y modal de edición con todos los campos y combos para valores normalizados (categoría, cuenta contable, tipo movimiento, status, medio pago, moneda, origen archivo).</v>
+        <v>Proyección de ingresos, egresos, G/P y ratios para los próximos 3 meses con configuración (mediana/promedio, meses de historia 3/6/12/24), ventana rodante; Int. por caución proyectado en cadena desde último real (G/P+interés); disclaimer de metodología bajo la proyección.</v>
       </c>
       <c r="C7">
-        <v>45000</v>
+        <v>55000</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Bitácora y documentación</v>
+        <v>Listado y edición completa de transacciones</v>
       </c>
       <c r="B8" t="str">
-        <v>Implementación de la bitácora en Excel (Log, Resumen, Versiones, Ref Git y Vercel, Presupuesto) y documentación funcional básica para el uso de la app.</v>
+        <v>Solapa Todas las transacciones con listado completo, filtros por mes y categoría, y modal de edición con todos los campos y combos para valores normalizados (categoría, cuenta contable, tipo movimiento, status, medio pago, moneda, origen archivo).</v>
       </c>
       <c r="C8">
-        <v>120000</v>
+        <v>45000</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Integración y despliegue</v>
+        <v>Bitácora y documentación</v>
       </c>
       <c r="B9" t="str">
-        <v>Configuración de repositorio Git/GitHub, flujo de despliegue a Vercel y ajustes de configuración (vercel.json, conexión con Supabase).</v>
+        <v>Implementación de la bitácora en Excel (Log, Resumen, Versiones, Ref Git y Vercel, Presupuesto) y documentación funcional básica para el uso de la app.</v>
       </c>
       <c r="C9">
-        <v>90000</v>
+        <v>120000</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
+        <v>Integración y despliegue</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Configuración de repositorio Git/GitHub, flujo de despliegue a Vercel y ajustes de configuración (vercel.json, conexión con Supabase).</v>
+      </c>
+      <c r="C10">
+        <v>90000</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
         <v>Mantenimiento y soporte inicial</v>
       </c>
-      <c r="B10" t="str">
+      <c r="B11" t="str">
         <v>Soporte post–implementación, pequeños ajustes funcionales y acompañamiento durante el primer período de uso.</v>
       </c>
-      <c r="C10">
+      <c r="C11">
         <v>80000</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
v1.18: ventana rodante, Int T-1 último día anterior, G/P acum inicio día
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E50"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -1243,9 +1243,26 @@
         <v>Implementacion</v>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>01/03/2026</v>
+      </c>
+      <c r="B50" t="str">
+        <v>10:00</v>
+      </c>
+      <c r="C50" t="str">
+        <v>Ventana rodante e Int T-1 y G/P acum inicio día</v>
+      </c>
+      <c r="D50" t="str">
+        <v>Ventana rodante: numReal hace que mes 2 y 3 proyectados usen menos reales + proyectados (ingresos/egresos distintos). Int T-1 día 1 = (Int T-1 + Int T) del último día del mes anterior (desde detalle real o prevRes). G/P acum en marcha (real y proyectado) = valor al inicio del día, no incluye ese día.</v>
+      </c>
+      <c r="E50" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E49"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E50"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1607,7 +1624,7 @@
         <v>Int. por caución proyectado</v>
       </c>
       <c r="B44" t="str">
-        <v>Punto de partida = G/P Total real (Total de la tabla) + interés acumulado; tasa = promedio del último mes real; días naturales del mes (31 ene, 28/29 feb, etc.); Int T-1 día 1 = interés acumulado real. Modal marcha: desglose G/P acum Total real + Int. acum = Base partida; columna G/P acum muestra solo G/P (Día 1 = Total real).</v>
+        <v>Punto de partida = G/P Total real + interés acumulado; tasa = promedio último mes real; días naturales; Int T-1 día 1 = (Int T-1 + Int T) último día del mes anterior. G/P acum en marcha = al inicio de cada día (real y proyectado). Ventana rodante: ingresos/egresos distintos por mes.</v>
       </c>
     </row>
     <row r="45">
@@ -1714,7 +1731,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C20"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1930,9 +1947,20 @@
         <v>Proyección: punto de partida = G/P Total real (no último mes); tasa = promedio último mes real; días naturales por mes; Int T-1 día 1 = interés acumulado real; modal marcha proyectado con desglose (G/P acum Total real + Int. acum) y columna G/P acum solo G/P (Día 1 = Total real). Despliegue a producción.</v>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>1.18</v>
+      </c>
+      <c r="B20" t="str">
+        <v>01/03/2026</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Ventana rodante: ingresos/egresos/G/P distintos por mes (drop real cuando pocos meses). Int T-1 día 1 = (Int T-1 + Int T) último día del mes anterior (real o proyectado). G/P acum en marcha = inicio del día (real y proyectado), no incluye ese día. Despliegue a producción.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C20"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.19: unificación botones/iconos, escala combo % caución
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E51"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -1260,16 +1260,33 @@
         <v>Implementacion</v>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>27/02/2026</v>
+      </c>
+      <c r="B51" t="str">
+        <v>12:00</v>
+      </c>
+      <c r="C51" t="str">
+        <v>Unificación botones e iconos</v>
+      </c>
+      <c r="D51" t="str">
+        <v>Mismo estilo en todos los botones: icono SVG + texto. Sidebar (chevron, home, engranaje), tabs con iconos, exportar con icono descarga, modales (Guardar/Cerrar/Excluir/Eliminar con iconos). Iconos solos (cerrar, editar, alerta) en SVG. Escala combo % G/P en caución de 5 en 5.</v>
+      </c>
+      <c r="E51" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E50"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E51"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B45"/>
+  <dimension ref="A1:B47"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -1635,9 +1652,25 @@
         <v>Debajo de las filas proyectadas, texto en letra chica y gris oscuro que explica la metodología: Mediana/Promedio de N meses, ventana rodante, y cálculo de Int. por caución proyectado.</v>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>Botones e iconos unificados</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Todos los botones con mismo estilo: icono SVG + texto. Sidebar (chevron, home, engranaje), tabs con iconos, exportar con icono descarga, modales con iconos (Guardar, Cerrar, Excluir, Eliminar). Iconos solos (cerrar, editar, alerta) en SVG.</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>Configuración % G/P en caución</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Combo "% G/P acum. en caución" en Configuración con escala de 5 en 5 (100, 95, 90… hasta 0). Por defecto 100 %; menor % = más liquidez (menos interés por caución).</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B45"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B47"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1731,7 +1764,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1958,9 +1991,20 @@
         <v>Ventana rodante: ingresos/egresos/G/P distintos por mes (drop real cuando pocos meses). Int T-1 día 1 = (Int T-1 + Int T) último día del mes anterior (real o proyectado). G/P acum en marcha = inicio del día (real y proyectado), no incluye ese día. Despliegue a producción.</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>1.19</v>
+      </c>
+      <c r="B21" t="str">
+        <v>27/02/2026</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Unificación de botones e iconos: mismo estilo (icono SVG + texto) en sidebar, tabs, exportar, modales; iconos solos (cerrar, editar, alerta) en SVG. Escala combo % G/P en caución de 5 en 5 (100, 95, 90…). Despliegue a producción.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C21"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.20: Caución (x% cash), quitar icono %
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E52"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -1277,16 +1277,33 @@
         <v>Implementacion</v>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>27/02/2026</v>
+      </c>
+      <c r="B52" t="str">
+        <v>12:30</v>
+      </c>
+      <c r="C52" t="str">
+        <v>Etiqueta Caución (x% cash)</v>
+      </c>
+      <c r="D52" t="str">
+        <v>Simplificar texto Int. por caución a Caución (x% cash) en cabecera de flujo por mes; x = valor del parámetro % G/P en caución. Quitar icono % a la izquierda. Modales de marcha y disclaimer con Caución.</v>
+      </c>
+      <c r="E52" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E51"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E52"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B47"/>
+  <dimension ref="A1:B48"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -1668,9 +1685,17 @@
         <v>Combo "% G/P acum. en caución" en Configuración con escala de 5 en 5 (100, 95, 90… hasta 0). Por defecto 100 %; menor % = más liquidez (menos interés por caución).</v>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>Etiqueta Caución (x% cash)</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Columna en flujo por mes: cabecera "Caución (x% cash)" donde x es el valor del parámetro % G/P; sin icono % a la izquierda. Modales de marcha y disclaimer usan "Caución".</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B47"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B48"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1764,7 +1789,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C22"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -2002,9 +2027,20 @@
         <v>Unificación de botones e iconos: mismo estilo (icono SVG + texto) en sidebar, tabs, exportar, modales; iconos solos (cerrar, editar, alerta) en SVG. Escala combo % G/P en caución de 5 en 5 (100, 95, 90…). Despliegue a producción.</v>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>1.20</v>
+      </c>
+      <c r="B22" t="str">
+        <v>27/02/2026</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Simplificar etiqueta: Int. por caución pasa a Caución (x% cash) en cabecera de flujo (x = parámetro % G/P); quitar icono % a la izquierda; modales y disclaimer con texto Caución. Despliegue a producción.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C22"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.21: meses a proyectar, config por usuario en Supabase
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E54"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -1294,16 +1294,50 @@
         <v>Implementacion</v>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>27/02/2026</v>
+      </c>
+      <c r="B53" t="str">
+        <v>13:00</v>
+      </c>
+      <c r="C53" t="str">
+        <v>Meses a proyectar en Configuración</v>
+      </c>
+      <c r="D53" t="str">
+        <v>Nuevo parámetro en Configuración: Meses a proyectar (1, 2, 3, 4, 5, 6, 12). Flujo por mes y Evolución muestran esa cantidad de meses proyectados. proyeccionDesdeSerie generalizada a N meses.</v>
+      </c>
+      <c r="E53" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>27/02/2026</v>
+      </c>
+      <c r="B54" t="str">
+        <v>13:15</v>
+      </c>
+      <c r="C54" t="str">
+        <v>Config dashboard por usuario en Supabase</v>
+      </c>
+      <c r="D54" t="str">
+        <v>Tabla config_dashboard en Supabase (user_id, proyeccion_metodo, proyeccion_meses, proyeccion_cantidad, pct_caucion). RLS por usuario. Al cargar: sync desde Supabase (Auth anónimo); al guardar: upsert en Supabase. Fallback a localStorage si no hay usuario.</v>
+      </c>
+      <c r="E54" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E52"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E54"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B48"/>
+  <dimension ref="A1:B50"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -1693,9 +1727,25 @@
         <v>Columna en flujo por mes: cabecera "Caución (x% cash)" donde x es el valor del parámetro % G/P; sin icono % a la izquierda. Modales de marcha y disclaimer usan "Caución".</v>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>Meses a proyectar</v>
+      </c>
+      <c r="B49" t="str">
+        <v>En Configuración: combo Meses a proyectar (1, 2, 3, 4, 5, 6, 12). Flujo por mes y Evolución muestran esa cantidad de columnas/filas proyectadas.</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>Config por usuario en Supabase</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Tabla config_dashboard (user_id, proyección y caución). Con Auth anónimo se sincroniza al cargar y al guardar; la config persiste por usuario en la base. Migración: supabase_config_dashboard.sql.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B48"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B50"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1789,7 +1839,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -2038,9 +2088,20 @@
         <v>Simplificar etiqueta: Int. por caución pasa a Caución (x% cash) en cabecera de flujo (x = parámetro % G/P); quitar icono % a la izquierda; modales y disclaimer con texto Caución. Despliegue a producción.</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>1.21</v>
+      </c>
+      <c r="B23" t="str">
+        <v>27/02/2026</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Config por usuario en Supabase: parámetro Meses a proyectar (1-12) en Configuración; tabla config_dashboard (user_id, proyección y caución); sync al cargar y al guardar con Auth anónimo. Despliegue a producción.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C23"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.22: Recorte % (cada lado) en Config; visible solo con Promedio recortado; proyeccion_recorte en config_dashboard
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:E56"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -1328,16 +1328,50 @@
         <v>Implementacion</v>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>27/02/2026</v>
+      </c>
+      <c r="B55" t="str">
+        <v>14:00</v>
+      </c>
+      <c r="C55" t="str">
+        <v>Recorte % (cada lado) en Configuración</v>
+      </c>
+      <c r="D55" t="str">
+        <v>Parámetro Recorte % (cada lado) en Configuración (0, 5, 10, 15, 20, 25) para el método Promedio recortado. Persistido en localStorage y columna proyeccion_recorte en config_dashboard (Supabase).</v>
+      </c>
+      <c r="E55" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>27/02/2026</v>
+      </c>
+      <c r="B56" t="str">
+        <v>14:10</v>
+      </c>
+      <c r="C56" t="str">
+        <v>Recorte % solo si Promedio recortado</v>
+      </c>
+      <c r="D56" t="str">
+        <v>El campo Recorte % (cada lado) se muestra en Configuración solo cuando el método elegido es Promedio recortado; al cambiar de método se oculta o muestra al instante.</v>
+      </c>
+      <c r="E56" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E54"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E56"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B50"/>
+  <dimension ref="A1:B51"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -1743,9 +1777,17 @@
         <v>Tabla config_dashboard (user_id, proyección y caución). Con Auth anónimo se sincroniza al cargar y al guardar; la config persiste por usuario en la base. Migración: supabase_config_dashboard.sql.</v>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>Recorte % (cada lado)</v>
+      </c>
+      <c r="B51" t="str">
+        <v>En Configuración, combo Recorte % (cada lado) (0, 5, 10, 15, 20, 25) visible solo cuando el método es Promedio recortado. Más % = más suavizado. Persistido en config_dashboard (proyeccion_recorte).</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B50"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B51"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1839,7 +1881,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C24"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -2099,9 +2141,20 @@
         <v>Config por usuario en Supabase: parámetro Meses a proyectar (1-12) en Configuración; tabla config_dashboard (user_id, proyección y caución); sync al cargar y al guardar con Auth anónimo. Despliegue a producción.</v>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>1.22</v>
+      </c>
+      <c r="B24" t="str">
+        <v>27/02/2026</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Parámetro Recorte % (cada lado) en Configuración (0-25); visible solo si método es Promedio recortado. Columna proyeccion_recorte en config_dashboard. Despliegue a producción.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C24"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.23: Parámetros por defecto sin datos de usuario (Método Promedio recortado, Recorte 20%, G/P caución 95%)
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:E57"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -1362,9 +1362,26 @@
         <v>Implementacion</v>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>27/02/2026</v>
+      </c>
+      <c r="B57" t="str">
+        <v>15:00</v>
+      </c>
+      <c r="C57" t="str">
+        <v>Parámetros por defecto sin datos de usuario</v>
+      </c>
+      <c r="D57" t="str">
+        <v>Si no hay config del usuario: Meses a proyectar 3, Método Promedio recortado, Recorte 20%, Meses de historia 6, % G/P acum. en caución 95%. Aplicado en getProyeccionConfig, getPctCaucion, sync y combos del modal.</v>
+      </c>
+      <c r="E57" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E56"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E57"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1881,7 +1898,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C25"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -2152,9 +2169,20 @@
         <v>Parámetro Recorte % (cada lado) en Configuración (0-25); visible solo si método es Promedio recortado. Columna proyeccion_recorte en config_dashboard. Despliegue a producción.</v>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>1.23</v>
+      </c>
+      <c r="B25" t="str">
+        <v>27/02/2026</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Valores por defecto sin datos de usuario: Meses a proyectar 3, Método Promedio recortado, Recorte 20%, Meses de historia 6, % G/P en caución 95%. Despliegue a producción.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C25"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.24: Demo cliente - leyenda datos ficticios al costado Evolución; SQL respaldo transacciones_fornitalia y carga monto×0,70
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -1898,7 +1898,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C26"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -2180,20 +2180,32 @@
         <v>Valores por defecto sin datos de usuario: Meses a proyectar 3, Método Promedio recortado, Recorte 20%, Meses de historia 6, % G/P en caución 95%. Despliegue a producción.</v>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>1.24</v>
+      </c>
+      <c r="B26" t="str">
+        <v>27/02/2026</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Demo potencial cliente: leyenda roja "Los datos presentados son ficticios..." al costado de Evolución; script SQL transacciones_fornitalia (respaldo) y carga con monto×0,70. Despliegue a producción.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C25"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C26"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:D11"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="90.83203125" customWidth="1"/>
-    <col min="3" max="3" width="24.83203125" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="22.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2204,7 +2216,10 @@
         <v>Descripción comercial</v>
       </c>
       <c r="C1" t="str">
-        <v>Importe sugerido (ARS)</v>
+        <v>Horas hombre</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Importe sugerido (USD)</v>
       </c>
     </row>
     <row r="2">
@@ -2215,7 +2230,10 @@
         <v>Relevamiento, limpieza y normalización de datos históricos de caja (campos de moneda, categorías, cuentas contables, flags de edición). Incluye lógica de excepciones y detección de inconsistencias.</v>
       </c>
       <c r="C2">
-        <v>250000</v>
+        <v>2</v>
+      </c>
+      <c r="D2">
+        <v>100</v>
       </c>
     </row>
     <row r="3">
@@ -2226,7 +2244,10 @@
         <v>Diseño y desarrollo del dashboard mensual (Flujo por mes, Resumen, alertas, modal By Categoría / By Cuenta, gráficos de serie mensual). Incluye formatos de moneda y visualizaciones.</v>
       </c>
       <c r="C3">
-        <v>320000</v>
+        <v>100</v>
+      </c>
+      <c r="D3">
+        <v>5000</v>
       </c>
     </row>
     <row r="4">
@@ -2237,7 +2258,10 @@
         <v>Detección de potencial duplicado (fecha, monto, tipo, cliente, descripción similar), tipo de error (inconsistencia / duplicado), filtro por tipo, modal de comparación con id_origen y Cliente, acciones anular o eliminar registro.</v>
       </c>
       <c r="C4">
-        <v>85000</v>
+        <v>25</v>
+      </c>
+      <c r="D4">
+        <v>1250</v>
       </c>
     </row>
     <row r="5">
@@ -2248,7 +2272,10 @@
         <v>Solapa Evolución: tabla dinámica con filas por Categoría o Cuenta contable y columnas por Período (Diario o Mensual). Neto por celda en moneda seleccionada.</v>
       </c>
       <c r="C5">
-        <v>55000</v>
+        <v>20</v>
+      </c>
+      <c r="D5">
+        <v>1000</v>
       </c>
     </row>
     <row r="6">
@@ -2259,7 +2286,10 @@
         <v>Columna Int. por caución en flujo por mes: cálculo de interés mensual por reinversión del sobrante a un día con tasa de serie de cauciones. Carga de Excel al refrescar, modal de marcha de cálculo (G/P acum, Base, Tasa, Int T). Incluye soporte para múltiples formatos de fecha y columna tasa_diaria.</v>
       </c>
       <c r="C6">
-        <v>50000</v>
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>900</v>
       </c>
     </row>
     <row r="7">
@@ -2270,7 +2300,10 @@
         <v>Proyección de ingresos, egresos, G/P y ratios para los próximos 3 meses con configuración (mediana/promedio, meses de historia 3/6/12/24), ventana rodante; Int. por caución proyectado en cadena desde último real (G/P+interés); disclaimer de metodología bajo la proyección.</v>
       </c>
       <c r="C7">
-        <v>55000</v>
+        <v>30</v>
+      </c>
+      <c r="D7">
+        <v>1500</v>
       </c>
     </row>
     <row r="8">
@@ -2281,7 +2314,10 @@
         <v>Solapa Todas las transacciones con listado completo, filtros por mes y categoría, y modal de edición con todos los campos y combos para valores normalizados (categoría, cuenta contable, tipo movimiento, status, medio pago, moneda, origen archivo).</v>
       </c>
       <c r="C8">
-        <v>45000</v>
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>1100</v>
       </c>
     </row>
     <row r="9">
@@ -2292,7 +2328,10 @@
         <v>Implementación de la bitácora en Excel (Log, Resumen, Versiones, Ref Git y Vercel, Presupuesto) y documentación funcional básica para el uso de la app.</v>
       </c>
       <c r="C9">
-        <v>120000</v>
+        <v>35</v>
+      </c>
+      <c r="D9">
+        <v>1750</v>
       </c>
     </row>
     <row r="10">
@@ -2303,7 +2342,10 @@
         <v>Configuración de repositorio Git/GitHub, flujo de despliegue a Vercel y ajustes de configuración (vercel.json, conexión con Supabase).</v>
       </c>
       <c r="C10">
-        <v>90000</v>
+        <v>30</v>
+      </c>
+      <c r="D10">
+        <v>1500</v>
       </c>
     </row>
     <row r="11">
@@ -2314,12 +2356,15 @@
         <v>Soporte post–implementación, pequeños ajustes funcionales y acompañamiento durante el primer período de uso.</v>
       </c>
       <c r="C11">
-        <v>80000</v>
+        <v>28</v>
+      </c>
+      <c r="D11">
+        <v>1400</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
v1.25: Ayuda al clic en Comisiones/Ventas y Egresos/Ingresos; regla bitácora con tecnología e infraestructura
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E57"/>
+  <dimension ref="A1:E58"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -1379,9 +1379,26 @@
         <v>Implementacion</v>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>27/02/2026</v>
+      </c>
+      <c r="B58" t="str">
+        <v>16:00</v>
+      </c>
+      <c r="C58" t="str">
+        <v>Ayuda al clic en columnas flujo y regla bitácora</v>
+      </c>
+      <c r="D58" t="str">
+        <v>Columnas Comisiones/Ventas y Egresos/Ingresos: icono de ayuda que al clic muestra popover con texto (Comisiones: "Corresponde solo a las comisiones por venta."; Egresos: "Egresos - Comisiones por Venta / Ingresos"). Regla bitácora: sección tecnología e infraestructura y refuerzo para actualizar todas las solapas que correspondan.</v>
+      </c>
+      <c r="E58" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E57"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E58"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1439,15 +1456,15 @@
         <v>Comisiones/Ventas %</v>
       </c>
       <c r="B6" t="str">
-        <v>Columna: porcentaje comisiones (egresos comisión desde Sueldos) sobre ventas del mes.</v>
+        <v>Columna: porcentaje comisiones (egresos comisión desde Sueldos) sobre ventas del mes. Icono de ayuda al clic: "Corresponde solo a las comisiones por venta."</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Egr s/com. / Ingresos</v>
+        <v>Egresos / Ingresos</v>
       </c>
       <c r="B7" t="str">
-        <v>Columna: porcentaje (egresos sin comisiones) sobre ingresos del mes.</v>
+        <v>Columna Egresos (icono ayuda) / Ingresos: porcentaje (egresos sin comisiones) sobre ingresos. Ayuda al clic: "Egresos - Comisiones por Venta / Ingresos".</v>
       </c>
     </row>
     <row r="8">
@@ -1898,7 +1915,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C27"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -2191,9 +2208,20 @@
         <v>Demo potencial cliente: leyenda roja "Los datos presentados son ficticios..." al costado de Evolución; script SQL transacciones_fornitalia (respaldo) y carga con monto×0,70. Despliegue a producción.</v>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>1.25</v>
+      </c>
+      <c r="B27" t="str">
+        <v>27/02/2026</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Ayuda al clic en columnas Comisiones/Ventas y Egresos/Ingresos (popover con texto explicativo). Regla bitácora: tecnología e infraestructura y actualizar todas las solapas. Despliegue a producción.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C26"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C27"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.26: Alerta desvío con categoría en negrita sin comillas
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E58"/>
+  <dimension ref="A1:E59"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -1381,10 +1381,10 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>27/02/2026</v>
+        <v>01/03/2026</v>
       </c>
       <c r="B58" t="str">
-        <v>16:00</v>
+        <v>23:45</v>
       </c>
       <c r="C58" t="str">
         <v>Ayuda al clic en columnas flujo y regla bitácora</v>
@@ -1396,9 +1396,26 @@
         <v>Implementacion</v>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>01/03/2026</v>
+      </c>
+      <c r="B59" t="str">
+        <v>23:45</v>
+      </c>
+      <c r="C59" t="str">
+        <v>Alerta desvío: categoría en negrita sin comillas</v>
+      </c>
+      <c r="D59" t="str">
+        <v>En el mensaje de alerta de desvío de categoría, reemplazar la categoría entre comillas por la categoría en negrita (sin comillas).</v>
+      </c>
+      <c r="E59" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E58"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E59"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1915,7 +1932,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C28"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -2213,15 +2230,26 @@
         <v>1.25</v>
       </c>
       <c r="B27" t="str">
-        <v>27/02/2026</v>
+        <v>01/03/2026</v>
       </c>
       <c r="C27" t="str">
         <v>Ayuda al clic en columnas Comisiones/Ventas y Egresos/Ingresos (popover con texto explicativo). Regla bitácora: tecnología e infraestructura y actualizar todas las solapas. Despliegue a producción.</v>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>1.26</v>
+      </c>
+      <c r="B28" t="str">
+        <v>01/03/2026</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Mensaje de alerta de desvío: categoría en negrita sin comillas. Despliegue a producción.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C27"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C28"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2272,10 +2300,10 @@
         <v>Diseño y desarrollo del dashboard mensual (Flujo por mes, Resumen, alertas, modal By Categoría / By Cuenta, gráficos de serie mensual). Incluye formatos de moneda y visualizaciones.</v>
       </c>
       <c r="C3">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="D3">
-        <v>5000</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="4">
@@ -2286,10 +2314,10 @@
         <v>Detección de potencial duplicado (fecha, monto, tipo, cliente, descripción similar), tipo de error (inconsistencia / duplicado), filtro por tipo, modal de comparación con id_origen y Cliente, acciones anular o eliminar registro.</v>
       </c>
       <c r="C4">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="D4">
-        <v>1250</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5">
@@ -2300,10 +2328,10 @@
         <v>Solapa Evolución: tabla dinámica con filas por Categoría o Cuenta contable y columnas por Período (Diario o Mensual). Neto por celda en moneda seleccionada.</v>
       </c>
       <c r="C5">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="D5">
-        <v>1000</v>
+        <v>250</v>
       </c>
     </row>
     <row r="6">
@@ -2314,10 +2342,10 @@
         <v>Columna Int. por caución en flujo por mes: cálculo de interés mensual por reinversión del sobrante a un día con tasa de serie de cauciones. Carga de Excel al refrescar, modal de marcha de cálculo (G/P acum, Base, Tasa, Int T). Incluye soporte para múltiples formatos de fecha y columna tasa_diaria.</v>
       </c>
       <c r="C6">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="D6">
-        <v>900</v>
+        <v>250</v>
       </c>
     </row>
     <row r="7">
@@ -2328,10 +2356,10 @@
         <v>Proyección de ingresos, egresos, G/P y ratios para los próximos 3 meses con configuración (mediana/promedio, meses de historia 3/6/12/24), ventana rodante; Int. por caución proyectado en cadena desde último real (G/P+interés); disclaimer de metodología bajo la proyección.</v>
       </c>
       <c r="C7">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="D7">
-        <v>1500</v>
+        <v>250</v>
       </c>
     </row>
     <row r="8">
@@ -2342,10 +2370,10 @@
         <v>Solapa Todas las transacciones con listado completo, filtros por mes y categoría, y modal de edición con todos los campos y combos para valores normalizados (categoría, cuenta contable, tipo movimiento, status, medio pago, moneda, origen archivo).</v>
       </c>
       <c r="C8">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="D8">
-        <v>1100</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9">
@@ -2356,10 +2384,10 @@
         <v>Implementación de la bitácora en Excel (Log, Resumen, Versiones, Ref Git y Vercel, Presupuesto) y documentación funcional básica para el uso de la app.</v>
       </c>
       <c r="C9">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="D9">
-        <v>1750</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10">
@@ -2370,10 +2398,10 @@
         <v>Configuración de repositorio Git/GitHub, flujo de despliegue a Vercel y ajustes de configuración (vercel.json, conexión con Supabase).</v>
       </c>
       <c r="C10">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="D10">
-        <v>1500</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11">
@@ -2384,10 +2412,10 @@
         <v>Soporte post–implementación, pequeños ajustes funcionales y acompañamiento durante el primer período de uso.</v>
       </c>
       <c r="C11">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="D11">
-        <v>1400</v>
+        <v>250</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
v1.27: Novedades del Negocio (Edge Function Gemini), bitácora y presentación
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -8,6 +8,7 @@
     <sheet name="Ref Git y Vercel" sheetId="3" r:id="rId3"/>
     <sheet name="Versiones" sheetId="4" r:id="rId4"/>
     <sheet name="Presupuesto" sheetId="5" r:id="rId5"/>
+    <sheet name="Tecnología" sheetId="6" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
@@ -401,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E59"/>
+  <dimension ref="A1:E60"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -1381,10 +1382,10 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>01/03/2026</v>
+        <v>02/03/2026</v>
       </c>
       <c r="B58" t="str">
-        <v>23:45</v>
+        <v>10:17</v>
       </c>
       <c r="C58" t="str">
         <v>Ayuda al clic en columnas flujo y regla bitácora</v>
@@ -1398,10 +1399,10 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>01/03/2026</v>
+        <v>02/03/2026</v>
       </c>
       <c r="B59" t="str">
-        <v>23:45</v>
+        <v>10:17</v>
       </c>
       <c r="C59" t="str">
         <v>Alerta desvío: categoría en negrita sin comillas</v>
@@ -1413,16 +1414,33 @@
         <v>Implementacion</v>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>02/03/2026</v>
+      </c>
+      <c r="B60" t="str">
+        <v>10:17</v>
+      </c>
+      <c r="C60" t="str">
+        <v>Novedades del Negocio y despliegue v1.27</v>
+      </c>
+      <c r="D60" t="str">
+        <v>Sección Novedades del Negocio en sidebar: Edge Function get-novedades-negocio (Gemini + google_search) para importadores y comercios de hornos en Argentina. Config GEMINI_API_KEY en Supabase. Despliegue a producción.</v>
+      </c>
+      <c r="E60" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E59"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E60"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B51"/>
+  <dimension ref="A1:B52"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -1836,9 +1854,17 @@
         <v>En Configuración, combo Recorte % (cada lado) (0, 5, 10, 15, 20, 25) visible solo cuando el método es Promedio recortado. Más % = más suavizado. Persistido en config_dashboard (proyeccion_recorte).</v>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>Novedades del Negocio</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Ítem en sidebar que abre una vista con importadores de hornos y comercios de venta de hornos en Argentina (Buenos Aires). Datos recuperados por IA (Edge Function con Gemini + google_search). Nombre, dirección, teléfono y web por contacto.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B51"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B52"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1932,7 +1958,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C29"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -2230,7 +2256,7 @@
         <v>1.25</v>
       </c>
       <c r="B27" t="str">
-        <v>01/03/2026</v>
+        <v>02/03/2026</v>
       </c>
       <c r="C27" t="str">
         <v>Ayuda al clic en columnas Comisiones/Ventas y Egresos/Ingresos (popover con texto explicativo). Regla bitácora: tecnología e infraestructura y actualizar todas las solapas. Despliegue a producción.</v>
@@ -2241,15 +2267,26 @@
         <v>1.26</v>
       </c>
       <c r="B28" t="str">
-        <v>01/03/2026</v>
+        <v>02/03/2026</v>
       </c>
       <c r="C28" t="str">
         <v>Mensaje de alerta de desvío: categoría en negrita sin comillas. Despliegue a producción.</v>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>1.27</v>
+      </c>
+      <c r="B29" t="str">
+        <v>02/03/2026</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Novedades del Negocio: sección en sidebar con importadores y comercios de hornos en Argentina (Edge Function Gemini + google_search). Despliegue a producción.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C28"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C29"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2275,7 +2312,7 @@
         <v>Horas hombre</v>
       </c>
       <c r="D1" t="str">
-        <v>Importe sugerido (USD)</v>
+        <v>Importe (USD)</v>
       </c>
     </row>
     <row r="2">
@@ -2289,7 +2326,7 @@
         <v>2</v>
       </c>
       <c r="D2">
-        <v>100</v>
+        <v>200</v>
       </c>
     </row>
     <row r="3">
@@ -2303,7 +2340,7 @@
         <v>25</v>
       </c>
       <c r="D3">
-        <v>1250</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="4">
@@ -2317,7 +2354,7 @@
         <v>2</v>
       </c>
       <c r="D4">
-        <v>100</v>
+        <v>200</v>
       </c>
     </row>
     <row r="5">
@@ -2331,7 +2368,7 @@
         <v>5</v>
       </c>
       <c r="D5">
-        <v>250</v>
+        <v>500</v>
       </c>
     </row>
     <row r="6">
@@ -2345,7 +2382,7 @@
         <v>5</v>
       </c>
       <c r="D6">
-        <v>250</v>
+        <v>500</v>
       </c>
     </row>
     <row r="7">
@@ -2359,7 +2396,7 @@
         <v>5</v>
       </c>
       <c r="D7">
-        <v>250</v>
+        <v>500</v>
       </c>
     </row>
     <row r="8">
@@ -2373,7 +2410,7 @@
         <v>2</v>
       </c>
       <c r="D8">
-        <v>100</v>
+        <v>200</v>
       </c>
     </row>
     <row r="9">
@@ -2387,7 +2424,7 @@
         <v>2</v>
       </c>
       <c r="D9">
-        <v>100</v>
+        <v>200</v>
       </c>
     </row>
     <row r="10">
@@ -2401,7 +2438,7 @@
         <v>2</v>
       </c>
       <c r="D10">
-        <v>100</v>
+        <v>200</v>
       </c>
     </row>
     <row r="11">
@@ -2415,7 +2452,7 @@
         <v>5</v>
       </c>
       <c r="D11">
-        <v>250</v>
+        <v>500</v>
       </c>
     </row>
   </sheetData>
@@ -2423,4 +2460,67 @@
     <ignoredError numberStoredAsText="1" sqref="A1:D11"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B6"/>
+  <cols>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="95.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Componente</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Detalle</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Frontend</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Una sola página dashboard-flujo-caja.html (HTML, CSS, JavaScript en el mismo archivo). Sin framework; llamadas a Supabase desde el cliente.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Datos</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Supabase (PostgreSQL). Tablas: transacciones, tipo_de_cambio, config_dashboard. Scripts SQL (supabase_*.sql) se ejecutan en Supabase SQL Editor.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Hosting</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Vercel. App en producción: fornitalia.vercel.app. Despliegue con vercel --prod tras push a main.</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Repositorio</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Git/GitHub, rama main.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Bitácora</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Node.js + SheetJS (xlsx). Script crear-bitacora-excel.js genera Bitacora_tareas.xlsx con las solapas Log, Resumen, Ref Git y Vercel, Versiones, Presupuesto, Tecnología.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B6"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
v1.28: favicon L&P centrado en círculo
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E60"/>
+  <dimension ref="A1:E61"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -1385,7 +1385,7 @@
         <v>02/03/2026</v>
       </c>
       <c r="B58" t="str">
-        <v>10:17</v>
+        <v>11:42</v>
       </c>
       <c r="C58" t="str">
         <v>Ayuda al clic en columnas flujo y regla bitácora</v>
@@ -1402,7 +1402,7 @@
         <v>02/03/2026</v>
       </c>
       <c r="B59" t="str">
-        <v>10:17</v>
+        <v>11:42</v>
       </c>
       <c r="C59" t="str">
         <v>Alerta desvío: categoría en negrita sin comillas</v>
@@ -1419,7 +1419,7 @@
         <v>02/03/2026</v>
       </c>
       <c r="B60" t="str">
-        <v>10:17</v>
+        <v>11:42</v>
       </c>
       <c r="C60" t="str">
         <v>Novedades del Negocio y despliegue v1.27</v>
@@ -1431,9 +1431,26 @@
         <v>Implementacion</v>
       </c>
     </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>02/03/2026</v>
+      </c>
+      <c r="B61" t="str">
+        <v>11:42</v>
+      </c>
+      <c r="C61" t="str">
+        <v>Favicon L&amp;P centrado</v>
+      </c>
+      <c r="D61" t="str">
+        <v>Ajuste del favicon: letras L y P (P reflejada) centradas en el círculo azul; posición y separación para que ambas se vean bien en pestaña y logo.</v>
+      </c>
+      <c r="E61" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E60"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E61"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1958,7 +1975,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C30"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -2284,9 +2301,20 @@
         <v>Novedades del Negocio: sección en sidebar con importadores y comercios de hornos en Argentina (Edge Function Gemini + google_search). Despliegue a producción.</v>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>1.28</v>
+      </c>
+      <c r="B30" t="str">
+        <v>02/03/2026</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Favicon L&amp;P: L y P dada vuelta centradas en el círculo azul; ajuste de posición y centrado. Despliegue a producción.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C29"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C30"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.29: errores id_origen/id_operacion, exclusiones duplicados, repoblar desde Excel
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:E62"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -1382,10 +1382,10 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>02/03/2026</v>
+        <v>03/03/2026</v>
       </c>
       <c r="B58" t="str">
-        <v>11:42</v>
+        <v>08:50</v>
       </c>
       <c r="C58" t="str">
         <v>Ayuda al clic en columnas flujo y regla bitácora</v>
@@ -1399,10 +1399,10 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>02/03/2026</v>
+        <v>03/03/2026</v>
       </c>
       <c r="B59" t="str">
-        <v>11:42</v>
+        <v>08:50</v>
       </c>
       <c r="C59" t="str">
         <v>Alerta desvío: categoría en negrita sin comillas</v>
@@ -1416,10 +1416,10 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>02/03/2026</v>
+        <v>03/03/2026</v>
       </c>
       <c r="B60" t="str">
-        <v>11:42</v>
+        <v>08:50</v>
       </c>
       <c r="C60" t="str">
         <v>Novedades del Negocio y despliegue v1.27</v>
@@ -1433,10 +1433,10 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>02/03/2026</v>
+        <v>03/03/2026</v>
       </c>
       <c r="B61" t="str">
-        <v>11:42</v>
+        <v>08:50</v>
       </c>
       <c r="C61" t="str">
         <v>Favicon L&amp;P centrado</v>
@@ -1448,9 +1448,26 @@
         <v>Implementacion</v>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="B62" t="str">
+        <v>08:50</v>
+      </c>
+      <c r="C62" t="str">
+        <v>Despliegue v1.29</v>
+      </c>
+      <c r="D62" t="str">
+        <v>Errores: id_origen/id_operacion en export y listado; modal duplicado con icono en campos distintos. Exclusiones duplicados (anulados, id_origen e id_operacion ambos distintos, montos 0). Sin disclaimer ficticios; repoblar desde Excel.</v>
+      </c>
+      <c r="E62" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E61"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E62"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1975,7 +1992,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C31"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -2273,7 +2290,7 @@
         <v>1.25</v>
       </c>
       <c r="B27" t="str">
-        <v>02/03/2026</v>
+        <v>03/03/2026</v>
       </c>
       <c r="C27" t="str">
         <v>Ayuda al clic en columnas Comisiones/Ventas y Egresos/Ingresos (popover con texto explicativo). Regla bitácora: tecnología e infraestructura y actualizar todas las solapas. Despliegue a producción.</v>
@@ -2284,7 +2301,7 @@
         <v>1.26</v>
       </c>
       <c r="B28" t="str">
-        <v>02/03/2026</v>
+        <v>03/03/2026</v>
       </c>
       <c r="C28" t="str">
         <v>Mensaje de alerta de desvío: categoría en negrita sin comillas. Despliegue a producción.</v>
@@ -2295,7 +2312,7 @@
         <v>1.27</v>
       </c>
       <c r="B29" t="str">
-        <v>02/03/2026</v>
+        <v>03/03/2026</v>
       </c>
       <c r="C29" t="str">
         <v>Novedades del Negocio: sección en sidebar con importadores y comercios de hornos en Argentina (Edge Function Gemini + google_search). Despliegue a producción.</v>
@@ -2306,15 +2323,26 @@
         <v>1.28</v>
       </c>
       <c r="B30" t="str">
-        <v>02/03/2026</v>
+        <v>03/03/2026</v>
       </c>
       <c r="C30" t="str">
         <v>Favicon L&amp;P: L y P dada vuelta centradas en el círculo azul; ajuste de posición y centrado. Despliegue a producción.</v>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>1.29</v>
+      </c>
+      <c r="B31" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Errores: export y listado con id_origen e id_operacion; modal duplicado con id_operacion e icono en campos que no coinciden. Exclusiones duplicados: anulados, id_origen e id_operacion ambos distintos, ambos montos 0. Quitar disclaimer datos ficticios; scripts e instrucciones para repoblar transacciones desde Excel. Despliegue a producción.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C30"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C31"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.30: errores orden y filtros categoría; flujo Anulado; export Tipo_Cambio Monto_ARS Monto_USD
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E62"/>
+  <dimension ref="A1:E63"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -1385,7 +1385,7 @@
         <v>03/03/2026</v>
       </c>
       <c r="B58" t="str">
-        <v>08:50</v>
+        <v>18:06</v>
       </c>
       <c r="C58" t="str">
         <v>Ayuda al clic en columnas flujo y regla bitácora</v>
@@ -1402,7 +1402,7 @@
         <v>03/03/2026</v>
       </c>
       <c r="B59" t="str">
-        <v>08:50</v>
+        <v>18:06</v>
       </c>
       <c r="C59" t="str">
         <v>Alerta desvío: categoría en negrita sin comillas</v>
@@ -1419,7 +1419,7 @@
         <v>03/03/2026</v>
       </c>
       <c r="B60" t="str">
-        <v>08:50</v>
+        <v>18:06</v>
       </c>
       <c r="C60" t="str">
         <v>Novedades del Negocio y despliegue v1.27</v>
@@ -1436,7 +1436,7 @@
         <v>03/03/2026</v>
       </c>
       <c r="B61" t="str">
-        <v>08:50</v>
+        <v>18:06</v>
       </c>
       <c r="C61" t="str">
         <v>Favicon L&amp;P centrado</v>
@@ -1453,7 +1453,7 @@
         <v>03/03/2026</v>
       </c>
       <c r="B62" t="str">
-        <v>08:50</v>
+        <v>18:06</v>
       </c>
       <c r="C62" t="str">
         <v>Despliegue v1.29</v>
@@ -1465,9 +1465,26 @@
         <v>Implementacion</v>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="B63" t="str">
+        <v>18:06</v>
+      </c>
+      <c r="C63" t="str">
+        <v>Despliegue v1.30</v>
+      </c>
+      <c r="D63" t="str">
+        <v>Errores: orden tipo y monto; filtros categoría orig. y mostrada. Flujo filtro Anulado. Export Base con Tipo_Cambio, Monto_ARS, Monto_USD.</v>
+      </c>
+      <c r="E63" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E62"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E63"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1992,7 +2009,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C32"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -2340,9 +2357,20 @@
         <v>Errores: export y listado con id_origen e id_operacion; modal duplicado con id_operacion e icono en campos que no coinciden. Exclusiones duplicados: anulados, id_origen e id_operacion ambos distintos, ambos montos 0. Quitar disclaimer datos ficticios; scripts e instrucciones para repoblar transacciones desde Excel. Despliegue a producción.</v>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>1.30</v>
+      </c>
+      <c r="B32" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Errores: orden por tipo y monto descendente; filtros por categoría original y categoría mostrada. Flujo: filtro explícito status Anulado. Export Base Histórica: columnas Tipo_Cambio, Monto_ARS, Monto_USD con conversiones. Despliegue a producción.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C31"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C32"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.31: estructura ordenada (sql/, scripts/, docs/), regla estructura-proyecto y flujo desplegar
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E63"/>
+  <dimension ref="A1:E64"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -1382,10 +1382,10 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>03/03/2026</v>
+        <v>05/03/2026</v>
       </c>
       <c r="B58" t="str">
-        <v>18:06</v>
+        <v>10:43</v>
       </c>
       <c r="C58" t="str">
         <v>Ayuda al clic en columnas flujo y regla bitácora</v>
@@ -1399,10 +1399,10 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>03/03/2026</v>
+        <v>05/03/2026</v>
       </c>
       <c r="B59" t="str">
-        <v>18:06</v>
+        <v>10:43</v>
       </c>
       <c r="C59" t="str">
         <v>Alerta desvío: categoría en negrita sin comillas</v>
@@ -1416,10 +1416,10 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>03/03/2026</v>
+        <v>05/03/2026</v>
       </c>
       <c r="B60" t="str">
-        <v>18:06</v>
+        <v>10:43</v>
       </c>
       <c r="C60" t="str">
         <v>Novedades del Negocio y despliegue v1.27</v>
@@ -1433,10 +1433,10 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>03/03/2026</v>
+        <v>05/03/2026</v>
       </c>
       <c r="B61" t="str">
-        <v>18:06</v>
+        <v>10:43</v>
       </c>
       <c r="C61" t="str">
         <v>Favicon L&amp;P centrado</v>
@@ -1450,10 +1450,10 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>03/03/2026</v>
+        <v>05/03/2026</v>
       </c>
       <c r="B62" t="str">
-        <v>18:06</v>
+        <v>10:43</v>
       </c>
       <c r="C62" t="str">
         <v>Despliegue v1.29</v>
@@ -1467,10 +1467,10 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>03/03/2026</v>
+        <v>05/03/2026</v>
       </c>
       <c r="B63" t="str">
-        <v>18:06</v>
+        <v>10:43</v>
       </c>
       <c r="C63" t="str">
         <v>Despliegue v1.30</v>
@@ -1482,9 +1482,26 @@
         <v>Implementacion</v>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>05/03/2026</v>
+      </c>
+      <c r="B64" t="str">
+        <v>10:43</v>
+      </c>
+      <c r="C64" t="str">
+        <v>Despliegue v1.31</v>
+      </c>
+      <c r="D64" t="str">
+        <v>Estructura ordenada: sql/, scripts/, docs/. Regla estructura-proyecto. Bitácora y docs con rutas actualizadas.</v>
+      </c>
+      <c r="E64" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E63"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E64"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2009,7 +2026,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C33"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -2307,7 +2324,7 @@
         <v>1.25</v>
       </c>
       <c r="B27" t="str">
-        <v>03/03/2026</v>
+        <v>05/03/2026</v>
       </c>
       <c r="C27" t="str">
         <v>Ayuda al clic en columnas Comisiones/Ventas y Egresos/Ingresos (popover con texto explicativo). Regla bitácora: tecnología e infraestructura y actualizar todas las solapas. Despliegue a producción.</v>
@@ -2318,7 +2335,7 @@
         <v>1.26</v>
       </c>
       <c r="B28" t="str">
-        <v>03/03/2026</v>
+        <v>05/03/2026</v>
       </c>
       <c r="C28" t="str">
         <v>Mensaje de alerta de desvío: categoría en negrita sin comillas. Despliegue a producción.</v>
@@ -2329,7 +2346,7 @@
         <v>1.27</v>
       </c>
       <c r="B29" t="str">
-        <v>03/03/2026</v>
+        <v>05/03/2026</v>
       </c>
       <c r="C29" t="str">
         <v>Novedades del Negocio: sección en sidebar con importadores y comercios de hornos en Argentina (Edge Function Gemini + google_search). Despliegue a producción.</v>
@@ -2340,7 +2357,7 @@
         <v>1.28</v>
       </c>
       <c r="B30" t="str">
-        <v>03/03/2026</v>
+        <v>05/03/2026</v>
       </c>
       <c r="C30" t="str">
         <v>Favicon L&amp;P: L y P dada vuelta centradas en el círculo azul; ajuste de posición y centrado. Despliegue a producción.</v>
@@ -2351,7 +2368,7 @@
         <v>1.29</v>
       </c>
       <c r="B31" t="str">
-        <v>03/03/2026</v>
+        <v>05/03/2026</v>
       </c>
       <c r="C31" t="str">
         <v>Errores: export y listado con id_origen e id_operacion; modal duplicado con id_operacion e icono en campos que no coinciden. Exclusiones duplicados: anulados, id_origen e id_operacion ambos distintos, ambos montos 0. Quitar disclaimer datos ficticios; scripts e instrucciones para repoblar transacciones desde Excel. Despliegue a producción.</v>
@@ -2362,15 +2379,26 @@
         <v>1.30</v>
       </c>
       <c r="B32" t="str">
-        <v>03/03/2026</v>
+        <v>05/03/2026</v>
       </c>
       <c r="C32" t="str">
         <v>Errores: orden por tipo y monto descendente; filtros por categoría original y categoría mostrada. Flujo: filtro explícito status Anulado. Export Base Histórica: columnas Tipo_Cambio, Monto_ARS, Monto_USD con conversiones. Despliegue a producción.</v>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>1.31</v>
+      </c>
+      <c r="B33" t="str">
+        <v>05/03/2026</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Estructura ordenada del repo: sql/, scripts/, docs/. Regla estructura-proyecto (mantener carpetas y rutas). Referencias en bitácora y docs actualizadas. Despliegue a producción.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C32"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C33"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2575,7 +2603,7 @@
         <v>Datos</v>
       </c>
       <c r="B3" t="str">
-        <v>Supabase (PostgreSQL). Tablas: transacciones, tipo_de_cambio, config_dashboard. Scripts SQL (supabase_*.sql) se ejecutan en Supabase SQL Editor.</v>
+        <v>Supabase (PostgreSQL). Tablas: transacciones, tipo_de_cambio, config_dashboard. Scripts SQL en carpeta sql/ se ejecutan en Supabase SQL Editor.</v>
       </c>
     </row>
     <row r="4">
@@ -2599,7 +2627,7 @@
         <v>Bitácora</v>
       </c>
       <c r="B6" t="str">
-        <v>Node.js + SheetJS (xlsx). Script crear-bitacora-excel.js genera Bitacora_tareas.xlsx con las solapas Log, Resumen, Ref Git y Vercel, Versiones, Presupuesto, Tecnología.</v>
+        <v>Node.js + SheetJS (xlsx). Script scripts/crear-bitacora-excel.js genera Bitacora_tareas.xlsx con las solapas Log, Resumen, Ref Git y Vercel, Versiones, Presupuesto, Tecnología.</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
v1.33: paginación Supabase, reglas moneda MP/Morba, upload normalizado, informe PDF y Playwright
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E65"/>
+  <dimension ref="A1:E77"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -1382,10 +1382,10 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>16/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B58" t="str">
-        <v>18:12</v>
+        <v>19:06</v>
       </c>
       <c r="C58" t="str">
         <v>Ayuda al clic en columnas flujo y regla bitácora</v>
@@ -1399,10 +1399,10 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>16/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B59" t="str">
-        <v>18:12</v>
+        <v>19:06</v>
       </c>
       <c r="C59" t="str">
         <v>Alerta desvío: categoría en negrita sin comillas</v>
@@ -1416,10 +1416,10 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>16/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B60" t="str">
-        <v>18:12</v>
+        <v>19:06</v>
       </c>
       <c r="C60" t="str">
         <v>Novedades del Negocio y despliegue v1.27</v>
@@ -1433,10 +1433,10 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>16/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B61" t="str">
-        <v>18:12</v>
+        <v>19:06</v>
       </c>
       <c r="C61" t="str">
         <v>Favicon L&amp;P centrado</v>
@@ -1450,10 +1450,10 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>16/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B62" t="str">
-        <v>18:12</v>
+        <v>19:06</v>
       </c>
       <c r="C62" t="str">
         <v>Despliegue v1.29</v>
@@ -1467,10 +1467,10 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>16/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B63" t="str">
-        <v>18:12</v>
+        <v>19:06</v>
       </c>
       <c r="C63" t="str">
         <v>Despliegue v1.30</v>
@@ -1484,10 +1484,10 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>16/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B64" t="str">
-        <v>18:12</v>
+        <v>19:06</v>
       </c>
       <c r="C64" t="str">
         <v>Despliegue v1.31</v>
@@ -1501,10 +1501,10 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>16/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B65" t="str">
-        <v>18:12</v>
+        <v>19:06</v>
       </c>
       <c r="C65" t="str">
         <v>Despliegue v1.32</v>
@@ -1516,16 +1516,220 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B66" t="str">
+        <v>19:06</v>
+      </c>
+      <c r="C66" t="str">
+        <v>Normalización de Extracto Fornitalia</v>
+      </c>
+      <c r="D66" t="str">
+        <v>Nuevo script scripts/normalizar-extracto-fornitalia.js que toma docs/Extracto-Fornitalia.xlsx y genera docs/Extracto-Fornitalia-Normalizado.xlsx con hoja Normalizado: parseo numérico de montos, fecha ISO, inferencia de moneda (USD/ARS) y monto_ars derivado para facilitar reemplazo de tablas y análisis.</v>
+      </c>
+      <c r="E66" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B67" t="str">
+        <v>19:06</v>
+      </c>
+      <c r="C67" t="str">
+        <v>Upload controlado de extracto normalizado en app</v>
+      </c>
+      <c r="D67" t="str">
+        <v>En dashboard-flujo-caja.html se agrega modal de carga controlada del Excel normalizado: validación de hoja/campos/tipos, confirmación explícita REEMPLAZAR, generación de id_origen técnico por fila (timestamp+índice con hash de trazabilidad), borrado por lotes e inserción por lotes sobre transacciones. Se agrega SQL de soporte sql/supabase_upload_normalizado_controlado.sql.</v>
+      </c>
+      <c r="E67" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B68" t="str">
+        <v>19:06</v>
+      </c>
+      <c r="C68" t="str">
+        <v>Upload normalizado sin confirmación manual y log de excluidos</v>
+      </c>
+      <c r="D68" t="str">
+        <v>Ajuste del modal de carga: se elimina requisito de escribir REEMPLAZAR, los errores quedan informativos y se cargan solo filas válidas. Nueva solapa Excluidos upload y tabla Supabase transacciones_upload_excluidos para auditar filas excluidas (validación y Apertura/Cierre de Caja).</v>
+      </c>
+      <c r="E68" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B69" t="str">
+        <v>19:06</v>
+      </c>
+      <c r="C69" t="str">
+        <v>Ajuste final upload: no loguear Apertura/Cierre y réplica en Everfit</v>
+      </c>
+      <c r="D69" t="str">
+        <v>Se ajusta Fornitalia para excluir Apertura/Cierre de Caja sin registrarlos en log de excluidos. En Everfit se replica el flujo optimizado de carga (progreso visual y vaciado rápido de tabla) para comportamiento equivalente y mayor velocidad percibida.</v>
+      </c>
+      <c r="E69" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B70" t="str">
+        <v>19:06</v>
+      </c>
+      <c r="C70" t="str">
+        <v>Limpieza de log excluidos y normalización de mes/año en carga</v>
+      </c>
+      <c r="D70" t="str">
+        <v>Antes de guardar excluidos de un nuevo upload se limpia transacciones_upload_excluidos para evitar arrastre histórico. En cargarDatos se normalizan mes/anio (con fallback desde fecha) para asegurar que Flujo por mes refleje todos los meses del archivo cargado.</v>
+      </c>
+      <c r="E70" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B71" t="str">
+        <v>19:06</v>
+      </c>
+      <c r="C71" t="str">
+        <v>Excluidos upload: mostrar solo última corrida y habilitar DELETE</v>
+      </c>
+      <c r="D71" t="str">
+        <v>La solapa Excluidos upload ahora filtra por run_ref más reciente para no mezclar corridas históricas. SQL de soporte actualizado con política DELETE en transacciones_upload_excluidos para permitir limpieza previa por corrida desde la app.</v>
+      </c>
+      <c r="E71" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B72" t="str">
+        <v>19:06</v>
+      </c>
+      <c r="C72" t="str">
+        <v>Carga paginada desde Supabase (transacciones y tipo de cambio)</v>
+      </c>
+      <c r="D72" t="str">
+        <v>PostgREST limita por defecto ~1000 filas por consulta; cargarDatos ahora pide transacciones (no anuladas) y tipo_de_cambio en páginas de 1000 con .range hasta agotar, para que Flujo por mes y totales reflejen toda la base.</v>
+      </c>
+      <c r="E72" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B73" t="str">
+        <v>19:06</v>
+      </c>
+      <c r="C73" t="str">
+        <v>Reglas moneda: Mercado Pago y Transferencia Morba siempre ARS</v>
+      </c>
+      <c r="D73" t="str">
+        <v>En extracto el medio es Transferencia Morba (con b); todo eso y Mercado Pago va como ARS en normalizar-extracto, upload y esTransaccionUSD. Se mantiene detección de morva por posible typo.</v>
+      </c>
+      <c r="E73" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B74" t="str">
+        <v>19:06</v>
+      </c>
+      <c r="C74" t="str">
+        <v>Documento análisis normalización datos legacy</v>
+      </c>
+      <c r="D74" t="str">
+        <v>Nuevo docs/ANALISIS_NORMALIZACION_DATOS_LEGACY_FORNITALIA.md: inconsistencias (categorías ambiguas, cuenta contable, pares categoría-cuenta, medios de pago, campos vacíos/guion) y recomendaciones para el cliente sobre qué corregir en su base de origen.</v>
+      </c>
+      <c r="E74" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B75" t="str">
+        <v>19:06</v>
+      </c>
+      <c r="C75" t="str">
+        <v>Informe normalización: cantidades por fila y PDF/HTML</v>
+      </c>
+      <c r="D75" t="str">
+        <v>Tablas del análisis con columna Cant. (extracto Movimientos, N=3008). Salidas docs/ANALISIS_*.html y .pdf; scripts md-informe-a-html.js e informe-html-a-pdf.js; npm run informe-normalizacion-pdf con Playwright (devDependency como en Pandi).</v>
+      </c>
+      <c r="E75" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B76" t="str">
+        <v>19:06</v>
+      </c>
+      <c r="C76" t="str">
+        <v>Playwright en todos los repos LyP</v>
+      </c>
+      <c r="D76" t="str">
+        <v>Everfit, Fornitalia, MiGusto, Pandi y Sistema-Contable: devDependency playwright ^1.49.0 y script npm run playwright:install (chromium). Raíz LyP: README-Playwright.md.</v>
+      </c>
+      <c r="E76" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B77" t="str">
+        <v>19:06</v>
+      </c>
+      <c r="C77" t="str">
+        <v>Despliegue v1.33 producción</v>
+      </c>
+      <c r="D77" t="str">
+        <v>Push a main y vercel --prod: paginación Supabase, reglas moneda MP/Morba, informe normalización y herramientas PDF; package.json playwright.</v>
+      </c>
+      <c r="E77" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E65"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E77"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B52"/>
+  <dimension ref="A1:B56"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -1696,7 +1900,7 @@
         <v>Datos</v>
       </c>
       <c r="B21" t="str">
-        <v>Transacciones y tipo de cambio desde Supabase. Cotización faltante: se usa la fecha anterior disponible.</v>
+        <v>Transacciones y tipo de cambio desde Supabase (carga paginada de a 1000 filas por request para no truncar resultados). Cotización faltante: se usa la fecha anterior disponible.</v>
       </c>
     </row>
     <row r="22">
@@ -1752,7 +1956,7 @@
         <v>Campo moneda (BD)</v>
       </c>
       <c r="B28" t="str">
-        <v>Columna moneda en tabla transacciones (ARS/USD). Si está informada, el dashboard la usa; si no, infiere desde medio_pago (ej. "dolar" → USD). Export a Excel incluye moneda.</v>
+        <v>Columna moneda en tabla transacciones (ARS/USD). Si está informada, el dashboard la usa salvo reglas de negocio: Mercado Pago y Transferencia Morba siempre ARS para conversión (también morva por typo). Si moneda vacía, infiere desde textos/medio (dólar → USD). Export a Excel incluye moneda.</v>
       </c>
     </row>
     <row r="29">
@@ -1947,9 +2151,41 @@
         <v>Ítem en sidebar que abre una vista con importadores de hornos y comercios de venta de hornos en Argentina (Buenos Aires). Datos recuperados por IA (Edge Function con Gemini + google_search). Nombre, dirección, teléfono y web por contacto.</v>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>Normalización de extracto bancario</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Script utilitario que normaliza el extracto Excel en una hoja estructurada (Normalizado) con campos listos para tablas: fecha_iso, tipo, medio, categoría, cuenta, moneda inferida (USD/ARS; Mercado Pago y Transferencia Morba forzados a ARS), monto_original numérico, tipo_cambio y monto_ars.</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>Informe inconsistencias datos legacy (cliente)</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Documento docs/ANALISIS_NORMALIZACION_DATOS_LEGACY_FORNITALIA.md con tablas Cant./recomendaciones; .html y .pdf en docs/. Regenerar: npm run informe-normalizacion-html o npm run informe-normalizacion-pdf (Playwright+Chromium, alineado a stack Pandi); primera vez: npx playwright install chromium.</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>Upload de extracto normalizado</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Botón en la app para reemplazar transacciones desde un Excel normalizado (hoja Normalizado), con validación previa, confirmación de seguridad, generación de id_origen técnico y carga en lotes.</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>Log de excluidos en upload</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Nueva solapa Excluidos upload con registros no insertados por error o por regla de negocio (Apertura/Cierre de Caja), persistidos en Supabase para auditoría.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B52"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B56"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2043,7 +2279,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C35"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -2341,7 +2577,7 @@
         <v>1.25</v>
       </c>
       <c r="B27" t="str">
-        <v>16/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C27" t="str">
         <v>Ayuda al clic en columnas Comisiones/Ventas y Egresos/Ingresos (popover con texto explicativo). Regla bitácora: tecnología e infraestructura y actualizar todas las solapas. Despliegue a producción.</v>
@@ -2352,7 +2588,7 @@
         <v>1.26</v>
       </c>
       <c r="B28" t="str">
-        <v>16/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C28" t="str">
         <v>Mensaje de alerta de desvío: categoría en negrita sin comillas. Despliegue a producción.</v>
@@ -2363,7 +2599,7 @@
         <v>1.27</v>
       </c>
       <c r="B29" t="str">
-        <v>16/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C29" t="str">
         <v>Novedades del Negocio: sección en sidebar con importadores y comercios de hornos en Argentina (Edge Function Gemini + google_search). Despliegue a producción.</v>
@@ -2374,7 +2610,7 @@
         <v>1.28</v>
       </c>
       <c r="B30" t="str">
-        <v>16/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C30" t="str">
         <v>Favicon L&amp;P: L y P dada vuelta centradas en el círculo azul; ajuste de posición y centrado. Despliegue a producción.</v>
@@ -2385,7 +2621,7 @@
         <v>1.29</v>
       </c>
       <c r="B31" t="str">
-        <v>16/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C31" t="str">
         <v>Errores: export y listado con id_origen e id_operacion; modal duplicado con id_operacion e icono en campos que no coinciden. Exclusiones duplicados: anulados, id_origen e id_operacion ambos distintos, ambos montos 0. Quitar disclaimer datos ficticios; scripts e instrucciones para repoblar transacciones desde Excel. Despliegue a producción.</v>
@@ -2396,7 +2632,7 @@
         <v>1.30</v>
       </c>
       <c r="B32" t="str">
-        <v>16/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C32" t="str">
         <v>Errores: orden por tipo y monto descendente; filtros por categoría original y categoría mostrada. Flujo: filtro explícito status Anulado. Export Base Histórica: columnas Tipo_Cambio, Monto_ARS, Monto_USD con conversiones. Despliegue a producción.</v>
@@ -2407,7 +2643,7 @@
         <v>1.31</v>
       </c>
       <c r="B33" t="str">
-        <v>16/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C33" t="str">
         <v>Estructura ordenada del repo: sql/, scripts/, docs/. Regla estructura-proyecto (mantener carpetas y rutas). Referencias en bitácora y docs actualizadas. Despliegue a producción.</v>
@@ -2418,15 +2654,26 @@
         <v>1.32</v>
       </c>
       <c r="B34" t="str">
-        <v>16/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C34" t="str">
         <v>Modales: no cerrar al elegir opción de select (mousedown+click en backdrop). Helper setupBackdropCloseOnlyOnRealClick en todos los modales.</v>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>1.33</v>
+      </c>
+      <c r="B35" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Carga paginada transacciones y tipo_de_cambio (límite PostgREST). Reglas ARS Mercado Pago y Transferencia Morba en normalizador, upload y esTransaccionUSD. Upload excluidos: filtro última corrida; SQL DELETE en transacciones_upload_excluidos. Informe análisis normalización (docs MD/HTML/PDF) y scripts Playwright. DevDependency playwright y npm run playwright:install.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C34"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C35"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2460,7 +2707,7 @@
         <v>Normalización de datos</v>
       </c>
       <c r="B2" t="str">
-        <v>Relevamiento, limpieza y normalización de datos históricos de caja (campos de moneda, categorías, cuentas contables, flags de edición). Incluye lógica de excepciones y detección de inconsistencias.</v>
+        <v>Relevamiento, limpieza y normalización de datos históricos de caja (campos de moneda, categorías, cuentas contables, flags de edición). Incluye lógica de excepciones, detección de inconsistencias y carga controlada desde extracto normalizado.</v>
       </c>
       <c r="C2">
         <v>2</v>

</xml_diff>

<commit_message>
v1.37: flujo bruto/operativo, conciliación monto_cambio con informe PDF, bitácora
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E77"/>
+  <dimension ref="A1:E89"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -1382,10 +1382,10 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>19/03/2026</v>
+        <v>22/03/2026</v>
       </c>
       <c r="B58" t="str">
-        <v>19:06</v>
+        <v>20:53</v>
       </c>
       <c r="C58" t="str">
         <v>Ayuda al clic en columnas flujo y regla bitácora</v>
@@ -1399,10 +1399,10 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>19/03/2026</v>
+        <v>22/03/2026</v>
       </c>
       <c r="B59" t="str">
-        <v>19:06</v>
+        <v>20:53</v>
       </c>
       <c r="C59" t="str">
         <v>Alerta desvío: categoría en negrita sin comillas</v>
@@ -1416,10 +1416,10 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>19/03/2026</v>
+        <v>22/03/2026</v>
       </c>
       <c r="B60" t="str">
-        <v>19:06</v>
+        <v>20:53</v>
       </c>
       <c r="C60" t="str">
         <v>Novedades del Negocio y despliegue v1.27</v>
@@ -1433,10 +1433,10 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>19/03/2026</v>
+        <v>22/03/2026</v>
       </c>
       <c r="B61" t="str">
-        <v>19:06</v>
+        <v>20:53</v>
       </c>
       <c r="C61" t="str">
         <v>Favicon L&amp;P centrado</v>
@@ -1450,10 +1450,10 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>19/03/2026</v>
+        <v>22/03/2026</v>
       </c>
       <c r="B62" t="str">
-        <v>19:06</v>
+        <v>20:53</v>
       </c>
       <c r="C62" t="str">
         <v>Despliegue v1.29</v>
@@ -1467,10 +1467,10 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>19/03/2026</v>
+        <v>22/03/2026</v>
       </c>
       <c r="B63" t="str">
-        <v>19:06</v>
+        <v>20:53</v>
       </c>
       <c r="C63" t="str">
         <v>Despliegue v1.30</v>
@@ -1484,10 +1484,10 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>19/03/2026</v>
+        <v>22/03/2026</v>
       </c>
       <c r="B64" t="str">
-        <v>19:06</v>
+        <v>20:53</v>
       </c>
       <c r="C64" t="str">
         <v>Despliegue v1.31</v>
@@ -1501,10 +1501,10 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>19/03/2026</v>
+        <v>22/03/2026</v>
       </c>
       <c r="B65" t="str">
-        <v>19:06</v>
+        <v>20:53</v>
       </c>
       <c r="C65" t="str">
         <v>Despliegue v1.32</v>
@@ -1518,10 +1518,10 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>19/03/2026</v>
+        <v>22/03/2026</v>
       </c>
       <c r="B66" t="str">
-        <v>19:06</v>
+        <v>20:53</v>
       </c>
       <c r="C66" t="str">
         <v>Normalización de Extracto Fornitalia</v>
@@ -1535,10 +1535,10 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>19/03/2026</v>
+        <v>22/03/2026</v>
       </c>
       <c r="B67" t="str">
-        <v>19:06</v>
+        <v>20:53</v>
       </c>
       <c r="C67" t="str">
         <v>Upload controlado de extracto normalizado en app</v>
@@ -1552,10 +1552,10 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>19/03/2026</v>
+        <v>22/03/2026</v>
       </c>
       <c r="B68" t="str">
-        <v>19:06</v>
+        <v>20:53</v>
       </c>
       <c r="C68" t="str">
         <v>Upload normalizado sin confirmación manual y log de excluidos</v>
@@ -1569,10 +1569,10 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>19/03/2026</v>
+        <v>22/03/2026</v>
       </c>
       <c r="B69" t="str">
-        <v>19:06</v>
+        <v>20:53</v>
       </c>
       <c r="C69" t="str">
         <v>Ajuste final upload: no loguear Apertura/Cierre y réplica en Everfit</v>
@@ -1586,10 +1586,10 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>19/03/2026</v>
+        <v>22/03/2026</v>
       </c>
       <c r="B70" t="str">
-        <v>19:06</v>
+        <v>20:53</v>
       </c>
       <c r="C70" t="str">
         <v>Limpieza de log excluidos y normalización de mes/año en carga</v>
@@ -1603,10 +1603,10 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>19/03/2026</v>
+        <v>22/03/2026</v>
       </c>
       <c r="B71" t="str">
-        <v>19:06</v>
+        <v>20:53</v>
       </c>
       <c r="C71" t="str">
         <v>Excluidos upload: mostrar solo última corrida y habilitar DELETE</v>
@@ -1620,10 +1620,10 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>19/03/2026</v>
+        <v>22/03/2026</v>
       </c>
       <c r="B72" t="str">
-        <v>19:06</v>
+        <v>20:53</v>
       </c>
       <c r="C72" t="str">
         <v>Carga paginada desde Supabase (transacciones y tipo de cambio)</v>
@@ -1637,10 +1637,10 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>19/03/2026</v>
+        <v>22/03/2026</v>
       </c>
       <c r="B73" t="str">
-        <v>19:06</v>
+        <v>20:53</v>
       </c>
       <c r="C73" t="str">
         <v>Reglas moneda: Mercado Pago y Transferencia Morba siempre ARS</v>
@@ -1654,10 +1654,10 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>19/03/2026</v>
+        <v>22/03/2026</v>
       </c>
       <c r="B74" t="str">
-        <v>19:06</v>
+        <v>20:53</v>
       </c>
       <c r="C74" t="str">
         <v>Documento análisis normalización datos legacy</v>
@@ -1671,10 +1671,10 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>19/03/2026</v>
+        <v>22/03/2026</v>
       </c>
       <c r="B75" t="str">
-        <v>19:06</v>
+        <v>20:53</v>
       </c>
       <c r="C75" t="str">
         <v>Informe normalización: cantidades por fila y PDF/HTML</v>
@@ -1688,10 +1688,10 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>19/03/2026</v>
+        <v>22/03/2026</v>
       </c>
       <c r="B76" t="str">
-        <v>19:06</v>
+        <v>20:53</v>
       </c>
       <c r="C76" t="str">
         <v>Playwright en todos los repos LyP</v>
@@ -1705,10 +1705,10 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>19/03/2026</v>
+        <v>22/03/2026</v>
       </c>
       <c r="B77" t="str">
-        <v>19:06</v>
+        <v>20:53</v>
       </c>
       <c r="C77" t="str">
         <v>Despliegue v1.33 producción</v>
@@ -1720,16 +1720,220 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>22/03/2026</v>
+      </c>
+      <c r="B78" t="str">
+        <v>20:53</v>
+      </c>
+      <c r="C78" t="str">
+        <v>Análisis normalización: propuesta recategorización categoría–cuenta</v>
+      </c>
+      <c r="D78" t="str">
+        <v>Sección 8 en ANALISIS_NORMALIZACION_DATOS_LEGACY_FORNITALIA.md: modelo (catálogo, plan de cuentas, matriz permitida, validación al cargar, histórico) y tabla de beneficios (calidad, reporting, automatización, auditoría, evolución). Regenerar HTML/PDF con npm run informe-normalizacion-pdf si se entregan esos formatos.</v>
+      </c>
+      <c r="E78" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>22/03/2026</v>
+      </c>
+      <c r="B79" t="str">
+        <v>20:53</v>
+      </c>
+      <c r="C79" t="str">
+        <v>Análisis normalización: matriz concreta Ord. n y acción Editar/Nueva/Eliminar</v>
+      </c>
+      <c r="D79" t="str">
+        <v>Sección 8.3: tabla valor actual vs propuesto (categoría y cuenta contable), columna Acción (Editar, Nueva, Eliminar) y Ord. n para priorizar; filas ejemplo alineadas a §1–§3.</v>
+      </c>
+      <c r="E79" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>22/03/2026</v>
+      </c>
+      <c r="B80" t="str">
+        <v>20:53</v>
+      </c>
+      <c r="C80" t="str">
+        <v>Rubros IGJ/FACPCE y balance: doc de referencia</v>
+      </c>
+      <c r="D80" t="str">
+        <v>Nuevo docs/RUBROS_CONTABILIDAD_ARGENTINA_REFERENCIA.md: marco local (RT/IGJ), ejemplo importación mercaderías/hornos, asientos tránsito/CMV/IVA/ajuste inflación; §8.4 en ANALISIS enlaza rubro patrimonial con matriz y proyección de balance.</v>
+      </c>
+      <c r="E80" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>22/03/2026</v>
+      </c>
+      <c r="B81" t="str">
+        <v>20:53</v>
+      </c>
+      <c r="C81" t="str">
+        <v>Matriz borrador categoría–cuenta–rubro (Argentina)</v>
+      </c>
+      <c r="D81" t="str">
+        <v>docs/MATRIZ_CATEGORIA_CUENTA_RUBRO_BORRADOR.md: tabla sugerida BC/ER/TES con rubros tipo presentación IGJ; celdas a definir donde falta criterio contable; enlaces desde ANALISIS §8.4 y RUBROS_CONTABILIDAD.</v>
+      </c>
+      <c r="E81" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>22/03/2026</v>
+      </c>
+      <c r="B82" t="str">
+        <v>20:53</v>
+      </c>
+      <c r="C82" t="str">
+        <v>Análisis: §8.4 borrador rubro dentro del MD principal</v>
+      </c>
+      <c r="D82" t="str">
+        <v>Tabla categoría/cuenta/rubro incorporada en ANALISIS_NORMALIZACION tras §8.3; ex §8.4 pasa a §8.5; MATRIZ_CATEGORIA_CUENTA_RUBRO_BORRADOR.md como espejo alineado.</v>
+      </c>
+      <c r="E82" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>22/03/2026</v>
+      </c>
+      <c r="B83" t="str">
+        <v>20:53</v>
+      </c>
+      <c r="C83" t="str">
+        <v>Borrador rubro: excluir Apertura/Cierre de caja</v>
+      </c>
+      <c r="D83" t="str">
+        <v>§8.4 y MATRIZ: filas Apertura/Cierre eliminadas; párrafo y notas indican exclusión por definición (alineado a upload).</v>
+      </c>
+      <c r="E83" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>22/03/2026</v>
+      </c>
+      <c r="B84" t="str">
+        <v>20:53</v>
+      </c>
+      <c r="C84" t="str">
+        <v>Análisis financiero extracto → HTML/PDF</v>
+      </c>
+      <c r="D84" t="str">
+        <v>scripts/generar-analisis-financiero-pdf.js: métricas desde Extracto-Fornitalia.xlsx (resumen, mensual, estacionalidad/IQR, medios, calidad datos, cash management). Salida docs/ANALISIS_FINANCIERO_EXTRACTO_FORNITALIA.*; npm run analisis-financiero-pdf; fallback Chrome headless si Playwright sin Chromium.</v>
+      </c>
+      <c r="E84" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>22/03/2026</v>
+      </c>
+      <c r="B85" t="str">
+        <v>20:53</v>
+      </c>
+      <c r="C85" t="str">
+        <v>Dashboard v1.34: excluir traspasos internos del flujo</v>
+      </c>
+      <c r="D85" t="str">
+        <v>excluirCategoria amplía a Transferencia y Deposito/Depósito (misma regla que informe financiero); nota en panel Flujo por mes; APP_VERSION 1.34. Base histórica export sigue completa.</v>
+      </c>
+      <c r="E85" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>22/03/2026</v>
+      </c>
+      <c r="B86" t="str">
+        <v>20:53</v>
+      </c>
+      <c r="C86" t="str">
+        <v>Informe financiero PDF: MEP desde docs y textos</v>
+      </c>
+      <c r="D86" t="str">
+        <v>generar-analisis-financiero-pdf.js: carga usd_mep desde docs/tipos_cambio_global_rows.sql (o CSV docs/raíz); conversión USD alineada al dashboard; filas sin ARS excluidas de totales con conteo en meta y advertencias en HTML. README ANALISIS_FINANCIERO_EXTRACTO_README.md actualizado.</v>
+      </c>
+      <c r="E86" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>22/03/2026</v>
+      </c>
+      <c r="B87" t="str">
+        <v>20:53</v>
+      </c>
+      <c r="C87" t="str">
+        <v>Dashboard v1.35: flujo alineado al informe PDF + solapa traspasos</v>
+      </c>
+      <c r="D87" t="str">
+        <v>Tarjetas y tabla Flujo por mes: totales extracto (con traspasos) vs G/P operativo; columnas Neto bruto y G/P operativo. excluirFilaFlujoOperativo (Anulado, apertura/cierre heurística, Transferencia/Depósito). Evolución y duplicados con la misma base. Solapa Traspasos internos con listado. APP_VERSION 1.35.</v>
+      </c>
+      <c r="E87" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>22/03/2026</v>
+      </c>
+      <c r="B88" t="str">
+        <v>20:53</v>
+      </c>
+      <c r="C88" t="str">
+        <v>Dashboard v1.36: ARS con monto_cambio y tipo_cambio (concilia PDF)</v>
+      </c>
+      <c r="D88" t="str">
+        <v>fetch transacciones incluye tipo_cambio y monto_cambio. montoConvertido en ARS prioriza monto_cambio (Monto en $), luego TC fila, luego tabla (como generar-analisis-financiero-pdf.js). Flujo por mes usa montoConvertido unificado. Nota en panel Flujo. APP_VERSION 1.36.</v>
+      </c>
+      <c r="E88" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>22/03/2026</v>
+      </c>
+      <c r="B89" t="str">
+        <v>20:53</v>
+      </c>
+      <c r="C89" t="str">
+        <v>Despliegue v1.37 producción</v>
+      </c>
+      <c r="D89" t="str">
+        <v>Push a main y Vercel --prod: versiones 1.34–1.37 en bitácora; APP_VERSION 1.37; flujo bruto/operativo, Traspasos internos, conciliación monto_cambio con informe PDF; script informe financiero MEP en docs.</v>
+      </c>
+      <c r="E89" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E77"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E89"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B56"/>
+  <dimension ref="A1:B58"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -1748,7 +1952,7 @@
         <v>Flujo de caja por mes</v>
       </c>
       <c r="B2" t="str">
-        <v>Tabla con ingresos, egresos y balance por mes/año.</v>
+        <v>Tabla alineada al informe financiero PDF: columnas Ingresos y Egresos = totales del extracto (incluyen traspasos entre cuentas); Neto bruto; G/P operativo sin Transferencia/Depósito ni Apertura/Cierre; ratios y Caución sobre operativo. Proyección solo sobre operativo.</v>
       </c>
     </row>
     <row r="3">
@@ -1756,7 +1960,7 @@
         <v>Resumen global</v>
       </c>
       <c r="B3" t="str">
-        <v>Totales: Total ingresos, Total egresos, Balance (en ARS o USD).</v>
+        <v>Cuatro tarjetas: Ingresos totales y Egresos totales del extracto (con traspasos), Neto caja (bruto) y G/P operativo (sin traspasos internos), en ARS o USD según selector.</v>
       </c>
     </row>
     <row r="4">
@@ -1764,7 +1968,7 @@
         <v>Moneda</v>
       </c>
       <c r="B4" t="str">
-        <v>Selector ARS / USD; conversión con tipos de cambio desde Supabase. Montos mostrados con $ (pesos) o US$ (dólares) a la izquierda.</v>
+        <v>Selector ARS / USD. En ARS: prioridad monto_cambio (Monto en $ del extracto en BD), tipo_cambio por fila y tabla tipo_de_cambio (MEP/CCL/Oficial); con MEP y datos cargados coincide con el informe PDF.</v>
       </c>
     </row>
     <row r="5">
@@ -1889,303 +2093,319 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Exclusiones</v>
+        <v>Exclusiones (flujo operativo)</v>
       </c>
       <c r="B20" t="str">
-        <v>No se incluyen transacciones anuladas ni categorías Apertura y Cierre.</v>
+        <v>No se incluyen en G/P operativo, Evolución ni Caución: anulados; apertura/cierre (categoría o heurística en fila); Transferencia ni Deposito/Depósito. Los traspasos se listan en la solapa Traspasos internos. Base histórica y Todas las transacciones siguen completas.</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Datos</v>
+        <v>Traspasos internos (solapa)</v>
       </c>
       <c r="B21" t="str">
-        <v>Transacciones y tipo de cambio desde Supabase (carga paginada de a 1000 filas por request para no truncar resultados). Cotización faltante: se usa la fecha anterior disponible.</v>
+        <v>Listado de movimientos categoría Transferencia o Deposito/Depósito (no anulados), con monto de registro y equivalente en moneda de vista.</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Menú lateral</v>
+        <v>Datos</v>
       </c>
       <c r="B22" t="str">
-        <v>Sidebar izquierdo colapsable/expandible; botón toggle (▶/◀); ítem Home por ahora; estado persistido en localStorage. Listo para ampliar con más ítems.</v>
+        <v>Transacciones y tipo de cambio desde Supabase (carga paginada de a 1000 filas por request para no truncar resultados). Cotización faltante: se usa la fecha anterior disponible.</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Repositorio Git (GitHub)</v>
+        <v>Menú lateral</v>
       </c>
       <c r="B23" t="str">
-        <v>Repo: https://github.com/lucasbustosmartin-coder/fornitalia. Rama main. .gitignore excluye node_modules, .venv, .env. Para actualizar: git add . ; git commit -m "mensaje" ; git push origin main.</v>
+        <v>Sidebar izquierdo colapsable/expandible; botón toggle (▶/◀); ítem Home por ahora; estado persistido en localStorage. Listo para ampliar con más ítems.</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>App en producción (Vercel)</v>
+        <v>Repositorio Git (GitHub)</v>
       </c>
       <c r="B24" t="str">
-        <v>URL pública: https://fornitalia.vercel.app/ (vercel.json reescribe / al dashboard). Cada push a main en GitHub dispara redeploy automático en Vercel. Proyecto: fornitalia, equipo Lucas Bustos, plan Hobby.</v>
+        <v>Repo: https://github.com/lucasbustosmartin-coder/fornitalia. Rama main. .gitignore excluye node_modules, .venv, .env. Para actualizar: git add . ; git commit -m "mensaje" ; git push origin main.</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Exportar a Excel</v>
+        <v>App en producción (Vercel)</v>
       </c>
       <c r="B25" t="str">
-        <v>Botón en la barra de la tabla (solo icono). Exporta la tabla de transacciones tal como está en Supabase: una hoja "Transacciones" con columnas fecha, mes, anio, tipo_movimiento, monto (valor numérico para fórmulas), status, medio_pago, moneda, descripcion, cliente, categoria, cat_desc, origen_archivo, cuenta_contable, editado, editado_detalle. Export Errores: monto también como número. Permite analizar y usar fórmulas en Excel.</v>
+        <v>URL pública: https://fornitalia.vercel.app/ (vercel.json reescribe / al dashboard). Cada push a main en GitHub dispara redeploy automático en Vercel. Proyecto: fornitalia, equipo Lucas Bustos, plan Hobby.</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Flujo de despliegue</v>
+        <v>Exportar a Excel</v>
       </c>
       <c r="B26" t="str">
-        <v>Al terminar cada tarea: el usuario prueba en local y confirma; recién entonces el asistente hace git add, commit y push (Vercel redepliega automático). No se despliega hasta confirmación.</v>
+        <v>Botón en la barra de la tabla (solo icono). Exporta la tabla de transacciones tal como está en Supabase: una hoja "Transacciones" con columnas fecha, mes, anio, tipo_movimiento, monto (valor numérico para fórmulas), status, medio_pago, moneda, descripcion, cliente, categoria, cat_desc, origen_archivo, cuenta_contable, editado, editado_detalle. Export Errores: monto también como número. Permite analizar y usar fórmulas en Excel.</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Versiones en bitácora</v>
+        <v>Flujo de despliegue</v>
       </c>
       <c r="B27" t="str">
-        <v>Hoja "Versiones" en Bitacora_tareas.xlsx: registro incremental (1.0, 1.1, …) con fecha y descripción de cada despliegue a Git/Vercel.</v>
+        <v>Al terminar cada tarea: el usuario prueba en local y confirma; recién entonces el asistente hace git add, commit y push (Vercel redepliega automático). No se despliega hasta confirmación.</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Campo moneda (BD)</v>
+        <v>Versiones en bitácora</v>
       </c>
       <c r="B28" t="str">
-        <v>Columna moneda en tabla transacciones (ARS/USD). Si está informada, el dashboard la usa salvo reglas de negocio: Mercado Pago y Transferencia Morba siempre ARS para conversión (también morva por typo). Si moneda vacía, infiere desde textos/medio (dólar → USD). Export a Excel incluye moneda.</v>
+        <v>Hoja "Versiones" en Bitacora_tareas.xlsx: registro incremental (1.0, 1.1, …) con fecha y descripción de cada despliegue a Git/Vercel.</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Edición desde modal Errores</v>
+        <v>Campo moneda (BD)</v>
       </c>
       <c r="B29" t="str">
-        <v>En el detalle de errores, icono de edición por registro. Abre modal para corregir: Categoría y Cuenta contable solo desde valores existentes en BD; Descripción libre. Al guardar se actualiza la fila y se marcan editado y editado_detalle (qué campos se editaron).</v>
+        <v>Columna moneda en tabla transacciones (ARS/USD). Si está informada, el dashboard la usa salvo reglas de negocio: Mercado Pago y Transferencia Morba siempre ARS para conversión (también morva por typo). Si moneda vacía, infiere desde textos/medio (dólar → USD). Export a Excel incluye moneda.</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Campos editado y editado_detalle</v>
+        <v>Edición desde modal Errores</v>
       </c>
       <c r="B30" t="str">
-        <v>En transacciones: editado (boolean) y editado_detalle (texto, ej. "Categoria, Descripcion, Cuenta Contable"). Migración supabase_transacciones_editado.sql. Export Excel los incluye.</v>
+        <v>En el detalle de errores, icono de edición por registro. Abre modal para corregir: Categoría y Cuenta contable solo desde valores existentes en BD; Descripción libre. Al guardar se actualiza la fila y se marcan editado y editado_detalle (qué campos se editaron).</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Tipo de error en Errores</v>
+        <v>Campos editado y editado_detalle</v>
       </c>
       <c r="B31" t="str">
-        <v>Tabla de errores muestra columna Tipo de error: Inconsistencia entre Categoria, Cuenta Contable y Descripcion; o Potencial registro duplicado. Export a Excel incluye tipo_error.</v>
+        <v>En transacciones: editado (boolean) y editado_detalle (texto, ej. "Categoria, Descripcion, Cuenta Contable"). Migración supabase_transacciones_editado.sql. Export Excel los incluye.</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Detección de potencial duplicado</v>
+        <v>Tipo de error en Errores</v>
       </c>
       <c r="B32" t="str">
-        <v>Registros con misma fecha, monto, tipo_movimiento y descripción similar se marcan como potencial duplicado. Icono Ver abre modal con comparación Este registro / Posible duplicado; acciones: Excluir de cálculos (anular) o Eliminar registro.</v>
+        <v>Tabla de errores muestra columna Tipo de error: Inconsistencia entre Categoria, Cuenta Contable y Descripcion; o Potencial registro duplicado. Export a Excel incluye tipo_error.</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Filtro por tipo de error</v>
+        <v>Detección de potencial duplicado</v>
       </c>
       <c r="B33" t="str">
-        <v>En la solapa Errores, selector para filtrar por tipo: Todos, Inconsistencia (categoría/cuenta/descripción), Potencial registro duplicado. La exportación a Excel exporta solo los registros visibles según el filtro.</v>
+        <v>Registros con misma fecha, monto, tipo_movimiento y descripción similar se marcan como potencial duplicado. Icono Ver abre modal con comparación Este registro / Posible duplicado; acciones: Excluir de cálculos (anular) o Eliminar registro.</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Duplicados: condición cliente</v>
+        <v>Filtro por tipo de error</v>
       </c>
       <c r="B34" t="str">
-        <v>Dos registros son potencial duplicado solo si coinciden en fecha, monto, tipo_movimiento, descripción similar y además cliente es igual; si cliente es distinto no se marcan como duplicado. Modal de comparación muestra id_origen y Cliente.</v>
+        <v>En la solapa Errores, selector para filtrar por tipo: Todos, Inconsistencia (categoría/cuenta/descripción), Potencial registro duplicado. La exportación a Excel exporta solo los registros visibles según el filtro.</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Regla bitácora</v>
+        <v>Duplicados: condición cliente</v>
       </c>
       <c r="B35" t="str">
-        <v>Actualizar todas las solapas necesarias: Log (siempre que haya tarea), Resumen (si cambia funcionalidad), Presupuesto (si agrega o cambia entregable comercial), Versiones (en despliegue). Regenerar Excel tras editar crear-bitacora-excel.js.</v>
+        <v>Dos registros son potencial duplicado solo si coinciden en fecha, monto, tipo_movimiento, descripción similar y además cliente es igual; si cliente es distinto no se marcan como duplicado. Modal de comparación muestra id_origen y Cliente.</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Evolución (tabla dinámica)</v>
+        <v>Regla bitácora</v>
       </c>
       <c r="B36" t="str">
-        <v>Solapa Evolución: Agrupar por = Categoría o Cuenta contable (fila); Período = Diario (fecha por día) o Mensual (MM-YYYY). Columnas = períodos, celdas = neto en moneda seleccionada, columna Total.</v>
+        <v>Actualizar todas las solapas necesarias: Log (siempre que haya tarea), Resumen (si cambia funcionalidad), Presupuesto (si agrega o cambia entregable comercial), Versiones (en despliegue). Regenerar Excel tras editar crear-bitacora-excel.js.</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Evolución: detalle al clic y exportar</v>
+        <v>Evolución (tabla dinámica)</v>
       </c>
       <c r="B37" t="str">
-        <v>Clic en un valor de la tabla Evolución abre modal con detalle: Fecha, Categoría, Descripción, Monto. Exportar Evolución a Excel exporta la tabla según filtros Agrupar por y Período.</v>
+        <v>Solapa Evolución: Agrupar por = Categoría o Cuenta contable (fila); Período = Diario (fecha por día) o Mensual (MM-YYYY). Columnas = períodos, celdas = neto en moneda seleccionada, columna Total.</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Exportaciones Excel</v>
+        <v>Evolución: detalle al clic y exportar</v>
       </c>
       <c r="B38" t="str">
-        <v>Todas las exportaciones incluyen una fila título con la moneda. Exportar Base Histórica (icono Excel) en la línea del selector de moneda; Exportar Evolución a Excel con el mismo icono.</v>
+        <v>Clic en un valor de la tabla Evolución abre modal con detalle: Fecha, Categoría, Descripción, Monto. Exportar Evolución a Excel exporta la tabla según filtros Agrupar por y Período.</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Evolución: orden ingreso/egreso</v>
+        <v>Exportaciones Excel</v>
       </c>
       <c r="B39" t="str">
-        <v>En la tabla Evolución las filas se muestran primero las de ingreso (total &gt;= 0) y luego las de egreso (total &lt; 0); dentro de cada grupo orden alfabético. Aplica tanto al agrupar por Categoría como por Cuenta contable.</v>
+        <v>Todas las exportaciones incluyen una fila título con la moneda. Exportar Base Histórica (icono Excel) en la línea del selector de moneda; Exportar Evolución a Excel con el mismo icono.</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Int. por caución</v>
+        <v>Evolución: orden ingreso/egreso</v>
       </c>
       <c r="B40" t="str">
-        <v>Columna en flujo por mes: interés mensual por colocar el sobrante de caja a la tasa diaria de la serie de cauciones. Carga Serie_Cauciones.xlsx al refrescar (o serie_cauciones.json si no hay Excel). Cálculo: base = G/P acumulado a la fecha + interés acumulado; Int T = base × tasa. Clic en el valor abre modal con marcha (G/P acum, Int T-1, Base, Tasa, Int T).</v>
+        <v>En la tabla Evolución las filas se muestran primero las de ingreso (total &gt;= 0) y luego las de egreso (total &lt; 0); dentro de cada grupo orden alfabético. Aplica tanto al agrupar por Categoría como por Cuenta contable.</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Todas las transacciones</v>
+        <v>Int. por caución</v>
       </c>
       <c r="B41" t="str">
-        <v>Solapa que lista todas las transacciones con todas las columnas. Filtros por mes y categoría. Botón Editar por registro abre modal de edición completa.</v>
+        <v>Columna en flujo por mes: interés mensual por colocar el sobrante de caja a la tasa diaria de la serie de cauciones. Carga Serie_Cauciones.xlsx al refrescar (o serie_cauciones.json si no hay Excel). Cálculo: base = G/P acumulado a la fecha + interés acumulado; Int T = base × tasa. Clic en el valor abre modal con marcha (G/P acum, Int T-1, Base, Tasa, Int T).</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Edición completa de registros</v>
+        <v>Todas las transacciones</v>
       </c>
       <c r="B42" t="str">
-        <v>Modal de edición con todos los campos: fecha, mes, año, tipo movimiento, monto, moneda, status, medio pago, categoría, cuenta contable, origen archivo, descripción, cliente, cat_desc, id_origen, id_operación. Combos para campos normalizados (valores existentes en BD). editado y editado_detalle al guardar.</v>
+        <v>Solapa que lista todas las transacciones con todas las columnas. Filtros por mes y categoría. Botón Editar por registro abre modal de edición completa.</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Proyección próximos 3 meses</v>
+        <v>Edición completa de registros</v>
       </c>
       <c r="B43" t="str">
-        <v>Debajo del total real en Flujo por mes: "Próximos 3 meses proyectados" con ventana rodante. Configuración (sidebar): método (Mediana/Promedio) y meses de historia (3, 6, 12, 24). Ingresos, egresos, G/P y ratios proyectados por mes.</v>
+        <v>Modal de edición con todos los campos: fecha, mes, año, tipo movimiento, monto, moneda, status, medio pago, categoría, cuenta contable, origen archivo, descripción, cliente, cat_desc, id_origen, id_operación. Combos para campos normalizados (valores existentes en BD). editado y editado_detalle al guardar.</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Int. por caución proyectado</v>
+        <v>Proyección próximos 3 meses</v>
       </c>
       <c r="B44" t="str">
-        <v>Punto de partida = G/P Total real + interés acumulado; tasa = promedio último mes real; días naturales; Int T-1 día 1 = (Int T-1 + Int T) último día del mes anterior. G/P acum en marcha = al inicio de cada día (real y proyectado). Ventana rodante: ingresos/egresos distintos por mes.</v>
+        <v>Debajo del total real en Flujo por mes: "Próximos 3 meses proyectados" con ventana rodante. Configuración (sidebar): método (Mediana/Promedio) y meses de historia (3, 6, 12, 24). Ingresos, egresos, G/P y ratios proyectados por mes.</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Disclaimer proyección</v>
+        <v>Int. por caución proyectado</v>
       </c>
       <c r="B45" t="str">
-        <v>Debajo de las filas proyectadas, texto en letra chica y gris oscuro que explica la metodología: Mediana/Promedio de N meses, ventana rodante, y cálculo de Int. por caución proyectado.</v>
+        <v>Punto de partida = G/P Total real + interés acumulado; tasa = promedio último mes real; días naturales; Int T-1 día 1 = (Int T-1 + Int T) último día del mes anterior. G/P acum en marcha = al inicio de cada día (real y proyectado). Ventana rodante: ingresos/egresos distintos por mes.</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Botones e iconos unificados</v>
+        <v>Disclaimer proyección</v>
       </c>
       <c r="B46" t="str">
-        <v>Todos los botones con mismo estilo: icono SVG + texto. Sidebar (chevron, home, engranaje), tabs con iconos, exportar con icono descarga, modales con iconos (Guardar, Cerrar, Excluir, Eliminar). Iconos solos (cerrar, editar, alerta) en SVG.</v>
+        <v>Debajo de las filas proyectadas, texto en letra chica y gris oscuro que explica la metodología: Mediana/Promedio de N meses, ventana rodante, y cálculo de Int. por caución proyectado.</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Configuración % G/P en caución</v>
+        <v>Botones e iconos unificados</v>
       </c>
       <c r="B47" t="str">
-        <v>Combo "% G/P acum. en caución" en Configuración con escala de 5 en 5 (100, 95, 90… hasta 0). Por defecto 100 %; menor % = más liquidez (menos interés por caución).</v>
+        <v>Todos los botones con mismo estilo: icono SVG + texto. Sidebar (chevron, home, engranaje), tabs con iconos, exportar con icono descarga, modales con iconos (Guardar, Cerrar, Excluir, Eliminar). Iconos solos (cerrar, editar, alerta) en SVG.</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Etiqueta Caución (x% cash)</v>
+        <v>Configuración % G/P en caución</v>
       </c>
       <c r="B48" t="str">
-        <v>Columna en flujo por mes: cabecera "Caución (x% cash)" donde x es el valor del parámetro % G/P; sin icono % a la izquierda. Modales de marcha y disclaimer usan "Caución".</v>
+        <v>Combo "% G/P acum. en caución" en Configuración con escala de 5 en 5 (100, 95, 90… hasta 0). Por defecto 100 %; menor % = más liquidez (menos interés por caución).</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Meses a proyectar</v>
+        <v>Etiqueta Caución (x% cash)</v>
       </c>
       <c r="B49" t="str">
-        <v>En Configuración: combo Meses a proyectar (1, 2, 3, 4, 5, 6, 12). Flujo por mes y Evolución muestran esa cantidad de columnas/filas proyectadas.</v>
+        <v>Columna en flujo por mes: cabecera "Caución (x% cash)" donde x es el valor del parámetro % G/P; sin icono % a la izquierda. Modales de marcha y disclaimer usan "Caución".</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Config por usuario en Supabase</v>
+        <v>Meses a proyectar</v>
       </c>
       <c r="B50" t="str">
-        <v>Tabla config_dashboard (user_id, proyección y caución). Con Auth anónimo se sincroniza al cargar y al guardar; la config persiste por usuario en la base. Migración: supabase_config_dashboard.sql.</v>
+        <v>En Configuración: combo Meses a proyectar (1, 2, 3, 4, 5, 6, 12). Flujo por mes y Evolución muestran esa cantidad de columnas/filas proyectadas.</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Recorte % (cada lado)</v>
+        <v>Config por usuario en Supabase</v>
       </c>
       <c r="B51" t="str">
-        <v>En Configuración, combo Recorte % (cada lado) (0, 5, 10, 15, 20, 25) visible solo cuando el método es Promedio recortado. Más % = más suavizado. Persistido en config_dashboard (proyeccion_recorte).</v>
+        <v>Tabla config_dashboard (user_id, proyección y caución). Con Auth anónimo se sincroniza al cargar y al guardar; la config persiste por usuario en la base. Migración: supabase_config_dashboard.sql.</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Novedades del Negocio</v>
+        <v>Recorte % (cada lado)</v>
       </c>
       <c r="B52" t="str">
-        <v>Ítem en sidebar que abre una vista con importadores de hornos y comercios de venta de hornos en Argentina (Buenos Aires). Datos recuperados por IA (Edge Function con Gemini + google_search). Nombre, dirección, teléfono y web por contacto.</v>
+        <v>En Configuración, combo Recorte % (cada lado) (0, 5, 10, 15, 20, 25) visible solo cuando el método es Promedio recortado. Más % = más suavizado. Persistido en config_dashboard (proyeccion_recorte).</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Normalización de extracto bancario</v>
+        <v>Novedades del Negocio</v>
       </c>
       <c r="B53" t="str">
-        <v>Script utilitario que normaliza el extracto Excel en una hoja estructurada (Normalizado) con campos listos para tablas: fecha_iso, tipo, medio, categoría, cuenta, moneda inferida (USD/ARS; Mercado Pago y Transferencia Morba forzados a ARS), monto_original numérico, tipo_cambio y monto_ars.</v>
+        <v>Ítem en sidebar que abre una vista con importadores de hornos y comercios de venta de hornos en Argentina (Buenos Aires). Datos recuperados por IA (Edge Function con Gemini + google_search). Nombre, dirección, teléfono y web por contacto.</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>Informe inconsistencias datos legacy (cliente)</v>
+        <v>Normalización de extracto bancario</v>
       </c>
       <c r="B54" t="str">
-        <v>Documento docs/ANALISIS_NORMALIZACION_DATOS_LEGACY_FORNITALIA.md con tablas Cant./recomendaciones; .html y .pdf en docs/. Regenerar: npm run informe-normalizacion-html o npm run informe-normalizacion-pdf (Playwright+Chromium, alineado a stack Pandi); primera vez: npx playwright install chromium.</v>
+        <v>Script utilitario que normaliza el extracto Excel en una hoja estructurada (Normalizado) con campos listos para tablas: fecha_iso, tipo, medio, categoría, cuenta, moneda inferida (USD/ARS; Mercado Pago y Transferencia Morba forzados a ARS), monto_original numérico, tipo_cambio y monto_ars.</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>Upload de extracto normalizado</v>
+        <v>Informe inconsistencias datos legacy (cliente)</v>
       </c>
       <c r="B55" t="str">
-        <v>Botón en la app para reemplazar transacciones desde un Excel normalizado (hoja Normalizado), con validación previa, confirmación de seguridad, generación de id_origen técnico y carga en lotes.</v>
+        <v>Documento docs/ANALISIS_NORMALIZACION_DATOS_LEGACY_FORNITALIA.md con tablas Cant./recomendaciones; .html y .pdf en docs/. Regenerar: npm run informe-normalizacion-html o npm run informe-normalizacion-pdf (Playwright+Chromium, alineado a stack Pandi); primera vez: npx playwright install chromium.</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
+        <v>Upload de extracto normalizado</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Botón en la app para reemplazar transacciones desde un Excel normalizado (hoja Normalizado), con validación previa, confirmación de seguridad, generación de id_origen técnico y carga en lotes.</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
         <v>Log de excluidos en upload</v>
       </c>
-      <c r="B56" t="str">
+      <c r="B57" t="str">
         <v>Nueva solapa Excluidos upload con registros no insertados por error o por regla de negocio (Apertura/Cierre de Caja), persistidos en Supabase para auditoría.</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>Análisis financiero extracto (PDF)</v>
+      </c>
+      <c r="B58" t="str">
+        <v>npm run analisis-financiero-pdf: métricas desde docs/Extracto-Fornitalia.xlsx; ARS vía Monto en $, TC por fila o MEP (docs/tipos_cambio_global_rows.sql o CSV); exclusiones y conteo de USD sin conversión en el informe. Ver docs/ANALISIS_FINANCIERO_EXTRACTO_README.md.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B56"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B58"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2279,7 +2499,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C39"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -2577,7 +2797,7 @@
         <v>1.25</v>
       </c>
       <c r="B27" t="str">
-        <v>19/03/2026</v>
+        <v>22/03/2026</v>
       </c>
       <c r="C27" t="str">
         <v>Ayuda al clic en columnas Comisiones/Ventas y Egresos/Ingresos (popover con texto explicativo). Regla bitácora: tecnología e infraestructura y actualizar todas las solapas. Despliegue a producción.</v>
@@ -2588,7 +2808,7 @@
         <v>1.26</v>
       </c>
       <c r="B28" t="str">
-        <v>19/03/2026</v>
+        <v>22/03/2026</v>
       </c>
       <c r="C28" t="str">
         <v>Mensaje de alerta de desvío: categoría en negrita sin comillas. Despliegue a producción.</v>
@@ -2599,7 +2819,7 @@
         <v>1.27</v>
       </c>
       <c r="B29" t="str">
-        <v>19/03/2026</v>
+        <v>22/03/2026</v>
       </c>
       <c r="C29" t="str">
         <v>Novedades del Negocio: sección en sidebar con importadores y comercios de hornos en Argentina (Edge Function Gemini + google_search). Despliegue a producción.</v>
@@ -2610,7 +2830,7 @@
         <v>1.28</v>
       </c>
       <c r="B30" t="str">
-        <v>19/03/2026</v>
+        <v>22/03/2026</v>
       </c>
       <c r="C30" t="str">
         <v>Favicon L&amp;P: L y P dada vuelta centradas en el círculo azul; ajuste de posición y centrado. Despliegue a producción.</v>
@@ -2621,7 +2841,7 @@
         <v>1.29</v>
       </c>
       <c r="B31" t="str">
-        <v>19/03/2026</v>
+        <v>22/03/2026</v>
       </c>
       <c r="C31" t="str">
         <v>Errores: export y listado con id_origen e id_operacion; modal duplicado con id_operacion e icono en campos que no coinciden. Exclusiones duplicados: anulados, id_origen e id_operacion ambos distintos, ambos montos 0. Quitar disclaimer datos ficticios; scripts e instrucciones para repoblar transacciones desde Excel. Despliegue a producción.</v>
@@ -2632,7 +2852,7 @@
         <v>1.30</v>
       </c>
       <c r="B32" t="str">
-        <v>19/03/2026</v>
+        <v>22/03/2026</v>
       </c>
       <c r="C32" t="str">
         <v>Errores: orden por tipo y monto descendente; filtros por categoría original y categoría mostrada. Flujo: filtro explícito status Anulado. Export Base Histórica: columnas Tipo_Cambio, Monto_ARS, Monto_USD con conversiones. Despliegue a producción.</v>
@@ -2643,7 +2863,7 @@
         <v>1.31</v>
       </c>
       <c r="B33" t="str">
-        <v>19/03/2026</v>
+        <v>22/03/2026</v>
       </c>
       <c r="C33" t="str">
         <v>Estructura ordenada del repo: sql/, scripts/, docs/. Regla estructura-proyecto (mantener carpetas y rutas). Referencias en bitácora y docs actualizadas. Despliegue a producción.</v>
@@ -2654,7 +2874,7 @@
         <v>1.32</v>
       </c>
       <c r="B34" t="str">
-        <v>19/03/2026</v>
+        <v>22/03/2026</v>
       </c>
       <c r="C34" t="str">
         <v>Modales: no cerrar al elegir opción de select (mousedown+click en backdrop). Helper setupBackdropCloseOnlyOnRealClick en todos los modales.</v>
@@ -2665,15 +2885,59 @@
         <v>1.33</v>
       </c>
       <c r="B35" t="str">
-        <v>19/03/2026</v>
+        <v>22/03/2026</v>
       </c>
       <c r="C35" t="str">
         <v>Carga paginada transacciones y tipo_de_cambio (límite PostgREST). Reglas ARS Mercado Pago y Transferencia Morba en normalizador, upload y esTransaccionUSD. Upload excluidos: filtro última corrida; SQL DELETE en transacciones_upload_excluidos. Informe análisis normalización (docs MD/HTML/PDF) y scripts Playwright. DevDependency playwright y npm run playwright:install.</v>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>1.34</v>
+      </c>
+      <c r="B36" t="str">
+        <v>22/03/2026</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Flujo operativo sin traspasos internos (Transferencia y Depósito); misma regla que informe PDF; nota en panel.</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>1.35</v>
+      </c>
+      <c r="B37" t="str">
+        <v>22/03/2026</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Flujo por mes alineado al PDF: ingresos/egresos brutos extracto, Neto bruto, G/P operativo; solapa Traspasos internos; excluirFilaFlujoOperativo y Evolución con misma base.</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>1.36</v>
+      </c>
+      <c r="B38" t="str">
+        <v>22/03/2026</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Select tipo_cambio y monto_cambio en transacciones; montoConvertido en ARS prioriza monto_cambio y TC de fila (concilia con informe PDF al centavo).</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>1.37</v>
+      </c>
+      <c r="B39" t="str">
+        <v>22/03/2026</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Despliegue a producción Vercel: informe financiero PDF con MEP desde docs; dashboard v1.37 con conciliación extracto.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C35"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C39"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.43: módulo seguridad, tablas sticky, scroll flujo y bitácora
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E89"/>
+  <dimension ref="A1:E100"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -1382,10 +1382,10 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="B58" t="str">
-        <v>20:53</v>
+        <v>20:30</v>
       </c>
       <c r="C58" t="str">
         <v>Ayuda al clic en columnas flujo y regla bitácora</v>
@@ -1399,10 +1399,10 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="B59" t="str">
-        <v>20:53</v>
+        <v>20:30</v>
       </c>
       <c r="C59" t="str">
         <v>Alerta desvío: categoría en negrita sin comillas</v>
@@ -1416,10 +1416,10 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="B60" t="str">
-        <v>20:53</v>
+        <v>20:30</v>
       </c>
       <c r="C60" t="str">
         <v>Novedades del Negocio y despliegue v1.27</v>
@@ -1433,10 +1433,10 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="B61" t="str">
-        <v>20:53</v>
+        <v>20:30</v>
       </c>
       <c r="C61" t="str">
         <v>Favicon L&amp;P centrado</v>
@@ -1450,10 +1450,10 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="B62" t="str">
-        <v>20:53</v>
+        <v>20:30</v>
       </c>
       <c r="C62" t="str">
         <v>Despliegue v1.29</v>
@@ -1467,10 +1467,10 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="B63" t="str">
-        <v>20:53</v>
+        <v>20:30</v>
       </c>
       <c r="C63" t="str">
         <v>Despliegue v1.30</v>
@@ -1484,10 +1484,10 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="B64" t="str">
-        <v>20:53</v>
+        <v>20:30</v>
       </c>
       <c r="C64" t="str">
         <v>Despliegue v1.31</v>
@@ -1501,10 +1501,10 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="B65" t="str">
-        <v>20:53</v>
+        <v>20:30</v>
       </c>
       <c r="C65" t="str">
         <v>Despliegue v1.32</v>
@@ -1518,10 +1518,10 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="B66" t="str">
-        <v>20:53</v>
+        <v>20:30</v>
       </c>
       <c r="C66" t="str">
         <v>Normalización de Extracto Fornitalia</v>
@@ -1535,10 +1535,10 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="B67" t="str">
-        <v>20:53</v>
+        <v>20:30</v>
       </c>
       <c r="C67" t="str">
         <v>Upload controlado de extracto normalizado en app</v>
@@ -1552,10 +1552,10 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="B68" t="str">
-        <v>20:53</v>
+        <v>20:30</v>
       </c>
       <c r="C68" t="str">
         <v>Upload normalizado sin confirmación manual y log de excluidos</v>
@@ -1569,10 +1569,10 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="B69" t="str">
-        <v>20:53</v>
+        <v>20:30</v>
       </c>
       <c r="C69" t="str">
         <v>Ajuste final upload: no loguear Apertura/Cierre y réplica en Everfit</v>
@@ -1586,10 +1586,10 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="B70" t="str">
-        <v>20:53</v>
+        <v>20:30</v>
       </c>
       <c r="C70" t="str">
         <v>Limpieza de log excluidos y normalización de mes/año en carga</v>
@@ -1603,10 +1603,10 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="B71" t="str">
-        <v>20:53</v>
+        <v>20:30</v>
       </c>
       <c r="C71" t="str">
         <v>Excluidos upload: mostrar solo última corrida y habilitar DELETE</v>
@@ -1620,10 +1620,10 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="B72" t="str">
-        <v>20:53</v>
+        <v>20:30</v>
       </c>
       <c r="C72" t="str">
         <v>Carga paginada desde Supabase (transacciones y tipo de cambio)</v>
@@ -1637,10 +1637,10 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="B73" t="str">
-        <v>20:53</v>
+        <v>20:30</v>
       </c>
       <c r="C73" t="str">
         <v>Reglas moneda: Mercado Pago y Transferencia Morba siempre ARS</v>
@@ -1654,10 +1654,10 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="B74" t="str">
-        <v>20:53</v>
+        <v>20:30</v>
       </c>
       <c r="C74" t="str">
         <v>Documento análisis normalización datos legacy</v>
@@ -1671,10 +1671,10 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="B75" t="str">
-        <v>20:53</v>
+        <v>20:30</v>
       </c>
       <c r="C75" t="str">
         <v>Informe normalización: cantidades por fila y PDF/HTML</v>
@@ -1688,10 +1688,10 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="B76" t="str">
-        <v>20:53</v>
+        <v>20:30</v>
       </c>
       <c r="C76" t="str">
         <v>Playwright en todos los repos LyP</v>
@@ -1705,10 +1705,10 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="B77" t="str">
-        <v>20:53</v>
+        <v>20:30</v>
       </c>
       <c r="C77" t="str">
         <v>Despliegue v1.33 producción</v>
@@ -1722,10 +1722,10 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="B78" t="str">
-        <v>20:53</v>
+        <v>20:30</v>
       </c>
       <c r="C78" t="str">
         <v>Análisis normalización: propuesta recategorización categoría–cuenta</v>
@@ -1739,10 +1739,10 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="B79" t="str">
-        <v>20:53</v>
+        <v>20:30</v>
       </c>
       <c r="C79" t="str">
         <v>Análisis normalización: matriz concreta Ord. n y acción Editar/Nueva/Eliminar</v>
@@ -1756,10 +1756,10 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="B80" t="str">
-        <v>20:53</v>
+        <v>20:30</v>
       </c>
       <c r="C80" t="str">
         <v>Rubros IGJ/FACPCE y balance: doc de referencia</v>
@@ -1773,10 +1773,10 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="B81" t="str">
-        <v>20:53</v>
+        <v>20:30</v>
       </c>
       <c r="C81" t="str">
         <v>Matriz borrador categoría–cuenta–rubro (Argentina)</v>
@@ -1790,10 +1790,10 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="B82" t="str">
-        <v>20:53</v>
+        <v>20:30</v>
       </c>
       <c r="C82" t="str">
         <v>Análisis: §8.4 borrador rubro dentro del MD principal</v>
@@ -1807,10 +1807,10 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="B83" t="str">
-        <v>20:53</v>
+        <v>20:30</v>
       </c>
       <c r="C83" t="str">
         <v>Borrador rubro: excluir Apertura/Cierre de caja</v>
@@ -1824,10 +1824,10 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="B84" t="str">
-        <v>20:53</v>
+        <v>20:30</v>
       </c>
       <c r="C84" t="str">
         <v>Análisis financiero extracto → HTML/PDF</v>
@@ -1841,10 +1841,10 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="B85" t="str">
-        <v>20:53</v>
+        <v>20:30</v>
       </c>
       <c r="C85" t="str">
         <v>Dashboard v1.34: excluir traspasos internos del flujo</v>
@@ -1858,10 +1858,10 @@
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="B86" t="str">
-        <v>20:53</v>
+        <v>20:30</v>
       </c>
       <c r="C86" t="str">
         <v>Informe financiero PDF: MEP desde docs y textos</v>
@@ -1875,10 +1875,10 @@
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="B87" t="str">
-        <v>20:53</v>
+        <v>20:30</v>
       </c>
       <c r="C87" t="str">
         <v>Dashboard v1.35: flujo alineado al informe PDF + solapa traspasos</v>
@@ -1892,10 +1892,10 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="B88" t="str">
-        <v>20:53</v>
+        <v>20:30</v>
       </c>
       <c r="C88" t="str">
         <v>Dashboard v1.36: ARS con monto_cambio y tipo_cambio (concilia PDF)</v>
@@ -1909,10 +1909,10 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="B89" t="str">
-        <v>20:53</v>
+        <v>20:30</v>
       </c>
       <c r="C89" t="str">
         <v>Despliegue v1.37 producción</v>
@@ -1924,16 +1924,203 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>24/03/2026</v>
+      </c>
+      <c r="B90" t="str">
+        <v>20:30</v>
+      </c>
+      <c r="C90" t="str">
+        <v>Informe financiero: sección Análisis de ventas</v>
+      </c>
+      <c r="D90" t="str">
+        <v>generar-analisis-financiero-pdf.js: sección 3 con performance (total, ticket, % s/ ingresos, CV mensual), día de semana y franja horaria, ranking Usuario y Cliente, serie mensual de ventas, referencia piso vs promedio/mediana egresos operativos y último mes con ventas vs egreso operativo. Renumeración secciones 4–9.</v>
+      </c>
+      <c r="E90" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>24/03/2026</v>
+      </c>
+      <c r="B91" t="str">
+        <v>20:30</v>
+      </c>
+      <c r="C91" t="str">
+        <v>Informe financiero: compras mercadería Hornos (proxy)</v>
+      </c>
+      <c r="D91" t="str">
+        <v>generar-analisis-financiero-pdf.js: sección 4 con restricciones explícitas; egreso + cuenta Hornos; tablas categoría/día/franja/usuario/cliente/mes; cruce mensual con ventas; ingresos cuenta Hornos excluidos informativos. README extracto actualizado. Secciones 5–10.</v>
+      </c>
+      <c r="E91" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>24/03/2026</v>
+      </c>
+      <c r="B92" t="str">
+        <v>20:30</v>
+      </c>
+      <c r="C92" t="str">
+        <v>Informe financiero: considerandos y cierre por sesión</v>
+      </c>
+      <c r="D92" t="str">
+        <v>Tablas finales en ventas, compras (proxy Hornos) y análisis financiero general: columna Considerando y Qué necesitamos para cerrar el análisis; ítems dinámicos (USD sin ARS, sin MEP, meses egreso cero). Helper htmlConsiderandosCierre. README extracto.</v>
+      </c>
+      <c r="E92" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>24/03/2026</v>
+      </c>
+      <c r="B93" t="str">
+        <v>20:30</v>
+      </c>
+      <c r="C93" t="str">
+        <v>Informe financiero: ventas por semana dentro del mes</v>
+      </c>
+      <c r="D93" t="str">
+        <v>generar-analisis-financiero-pdf.js: franjas 1–7, 8–14, 15–21, 22–fin por día calendario; totales período y desglose por mes con % semana 4 s/ mes; pico y % última franja global. Considerando en cierre ventas. README.</v>
+      </c>
+      <c r="E93" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>24/03/2026</v>
+      </c>
+      <c r="B94" t="str">
+        <v>20:30</v>
+      </c>
+      <c r="C94" t="str">
+        <v>PDF captura app dashboard para instructivo</v>
+      </c>
+      <c r="D94" t="str">
+        <v>scripts/dashboard-html-a-pdf.js: PDF desde dashboard-flujo-caja.html (Playwright, ancho 1440px, alto según documento, fondos). Salida docs/Dashboard_Flujo_Caja_App.pdf; npm run dashboard-app-pdf; fallback Chrome; DASHBOARD_PDF_WAIT_MS opcional.</v>
+      </c>
+      <c r="E94" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>24/03/2026</v>
+      </c>
+      <c r="B95" t="str">
+        <v>20:30</v>
+      </c>
+      <c r="C95" t="str">
+        <v>Módulo Seguridad (roles y permisos)</v>
+      </c>
+      <c r="D95" t="str">
+        <v>SQL supabase_seguridad_forfitalia.sql y supabase_admin_inicial_forfitalia.sql (admin lucas.bustos.martin@gmail.com). Login/registro/invitado anónimo; get_my_permissions; visor = solo Flujo por mes + Exportar Base Histórica; encargado/admin panel operador; admin asigna roles y toggles en app_role_permission. Vista Seguridad en sidebar. APP_VERSION 1.38.</v>
+      </c>
+      <c r="E95" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>24/03/2026</v>
+      </c>
+      <c r="B96" t="str">
+        <v>20:30</v>
+      </c>
+      <c r="C96" t="str">
+        <v>Registro: mensaje contraseña débil Supabase</v>
+      </c>
+      <c r="D96" t="str">
+        <v>mensajeErrorAuthSupabase para texto weak password; hint bajo campo contraseña; minlength 8; catch en signUp/signInWithPassword. APP_VERSION 1.39.</v>
+      </c>
+      <c r="E96" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>24/03/2026</v>
+      </c>
+      <c r="B97" t="str">
+        <v>20:30</v>
+      </c>
+      <c r="C97" t="str">
+        <v>Seguridad: listar solo usuarios con email</v>
+      </c>
+      <c r="D97" t="str">
+        <v>get_users_for_admin filtra email vacío (invitados anónimos en user_profiles). migracion_seguridad_listar_solo_usuarios_con_email.sql + filtro en cliente. APP_VERSION 1.40.</v>
+      </c>
+      <c r="E97" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>24/03/2026</v>
+      </c>
+      <c r="B98" t="str">
+        <v>20:30</v>
+      </c>
+      <c r="C98" t="str">
+        <v>Tablas: encabezados sticky LyP</v>
+      </c>
+      <c r="D98" t="str">
+        <v>flujo-table-wrap y errores-table-wrap con scroll acotado; thead sticky en flujo, errores, todas, traspasos, excluidos, referencia flujo, evolución (z-index esquina), modales y detalle anidado. overscroll-behavior / -webkit-overflow-scrolling. APP_VERSION 1.41.</v>
+      </c>
+      <c r="E98" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>24/03/2026</v>
+      </c>
+      <c r="B99" t="str">
+        <v>20:30</v>
+      </c>
+      <c r="C99" t="str">
+        <v>Flujo: scroll hasta el final de la tabla</v>
+      </c>
+      <c r="D99" t="str">
+        <v>flujo-table-wrap sin max-height ni scroll vertical interno (solo overflow-x); overscroll-y ya no contain en errores; evolución overscroll-y auto. El párrafo informativo no estaba dentro del wrap: el problema era doble scroll + contain. APP_VERSION 1.42.</v>
+      </c>
+      <c r="E99" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>24/03/2026</v>
+      </c>
+      <c r="B100" t="str">
+        <v>20:30</v>
+      </c>
+      <c r="C100" t="str">
+        <v>Despliegue v1.43 producción</v>
+      </c>
+      <c r="D100" t="str">
+        <v>Git push main y vercel --prod: seguridad, UX registro, lista usuarios con email, tablas sticky, scroll flujo; APP_VERSION 1.43.</v>
+      </c>
+      <c r="E100" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E89"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E100"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B58"/>
+  <dimension ref="A1:B61"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -2117,295 +2304,319 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Menú lateral</v>
+        <v>Tablas y scroll</v>
       </c>
       <c r="B23" t="str">
-        <v>Sidebar izquierdo colapsable/expandible; botón toggle (▶/◀); ítem Home por ahora; estado persistido en localStorage. Listo para ampliar con más ítems.</v>
+        <v>Encabezados de columna anclados (sticky) al desplazarse. Flujo por mes: scroll vertical de la página (sin caja con max-height) para llegar bien al pie de la tabla; scroll horizontal en el wrap si hace falta. Otras solapas listas anchas con scroll horizontal.</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Repositorio Git (GitHub)</v>
+        <v>Menú lateral</v>
       </c>
       <c r="B24" t="str">
-        <v>Repo: https://github.com/lucasbustosmartin-coder/fornitalia. Rama main. .gitignore excluye node_modules, .venv, .env. Para actualizar: git add . ; git commit -m "mensaje" ; git push origin main.</v>
+        <v>Sidebar izquierdo colapsable/expandible; botón toggle (▶/◀); Home, Novedades, Configuración, Seguridad (solo admin con permiso), Cerrar sesión; estado expandido en localStorage.</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>App en producción (Vercel)</v>
+        <v>Seguridad y roles</v>
       </c>
       <c r="B25" t="str">
-        <v>URL pública: https://fornitalia.vercel.app/ (vercel.json reescribe / al dashboard). Cada push a main en GitHub dispara redeploy automático en Vercel. Proyecto: fornitalia, equipo Lucas Bustos, plan Hobby.</v>
+        <v>Login con email/contraseña, registro o invitado anónimo (visor). Permisos desde Supabase: exportar_base_historica, dashboard_operador, assign_roles. Visor: solo solapa Flujo por mes y botón Exportar Base Histórica (sin edición ni solapa Errores en modal mes). Encargado/Admin: resto del dashboard. Admin: vista Seguridad (usuarios/roles y permisos por rol). La tabla de usuarios solo muestra cuentas con email (no sesiones anónimas). Sin SQL de seguridad desplegado, la app mantiene modo compatibilidad con acceso completo.</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Exportar a Excel</v>
+        <v>Registro y contraseña</v>
       </c>
       <c r="B26" t="str">
-        <v>Botón en la barra de la tabla (solo icono). Exporta la tabla de transacciones tal como está en Supabase: una hoja "Transacciones" con columnas fecha, mes, anio, tipo_movimiento, monto (valor numérico para fórmulas), status, medio_pago, moneda, descripcion, cliente, categoria, cat_desc, origen_archivo, cuenta_contable, editado, editado_detalle. Export Errores: monto también como número. Permite analizar y usar fórmulas en Excel.</v>
+        <v>Si Supabase rechaza la contraseña (débil o en listas de filtrados), el mensaje se muestra en español en pantalla; ayuda bajo el campo y mínimo 8 caracteres en el formulario.</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Flujo de despliegue</v>
+        <v>Repositorio Git (GitHub)</v>
       </c>
       <c r="B27" t="str">
-        <v>Al terminar cada tarea: el usuario prueba en local y confirma; recién entonces el asistente hace git add, commit y push (Vercel redepliega automático). No se despliega hasta confirmación.</v>
+        <v>Repo: https://github.com/lucasbustosmartin-coder/fornitalia. Rama main. .gitignore excluye node_modules, .venv, .env. Para actualizar: git add . ; git commit -m "mensaje" ; git push origin main.</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Versiones en bitácora</v>
+        <v>App en producción (Vercel)</v>
       </c>
       <c r="B28" t="str">
-        <v>Hoja "Versiones" en Bitacora_tareas.xlsx: registro incremental (1.0, 1.1, …) con fecha y descripción de cada despliegue a Git/Vercel.</v>
+        <v>URL pública: https://fornitalia.vercel.app/ (vercel.json reescribe / al dashboard). Cada push a main en GitHub dispara redeploy automático en Vercel. Proyecto: fornitalia, equipo Lucas Bustos, plan Hobby.</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Campo moneda (BD)</v>
+        <v>Exportar a Excel</v>
       </c>
       <c r="B29" t="str">
-        <v>Columna moneda en tabla transacciones (ARS/USD). Si está informada, el dashboard la usa salvo reglas de negocio: Mercado Pago y Transferencia Morba siempre ARS para conversión (también morva por typo). Si moneda vacía, infiere desde textos/medio (dólar → USD). Export a Excel incluye moneda.</v>
+        <v>Botón en la barra de la tabla (solo icono). Exporta la tabla de transacciones tal como está en Supabase: una hoja "Transacciones" con columnas fecha, mes, anio, tipo_movimiento, monto (valor numérico para fórmulas), status, medio_pago, moneda, descripcion, cliente, categoria, cat_desc, origen_archivo, cuenta_contable, editado, editado_detalle. Export Errores: monto también como número. Permite analizar y usar fórmulas en Excel.</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Edición desde modal Errores</v>
+        <v>Flujo de despliegue</v>
       </c>
       <c r="B30" t="str">
-        <v>En el detalle de errores, icono de edición por registro. Abre modal para corregir: Categoría y Cuenta contable solo desde valores existentes en BD; Descripción libre. Al guardar se actualiza la fila y se marcan editado y editado_detalle (qué campos se editaron).</v>
+        <v>Al terminar cada tarea: el usuario prueba en local y confirma; recién entonces el asistente hace git add, commit y push (Vercel redepliega automático). No se despliega hasta confirmación.</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Campos editado y editado_detalle</v>
+        <v>Versiones en bitácora</v>
       </c>
       <c r="B31" t="str">
-        <v>En transacciones: editado (boolean) y editado_detalle (texto, ej. "Categoria, Descripcion, Cuenta Contable"). Migración supabase_transacciones_editado.sql. Export Excel los incluye.</v>
+        <v>Hoja "Versiones" en Bitacora_tareas.xlsx: registro incremental (1.0, 1.1, …) con fecha y descripción de cada despliegue a Git/Vercel.</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Tipo de error en Errores</v>
+        <v>Campo moneda (BD)</v>
       </c>
       <c r="B32" t="str">
-        <v>Tabla de errores muestra columna Tipo de error: Inconsistencia entre Categoria, Cuenta Contable y Descripcion; o Potencial registro duplicado. Export a Excel incluye tipo_error.</v>
+        <v>Columna moneda en tabla transacciones (ARS/USD). Si está informada, el dashboard la usa salvo reglas de negocio: Mercado Pago y Transferencia Morba siempre ARS para conversión (también morva por typo). Si moneda vacía, infiere desde textos/medio (dólar → USD). Export a Excel incluye moneda.</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Detección de potencial duplicado</v>
+        <v>Edición desde modal Errores</v>
       </c>
       <c r="B33" t="str">
-        <v>Registros con misma fecha, monto, tipo_movimiento y descripción similar se marcan como potencial duplicado. Icono Ver abre modal con comparación Este registro / Posible duplicado; acciones: Excluir de cálculos (anular) o Eliminar registro.</v>
+        <v>En el detalle de errores, icono de edición por registro. Abre modal para corregir: Categoría y Cuenta contable solo desde valores existentes en BD; Descripción libre. Al guardar se actualiza la fila y se marcan editado y editado_detalle (qué campos se editaron).</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Filtro por tipo de error</v>
+        <v>Campos editado y editado_detalle</v>
       </c>
       <c r="B34" t="str">
-        <v>En la solapa Errores, selector para filtrar por tipo: Todos, Inconsistencia (categoría/cuenta/descripción), Potencial registro duplicado. La exportación a Excel exporta solo los registros visibles según el filtro.</v>
+        <v>En transacciones: editado (boolean) y editado_detalle (texto, ej. "Categoria, Descripcion, Cuenta Contable"). Migración supabase_transacciones_editado.sql. Export Excel los incluye.</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Duplicados: condición cliente</v>
+        <v>Tipo de error en Errores</v>
       </c>
       <c r="B35" t="str">
-        <v>Dos registros son potencial duplicado solo si coinciden en fecha, monto, tipo_movimiento, descripción similar y además cliente es igual; si cliente es distinto no se marcan como duplicado. Modal de comparación muestra id_origen y Cliente.</v>
+        <v>Tabla de errores muestra columna Tipo de error: Inconsistencia entre Categoria, Cuenta Contable y Descripcion; o Potencial registro duplicado. Export a Excel incluye tipo_error.</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Regla bitácora</v>
+        <v>Detección de potencial duplicado</v>
       </c>
       <c r="B36" t="str">
-        <v>Actualizar todas las solapas necesarias: Log (siempre que haya tarea), Resumen (si cambia funcionalidad), Presupuesto (si agrega o cambia entregable comercial), Versiones (en despliegue). Regenerar Excel tras editar crear-bitacora-excel.js.</v>
+        <v>Registros con misma fecha, monto, tipo_movimiento y descripción similar se marcan como potencial duplicado. Icono Ver abre modal con comparación Este registro / Posible duplicado; acciones: Excluir de cálculos (anular) o Eliminar registro.</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Evolución (tabla dinámica)</v>
+        <v>Filtro por tipo de error</v>
       </c>
       <c r="B37" t="str">
-        <v>Solapa Evolución: Agrupar por = Categoría o Cuenta contable (fila); Período = Diario (fecha por día) o Mensual (MM-YYYY). Columnas = períodos, celdas = neto en moneda seleccionada, columna Total.</v>
+        <v>En la solapa Errores, selector para filtrar por tipo: Todos, Inconsistencia (categoría/cuenta/descripción), Potencial registro duplicado. La exportación a Excel exporta solo los registros visibles según el filtro.</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Evolución: detalle al clic y exportar</v>
+        <v>Duplicados: condición cliente</v>
       </c>
       <c r="B38" t="str">
-        <v>Clic en un valor de la tabla Evolución abre modal con detalle: Fecha, Categoría, Descripción, Monto. Exportar Evolución a Excel exporta la tabla según filtros Agrupar por y Período.</v>
+        <v>Dos registros son potencial duplicado solo si coinciden en fecha, monto, tipo_movimiento, descripción similar y además cliente es igual; si cliente es distinto no se marcan como duplicado. Modal de comparación muestra id_origen y Cliente.</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Exportaciones Excel</v>
+        <v>Regla bitácora</v>
       </c>
       <c r="B39" t="str">
-        <v>Todas las exportaciones incluyen una fila título con la moneda. Exportar Base Histórica (icono Excel) en la línea del selector de moneda; Exportar Evolución a Excel con el mismo icono.</v>
+        <v>Actualizar todas las solapas necesarias: Log (siempre que haya tarea), Resumen (si cambia funcionalidad), Presupuesto (si agrega o cambia entregable comercial), Versiones (en despliegue). Regenerar Excel tras editar crear-bitacora-excel.js.</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Evolución: orden ingreso/egreso</v>
+        <v>Evolución (tabla dinámica)</v>
       </c>
       <c r="B40" t="str">
-        <v>En la tabla Evolución las filas se muestran primero las de ingreso (total &gt;= 0) y luego las de egreso (total &lt; 0); dentro de cada grupo orden alfabético. Aplica tanto al agrupar por Categoría como por Cuenta contable.</v>
+        <v>Solapa Evolución: Agrupar por = Categoría o Cuenta contable (fila); Período = Diario (fecha por día) o Mensual (MM-YYYY). Columnas = períodos, celdas = neto en moneda seleccionada, columna Total.</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Int. por caución</v>
+        <v>Evolución: detalle al clic y exportar</v>
       </c>
       <c r="B41" t="str">
-        <v>Columna en flujo por mes: interés mensual por colocar el sobrante de caja a la tasa diaria de la serie de cauciones. Carga Serie_Cauciones.xlsx al refrescar (o serie_cauciones.json si no hay Excel). Cálculo: base = G/P acumulado a la fecha + interés acumulado; Int T = base × tasa. Clic en el valor abre modal con marcha (G/P acum, Int T-1, Base, Tasa, Int T).</v>
+        <v>Clic en un valor de la tabla Evolución abre modal con detalle: Fecha, Categoría, Descripción, Monto. Exportar Evolución a Excel exporta la tabla según filtros Agrupar por y Período.</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Todas las transacciones</v>
+        <v>Exportaciones Excel</v>
       </c>
       <c r="B42" t="str">
-        <v>Solapa que lista todas las transacciones con todas las columnas. Filtros por mes y categoría. Botón Editar por registro abre modal de edición completa.</v>
+        <v>Todas las exportaciones incluyen una fila título con la moneda. Exportar Base Histórica (icono Excel) en la línea del selector de moneda; Exportar Evolución a Excel con el mismo icono.</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Edición completa de registros</v>
+        <v>Evolución: orden ingreso/egreso</v>
       </c>
       <c r="B43" t="str">
-        <v>Modal de edición con todos los campos: fecha, mes, año, tipo movimiento, monto, moneda, status, medio pago, categoría, cuenta contable, origen archivo, descripción, cliente, cat_desc, id_origen, id_operación. Combos para campos normalizados (valores existentes en BD). editado y editado_detalle al guardar.</v>
+        <v>En la tabla Evolución las filas se muestran primero las de ingreso (total &gt;= 0) y luego las de egreso (total &lt; 0); dentro de cada grupo orden alfabético. Aplica tanto al agrupar por Categoría como por Cuenta contable.</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Proyección próximos 3 meses</v>
+        <v>Int. por caución</v>
       </c>
       <c r="B44" t="str">
-        <v>Debajo del total real en Flujo por mes: "Próximos 3 meses proyectados" con ventana rodante. Configuración (sidebar): método (Mediana/Promedio) y meses de historia (3, 6, 12, 24). Ingresos, egresos, G/P y ratios proyectados por mes.</v>
+        <v>Columna en flujo por mes: interés mensual por colocar el sobrante de caja a la tasa diaria de la serie de cauciones. Carga Serie_Cauciones.xlsx al refrescar (o serie_cauciones.json si no hay Excel). Cálculo: base = G/P acumulado a la fecha + interés acumulado; Int T = base × tasa. Clic en el valor abre modal con marcha (G/P acum, Int T-1, Base, Tasa, Int T).</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Int. por caución proyectado</v>
+        <v>Todas las transacciones</v>
       </c>
       <c r="B45" t="str">
-        <v>Punto de partida = G/P Total real + interés acumulado; tasa = promedio último mes real; días naturales; Int T-1 día 1 = (Int T-1 + Int T) último día del mes anterior. G/P acum en marcha = al inicio de cada día (real y proyectado). Ventana rodante: ingresos/egresos distintos por mes.</v>
+        <v>Solapa que lista todas las transacciones con todas las columnas. Filtros por mes y categoría. Botón Editar por registro abre modal de edición completa.</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Disclaimer proyección</v>
+        <v>Edición completa de registros</v>
       </c>
       <c r="B46" t="str">
-        <v>Debajo de las filas proyectadas, texto en letra chica y gris oscuro que explica la metodología: Mediana/Promedio de N meses, ventana rodante, y cálculo de Int. por caución proyectado.</v>
+        <v>Modal de edición con todos los campos: fecha, mes, año, tipo movimiento, monto, moneda, status, medio pago, categoría, cuenta contable, origen archivo, descripción, cliente, cat_desc, id_origen, id_operación. Combos para campos normalizados (valores existentes en BD). editado y editado_detalle al guardar.</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Botones e iconos unificados</v>
+        <v>Proyección próximos 3 meses</v>
       </c>
       <c r="B47" t="str">
-        <v>Todos los botones con mismo estilo: icono SVG + texto. Sidebar (chevron, home, engranaje), tabs con iconos, exportar con icono descarga, modales con iconos (Guardar, Cerrar, Excluir, Eliminar). Iconos solos (cerrar, editar, alerta) en SVG.</v>
+        <v>Debajo del total real en Flujo por mes: "Próximos 3 meses proyectados" con ventana rodante. Configuración (sidebar): método (Mediana/Promedio) y meses de historia (3, 6, 12, 24). Ingresos, egresos, G/P y ratios proyectados por mes.</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Configuración % G/P en caución</v>
+        <v>Int. por caución proyectado</v>
       </c>
       <c r="B48" t="str">
-        <v>Combo "% G/P acum. en caución" en Configuración con escala de 5 en 5 (100, 95, 90… hasta 0). Por defecto 100 %; menor % = más liquidez (menos interés por caución).</v>
+        <v>Punto de partida = G/P Total real + interés acumulado; tasa = promedio último mes real; días naturales; Int T-1 día 1 = (Int T-1 + Int T) último día del mes anterior. G/P acum en marcha = al inicio de cada día (real y proyectado). Ventana rodante: ingresos/egresos distintos por mes.</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Etiqueta Caución (x% cash)</v>
+        <v>Disclaimer proyección</v>
       </c>
       <c r="B49" t="str">
-        <v>Columna en flujo por mes: cabecera "Caución (x% cash)" donde x es el valor del parámetro % G/P; sin icono % a la izquierda. Modales de marcha y disclaimer usan "Caución".</v>
+        <v>Debajo de las filas proyectadas, texto en letra chica y gris oscuro que explica la metodología: Mediana/Promedio de N meses, ventana rodante, y cálculo de Int. por caución proyectado.</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Meses a proyectar</v>
+        <v>Botones e iconos unificados</v>
       </c>
       <c r="B50" t="str">
-        <v>En Configuración: combo Meses a proyectar (1, 2, 3, 4, 5, 6, 12). Flujo por mes y Evolución muestran esa cantidad de columnas/filas proyectadas.</v>
+        <v>Todos los botones con mismo estilo: icono SVG + texto. Sidebar (chevron, home, engranaje), tabs con iconos, exportar con icono descarga, modales con iconos (Guardar, Cerrar, Excluir, Eliminar). Iconos solos (cerrar, editar, alerta) en SVG.</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Config por usuario en Supabase</v>
+        <v>Configuración % G/P en caución</v>
       </c>
       <c r="B51" t="str">
-        <v>Tabla config_dashboard (user_id, proyección y caución). Con Auth anónimo se sincroniza al cargar y al guardar; la config persiste por usuario en la base. Migración: supabase_config_dashboard.sql.</v>
+        <v>Combo "% G/P acum. en caución" en Configuración con escala de 5 en 5 (100, 95, 90… hasta 0). Por defecto 100 %; menor % = más liquidez (menos interés por caución).</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Recorte % (cada lado)</v>
+        <v>Etiqueta Caución (x% cash)</v>
       </c>
       <c r="B52" t="str">
-        <v>En Configuración, combo Recorte % (cada lado) (0, 5, 10, 15, 20, 25) visible solo cuando el método es Promedio recortado. Más % = más suavizado. Persistido en config_dashboard (proyeccion_recorte).</v>
+        <v>Columna en flujo por mes: cabecera "Caución (x% cash)" donde x es el valor del parámetro % G/P; sin icono % a la izquierda. Modales de marcha y disclaimer usan "Caución".</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Novedades del Negocio</v>
+        <v>Meses a proyectar</v>
       </c>
       <c r="B53" t="str">
-        <v>Ítem en sidebar que abre una vista con importadores de hornos y comercios de venta de hornos en Argentina (Buenos Aires). Datos recuperados por IA (Edge Function con Gemini + google_search). Nombre, dirección, teléfono y web por contacto.</v>
+        <v>En Configuración: combo Meses a proyectar (1, 2, 3, 4, 5, 6, 12). Flujo por mes y Evolución muestran esa cantidad de columnas/filas proyectadas.</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>Normalización de extracto bancario</v>
+        <v>Config por usuario en Supabase</v>
       </c>
       <c r="B54" t="str">
-        <v>Script utilitario que normaliza el extracto Excel en una hoja estructurada (Normalizado) con campos listos para tablas: fecha_iso, tipo, medio, categoría, cuenta, moneda inferida (USD/ARS; Mercado Pago y Transferencia Morba forzados a ARS), monto_original numérico, tipo_cambio y monto_ars.</v>
+        <v>Tabla config_dashboard (user_id, proyección y caución). Con Auth anónimo se sincroniza al cargar y al guardar; la config persiste por usuario en la base. Migración: supabase_config_dashboard.sql.</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>Informe inconsistencias datos legacy (cliente)</v>
+        <v>Recorte % (cada lado)</v>
       </c>
       <c r="B55" t="str">
-        <v>Documento docs/ANALISIS_NORMALIZACION_DATOS_LEGACY_FORNITALIA.md con tablas Cant./recomendaciones; .html y .pdf en docs/. Regenerar: npm run informe-normalizacion-html o npm run informe-normalizacion-pdf (Playwright+Chromium, alineado a stack Pandi); primera vez: npx playwright install chromium.</v>
+        <v>En Configuración, combo Recorte % (cada lado) (0, 5, 10, 15, 20, 25) visible solo cuando el método es Promedio recortado. Más % = más suavizado. Persistido en config_dashboard (proyeccion_recorte).</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>Upload de extracto normalizado</v>
+        <v>Novedades del Negocio</v>
       </c>
       <c r="B56" t="str">
-        <v>Botón en la app para reemplazar transacciones desde un Excel normalizado (hoja Normalizado), con validación previa, confirmación de seguridad, generación de id_origen técnico y carga en lotes.</v>
+        <v>Ítem en sidebar que abre una vista con importadores de hornos y comercios de venta de hornos en Argentina (Buenos Aires). Datos recuperados por IA (Edge Function con Gemini + google_search). Nombre, dirección, teléfono y web por contacto.</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>Log de excluidos en upload</v>
+        <v>Normalización de extracto bancario</v>
       </c>
       <c r="B57" t="str">
-        <v>Nueva solapa Excluidos upload con registros no insertados por error o por regla de negocio (Apertura/Cierre de Caja), persistidos en Supabase para auditoría.</v>
+        <v>Script utilitario que normaliza el extracto Excel en una hoja estructurada (Normalizado) con campos listos para tablas: fecha_iso, tipo, medio, categoría, cuenta, moneda inferida (USD/ARS; Mercado Pago y Transferencia Morba forzados a ARS), monto_original numérico, tipo_cambio y monto_ars.</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
+        <v>Informe inconsistencias datos legacy (cliente)</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Documento docs/ANALISIS_NORMALIZACION_DATOS_LEGACY_FORNITALIA.md con tablas Cant./recomendaciones; .html y .pdf en docs/. Regenerar: npm run informe-normalizacion-html o npm run informe-normalizacion-pdf (Playwright+Chromium, alineado a stack Pandi); primera vez: npx playwright install chromium.</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>Upload de extracto normalizado</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Botón en la app para reemplazar transacciones desde un Excel normalizado (hoja Normalizado), con validación previa, confirmación de seguridad, generación de id_origen técnico y carga en lotes.</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>Log de excluidos en upload</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Nueva solapa Excluidos upload con registros no insertados por error o por regla de negocio (Apertura/Cierre de Caja), persistidos en Supabase para auditoría.</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
         <v>Análisis financiero extracto (PDF)</v>
       </c>
-      <c r="B58" t="str">
+      <c r="B61" t="str">
         <v>npm run analisis-financiero-pdf: métricas desde docs/Extracto-Fornitalia.xlsx; ARS vía Monto en $, TC por fila o MEP (docs/tipos_cambio_global_rows.sql o CSV); exclusiones y conteo de USD sin conversión en el informe. Ver docs/ANALISIS_FINANCIERO_EXTRACTO_README.md.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B58"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B61"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2499,7 +2710,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C40"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -2797,7 +3008,7 @@
         <v>1.25</v>
       </c>
       <c r="B27" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="C27" t="str">
         <v>Ayuda al clic en columnas Comisiones/Ventas y Egresos/Ingresos (popover con texto explicativo). Regla bitácora: tecnología e infraestructura y actualizar todas las solapas. Despliegue a producción.</v>
@@ -2808,7 +3019,7 @@
         <v>1.26</v>
       </c>
       <c r="B28" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="C28" t="str">
         <v>Mensaje de alerta de desvío: categoría en negrita sin comillas. Despliegue a producción.</v>
@@ -2819,7 +3030,7 @@
         <v>1.27</v>
       </c>
       <c r="B29" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="C29" t="str">
         <v>Novedades del Negocio: sección en sidebar con importadores y comercios de hornos en Argentina (Edge Function Gemini + google_search). Despliegue a producción.</v>
@@ -2830,7 +3041,7 @@
         <v>1.28</v>
       </c>
       <c r="B30" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="C30" t="str">
         <v>Favicon L&amp;P: L y P dada vuelta centradas en el círculo azul; ajuste de posición y centrado. Despliegue a producción.</v>
@@ -2841,7 +3052,7 @@
         <v>1.29</v>
       </c>
       <c r="B31" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="C31" t="str">
         <v>Errores: export y listado con id_origen e id_operacion; modal duplicado con id_operacion e icono en campos que no coinciden. Exclusiones duplicados: anulados, id_origen e id_operacion ambos distintos, ambos montos 0. Quitar disclaimer datos ficticios; scripts e instrucciones para repoblar transacciones desde Excel. Despliegue a producción.</v>
@@ -2852,7 +3063,7 @@
         <v>1.30</v>
       </c>
       <c r="B32" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="C32" t="str">
         <v>Errores: orden por tipo y monto descendente; filtros por categoría original y categoría mostrada. Flujo: filtro explícito status Anulado. Export Base Histórica: columnas Tipo_Cambio, Monto_ARS, Monto_USD con conversiones. Despliegue a producción.</v>
@@ -2863,7 +3074,7 @@
         <v>1.31</v>
       </c>
       <c r="B33" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="C33" t="str">
         <v>Estructura ordenada del repo: sql/, scripts/, docs/. Regla estructura-proyecto (mantener carpetas y rutas). Referencias en bitácora y docs actualizadas. Despliegue a producción.</v>
@@ -2874,7 +3085,7 @@
         <v>1.32</v>
       </c>
       <c r="B34" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="C34" t="str">
         <v>Modales: no cerrar al elegir opción de select (mousedown+click en backdrop). Helper setupBackdropCloseOnlyOnRealClick en todos los modales.</v>
@@ -2885,7 +3096,7 @@
         <v>1.33</v>
       </c>
       <c r="B35" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="C35" t="str">
         <v>Carga paginada transacciones y tipo_de_cambio (límite PostgREST). Reglas ARS Mercado Pago y Transferencia Morba en normalizador, upload y esTransaccionUSD. Upload excluidos: filtro última corrida; SQL DELETE en transacciones_upload_excluidos. Informe análisis normalización (docs MD/HTML/PDF) y scripts Playwright. DevDependency playwright y npm run playwright:install.</v>
@@ -2896,7 +3107,7 @@
         <v>1.34</v>
       </c>
       <c r="B36" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="C36" t="str">
         <v>Flujo operativo sin traspasos internos (Transferencia y Depósito); misma regla que informe PDF; nota en panel.</v>
@@ -2907,7 +3118,7 @@
         <v>1.35</v>
       </c>
       <c r="B37" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="C37" t="str">
         <v>Flujo por mes alineado al PDF: ingresos/egresos brutos extracto, Neto bruto, G/P operativo; solapa Traspasos internos; excluirFilaFlujoOperativo y Evolución con misma base.</v>
@@ -2918,7 +3129,7 @@
         <v>1.36</v>
       </c>
       <c r="B38" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="C38" t="str">
         <v>Select tipo_cambio y monto_cambio en transacciones; montoConvertido en ARS prioriza monto_cambio y TC de fila (concilia con informe PDF al centavo).</v>
@@ -2929,22 +3140,33 @@
         <v>1.37</v>
       </c>
       <c r="B39" t="str">
-        <v>22/03/2026</v>
+        <v>24/03/2026</v>
       </c>
       <c r="C39" t="str">
         <v>Despliegue a producción Vercel: informe financiero PDF con MEP desde docs; dashboard v1.37 con conciliación extracto.</v>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>1.43</v>
+      </c>
+      <c r="B40" t="str">
+        <v>24/03/2026</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Módulo Seguridad (login/registro/invitado, roles, permisos, vista Seguridad); get_users_for_admin solo email; mensajes registro Supabase; thead sticky en tablas; scroll vertical flujo por página (v1.42); APP_VERSION 1.43. Push main y Vercel producción.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C39"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C40"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="90.83203125" customWidth="1"/>
@@ -3094,21 +3316,35 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
+        <v>Seguridad y roles (dashboard)</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Autenticación email/anónimo, roles Admin/Encargado/Visor, permisos en Supabase (RPC y RLS), pantalla Seguridad para asignar roles y toggles por rol; visor restringido a Flujo por mes y exportar base histórica.</v>
+      </c>
+      <c r="C11">
+        <v>18</v>
+      </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
         <v>Mantenimiento y soporte inicial</v>
       </c>
-      <c r="B11" t="str">
+      <c r="B12" t="str">
         <v>Soporte post–implementación, pequeños ajustes funcionales y acompañamiento durante el primer período de uso.</v>
       </c>
-      <c r="C11">
+      <c r="C12">
         <v>5</v>
       </c>
-      <c r="D11">
+      <c r="D12">
         <v>500</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D12"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.49: caución alineada app/informe, tasas y serie_cauciones; bitácora y despliegue
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E100"/>
+  <dimension ref="A1:E116"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -1382,10 +1382,10 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B58" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C58" t="str">
         <v>Ayuda al clic en columnas flujo y regla bitácora</v>
@@ -1399,10 +1399,10 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B59" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C59" t="str">
         <v>Alerta desvío: categoría en negrita sin comillas</v>
@@ -1416,10 +1416,10 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B60" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C60" t="str">
         <v>Novedades del Negocio y despliegue v1.27</v>
@@ -1433,10 +1433,10 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B61" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C61" t="str">
         <v>Favicon L&amp;P centrado</v>
@@ -1450,10 +1450,10 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B62" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C62" t="str">
         <v>Despliegue v1.29</v>
@@ -1467,10 +1467,10 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B63" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C63" t="str">
         <v>Despliegue v1.30</v>
@@ -1484,10 +1484,10 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B64" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C64" t="str">
         <v>Despliegue v1.31</v>
@@ -1501,10 +1501,10 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B65" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C65" t="str">
         <v>Despliegue v1.32</v>
@@ -1518,10 +1518,10 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B66" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C66" t="str">
         <v>Normalización de Extracto Fornitalia</v>
@@ -1535,10 +1535,10 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B67" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C67" t="str">
         <v>Upload controlado de extracto normalizado en app</v>
@@ -1552,10 +1552,10 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B68" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C68" t="str">
         <v>Upload normalizado sin confirmación manual y log de excluidos</v>
@@ -1569,10 +1569,10 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B69" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C69" t="str">
         <v>Ajuste final upload: no loguear Apertura/Cierre y réplica en Everfit</v>
@@ -1586,10 +1586,10 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B70" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C70" t="str">
         <v>Limpieza de log excluidos y normalización de mes/año en carga</v>
@@ -1603,10 +1603,10 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B71" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C71" t="str">
         <v>Excluidos upload: mostrar solo última corrida y habilitar DELETE</v>
@@ -1620,10 +1620,10 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B72" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C72" t="str">
         <v>Carga paginada desde Supabase (transacciones y tipo de cambio)</v>
@@ -1637,10 +1637,10 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B73" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C73" t="str">
         <v>Reglas moneda: Mercado Pago y Transferencia Morba siempre ARS</v>
@@ -1654,10 +1654,10 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B74" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C74" t="str">
         <v>Documento análisis normalización datos legacy</v>
@@ -1671,10 +1671,10 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B75" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C75" t="str">
         <v>Informe normalización: cantidades por fila y PDF/HTML</v>
@@ -1688,10 +1688,10 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B76" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C76" t="str">
         <v>Playwright en todos los repos LyP</v>
@@ -1705,10 +1705,10 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B77" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C77" t="str">
         <v>Despliegue v1.33 producción</v>
@@ -1722,10 +1722,10 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B78" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C78" t="str">
         <v>Análisis normalización: propuesta recategorización categoría–cuenta</v>
@@ -1739,10 +1739,10 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B79" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C79" t="str">
         <v>Análisis normalización: matriz concreta Ord. n y acción Editar/Nueva/Eliminar</v>
@@ -1756,10 +1756,10 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B80" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C80" t="str">
         <v>Rubros IGJ/FACPCE y balance: doc de referencia</v>
@@ -1773,10 +1773,10 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B81" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C81" t="str">
         <v>Matriz borrador categoría–cuenta–rubro (Argentina)</v>
@@ -1790,10 +1790,10 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B82" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C82" t="str">
         <v>Análisis: §8.4 borrador rubro dentro del MD principal</v>
@@ -1807,10 +1807,10 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B83" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C83" t="str">
         <v>Borrador rubro: excluir Apertura/Cierre de caja</v>
@@ -1824,10 +1824,10 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B84" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C84" t="str">
         <v>Análisis financiero extracto → HTML/PDF</v>
@@ -1841,10 +1841,10 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B85" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C85" t="str">
         <v>Dashboard v1.34: excluir traspasos internos del flujo</v>
@@ -1858,10 +1858,10 @@
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B86" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C86" t="str">
         <v>Informe financiero PDF: MEP desde docs y textos</v>
@@ -1875,10 +1875,10 @@
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B87" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C87" t="str">
         <v>Dashboard v1.35: flujo alineado al informe PDF + solapa traspasos</v>
@@ -1892,10 +1892,10 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B88" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C88" t="str">
         <v>Dashboard v1.36: ARS con monto_cambio y tipo_cambio (concilia PDF)</v>
@@ -1909,10 +1909,10 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B89" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C89" t="str">
         <v>Despliegue v1.37 producción</v>
@@ -1926,10 +1926,10 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B90" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C90" t="str">
         <v>Informe financiero: sección Análisis de ventas</v>
@@ -1943,10 +1943,10 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B91" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C91" t="str">
         <v>Informe financiero: compras mercadería Hornos (proxy)</v>
@@ -1960,10 +1960,10 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B92" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C92" t="str">
         <v>Informe financiero: considerandos y cierre por sesión</v>
@@ -1977,10 +1977,10 @@
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B93" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C93" t="str">
         <v>Informe financiero: ventas por semana dentro del mes</v>
@@ -1994,10 +1994,10 @@
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B94" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C94" t="str">
         <v>PDF captura app dashboard para instructivo</v>
@@ -2011,10 +2011,10 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B95" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C95" t="str">
         <v>Módulo Seguridad (roles y permisos)</v>
@@ -2028,10 +2028,10 @@
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B96" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C96" t="str">
         <v>Registro: mensaje contraseña débil Supabase</v>
@@ -2045,10 +2045,10 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B97" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C97" t="str">
         <v>Seguridad: listar solo usuarios con email</v>
@@ -2062,10 +2062,10 @@
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B98" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C98" t="str">
         <v>Tablas: encabezados sticky LyP</v>
@@ -2079,10 +2079,10 @@
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B99" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C99" t="str">
         <v>Flujo: scroll hasta el final de la tabla</v>
@@ -2096,10 +2096,10 @@
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="B100" t="str">
-        <v>20:30</v>
+        <v>20:23</v>
       </c>
       <c r="C100" t="str">
         <v>Despliegue v1.43 producción</v>
@@ -2111,9 +2111,281 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>25/03/2026</v>
+      </c>
+      <c r="B101" t="str">
+        <v>20:23</v>
+      </c>
+      <c r="C101" t="str">
+        <v>Excel plan normalización para Gerencia de Sistemas</v>
+      </c>
+      <c r="D101" t="str">
+        <v>scripts/generar-excel-plan-normalizacion-desde-normalizado.js: lee docs/Extracto-Fornitalia-Normalizado.xlsx (Normalizado) y genera docs/Extracto-Fornitalia-Plan-Normalizacion-GS.xlsx con columnas marcar/recomendación (categoría, cuenta, relación cat–cuenta), medio vacío/guion, vacíos, typo comisión en texto, validaciones sugeridas por fila; hojas Validaciones_sistema y Resumen_conteos. npm run plan-normalizacion-excel.</v>
+      </c>
+      <c r="E101" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v>25/03/2026</v>
+      </c>
+      <c r="B102" t="str">
+        <v>20:23</v>
+      </c>
+      <c r="C102" t="str">
+        <v>Ventas.xlsx: normalización, conciliación e informe por vendedor</v>
+      </c>
+      <c r="D102" t="str">
+        <v>scripts/lib/ventas-auxiliar-fornitalia.js y normalizar-extracto-ventas-fornitalia.js: columna A en bloques de 7 (op, email, monto ARS, fechas serie, etiqueta, vendedor) → docs/Ventas-Normalizado.xlsx. generar-analisis-financiero-pdf.js: cruce por N° Operación con extracto, tabla conciliación, ranking ventas por vendedor real cuando aplica. npm run normalizar-ventas-excel; README extracto actualizado.</v>
+      </c>
+      <c r="E102" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>25/03/2026</v>
+      </c>
+      <c r="B103" t="str">
+        <v>20:23</v>
+      </c>
+      <c r="C103" t="str">
+        <v>Informe financiero: ventas solo extracto; diagnóstico Ventas_2</v>
+      </c>
+      <c r="D103" t="str">
+        <v>Revertido en generar-analisis-financiero-pdf.js el uso de archivo auxiliar en ranking/conciliación de ventas hasta definir fuente de verdad. scripts/diagnostico-conciliacion-ventas-2-julio.js y npm run diagnostico-ventas-2-julio: cruce julio 2025 Ventas_2 vs extracto. README extracto actualizado.</v>
+      </c>
+      <c r="E103" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v>25/03/2026</v>
+      </c>
+      <c r="B104" t="str">
+        <v>20:23</v>
+      </c>
+      <c r="C104" t="str">
+        <v>Excluir marzo 2026 (mes no cerrado) en app e informe</v>
+      </c>
+      <c r="D104" t="str">
+        <v>dashboard-flujo-caja.html: filtro tras cargar datos + nota bajo título Flujo; APP_VERSION 1.44. generar-analisis-financiero-pdf.js: omite filas marzo 2026 (Mes/Año o fecha), metadatos y considerandos. README extracto. Misma regla documentada en código para alinear con mes cerrado.</v>
+      </c>
+      <c r="E104" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>25/03/2026</v>
+      </c>
+      <c r="B105" t="str">
+        <v>20:23</v>
+      </c>
+      <c r="C105" t="str">
+        <v>Compras_v1: normalización y conciliación con extracto</v>
+      </c>
+      <c r="D105" t="str">
+        <v>Conciliación alineada al informe: solo Egreso + cuenta Hornos (misma lógica ARS/MEP que generar-analisis-financiero-pdf.js). fornitalia-informe-compras-hornos.js. Salida docs/Compras_v1-Normalizado.xlsx y docs/Extracto-Compras-Informe-Hornos.xlsx. npm run normalizar-compras-v1.</v>
+      </c>
+      <c r="E105" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>25/03/2026</v>
+      </c>
+      <c r="B106" t="str">
+        <v>20:23</v>
+      </c>
+      <c r="C106" t="str">
+        <v>Diagnóstico Fornitalia_Movimientos vs Extracto</v>
+      </c>
+      <c r="D106" t="str">
+        <v>docs/DIAGNOSTICO_FORNITALIA_MOVIMIENTOS_VS_EXTRACTO.md: comparación 3008 filas, mapa columnas, IDs (ComprobantePago, Impuesto, CierreCaja), impacto import/PDF/app/Supabase; sin reemplazo implementado.</v>
+      </c>
+      <c r="E106" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v>25/03/2026</v>
+      </c>
+      <c r="B107" t="str">
+        <v>20:23</v>
+      </c>
+      <c r="C107" t="str">
+        <v>Fuente movimientos: Fornitalia_Movimientos + canon + IDs en carga</v>
+      </c>
+      <c r="D107" t="str">
+        <v>scripts/lib/fornitalia-docs-paths.js y fornitalia-movimiento-row-canon.js. Entrada preferida docs/Fornitalia_Movimientos.xlsx; fallback Extracto-Fornitalia.xlsx. normalizar-extracto-fornitalia.js y PDF/compras/ventas/diagnóstico usan resolveMovimientosXlsxPath. Normalizado incluye id_cierre_caja, id_comprobante_pago, id_impuesto, cat_desc. dashboard upload mapea esos campos; APP_VERSION 1.45. sql/supabase_indices_transacciones_id_lookup.sql opcional. npm run normalizar-extracto.</v>
+      </c>
+      <c r="E107" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="str">
+        <v>25/03/2026</v>
+      </c>
+      <c r="B108" t="str">
+        <v>20:23</v>
+      </c>
+      <c r="C108" t="str">
+        <v>Informe normalización datos legacy: fuente y validaciones futuras</v>
+      </c>
+      <c r="D108" t="str">
+        <v>ANALISIS_NORMALIZACION_DATOS_LEGACY_FORNITALIA.md: alcance Fornitalia_Movimientos + pipeline normalizar-extracto/upload; §0 IDs/CatDesc/Status; §5 CatDesc; §7 plan GS; pie actualizado. MATRIZ y RUBROS referencia. informe-html-a-pdf.js fallback Chrome. Regenerados .html/.pdf.</v>
+      </c>
+      <c r="E108" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="str">
+        <v>25/03/2026</v>
+      </c>
+      <c r="B109" t="str">
+        <v>20:23</v>
+      </c>
+      <c r="C109" t="str">
+        <v>Informe financiero: saldo por caja al cierre de mes (ARS y USD)</v>
+      </c>
+      <c r="D109" t="str">
+        <v>generar-analisis-financiero-pdf.js: sección 6 con tablas separadas por moneda inferida; acumulado por Medio de pago hasta último día de cada mes (Ingreso +, Egreso −); USD con Monto en dólares sin TC; ARS con reglas del informe; hasta 15 medios + Otros + Total. Sección 7 aclara egresos del período vs saldo acumulado. Secciones 8–11 renumeradas. npm run analisis-financiero-pdf.</v>
+      </c>
+      <c r="E109" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="str">
+        <v>25/03/2026</v>
+      </c>
+      <c r="B110" t="str">
+        <v>20:23</v>
+      </c>
+      <c r="C110" t="str">
+        <v>Informe financiero §6: saldo caja sin conversión</v>
+      </c>
+      <c r="D110" t="str">
+        <v>Saldo por caja: ARS solo con montoNativoArsSinConversion (Monto, fallback Monto en $) — sin MEP/TC; USD solo Monto en USD. Texto HTML aclara que el apartado es moneda de registro vs resto del informe en ARS equivalente.</v>
+      </c>
+      <c r="E110" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="str">
+        <v>25/03/2026</v>
+      </c>
+      <c r="B111" t="str">
+        <v>20:23</v>
+      </c>
+      <c r="C111" t="str">
+        <v>Informe §6: medio “Efectivo Dolar” solo en tabla USD</v>
+      </c>
+      <c r="D111" t="str">
+        <v>medioNombreIndicaCajaUsd / medioNombreIndicaCajaSoloPesos: prioridad por nombre del medio en saldo por caja.</v>
+      </c>
+      <c r="E111" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="str">
+        <v>25/03/2026</v>
+      </c>
+      <c r="B112" t="str">
+        <v>20:23</v>
+      </c>
+      <c r="C112" t="str">
+        <v>Convención Pesos=ARS y Dolar=USD en inferCurrency</v>
+      </c>
+      <c r="D112" t="str">
+        <v>Helpers aplicados al inicio de inferCurrency (y §6 saldo caja); párrafo §1 moneda de origen; README extracto. Una caja/medio = una moneda en origen; alinear normalización/import.</v>
+      </c>
+      <c r="E112" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="str">
+        <v>25/03/2026</v>
+      </c>
+      <c r="B113" t="str">
+        <v>20:23</v>
+      </c>
+      <c r="C113" t="str">
+        <v>Maestro único caja→moneda (Fornitalia)</v>
+      </c>
+      <c r="D113" t="str">
+        <v>scripts/lib/fornitalia-moneda-por-medio.js: tabla Medio/Moneda (Galicia, MercadoPago, Efectivo Pesos, Morba, Credicoop, -, Galicia Dolar, Efectivo Dolar). Uso en generar-analisis-financiero-pdf.js, normalizar-extracto-fornitalia.js y dashboard MEDIO_MONEDA_FORNITALIA_TABLA + import. APP_VERSION 1.46.</v>
+      </c>
+      <c r="E113" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="str">
+        <v>25/03/2026</v>
+      </c>
+      <c r="B114" t="str">
+        <v>20:23</v>
+      </c>
+      <c r="C114" t="str">
+        <v>Caución solo ARS + informe §8 oportunidad</v>
+      </c>
+      <c r="D114" t="str">
+        <v>dashboard-flujo-caja.html v1.47: flujo/proyección caución con montos en ARS solo si moneda de origen ARS (tasas en ARS); UI y modales en pesos. generar-analisis-financiero-pdf.js: sección 8 Oportunidad de inversión no realizada (tabla mes × interés ARS, total, metodología, serie_cauciones.json); considerando si falta serie; secciones 9–12 renumeradas. npm run analisis-financiero-pdf.</v>
+      </c>
+      <c r="E114" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="str">
+        <v>25/03/2026</v>
+      </c>
+      <c r="B115" t="str">
+        <v>20:23</v>
+      </c>
+      <c r="C115" t="str">
+        <v>Caución informe = app: tasa y filtro USD</v>
+      </c>
+      <c r="D115" t="str">
+        <v>APP_VERSION 1.48. serie_cauciones.json antiguo guardaba TNA%/365 sin ÷100 (~100×): normalizeTasaCaucionDiaria en PDF y dashboard (umbral 0,02). convertir-serie-cauciones.js: fechas Date/ISO además de serial Excel. JSON regenerado desde Serie_Cauciones.xlsx. Caución PDF: esTransaccionUSDPdf + montoPesos; Moneda/CatDesc en rowToLegacyExtractoShape.</v>
+      </c>
+      <c r="E115" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="str">
+        <v>25/03/2026</v>
+      </c>
+      <c r="B116" t="str">
+        <v>20:23</v>
+      </c>
+      <c r="C116" t="str">
+        <v>Despliegue v1.49 producción</v>
+      </c>
+      <c r="D116" t="str">
+        <v>Push a main y vercel --prod: APP_VERSION 1.49; caución con normalizeTasaCaucionDiaria; informe PDF §8 alineado; serie_cauciones.json regenerado; canon Moneda/CatDesc.</v>
+      </c>
+      <c r="E116" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E100"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E116"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2139,7 +2411,7 @@
         <v>Flujo de caja por mes</v>
       </c>
       <c r="B2" t="str">
-        <v>Tabla alineada al informe financiero PDF: columnas Ingresos y Egresos = totales del extracto (incluyen traspasos entre cuentas); Neto bruto; G/P operativo sin Transferencia/Depósito ni Apertura/Cierre; ratios y Caución sobre operativo. Proyección solo sobre operativo.</v>
+        <v>Tabla alineada al informe financiero PDF: columnas Ingresos y Egresos = totales del libro de movimientos (incluyen traspasos entre cuentas); Neto bruto; G/P operativo sin Transferencia/Depósito ni Apertura/Cierre; ratios y columna Caución (mismo criterio que esTransaccionUSD, montos en pesos; tasas desde serie_cauciones.json o Serie_Cauciones.xlsx; normalización automática si el JSON está en escala antigua; % configurable). Proyección de caución en ARS con la misma base. Meses abiertos no cerrados (p. ej. marzo 2026) excluidos de la vista y del export hasta cerrar el período.</v>
       </c>
     </row>
     <row r="3">
@@ -2147,7 +2419,7 @@
         <v>Resumen global</v>
       </c>
       <c r="B3" t="str">
-        <v>Cuatro tarjetas: Ingresos totales y Egresos totales del extracto (con traspasos), Neto caja (bruto) y G/P operativo (sin traspasos internos), en ARS o USD según selector.</v>
+        <v>Cuatro tarjetas: Ingresos totales y Egresos totales del libro de movimientos (con traspasos), Neto caja (bruto) y G/P operativo (sin traspasos internos), en ARS o USD según selector.</v>
       </c>
     </row>
     <row r="4">
@@ -2155,7 +2427,7 @@
         <v>Moneda</v>
       </c>
       <c r="B4" t="str">
-        <v>Selector ARS / USD. En ARS: prioridad monto_cambio (Monto en $ del extracto en BD), tipo_cambio por fila y tabla tipo_de_cambio (MEP/CCL/Oficial); con MEP y datos cargados coincide con el informe PDF.</v>
+        <v>Selector ARS / USD. Maestro caja→moneda (medio de pago) alineado a scripts/lib/fornitalia-moneda-por-medio.js en import normalizado y en esTransaccionUSD. En ARS: prioridad monto_cambio, tipo_cambio por fila y tabla tipo_de_cambio (MEP/CCL/Oficial); con MEP y datos cargados coincide con el informe PDF.</v>
       </c>
     </row>
     <row r="5">
@@ -2579,7 +2851,7 @@
         <v>Normalización de extracto bancario</v>
       </c>
       <c r="B57" t="str">
-        <v>Script utilitario que normaliza el extracto Excel en una hoja estructurada (Normalizado) con campos listos para tablas: fecha_iso, tipo, medio, categoría, cuenta, moneda inferida (USD/ARS; Mercado Pago y Transferencia Morba forzados a ARS), monto_original numérico, tipo_cambio y monto_ars.</v>
+        <v>npm run normalizar-extracto: lee Fornitalia_Movimientos.xlsx (o Extracto legado), hoja Normalizado con fecha_iso, tipo, medio, categoría, cuenta, moneda inferida, monto_original, tipo_cambio, monto_ars, id_cierre_caja, id_comprobante_pago, id_impuesto, cat_desc cuando vienen del export.</v>
       </c>
     </row>
     <row r="58">
@@ -2587,7 +2859,7 @@
         <v>Informe inconsistencias datos legacy (cliente)</v>
       </c>
       <c r="B58" t="str">
-        <v>Documento docs/ANALISIS_NORMALIZACION_DATOS_LEGACY_FORNITALIA.md con tablas Cant./recomendaciones; .html y .pdf en docs/. Regenerar: npm run informe-normalizacion-html o npm run informe-normalizacion-pdf (Playwright+Chromium, alineado a stack Pandi); primera vez: npx playwright install chromium.</v>
+        <v>docs/ANALISIS_NORMALIZACION_DATOS_LEGACY_FORNITALIA.md alineado a Fornitalia_Movimientos.xlsx, §0 validaciones IDs/CatDesc, pipeline normalizar-extracto. Regenerar: npm run informe-normalizacion-html / informe-normalizacion-pdf; PDF con Playwright o Chrome headless (informe-html-a-pdf.js).</v>
       </c>
     </row>
     <row r="59">
@@ -2595,7 +2867,7 @@
         <v>Upload de extracto normalizado</v>
       </c>
       <c r="B59" t="str">
-        <v>Botón en la app para reemplazar transacciones desde un Excel normalizado (hoja Normalizado), con validación previa, confirmación de seguridad, generación de id_origen técnico y carga en lotes.</v>
+        <v>Botón en la app para reemplazar transacciones desde la hoja Normalizado (generada con npm run normalizar-extracto desde Fornitalia_Movimientos), con validación previa, IDs y cat_desc persistidos cuando existen, confirmación de seguridad, id_origen técnico y carga en lotes.</v>
       </c>
     </row>
     <row r="60">
@@ -2611,7 +2883,7 @@
         <v>Análisis financiero extracto (PDF)</v>
       </c>
       <c r="B61" t="str">
-        <v>npm run analisis-financiero-pdf: métricas desde docs/Extracto-Fornitalia.xlsx; ARS vía Monto en $, TC por fila o MEP (docs/tipos_cambio_global_rows.sql o CSV); exclusiones y conteo de USD sin conversión en el informe. Ver docs/ANALISIS_FINANCIERO_EXTRACTO_README.md.</v>
+        <v>npm run analisis-financiero-pdf: métricas desde Fornitalia_Movimientos.xlsx (fallback Extracto legado); ARS vía MontoCambio/Monto en $, TC por fila o MEP; exclusiones y USD sin conversión. Ver docs/ANALISIS_FINANCIERO_EXTRACTO_README.md.</v>
       </c>
     </row>
   </sheetData>
@@ -2710,7 +2982,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:C41"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -3008,7 +3280,7 @@
         <v>1.25</v>
       </c>
       <c r="B27" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="C27" t="str">
         <v>Ayuda al clic en columnas Comisiones/Ventas y Egresos/Ingresos (popover con texto explicativo). Regla bitácora: tecnología e infraestructura y actualizar todas las solapas. Despliegue a producción.</v>
@@ -3019,7 +3291,7 @@
         <v>1.26</v>
       </c>
       <c r="B28" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="C28" t="str">
         <v>Mensaje de alerta de desvío: categoría en negrita sin comillas. Despliegue a producción.</v>
@@ -3030,7 +3302,7 @@
         <v>1.27</v>
       </c>
       <c r="B29" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="C29" t="str">
         <v>Novedades del Negocio: sección en sidebar con importadores y comercios de hornos en Argentina (Edge Function Gemini + google_search). Despliegue a producción.</v>
@@ -3041,7 +3313,7 @@
         <v>1.28</v>
       </c>
       <c r="B30" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="C30" t="str">
         <v>Favicon L&amp;P: L y P dada vuelta centradas en el círculo azul; ajuste de posición y centrado. Despliegue a producción.</v>
@@ -3052,7 +3324,7 @@
         <v>1.29</v>
       </c>
       <c r="B31" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="C31" t="str">
         <v>Errores: export y listado con id_origen e id_operacion; modal duplicado con id_operacion e icono en campos que no coinciden. Exclusiones duplicados: anulados, id_origen e id_operacion ambos distintos, ambos montos 0. Quitar disclaimer datos ficticios; scripts e instrucciones para repoblar transacciones desde Excel. Despliegue a producción.</v>
@@ -3063,7 +3335,7 @@
         <v>1.30</v>
       </c>
       <c r="B32" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="C32" t="str">
         <v>Errores: orden por tipo y monto descendente; filtros por categoría original y categoría mostrada. Flujo: filtro explícito status Anulado. Export Base Histórica: columnas Tipo_Cambio, Monto_ARS, Monto_USD con conversiones. Despliegue a producción.</v>
@@ -3074,7 +3346,7 @@
         <v>1.31</v>
       </c>
       <c r="B33" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="C33" t="str">
         <v>Estructura ordenada del repo: sql/, scripts/, docs/. Regla estructura-proyecto (mantener carpetas y rutas). Referencias en bitácora y docs actualizadas. Despliegue a producción.</v>
@@ -3085,7 +3357,7 @@
         <v>1.32</v>
       </c>
       <c r="B34" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="C34" t="str">
         <v>Modales: no cerrar al elegir opción de select (mousedown+click en backdrop). Helper setupBackdropCloseOnlyOnRealClick en todos los modales.</v>
@@ -3096,7 +3368,7 @@
         <v>1.33</v>
       </c>
       <c r="B35" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="C35" t="str">
         <v>Carga paginada transacciones y tipo_de_cambio (límite PostgREST). Reglas ARS Mercado Pago y Transferencia Morba en normalizador, upload y esTransaccionUSD. Upload excluidos: filtro última corrida; SQL DELETE en transacciones_upload_excluidos. Informe análisis normalización (docs MD/HTML/PDF) y scripts Playwright. DevDependency playwright y npm run playwright:install.</v>
@@ -3107,7 +3379,7 @@
         <v>1.34</v>
       </c>
       <c r="B36" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="C36" t="str">
         <v>Flujo operativo sin traspasos internos (Transferencia y Depósito); misma regla que informe PDF; nota en panel.</v>
@@ -3118,7 +3390,7 @@
         <v>1.35</v>
       </c>
       <c r="B37" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="C37" t="str">
         <v>Flujo por mes alineado al PDF: ingresos/egresos brutos extracto, Neto bruto, G/P operativo; solapa Traspasos internos; excluirFilaFlujoOperativo y Evolución con misma base.</v>
@@ -3129,7 +3401,7 @@
         <v>1.36</v>
       </c>
       <c r="B38" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="C38" t="str">
         <v>Select tipo_cambio y monto_cambio en transacciones; montoConvertido en ARS prioriza monto_cambio y TC de fila (concilia con informe PDF al centavo).</v>
@@ -3140,7 +3412,7 @@
         <v>1.37</v>
       </c>
       <c r="B39" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="C39" t="str">
         <v>Despliegue a producción Vercel: informe financiero PDF con MEP desde docs; dashboard v1.37 con conciliación extracto.</v>
@@ -3151,15 +3423,26 @@
         <v>1.43</v>
       </c>
       <c r="B40" t="str">
-        <v>24/03/2026</v>
+        <v>25/03/2026</v>
       </c>
       <c r="C40" t="str">
         <v>Módulo Seguridad (login/registro/invitado, roles, permisos, vista Seguridad); get_users_for_admin solo email; mensajes registro Supabase; thead sticky en tablas; scroll vertical flujo por página (v1.42); APP_VERSION 1.43. Push main y Vercel producción.</v>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>1.49</v>
+      </c>
+      <c r="B41" t="str">
+        <v>25/03/2026</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Caución: normalización de escala de tasas (JSON legado vs fracción diaria Excel); informe financiero §8 coherente con app (esTransaccionUSD, montos en pesos); convertir-serie-cauciones.js con fechas Date/ISO; serie_cauciones.json alineado a Serie_Cauciones.xlsx. Despliegue a producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C40"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C41"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.57: matriz en Evolución y vistas, meses excluidos en Config, edición costo directo/indirecto, ayuda flujo en ícono, SQL meses_excluidos; bitácora.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E116"/>
+  <dimension ref="A1:E138"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -861,10 +861,10 @@
         <v>18:00</v>
       </c>
       <c r="C27" t="str">
-        <v>Excepción errores: Alquileres y Servicios / Alquiler</v>
+        <v>Excepción errores: Alquileres y Servicios / Alquiler (+ más pares)</v>
       </c>
       <c r="D27" t="str">
-        <v>Si la categoría es Alquiler (mostrada como Alquileres y Servicios) y la cuenta contable es Alquiler, se considera consistente y no entra en el log de errores de clasificación.</v>
+        <v>Alquiler o Alquileres y Servicios con cuenta Alquiler, Electricidad, Internet o Telefonia; Impuestos/IIBB; Logistica/Fletes y Transportes; Activos/Hornos; Mantenimiento/Ferreteria; Sueldos/Comisiones o Comisones Venta(s); Marketing/Creación de Contenido; Honorarios/Honorarios Contable(s). Norm sin acentos.</v>
       </c>
       <c r="E27" t="str">
         <v>Diagnostico</v>
@@ -1382,10 +1382,10 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B58" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C58" t="str">
         <v>Ayuda al clic en columnas flujo y regla bitácora</v>
@@ -1399,10 +1399,10 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B59" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C59" t="str">
         <v>Alerta desvío: categoría en negrita sin comillas</v>
@@ -1416,10 +1416,10 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B60" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C60" t="str">
         <v>Novedades del Negocio y despliegue v1.27</v>
@@ -1433,10 +1433,10 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B61" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C61" t="str">
         <v>Favicon L&amp;P centrado</v>
@@ -1450,10 +1450,10 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B62" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C62" t="str">
         <v>Despliegue v1.29</v>
@@ -1467,10 +1467,10 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B63" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C63" t="str">
         <v>Despliegue v1.30</v>
@@ -1484,10 +1484,10 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B64" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C64" t="str">
         <v>Despliegue v1.31</v>
@@ -1501,10 +1501,10 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B65" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C65" t="str">
         <v>Despliegue v1.32</v>
@@ -1518,10 +1518,10 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B66" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C66" t="str">
         <v>Normalización de Extracto Fornitalia</v>
@@ -1535,10 +1535,10 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B67" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C67" t="str">
         <v>Upload controlado de extracto normalizado en app</v>
@@ -1552,10 +1552,10 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B68" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C68" t="str">
         <v>Upload normalizado sin confirmación manual y log de excluidos</v>
@@ -1569,10 +1569,10 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B69" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C69" t="str">
         <v>Ajuste final upload: no loguear Apertura/Cierre y réplica en Everfit</v>
@@ -1586,10 +1586,10 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B70" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C70" t="str">
         <v>Limpieza de log excluidos y normalización de mes/año en carga</v>
@@ -1603,10 +1603,10 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B71" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C71" t="str">
         <v>Excluidos upload: mostrar solo última corrida y habilitar DELETE</v>
@@ -1620,10 +1620,10 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B72" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C72" t="str">
         <v>Carga paginada desde Supabase (transacciones y tipo de cambio)</v>
@@ -1637,10 +1637,10 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B73" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C73" t="str">
         <v>Reglas moneda: Mercado Pago y Transferencia Morba siempre ARS</v>
@@ -1654,10 +1654,10 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B74" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C74" t="str">
         <v>Documento análisis normalización datos legacy</v>
@@ -1671,10 +1671,10 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B75" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C75" t="str">
         <v>Informe normalización: cantidades por fila y PDF/HTML</v>
@@ -1688,10 +1688,10 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B76" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C76" t="str">
         <v>Playwright en todos los repos LyP</v>
@@ -1705,10 +1705,10 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B77" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C77" t="str">
         <v>Despliegue v1.33 producción</v>
@@ -1722,10 +1722,10 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B78" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C78" t="str">
         <v>Análisis normalización: propuesta recategorización categoría–cuenta</v>
@@ -1739,10 +1739,10 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B79" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C79" t="str">
         <v>Análisis normalización: matriz concreta Ord. n y acción Editar/Nueva/Eliminar</v>
@@ -1756,10 +1756,10 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B80" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C80" t="str">
         <v>Rubros IGJ/FACPCE y balance: doc de referencia</v>
@@ -1773,10 +1773,10 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B81" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C81" t="str">
         <v>Matriz borrador categoría–cuenta–rubro (Argentina)</v>
@@ -1790,10 +1790,10 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B82" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C82" t="str">
         <v>Análisis: §8.4 borrador rubro dentro del MD principal</v>
@@ -1807,10 +1807,10 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B83" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C83" t="str">
         <v>Borrador rubro: excluir Apertura/Cierre de caja</v>
@@ -1824,10 +1824,10 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B84" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C84" t="str">
         <v>Análisis financiero extracto → HTML/PDF</v>
@@ -1841,10 +1841,10 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B85" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C85" t="str">
         <v>Dashboard v1.34: excluir traspasos internos del flujo</v>
@@ -1858,10 +1858,10 @@
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B86" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C86" t="str">
         <v>Informe financiero PDF: MEP desde docs y textos</v>
@@ -1875,10 +1875,10 @@
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B87" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C87" t="str">
         <v>Dashboard v1.35: flujo alineado al informe PDF + solapa traspasos</v>
@@ -1892,10 +1892,10 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B88" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C88" t="str">
         <v>Dashboard v1.36: ARS con monto_cambio y tipo_cambio (concilia PDF)</v>
@@ -1909,10 +1909,10 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B89" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C89" t="str">
         <v>Despliegue v1.37 producción</v>
@@ -1926,10 +1926,10 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B90" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C90" t="str">
         <v>Informe financiero: sección Análisis de ventas</v>
@@ -1943,10 +1943,10 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B91" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C91" t="str">
         <v>Informe financiero: compras mercadería Hornos (proxy)</v>
@@ -1960,10 +1960,10 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B92" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C92" t="str">
         <v>Informe financiero: considerandos y cierre por sesión</v>
@@ -1977,10 +1977,10 @@
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B93" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C93" t="str">
         <v>Informe financiero: ventas por semana dentro del mes</v>
@@ -1994,10 +1994,10 @@
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B94" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C94" t="str">
         <v>PDF captura app dashboard para instructivo</v>
@@ -2011,10 +2011,10 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B95" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C95" t="str">
         <v>Módulo Seguridad (roles y permisos)</v>
@@ -2028,10 +2028,10 @@
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B96" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C96" t="str">
         <v>Registro: mensaje contraseña débil Supabase</v>
@@ -2045,10 +2045,10 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B97" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C97" t="str">
         <v>Seguridad: listar solo usuarios con email</v>
@@ -2062,10 +2062,10 @@
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B98" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C98" t="str">
         <v>Tablas: encabezados sticky LyP</v>
@@ -2079,10 +2079,10 @@
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B99" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C99" t="str">
         <v>Flujo: scroll hasta el final de la tabla</v>
@@ -2096,10 +2096,10 @@
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B100" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C100" t="str">
         <v>Despliegue v1.43 producción</v>
@@ -2113,10 +2113,10 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B101" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C101" t="str">
         <v>Excel plan normalización para Gerencia de Sistemas</v>
@@ -2130,10 +2130,10 @@
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B102" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C102" t="str">
         <v>Ventas.xlsx: normalización, conciliación e informe por vendedor</v>
@@ -2147,10 +2147,10 @@
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B103" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C103" t="str">
         <v>Informe financiero: ventas solo extracto; diagnóstico Ventas_2</v>
@@ -2164,10 +2164,10 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B104" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C104" t="str">
         <v>Excluir marzo 2026 (mes no cerrado) en app e informe</v>
@@ -2181,10 +2181,10 @@
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B105" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C105" t="str">
         <v>Compras_v1: normalización y conciliación con extracto</v>
@@ -2198,10 +2198,10 @@
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B106" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C106" t="str">
         <v>Diagnóstico Fornitalia_Movimientos vs Extracto</v>
@@ -2215,10 +2215,10 @@
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B107" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C107" t="str">
         <v>Fuente movimientos: Fornitalia_Movimientos + canon + IDs en carga</v>
@@ -2232,10 +2232,10 @@
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B108" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C108" t="str">
         <v>Informe normalización datos legacy: fuente y validaciones futuras</v>
@@ -2249,10 +2249,10 @@
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B109" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C109" t="str">
         <v>Informe financiero: saldo por caja al cierre de mes (ARS y USD)</v>
@@ -2266,10 +2266,10 @@
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B110" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C110" t="str">
         <v>Informe financiero §6: saldo caja sin conversión</v>
@@ -2283,10 +2283,10 @@
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B111" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C111" t="str">
         <v>Informe §6: medio “Efectivo Dolar” solo en tabla USD</v>
@@ -2300,10 +2300,10 @@
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B112" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C112" t="str">
         <v>Convención Pesos=ARS y Dolar=USD en inferCurrency</v>
@@ -2317,10 +2317,10 @@
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B113" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C113" t="str">
         <v>Maestro único caja→moneda (Fornitalia)</v>
@@ -2334,10 +2334,10 @@
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B114" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C114" t="str">
         <v>Caución solo ARS + informe §8 oportunidad</v>
@@ -2351,10 +2351,10 @@
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B115" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C115" t="str">
         <v>Caución informe = app: tasa y filtro USD</v>
@@ -2368,10 +2368,10 @@
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="B116" t="str">
-        <v>20:23</v>
+        <v>12:54</v>
       </c>
       <c r="C116" t="str">
         <v>Despliegue v1.49 producción</v>
@@ -2383,16 +2383,390 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="117">
+      <c r="A117" t="str">
+        <v>08/05/2026</v>
+      </c>
+      <c r="B117" t="str">
+        <v>12:54</v>
+      </c>
+      <c r="C117" t="str">
+        <v>Base Fornitalia Compras vs movimientos</v>
+      </c>
+      <c r="D117" t="str">
+        <v>docs/Base Fornitalia Compras.xlsx (Compras+Detalle). scripts/lib/fornitalia-base-compras.js y fornitalia-docs-paths resolveBaseComprasXlsxPath. procesarMovimientosEgresosOperativosCaja en fornitalia-informe-compras-hornos.js. conciliar-base-compras-movimientos.js → docs/Base-Compras-Conciliacion-Caja.xlsx. npm run conciliar-base-compras. README extracto.</v>
+      </c>
+      <c r="E117" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="str">
+        <v>08/05/2026</v>
+      </c>
+      <c r="B118" t="str">
+        <v>12:54</v>
+      </c>
+      <c r="C118" t="str">
+        <v>Informe normalización: §5.1 uso por usuario</v>
+      </c>
+      <c r="D118" t="str">
+        <v>ANALISIS_NORMALIZACION_DATOS_LEGACY_FORNITALIA.md: subsección estadística distribución por usuario (no anulados). scripts/actualizar-seccion-usuario-informe-normalizacion.js; npm run informe-normalizacion actualiza tabla desde Fornitalia_Movimientos.xlsx.</v>
+      </c>
+      <c r="E118" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="str">
+        <v>08/05/2026</v>
+      </c>
+      <c r="B119" t="str">
+        <v>12:54</v>
+      </c>
+      <c r="C119" t="str">
+        <v>Compras Excel sistemas: normalización y cruce con base</v>
+      </c>
+      <c r="D119" t="str">
+        <v>scripts/lib/fornitalia-fecha-argentina.js: fechas Argentina (dd/mm/yyyy texto, serial Excel, ISO) alineadas a Base Compras y extracto. normalizar-compras-excel-sistemas.js → docs/Compras-Excel-Sistemas-Normalizado.xlsx desde docs/Excel/Compras.xlsx. conciliar-compras-sistemas-vs-base.js → docs/Compras-Sistemas-vs-Base.xlsx (join por ID con Base Fornitalia Compras). normalizar-extracto-fornitalia.js delega fecha_iso en la misma función. resolveComprasExcelSistemasPath en fornitalia-docs-paths. npm run normalizar-compras-excel-sistemas; npm run conciliar-compras-sistemas-vs-base.</v>
+      </c>
+      <c r="E119" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="str">
+        <v>08/05/2026</v>
+      </c>
+      <c r="B120" t="str">
+        <v>12:54</v>
+      </c>
+      <c r="C120" t="str">
+        <v>Base compras enriquecida desde export sistemas</v>
+      </c>
+      <c r="D120" t="str">
+        <v>fornitalia-compras-sistemas-extra.js: columnas VersionApp_CO, Creado por, Creado, Modificado, Tipo de elemento por ID. excelSerialToIsoDateTime en fornitalia-fecha-argentina. enriquecer-base-compras-desde-excel-sistemas.js → docs/Base-Fornitalia-Compras-Enriquecida.xlsx (Compras ampliada + Creado_ISO/Modificado_ISO + Enriquecido_sistemas; Detalle copiado). loadBaseFornitaliaCompras(..., { mergeSistemasXlsxPath }) opcional. npm run enriquecer-base-compras-sistemas.</v>
+      </c>
+      <c r="E120" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="str">
+        <v>08/05/2026</v>
+      </c>
+      <c r="B121" t="str">
+        <v>12:54</v>
+      </c>
+      <c r="C121" t="str">
+        <v>Compras sistemas vs movimientos (Supabase)</v>
+      </c>
+      <c r="D121" t="str">
+        <v>conciliar-compras-sistemas-transacciones.js: ID=nro_operacion; Egreso; suma ARS sin Impuestos vs TotalBruto; Percepciones_Impuesto_Compras (IDCompra_PIC) suma Importe_PIC; Diferencia_mas_percepciones_PIC y Concilia_ajustada_PIC; resolvePercepcionesImpuestoComprasPath. → docs/Compras-Sistemas-vs-Transacciones.xlsx. npm run conciliar-compras-sistemas-transacciones.</v>
+      </c>
+      <c r="E121" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="str">
+        <v>08/05/2026</v>
+      </c>
+      <c r="B122" t="str">
+        <v>12:54</v>
+      </c>
+      <c r="C122" t="str">
+        <v>Detalle operaciones ventas: normalización e informe PDF</v>
+      </c>
+      <c r="D122" t="str">
+        <v>docs/Excel/Detalle_De_Operaciones + Resumen_Operaciones: líneas Status Activo, Tipo_RO Venta (no cotización), operación no anulada en resumen; ranking top 15 productos por Total_DO y % sobre total detalle en generar-analisis-financiero-pdf.js (sección Análisis de ventas). scripts/lib/fornitalia-detalle-operaciones-ventas.js; normalizar-detalle-operaciones-ventas.js → docs/Detalle-Operaciones-Ventas-Normalizado.xlsx; rutas FORNITALIA_DETALLE_OPERACIONES_XLSX / FORNITALIA_RESUMEN_OPERACIONES_XLSX opcionales.</v>
+      </c>
+      <c r="E122" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="str">
+        <v>08/05/2026</v>
+      </c>
+      <c r="B123" t="str">
+        <v>12:54</v>
+      </c>
+      <c r="C123" t="str">
+        <v>Conciliación detalle ventas vs movimientos por ID operación</v>
+      </c>
+      <c r="D123" t="str">
+        <v>conciliar-detalle-ventas-movimientos.js: suma Total_DO por IDOperacion_DO vs suma ARS (Ingreso Ventas, mismo monto ARS que informe PDF) por N° Operación; columna Concilia Y/N con tolerancia 1 ARS. Salida docs/Detalle-Ventas-vs-Movimientos-Conciliacion.xlsx (Por_operacion, Resumen, Ventas_sin_ID_operacion). lib/fornitalia-monto-ars-informe-pdf.js. npm run conciliar-detalle-ventas-movimientos.</v>
+      </c>
+      <c r="E123" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="str">
+        <v>08/05/2026</v>
+      </c>
+      <c r="B124" t="str">
+        <v>12:54</v>
+      </c>
+      <c r="C124" t="str">
+        <v>Ranking productos proxy: cierre feb 2026 y % sobre extracto</v>
+      </c>
+      <c r="D124" t="str">
+        <v>Detalle operaciones: solo operaciones con mes en resumen ≤ 2026-02 (excl. marzo en adelante). Informe PDF: monto proxy = % composición Total_DO del detalle (período) × total ventas extracto hasta ese mes; tabla y considerandos actualizados. MES_CLAVE_MAX_VENTAS_CIERRE en fornitalia-detalle-operaciones-ventas.js. normalizar-detalle y conciliar con mismo filtro de mes.</v>
+      </c>
+      <c r="E124" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="str">
+        <v>08/05/2026</v>
+      </c>
+      <c r="B125" t="str">
+        <v>12:54</v>
+      </c>
+      <c r="C125" t="str">
+        <v>Informe PDF: ranking por vendedor (Resumen_Operaciones)</v>
+      </c>
+      <c r="D125" t="str">
+        <v>Reemplazo del ranking por Usuario del extracto: fornitalia-resumen-operaciones-vendedor.js lee Tabla (Vendedor_RO, Tipo Venta, no anulado), cruce por N° operación = ID. generar-analisis-financiero-pdf.js: rankVendedores y sección «Ranking por vendedor (resumen operaciones)».</v>
+      </c>
+      <c r="E125" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="str">
+        <v>08/05/2026</v>
+      </c>
+      <c r="B126" t="str">
+        <v>12:54</v>
+      </c>
+      <c r="C126" t="str">
+        <v>Informe normalización §8.4: matriz desde Exportación cuentas v2</v>
+      </c>
+      <c r="D126" t="str">
+        <v>scripts/actualizar-seccion-84-matriz-normalizacion.js lee docs/Exportación_cuentas_contables_v2.xlsx (Matriz_Cuenta_Contable_Balance + Cuentas contables) y reemplaza la tabla del §8.4 en ANALISIS_NORMALIZACION_DATOS_LEGACY_FORNITALIA.md entre marcadores; Dudas cuando Categoría vacía; nota revisión contador/a. Intro y comando regeneración en el .md.</v>
+      </c>
+      <c r="E126" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="str">
+        <v>08/05/2026</v>
+      </c>
+      <c r="B127" t="str">
+        <v>12:54</v>
+      </c>
+      <c r="C127" t="str">
+        <v>Informe normalización: npm siempre genera PDF</v>
+      </c>
+      <c r="D127" t="str">
+        <v>package.json: informe-normalizacion ejecuta §84 + usuario + HTML + Playwright PDF; informe-normalizacion-html y -pdf delegan en el mismo; informe-normalizacion-solo-html sin PDF. Documentación y script usuario actualizados.</v>
+      </c>
+      <c r="E127" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="str">
+        <v>08/05/2026</v>
+      </c>
+      <c r="B128" t="str">
+        <v>12:54</v>
+      </c>
+      <c r="C128" t="str">
+        <v>Informe §8.4: columnas Nombre/Rama/Categoría Balance</v>
+      </c>
+      <c r="D128" t="str">
+        <v>actualizar-seccion-84-matriz-normalizacion.js: tabla con Nombre Balance, Rama Balance y Categoría Balance (Excel Nombre, Rama, Categoría) antes de Dudas; intro §8.4 actualizada.</v>
+      </c>
+      <c r="E128" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="str">
+        <v>08/05/2026</v>
+      </c>
+      <c r="B129" t="str">
+        <v>12:54</v>
+      </c>
+      <c r="C129" t="str">
+        <v>Dashboard: edición errores — feedback guardado Supabase</v>
+      </c>
+      <c r="D129" t="str">
+        <v>Modal editar: aviso si no hay cambios (antes cerraba sin UPDATE a transacciones); validación id y .select tras update si 0 filas; nota contextual inconsistencia categoría/cuenta/descripción. APP_VERSION 1.50.</v>
+      </c>
+      <c r="E129" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="str">
+        <v>08/05/2026</v>
+      </c>
+      <c r="B130" t="str">
+        <v>12:54</v>
+      </c>
+      <c r="C130" t="str">
+        <v>Dashboard: refresh tras guardar edición</v>
+      </c>
+      <c r="D130" t="str">
+        <v>Tras UPDATE: await cargarDatos antes de cerrar modal editar; try/catch si falla recarga; si el modal del mes sigue abierto, abrirModal de nuevo con ultimoModalMesAnio/Mes para regenerar HTML (By Categoria / detalle). APP_VERSION 1.51.</v>
+      </c>
+      <c r="E130" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="str">
+        <v>08/05/2026</v>
+      </c>
+      <c r="B131" t="str">
+        <v>12:54</v>
+      </c>
+      <c r="C131" t="str">
+        <v>Errores clasificación: exclusiones cat/cuenta</v>
+      </c>
+      <c r="D131" t="str">
+        <v>esParCategoriaCuentaExcluidoErrores: Impuestos/IIBB; Logistica/Fletes y Transportes; Alquiler o Alquileres y Servicios con Alquiler Electricidad Internet Telefonia; Activos/Hornos; Mantenimiento o Manteniemiento/Ferreteria (norm sin acentos). APP_VERSION 1.52.</v>
+      </c>
+      <c r="E131" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="str">
+        <v>08/05/2026</v>
+      </c>
+      <c r="B132" t="str">
+        <v>12:54</v>
+      </c>
+      <c r="C132" t="str">
+        <v>Errores clasificación: más exclusiones cat/cuenta</v>
+      </c>
+      <c r="D132" t="str">
+        <v>Sueldos + Comisiones/Comisones Venta(s) y typo Comisoiones Venta; Marketing + Creación de Contenido; Honorarios + Honorarios Contable(s). APP_VERSION 1.53.</v>
+      </c>
+      <c r="E132" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="str">
+        <v>08/05/2026</v>
+      </c>
+      <c r="B133" t="str">
+        <v>12:54</v>
+      </c>
+      <c r="C133" t="str">
+        <v>Todas las transacciones: filtro cuenta contable</v>
+      </c>
+      <c r="D133" t="str">
+        <v>Select filtro-todas-cuenta-contable; opciones únicas desde cache (vacío → Sin cuenta contable); combina con mes/categoría/tipo/id operación. APP_VERSION 1.54.</v>
+      </c>
+      <c r="E133" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="str">
+        <v>08/05/2026</v>
+      </c>
+      <c r="B134" t="str">
+        <v>12:54</v>
+      </c>
+      <c r="C134" t="str">
+        <v>Dashboard: vistas con categoría/cuenta de matriz</v>
+      </c>
+      <c r="D134" t="str">
+        <v>Evolución y export agrupan por nueva_categoria / nueva_cuenta_contable con fallback (helpers categoriaDistribucionFlujo / cuentaDistribucionFlujo). Proyección flujo por mes y alertas de desvío % coherentes con matriz. Todas las transacciones: filtros y columnas principales por matriz; columnas BD nueva_* aparte. Traspasos: categoría/cuenta extracto + matriz. Errores: columnas y filtro por matriz; export Excel categoria_matriz y cuenta_matriz. Modal mes: pestañas y tablas etiquetadas matriz; modal proyección encabezado agrupación (matriz).</v>
+      </c>
+      <c r="E134" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="str">
+        <v>08/05/2026</v>
+      </c>
+      <c r="B135" t="str">
+        <v>12:54</v>
+      </c>
+      <c r="C135" t="str">
+        <v>Config: excluir meses de totales y flujo</v>
+      </c>
+      <c r="D135" t="str">
+        <v>Inclusión por mes en Configuración: interruptores por mes con datos; meses_excluidos en localStorage y Supabase (sql/supabase_config_dashboard_meses_excluidos.sql). Cache completo; excluirFilaFlujoOperativo incluye mes excluido. Default legacy marzo 2026 sin preferencia. Duplicados sin filtro por mes. APP_VERSION 1.55.</v>
+      </c>
+      <c r="E135" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="str">
+        <v>08/05/2026</v>
+      </c>
+      <c r="B136" t="str">
+        <v>12:54</v>
+      </c>
+      <c r="C136" t="str">
+        <v>Modal editar: costo directo e indirecto</v>
+      </c>
+      <c r="D136" t="str">
+        <v>Select Y/N/vacío para costo_directo y costo_indirecto; UPDATE en transacciones y editado_detalle. APP_VERSION 1.56.</v>
+      </c>
+      <c r="E136" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="str">
+        <v>08/05/2026</v>
+      </c>
+      <c r="B137" t="str">
+        <v>12:54</v>
+      </c>
+      <c r="C137" t="str">
+        <v>Flujo por mes: ayuda informe PDF en icono</v>
+      </c>
+      <c r="D137" t="str">
+        <v>Texto largo reemplazado por botón th-help--inline; popover enriquecido desde template template-flujo-informe-pdf (data-help-template).</v>
+      </c>
+      <c r="E137" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="str">
+        <v>08/05/2026</v>
+      </c>
+      <c r="B138" t="str">
+        <v>12:54</v>
+      </c>
+      <c r="C138" t="str">
+        <v>Excel Categoria_CCSis: solapa resumen sin duplicar</v>
+      </c>
+      <c r="D138" t="str">
+        <v>scripts/completar-matriz-ccsis-desde-normalizado.js: solapa Resumen_Confirmados_cat_cuenta (categoria, cuenta_contable, # Registros, Monto_ARS) agregado único desde Extracto-Fornitalia-Normalizado solo Confirmado; no modifica solapas Matriz_*. npm run completar-matriz-ccsis-normalizado.</v>
+      </c>
+      <c r="E138" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E116"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E138"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B61"/>
+  <dimension ref="A1:B62"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -2411,7 +2785,7 @@
         <v>Flujo de caja por mes</v>
       </c>
       <c r="B2" t="str">
-        <v>Tabla alineada al informe financiero PDF: columnas Ingresos y Egresos = totales del libro de movimientos (incluyen traspasos entre cuentas); Neto bruto; G/P operativo sin Transferencia/Depósito ni Apertura/Cierre; ratios y columna Caución (mismo criterio que esTransaccionUSD, montos en pesos; tasas desde serie_cauciones.json o Serie_Cauciones.xlsx; normalización automática si el JSON está en escala antigua; % configurable). Proyección de caución en ARS con la misma base. Meses abiertos no cerrados (p. ej. marzo 2026) excluidos de la vista y del export hasta cerrar el período.</v>
+        <v>Tabla alineada al informe financiero PDF: columnas Ingresos y Egresos = totales del libro de movimientos (incluyen traspasos entre cuentas); Neto bruto; G/P operativo sin Transferencia/Depósito ni Apertura/Cierre; ratios y columna Caución (mismo criterio que esTransaccionUSD, montos en pesos; tasas desde serie_cauciones.json o Serie_Cauciones.xlsx; normalización automática si el JSON está en escala antigua; % configurable). Proyección de caución en ARS con la misma base. Meses excluidos por Configuración → Inclusión por mes no aparecen en filas ni totales agregados. Icono de ayuda discreto sobre la tabla abre el texto detallado de alineación al PDF (popover).</v>
       </c>
     </row>
     <row r="3">
@@ -2475,23 +2849,23 @@
         <v>Detalle por mes</v>
       </c>
       <c r="B10" t="str">
-        <v>Clic en una fila de mes abre modal con dos solapas: By Categoria y By Cuenta Contable.</v>
+        <v>Clic en una fila de mes abre modal con dos solapas: por categoría (matriz) y por cuenta (matriz).</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>By Categoria</v>
+        <v>Por categoría (matriz)</v>
       </c>
       <c r="B11" t="str">
-        <v>Solapa del modal: detalle agrupado por categoría (Sueldos, Comisiones, etc.) con botón Ver para listado de transacciones.</v>
+        <v>Solapa del modal: detalle agrupado por nueva_categoria con fallback a extracto/validación (categoriaDistribucionFlujo); bloques Ingresos / Costo directo / indirecto / Otros costos; Ver para listado de transacciones.</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>By Cuenta Contable</v>
+        <v>Por cuenta (matriz)</v>
       </c>
       <c r="B12" t="str">
-        <v>Solapa del modal: detalle agrupado por cuenta_contable; misma tabla con Monto y Ver para ver transacciones.</v>
+        <v>Solapa del modal: detalle agrupado por nueva_cuenta_contable con fallback (cuentaDistribucionFlujo); misma estructura y botón Gráfico.</v>
       </c>
     </row>
     <row r="13">
@@ -2499,7 +2873,7 @@
         <v>Gráfico serie mensual</v>
       </c>
       <c r="B13" t="str">
-        <v>Botón "Gráfico" en cada fila de categoría/cuenta: abre modal con gráfico de barras de la serie mensual (neto por mes) para esa categoría o cuenta, en la moneda seleccionada.</v>
+        <v>Botón "Gráfico" en cada fila de categoría o cuenta de matriz: modal con serie mensual (neto por mes) para esa clave, en la moneda seleccionada.</v>
       </c>
     </row>
     <row r="14">
@@ -2539,356 +2913,364 @@
         <v>Alertas por mes</v>
       </c>
       <c r="B18" t="str">
-        <v>Avisos: mes sin egresos; sin registros de Sueldos, Comisiones, Alquileres o Impuestos; desvío % de categoría vs mes anterior.</v>
+        <v>Avisos: mes sin egresos; sin registros de Sueldos, Comisiones, Alquileres o Impuestos; desvío % de categoría (matriz) vs mes anterior.</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Sin cotización</v>
+        <v>Inclusión por mes (Configuración)</v>
       </c>
       <c r="B19" t="str">
-        <v>Pestaña con transacciones que no tienen tipo de cambio (excluidas del resumen).</v>
+        <v>Interruptores por cada mes con movimientos: incluir o excluir del flujo por mes, tarjetas de resumen, Evolución, Caución y agregados que usan excluirFilaFlujoOperativo. Persistencia localStorage y columna meses_excluidos en config_dashboard. Sin afectar duplicados ni export de base histórica.</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Exclusiones (flujo operativo)</v>
+        <v>Sin cotización</v>
       </c>
       <c r="B20" t="str">
-        <v>No se incluyen en G/P operativo, Evolución ni Caución: anulados; apertura/cierre (categoría o heurística en fila); Transferencia ni Deposito/Depósito. Los traspasos se listan en la solapa Traspasos internos. Base histórica y Todas las transacciones siguen completas.</v>
+        <v>Pestaña con transacciones que no tienen tipo de cambio (excluidas del resumen).</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Traspasos internos (solapa)</v>
+        <v>Exclusiones (flujo operativo)</v>
       </c>
       <c r="B21" t="str">
-        <v>Listado de movimientos categoría Transferencia o Deposito/Depósito (no anulados), con monto de registro y equivalente en moneda de vista.</v>
+        <v>No se incluyen en G/P operativo, Evolución ni Caución: anulados; apertura/cierre (categoría o heurística en fila); Transferencia ni Deposito/Depósito; meses desmarcados en Configuración → Inclusión por mes (meses_excluidos en Supabase/localStorage). Traspasos en solapa dedicada. Base histórica y Todas las transacciones siguen completas.</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Datos</v>
+        <v>Traspasos internos (solapa)</v>
       </c>
       <c r="B22" t="str">
-        <v>Transacciones y tipo de cambio desde Supabase (carga paginada de a 1000 filas por request para no truncar resultados). Cotización faltante: se usa la fecha anterior disponible.</v>
+        <v>Listado de movimientos con categoría extracto Transferencia o Deposito/Depósito (no anulados), con monto de registro y equivalente en moneda de vista; columnas extracto y categoría/cuenta de matriz (nueva en BD o fallback).</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Tablas y scroll</v>
+        <v>Datos</v>
       </c>
       <c r="B23" t="str">
-        <v>Encabezados de columna anclados (sticky) al desplazarse. Flujo por mes: scroll vertical de la página (sin caja con max-height) para llegar bien al pie de la tabla; scroll horizontal en el wrap si hace falta. Otras solapas listas anchas con scroll horizontal.</v>
+        <v>Transacciones y tipo de cambio desde Supabase (carga paginada de a 1000 filas por request para no truncar resultados). Cotización faltante: se usa la fecha anterior disponible.</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Menú lateral</v>
+        <v>Tablas y scroll</v>
       </c>
       <c r="B24" t="str">
-        <v>Sidebar izquierdo colapsable/expandible; botón toggle (▶/◀); Home, Novedades, Configuración, Seguridad (solo admin con permiso), Cerrar sesión; estado expandido en localStorage.</v>
+        <v>Encabezados de columna anclados (sticky) al desplazarse. Flujo por mes: scroll vertical de la página (sin caja con max-height) para llegar bien al pie de la tabla; scroll horizontal en el wrap si hace falta. Otras solapas listas anchas con scroll horizontal.</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Seguridad y roles</v>
+        <v>Menú lateral</v>
       </c>
       <c r="B25" t="str">
-        <v>Login con email/contraseña, registro o invitado anónimo (visor). Permisos desde Supabase: exportar_base_historica, dashboard_operador, assign_roles. Visor: solo solapa Flujo por mes y botón Exportar Base Histórica (sin edición ni solapa Errores en modal mes). Encargado/Admin: resto del dashboard. Admin: vista Seguridad (usuarios/roles y permisos por rol). La tabla de usuarios solo muestra cuentas con email (no sesiones anónimas). Sin SQL de seguridad desplegado, la app mantiene modo compatibilidad con acceso completo.</v>
+        <v>Sidebar izquierdo colapsable/expandible; botón toggle (▶/◀); Home, Novedades, Configuración, Seguridad (solo admin con permiso), Cerrar sesión; estado expandido en localStorage.</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Registro y contraseña</v>
+        <v>Seguridad y roles</v>
       </c>
       <c r="B26" t="str">
-        <v>Si Supabase rechaza la contraseña (débil o en listas de filtrados), el mensaje se muestra en español en pantalla; ayuda bajo el campo y mínimo 8 caracteres en el formulario.</v>
+        <v>Login con email/contraseña, registro o invitado anónimo (visor). Permisos desde Supabase: exportar_base_historica, dashboard_operador, assign_roles. Visor: solo solapa Flujo por mes y botón Exportar Base Histórica (sin edición ni solapa Errores en modal mes). Encargado/Admin: resto del dashboard. Admin: vista Seguridad (usuarios/roles y permisos por rol). La tabla de usuarios solo muestra cuentas con email (no sesiones anónimas). Sin SQL de seguridad desplegado, la app mantiene modo compatibilidad con acceso completo.</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Repositorio Git (GitHub)</v>
+        <v>Registro y contraseña</v>
       </c>
       <c r="B27" t="str">
-        <v>Repo: https://github.com/lucasbustosmartin-coder/fornitalia. Rama main. .gitignore excluye node_modules, .venv, .env. Para actualizar: git add . ; git commit -m "mensaje" ; git push origin main.</v>
+        <v>Si Supabase rechaza la contraseña (débil o en listas de filtrados), el mensaje se muestra en español en pantalla; ayuda bajo el campo y mínimo 8 caracteres en el formulario.</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>App en producción (Vercel)</v>
+        <v>Repositorio Git (GitHub)</v>
       </c>
       <c r="B28" t="str">
-        <v>URL pública: https://fornitalia.vercel.app/ (vercel.json reescribe / al dashboard). Cada push a main en GitHub dispara redeploy automático en Vercel. Proyecto: fornitalia, equipo Lucas Bustos, plan Hobby.</v>
+        <v>Repo: https://github.com/lucasbustosmartin-coder/fornitalia. Rama main. .gitignore excluye node_modules, .venv, .env. Para actualizar: git add . ; git commit -m "mensaje" ; git push origin main.</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Exportar a Excel</v>
+        <v>App en producción (Vercel)</v>
       </c>
       <c r="B29" t="str">
-        <v>Botón en la barra de la tabla (solo icono). Exporta la tabla de transacciones tal como está en Supabase: una hoja "Transacciones" con columnas fecha, mes, anio, tipo_movimiento, monto (valor numérico para fórmulas), status, medio_pago, moneda, descripcion, cliente, categoria, cat_desc, origen_archivo, cuenta_contable, editado, editado_detalle. Export Errores: monto también como número. Permite analizar y usar fórmulas en Excel.</v>
+        <v>URL pública: https://fornitalia.vercel.app/ (vercel.json reescribe / al dashboard). Cada push a main en GitHub dispara redeploy automático en Vercel. Proyecto: fornitalia, equipo Lucas Bustos, plan Hobby.</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Flujo de despliegue</v>
+        <v>Exportar a Excel</v>
       </c>
       <c r="B30" t="str">
-        <v>Al terminar cada tarea: el usuario prueba en local y confirma; recién entonces el asistente hace git add, commit y push (Vercel redepliega automático). No se despliega hasta confirmación.</v>
+        <v>Botón en la barra de la tabla (solo icono). Exporta la tabla de transacciones tal como está en Supabase: una hoja "Transacciones" con columnas fecha, mes, anio, tipo_movimiento, monto (valor numérico para fórmulas), status, medio_pago, moneda, descripcion, cliente, categoria, cat_desc, origen_archivo, cuenta_contable, editado, editado_detalle. Export Errores: incluye categoria_matriz y cuenta_matriz (misma lógica que el dashboard); monto como número.</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Versiones en bitácora</v>
+        <v>Flujo de despliegue</v>
       </c>
       <c r="B31" t="str">
-        <v>Hoja "Versiones" en Bitacora_tareas.xlsx: registro incremental (1.0, 1.1, …) con fecha y descripción de cada despliegue a Git/Vercel.</v>
+        <v>Al terminar cada tarea: el usuario prueba en local y confirma; recién entonces el asistente hace git add, commit y push (Vercel redepliega automático). No se despliega hasta confirmación.</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Campo moneda (BD)</v>
+        <v>Versiones en bitácora</v>
       </c>
       <c r="B32" t="str">
-        <v>Columna moneda en tabla transacciones (ARS/USD). Si está informada, el dashboard la usa salvo reglas de negocio: Mercado Pago y Transferencia Morba siempre ARS para conversión (también morva por typo). Si moneda vacía, infiere desde textos/medio (dólar → USD). Export a Excel incluye moneda.</v>
+        <v>Hoja "Versiones" en Bitacora_tareas.xlsx: registro incremental (1.0, 1.1, …) con fecha y descripción de cada despliegue a Git/Vercel.</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Edición desde modal Errores</v>
+        <v>Campo moneda (BD)</v>
       </c>
       <c r="B33" t="str">
-        <v>En el detalle de errores, icono de edición por registro. Abre modal para corregir: Categoría y Cuenta contable solo desde valores existentes en BD; Descripción libre. Al guardar se actualiza la fila y se marcan editado y editado_detalle (qué campos se editaron).</v>
+        <v>Columna moneda en tabla transacciones (ARS/USD). Si está informada, el dashboard la usa salvo reglas de negocio: Mercado Pago y Transferencia Morba siempre ARS para conversión (también morva por typo). Si moneda vacía, infiere desde textos/medio (dólar → USD). Export a Excel incluye moneda.</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Campos editado y editado_detalle</v>
+        <v>Edición desde modal Errores</v>
       </c>
       <c r="B34" t="str">
-        <v>En transacciones: editado (boolean) y editado_detalle (texto, ej. "Categoria, Descripcion, Cuenta Contable"). Migración supabase_transacciones_editado.sql. Export Excel los incluye.</v>
+        <v>En el detalle de errores, icono de edición por registro. Abre modal para corregir: Categoría y Cuenta contable solo desde valores existentes en BD; Descripción libre. UPDATE en transacciones solo si hubo cambios respecto a la fila; si no, aviso (antes el modal cerraba sin guardar). Tras UPDATE se verifica que haya filas actualizadas; nota contextual para inconsistencia categoría/cuenta/descripción. editado y editado_detalle al guardar con cambios.</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Tipo de error en Errores</v>
+        <v>Campos editado y editado_detalle</v>
       </c>
       <c r="B35" t="str">
-        <v>Tabla de errores muestra columna Tipo de error: Inconsistencia entre Categoria, Cuenta Contable y Descripcion; o Potencial registro duplicado. Export a Excel incluye tipo_error.</v>
+        <v>En transacciones: editado (boolean) y editado_detalle (texto, ej. "Categoria, Descripcion, Cuenta Contable"). Migración supabase_transacciones_editado.sql. Export Excel los incluye.</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Detección de potencial duplicado</v>
+        <v>Tipo de error en Errores</v>
       </c>
       <c r="B36" t="str">
-        <v>Registros con misma fecha, monto, tipo_movimiento y descripción similar se marcan como potencial duplicado. Icono Ver abre modal con comparación Este registro / Posible duplicado; acciones: Excluir de cálculos (anular) o Eliminar registro.</v>
+        <v>Tabla de errores muestra columna Tipo de error: Inconsistencia entre Categoria, Cuenta Contable y Descripcion; o Potencial registro duplicado. Excepciones explícitas cat/cuenta (Impuestos/IIBB, Logistica/Fletes, Alquileres varias cuentas, Activos/Hornos, Mantenimiento/Ferreteria, Sueldos/Comisiones Ventas y variantes, Marketing/Creación contenido, Honorarios/Honorarios Contables) no marcan inconsistencia. Export a Excel incluye tipo_error.</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Filtro por tipo de error</v>
+        <v>Detección de potencial duplicado</v>
       </c>
       <c r="B37" t="str">
-        <v>En la solapa Errores, selector para filtrar por tipo: Todos, Inconsistencia (categoría/cuenta/descripción), Potencial registro duplicado. La exportación a Excel exporta solo los registros visibles según el filtro.</v>
+        <v>Registros con misma fecha, monto, tipo_movimiento y descripción similar se marcan como potencial duplicado. Icono Ver abre modal con comparación Este registro / Posible duplicado; acciones: Excluir de cálculos (anular) o Eliminar registro.</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Duplicados: condición cliente</v>
+        <v>Filtro por tipo de error</v>
       </c>
       <c r="B38" t="str">
-        <v>Dos registros son potencial duplicado solo si coinciden en fecha, monto, tipo_movimiento, descripción similar y además cliente es igual; si cliente es distinto no se marcan como duplicado. Modal de comparación muestra id_origen y Cliente.</v>
+        <v>En la solapa Errores, selector para filtrar por tipo: Todos, Inconsistencia (categoría/cuenta/descripción), Potencial registro duplicado. La exportación a Excel exporta solo los registros visibles según el filtro.</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Regla bitácora</v>
+        <v>Duplicados: condición cliente</v>
       </c>
       <c r="B39" t="str">
-        <v>Actualizar todas las solapas necesarias: Log (siempre que haya tarea), Resumen (si cambia funcionalidad), Presupuesto (si agrega o cambia entregable comercial), Versiones (en despliegue). Regenerar Excel tras editar crear-bitacora-excel.js.</v>
+        <v>Dos registros son potencial duplicado solo si coinciden en fecha, monto, tipo_movimiento, descripción similar y además cliente es igual; si cliente es distinto no se marcan como duplicado. Modal de comparación muestra id_origen y Cliente.</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Evolución (tabla dinámica)</v>
+        <v>Regla bitácora</v>
       </c>
       <c r="B40" t="str">
-        <v>Solapa Evolución: Agrupar por = Categoría o Cuenta contable (fila); Período = Diario (fecha por día) o Mensual (MM-YYYY). Columnas = períodos, celdas = neto en moneda seleccionada, columna Total.</v>
+        <v>Actualizar todas las solapas necesarias: Log (siempre que haya tarea), Resumen (si cambia funcionalidad), Presupuesto (si agrega o cambia entregable comercial), Versiones (en despliegue). Regenerar Excel tras editar crear-bitacora-excel.js.</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Evolución: detalle al clic y exportar</v>
+        <v>Evolución (tabla dinámica)</v>
       </c>
       <c r="B41" t="str">
-        <v>Clic en un valor de la tabla Evolución abre modal con detalle: Fecha, Categoría, Descripción, Monto. Exportar Evolución a Excel exporta la tabla según filtros Agrupar por y Período.</v>
+        <v>Solapa Evolución: Agrupar por = Nueva categoría (matriz) o Nueva cuenta contable (matriz) —prioriza nueva_categoria / nueva_cuenta_contable en BD y si faltan usa extracto con validación—; Período = Diario o Mensual (MM-YYYY). Columnas = períodos, celdas = neto en moneda seleccionada, columna Total.</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Exportaciones Excel</v>
+        <v>Evolución: detalle al clic y exportar</v>
       </c>
       <c r="B42" t="str">
-        <v>Todas las exportaciones incluyen una fila título con la moneda. Exportar Base Histórica (icono Excel) en la línea del selector de moneda; Exportar Evolución a Excel con el mismo icono.</v>
+        <v>Clic en un valor abre modal con detalle: Fecha, Categoría (matriz), Cuenta (matriz), Descripción, Monto. Exportar Evolución a Excel: primera columna con el mismo criterio de agrupación.</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Evolución: orden ingreso/egreso</v>
+        <v>Exportaciones Excel</v>
       </c>
       <c r="B43" t="str">
-        <v>En la tabla Evolución las filas se muestran primero las de ingreso (total &gt;= 0) y luego las de egreso (total &lt; 0); dentro de cada grupo orden alfabético. Aplica tanto al agrupar por Categoría como por Cuenta contable.</v>
+        <v>Todas las exportaciones incluyen una fila título con la moneda. Exportar Base Histórica (icono Excel) en la línea del selector de moneda; Exportar Evolución a Excel con el mismo icono.</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Int. por caución</v>
+        <v>Evolución: orden ingreso/egreso</v>
       </c>
       <c r="B44" t="str">
-        <v>Columna en flujo por mes: interés mensual por colocar el sobrante de caja a la tasa diaria de la serie de cauciones. Carga Serie_Cauciones.xlsx al refrescar (o serie_cauciones.json si no hay Excel). Cálculo: base = G/P acumulado a la fecha + interés acumulado; Int T = base × tasa. Clic en el valor abre modal con marcha (G/P acum, Int T-1, Base, Tasa, Int T).</v>
+        <v>En la tabla Evolución las filas se muestran primero las de ingreso (total &gt;= 0) y luego las de egreso (total &lt; 0); dentro de cada grupo orden alfabético. Aplica al agrupar por categoría o cuenta de matriz.</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Todas las transacciones</v>
+        <v>Int. por caución</v>
       </c>
       <c r="B45" t="str">
-        <v>Solapa que lista todas las transacciones con todas las columnas. Filtros por mes y categoría. Botón Editar por registro abre modal de edición completa.</v>
+        <v>Columna en flujo por mes: interés mensual por colocar el sobrante de caja a la tasa diaria de la serie de cauciones. Carga Serie_Cauciones.xlsx al refrescar (o serie_cauciones.json si no hay Excel). Cálculo: base = G/P acumulado a la fecha + interés acumulado; Int T = base × tasa. Clic en el valor abre modal con marcha (G/P acum, Int T-1, Base, Tasa, Int T).</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Edición completa de registros</v>
+        <v>Todas las transacciones</v>
       </c>
       <c r="B46" t="str">
-        <v>Modal de edición con todos los campos: fecha, mes, año, tipo movimiento, monto, moneda, status, medio pago, categoría, cuenta contable, origen archivo, descripción, cliente, cat_desc, id_origen, id_operación. Combos para campos normalizados (valores existentes en BD). editado y editado_detalle al guardar.</v>
+        <v>Solapa que lista todas las transacciones con todas las columnas. Filtros por mes, categoría (matriz) y cuenta (matriz) —misma prioridad nueva_* que Evolución—, tipo (Ingreso/Egreso) e id operación (texto). Columnas principales cat/cuenta por matriz; columnas nueva_* como en BD. Botón Editar por registro abre modal de edición completa.</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Proyección próximos 3 meses</v>
+        <v>Edición completa de registros</v>
       </c>
       <c r="B47" t="str">
-        <v>Debajo del total real en Flujo por mes: "Próximos 3 meses proyectados" con ventana rodante. Configuración (sidebar): método (Mediana/Promedio) y meses de historia (3, 6, 12, 24). Ingresos, egresos, G/P y ratios proyectados por mes.</v>
+        <v>Modal de edición con todos los campos: fecha, mes, año, tipo movimiento, monto, moneda, status, medio pago, categoría, cuenta contable, costo_directo y costo_indirecto (Y/N o vacío), origen archivo, descripción, cliente, cat_desc, id_origen, id_operación. Combos para campos normalizados (valores existentes en BD). editado y editado_detalle al guardar. Tras guardar OK: recarga datos, recalcula flujo, y si el modal de detalle del mes sigue abierto se vuelve a armar ese modal para no mostrar HTML viejo.</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Int. por caución proyectado</v>
+        <v>Proyección próximos 3 meses</v>
       </c>
       <c r="B48" t="str">
-        <v>Punto de partida = G/P Total real + interés acumulado; tasa = promedio último mes real; días naturales; Int T-1 día 1 = (Int T-1 + Int T) último día del mes anterior. G/P acum en marcha = al inicio de cada día (real y proyectado). Ventana rodante: ingresos/egresos distintos por mes.</v>
+        <v>Debajo del total real en Flujo por mes: "Próximos 3 meses proyectados" con ventana rodante. Configuración (sidebar): método (Mediana/Promedio) y meses de historia (3, 6, 12, 24). Ingresos, egresos, G/P y ratios proyectados por mes.</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Disclaimer proyección</v>
+        <v>Int. por caución proyectado</v>
       </c>
       <c r="B49" t="str">
-        <v>Debajo de las filas proyectadas, texto en letra chica y gris oscuro que explica la metodología: Mediana/Promedio de N meses, ventana rodante, y cálculo de Int. por caución proyectado.</v>
+        <v>Punto de partida = G/P Total real + interés acumulado; tasa = promedio último mes real; días naturales; Int T-1 día 1 = (Int T-1 + Int T) último día del mes anterior. G/P acum en marcha = al inicio de cada día (real y proyectado). Ventana rodante: ingresos/egresos distintos por mes.</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Botones e iconos unificados</v>
+        <v>Disclaimer proyección</v>
       </c>
       <c r="B50" t="str">
-        <v>Todos los botones con mismo estilo: icono SVG + texto. Sidebar (chevron, home, engranaje), tabs con iconos, exportar con icono descarga, modales con iconos (Guardar, Cerrar, Excluir, Eliminar). Iconos solos (cerrar, editar, alerta) en SVG.</v>
+        <v>Debajo de las filas proyectadas, texto en letra chica y gris oscuro que explica la metodología: Mediana/Promedio de N meses, ventana rodante, y cálculo de Int. por caución proyectado.</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Configuración % G/P en caución</v>
+        <v>Botones e iconos unificados</v>
       </c>
       <c r="B51" t="str">
-        <v>Combo "% G/P acum. en caución" en Configuración con escala de 5 en 5 (100, 95, 90… hasta 0). Por defecto 100 %; menor % = más liquidez (menos interés por caución).</v>
+        <v>Todos los botones con mismo estilo: icono SVG + texto. Sidebar (chevron, home, engranaje), tabs con iconos, exportar con icono descarga, modales con iconos (Guardar, Cerrar, Excluir, Eliminar). Iconos solos (cerrar, editar, alerta) en SVG.</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Etiqueta Caución (x% cash)</v>
+        <v>Configuración % G/P en caución</v>
       </c>
       <c r="B52" t="str">
-        <v>Columna en flujo por mes: cabecera "Caución (x% cash)" donde x es el valor del parámetro % G/P; sin icono % a la izquierda. Modales de marcha y disclaimer usan "Caución".</v>
+        <v>Combo "% G/P acum. en caución" en Configuración con escala de 5 en 5 (100, 95, 90… hasta 0). Por defecto 100 %; menor % = más liquidez (menos interés por caución).</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Meses a proyectar</v>
+        <v>Etiqueta Caución (x% cash)</v>
       </c>
       <c r="B53" t="str">
-        <v>En Configuración: combo Meses a proyectar (1, 2, 3, 4, 5, 6, 12). Flujo por mes y Evolución muestran esa cantidad de columnas/filas proyectadas.</v>
+        <v>Columna en flujo por mes: cabecera "Caución (x% cash)" donde x es el valor del parámetro % G/P; sin icono % a la izquierda. Modales de marcha y disclaimer usan "Caución".</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>Config por usuario en Supabase</v>
+        <v>Meses a proyectar</v>
       </c>
       <c r="B54" t="str">
-        <v>Tabla config_dashboard (user_id, proyección y caución). Con Auth anónimo se sincroniza al cargar y al guardar; la config persiste por usuario en la base. Migración: supabase_config_dashboard.sql.</v>
+        <v>En Configuración: combo Meses a proyectar (1, 2, 3, 4, 5, 6, 12). Flujo por mes y Evolución muestran esa cantidad de columnas/filas proyectadas.</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>Recorte % (cada lado)</v>
+        <v>Config por usuario en Supabase</v>
       </c>
       <c r="B55" t="str">
-        <v>En Configuración, combo Recorte % (cada lado) (0, 5, 10, 15, 20, 25) visible solo cuando el método es Promedio recortado. Más % = más suavizado. Persistido en config_dashboard (proyeccion_recorte).</v>
+        <v>Tabla config_dashboard (user_id, proyección, caución, alertas y meses_excluidos JSON). Con Auth anónimo se sincroniza al cargar y al guardar; la config persiste por usuario en la base. Migración: supabase_config_dashboard.sql; meses excluidos: supabase_config_dashboard_meses_excluidos.sql.</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>Novedades del Negocio</v>
+        <v>Recorte % (cada lado)</v>
       </c>
       <c r="B56" t="str">
-        <v>Ítem en sidebar que abre una vista con importadores de hornos y comercios de venta de hornos en Argentina (Buenos Aires). Datos recuperados por IA (Edge Function con Gemini + google_search). Nombre, dirección, teléfono y web por contacto.</v>
+        <v>En Configuración, combo Recorte % (cada lado) (0, 5, 10, 15, 20, 25) visible solo cuando el método es Promedio recortado. Más % = más suavizado. Persistido en config_dashboard (proyeccion_recorte).</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>Normalización de extracto bancario</v>
+        <v>Novedades del Negocio</v>
       </c>
       <c r="B57" t="str">
-        <v>npm run normalizar-extracto: lee Fornitalia_Movimientos.xlsx (o Extracto legado), hoja Normalizado con fecha_iso, tipo, medio, categoría, cuenta, moneda inferida, monto_original, tipo_cambio, monto_ars, id_cierre_caja, id_comprobante_pago, id_impuesto, cat_desc cuando vienen del export.</v>
+        <v>Ítem en sidebar que abre una vista con importadores de hornos y comercios de venta de hornos en Argentina (Buenos Aires). Datos recuperados por IA (Edge Function con Gemini + google_search). Nombre, dirección, teléfono y web por contacto.</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>Informe inconsistencias datos legacy (cliente)</v>
+        <v>Normalización de extracto bancario</v>
       </c>
       <c r="B58" t="str">
-        <v>docs/ANALISIS_NORMALIZACION_DATOS_LEGACY_FORNITALIA.md alineado a Fornitalia_Movimientos.xlsx, §0 validaciones IDs/CatDesc, pipeline normalizar-extracto. Regenerar: npm run informe-normalizacion-html / informe-normalizacion-pdf; PDF con Playwright o Chrome headless (informe-html-a-pdf.js).</v>
+        <v>npm run normalizar-extracto: lee Fornitalia_Movimientos.xlsx (o Extracto legado), hoja Normalizado con fecha_iso, tipo, medio, categoría, cuenta, moneda inferida, monto_original, tipo_cambio, monto_ars, id_cierre_caja, id_comprobante_pago, id_impuesto, cat_desc cuando vienen del export.</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>Upload de extracto normalizado</v>
+        <v>Informe inconsistencias datos legacy (cliente)</v>
       </c>
       <c r="B59" t="str">
-        <v>Botón en la app para reemplazar transacciones desde la hoja Normalizado (generada con npm run normalizar-extracto desde Fornitalia_Movimientos), con validación previa, IDs y cat_desc persistidos cuando existen, confirmación de seguridad, id_origen técnico y carga en lotes.</v>
+        <v>docs/ANALISIS_NORMALIZACION_DATOS_LEGACY_FORNITALIA.md alineado a Fornitalia_Movimientos.xlsx, §0 validaciones IDs/CatDesc, pipeline normalizar-extracto. Regenerar HTML+PDF: npm run informe-normalizacion (informe-normalizacion-solo-html solo si hace falta iterar sin Playwright).</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>Log de excluidos en upload</v>
+        <v>Upload de extracto normalizado</v>
       </c>
       <c r="B60" t="str">
-        <v>Nueva solapa Excluidos upload con registros no insertados por error o por regla de negocio (Apertura/Cierre de Caja), persistidos en Supabase para auditoría.</v>
+        <v>Botón en la app para reemplazar transacciones desde la hoja Normalizado (generada con npm run normalizar-extracto desde Fornitalia_Movimientos), con validación previa, IDs y cat_desc persistidos cuando existen, confirmación de seguridad, id_origen técnico y carga en lotes.</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
+        <v>Log de excluidos en upload</v>
+      </c>
+      <c r="B61" t="str">
+        <v>Nueva solapa Excluidos upload con registros no insertados por error o por regla de negocio (Apertura/Cierre de Caja), persistidos en Supabase para auditoría.</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
         <v>Análisis financiero extracto (PDF)</v>
       </c>
-      <c r="B61" t="str">
-        <v>npm run analisis-financiero-pdf: métricas desde Fornitalia_Movimientos.xlsx (fallback Extracto legado); ARS vía MontoCambio/Monto en $, TC por fila o MEP; exclusiones y USD sin conversión. Ver docs/ANALISIS_FINANCIERO_EXTRACTO_README.md.</v>
+      <c r="B62" t="str">
+        <v>npm run analisis-financiero-pdf: métricas desde Fornitalia_Movimientos.xlsx (fallback Extracto legado); ARS vía MontoCambio/Monto en $, TC por fila o MEP; exclusiones y USD sin conversión. Sección ventas: ranking por vendedor desde Resumen_Operaciones (Tabla, Vendedor_RO) por N° operación; ranking proxy por producto (detalle hasta mes cierre feb 2026). Ver docs/ANALISIS_FINANCIERO_EXTRACTO_README.md.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B61"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B62"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2982,7 +3364,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C42"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -3280,7 +3662,7 @@
         <v>1.25</v>
       </c>
       <c r="B27" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="C27" t="str">
         <v>Ayuda al clic en columnas Comisiones/Ventas y Egresos/Ingresos (popover con texto explicativo). Regla bitácora: tecnología e infraestructura y actualizar todas las solapas. Despliegue a producción.</v>
@@ -3291,7 +3673,7 @@
         <v>1.26</v>
       </c>
       <c r="B28" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="C28" t="str">
         <v>Mensaje de alerta de desvío: categoría en negrita sin comillas. Despliegue a producción.</v>
@@ -3302,7 +3684,7 @@
         <v>1.27</v>
       </c>
       <c r="B29" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="C29" t="str">
         <v>Novedades del Negocio: sección en sidebar con importadores y comercios de hornos en Argentina (Edge Function Gemini + google_search). Despliegue a producción.</v>
@@ -3313,7 +3695,7 @@
         <v>1.28</v>
       </c>
       <c r="B30" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="C30" t="str">
         <v>Favicon L&amp;P: L y P dada vuelta centradas en el círculo azul; ajuste de posición y centrado. Despliegue a producción.</v>
@@ -3324,7 +3706,7 @@
         <v>1.29</v>
       </c>
       <c r="B31" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="C31" t="str">
         <v>Errores: export y listado con id_origen e id_operacion; modal duplicado con id_operacion e icono en campos que no coinciden. Exclusiones duplicados: anulados, id_origen e id_operacion ambos distintos, ambos montos 0. Quitar disclaimer datos ficticios; scripts e instrucciones para repoblar transacciones desde Excel. Despliegue a producción.</v>
@@ -3335,7 +3717,7 @@
         <v>1.30</v>
       </c>
       <c r="B32" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="C32" t="str">
         <v>Errores: orden por tipo y monto descendente; filtros por categoría original y categoría mostrada. Flujo: filtro explícito status Anulado. Export Base Histórica: columnas Tipo_Cambio, Monto_ARS, Monto_USD con conversiones. Despliegue a producción.</v>
@@ -3346,7 +3728,7 @@
         <v>1.31</v>
       </c>
       <c r="B33" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="C33" t="str">
         <v>Estructura ordenada del repo: sql/, scripts/, docs/. Regla estructura-proyecto (mantener carpetas y rutas). Referencias en bitácora y docs actualizadas. Despliegue a producción.</v>
@@ -3357,7 +3739,7 @@
         <v>1.32</v>
       </c>
       <c r="B34" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="C34" t="str">
         <v>Modales: no cerrar al elegir opción de select (mousedown+click en backdrop). Helper setupBackdropCloseOnlyOnRealClick en todos los modales.</v>
@@ -3368,7 +3750,7 @@
         <v>1.33</v>
       </c>
       <c r="B35" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="C35" t="str">
         <v>Carga paginada transacciones y tipo_de_cambio (límite PostgREST). Reglas ARS Mercado Pago y Transferencia Morba en normalizador, upload y esTransaccionUSD. Upload excluidos: filtro última corrida; SQL DELETE en transacciones_upload_excluidos. Informe análisis normalización (docs MD/HTML/PDF) y scripts Playwright. DevDependency playwright y npm run playwright:install.</v>
@@ -3379,7 +3761,7 @@
         <v>1.34</v>
       </c>
       <c r="B36" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="C36" t="str">
         <v>Flujo operativo sin traspasos internos (Transferencia y Depósito); misma regla que informe PDF; nota en panel.</v>
@@ -3390,7 +3772,7 @@
         <v>1.35</v>
       </c>
       <c r="B37" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="C37" t="str">
         <v>Flujo por mes alineado al PDF: ingresos/egresos brutos extracto, Neto bruto, G/P operativo; solapa Traspasos internos; excluirFilaFlujoOperativo y Evolución con misma base.</v>
@@ -3401,7 +3783,7 @@
         <v>1.36</v>
       </c>
       <c r="B38" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="C38" t="str">
         <v>Select tipo_cambio y monto_cambio en transacciones; montoConvertido en ARS prioriza monto_cambio y TC de fila (concilia con informe PDF al centavo).</v>
@@ -3412,7 +3794,7 @@
         <v>1.37</v>
       </c>
       <c r="B39" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="C39" t="str">
         <v>Despliegue a producción Vercel: informe financiero PDF con MEP desde docs; dashboard v1.37 con conciliación extracto.</v>
@@ -3423,7 +3805,7 @@
         <v>1.43</v>
       </c>
       <c r="B40" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="C40" t="str">
         <v>Módulo Seguridad (login/registro/invitado, roles, permisos, vista Seguridad); get_users_for_admin solo email; mensajes registro Supabase; thead sticky en tablas; scroll vertical flujo por página (v1.42); APP_VERSION 1.43. Push main y Vercel producción.</v>
@@ -3434,15 +3816,26 @@
         <v>1.49</v>
       </c>
       <c r="B41" t="str">
-        <v>25/03/2026</v>
+        <v>08/05/2026</v>
       </c>
       <c r="C41" t="str">
         <v>Caución: normalización de escala de tasas (JSON legado vs fracción diaria Excel); informe financiero §8 coherente con app (esTransaccionUSD, montos en pesos); convertir-serie-cauciones.js con fechas Date/ISO; serie_cauciones.json alineado a Serie_Cauciones.xlsx. Despliegue a producción Vercel.</v>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>1.57</v>
+      </c>
+      <c r="B42" t="str">
+        <v>08/05/2026</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Dashboard: Evolución y agregados con categoría/cuenta matriz (nueva_* + fallback); Configuración Inclusión por mes (meses_excluidos localStorage + Supabase, sql supabase_config_dashboard_meses_excluidos.sql); modal editar costo_directo y costo_indirecto; ayuda informe PDF tras ícono en Flujo por mes (popover template); duplicados sin filtrar por mes excluido; APP_VERSION 1.57. Despliegue producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C41"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C42"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3634,7 +4027,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="95.83203125" customWidth="1"/>
@@ -3688,9 +4081,17 @@
         <v>Node.js + SheetJS (xlsx). Script scripts/crear-bitacora-excel.js genera Bitacora_tareas.xlsx con las solapas Log, Resumen, Ref Git y Vercel, Versiones, Presupuesto, Tecnología.</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Conciliación compras</v>
+      </c>
+      <c r="B7" t="str">
+        <v>npm run conciliar-base-compras: cruza docs/Base Fornitalia Compras.xlsx con Fornitalia_Movimientos.xlsx; salida docs/Base-Compras-Conciliacion-Caja.xlsx.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
v1.58: scroll modal detalle, conversión montos, edición matriz, bitácora con fechas históricas; despliegue.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E138"/>
+  <dimension ref="A1:E144"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -2748,18 +2748,120 @@
         <v>12:54</v>
       </c>
       <c r="C138" t="str">
+        <v>Despliegue v1.57 producción</v>
+      </c>
+      <c r="D138" t="str">
+        <v>Push main y vercel --prod: matriz en vistas, meses excluidos Config, edición flags costo, ayuda flujo, migración SQL meses_excluidos documentada.</v>
+      </c>
+      <c r="E138" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="str">
+        <v>13/05/2026</v>
+      </c>
+      <c r="B139" t="str">
+        <v>13:55</v>
+      </c>
+      <c r="C139" t="str">
         <v>Excel Categoria_CCSis: solapa resumen sin duplicar</v>
       </c>
-      <c r="D138" t="str">
+      <c r="D139" t="str">
         <v>scripts/completar-matriz-ccsis-desde-normalizado.js: solapa Resumen_Confirmados_cat_cuenta (categoria, cuenta_contable, # Registros, Monto_ARS) agregado único desde Extracto-Fornitalia-Normalizado solo Confirmado; no modifica solapas Matriz_*. npm run completar-matriz-ccsis-normalizado.</v>
       </c>
-      <c r="E138" t="str">
-        <v>Diagnostico</v>
+      <c r="E139" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="str">
+        <v>13/05/2026</v>
+      </c>
+      <c r="B140" t="str">
+        <v>13:55</v>
+      </c>
+      <c r="C140" t="str">
+        <v>Modal mes: scroll en detalle por categoría</v>
+      </c>
+      <c r="D140" t="str">
+        <v>Cuerpo del modal con scroll vertical; detalle expandido (ojito) en contenedor con altura máxima y encabezados fijos.</v>
+      </c>
+      <c r="E140" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="str">
+        <v>13/05/2026</v>
+      </c>
+      <c r="B141" t="str">
+        <v>13:55</v>
+      </c>
+      <c r="C141" t="str">
+        <v>Conversión ARS en dashboard (USD y monto)</v>
+      </c>
+      <c r="D141" t="str">
+        <v>montoConvertido: USD con monto × tipo_cambio o cotización de tabla; movimientos ARS usan monto (no monto_cambio desalineado). Ayuda Flujo actualizada.</v>
+      </c>
+      <c r="E141" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="str">
+        <v>13/05/2026</v>
+      </c>
+      <c r="B142" t="str">
+        <v>13:55</v>
+      </c>
+      <c r="C142" t="str">
+        <v>Modal editar: nueva categoría y cuenta matriz</v>
+      </c>
+      <c r="D142" t="str">
+        <v>Select nueva_categoria y nueva_cuenta_contable en edición completa; persistencia en transacciones y editado_detalle.</v>
+      </c>
+      <c r="E142" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="str">
+        <v>13/05/2026</v>
+      </c>
+      <c r="B143" t="str">
+        <v>13:55</v>
+      </c>
+      <c r="C143" t="str">
+        <v>Bitácora: fechas históricas al regenerar</v>
+      </c>
+      <c r="D143" t="str">
+        <v>crear-bitacora-excel.js conserva Fecha/Hora de Log y Versiones ya escritas en Bitacora_tareas.xlsx; regla bitacora-tareas sin reescribir filas antiguas.</v>
+      </c>
+      <c r="E143" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="str">
+        <v>13/05/2026</v>
+      </c>
+      <c r="B144" t="str">
+        <v>13:55</v>
+      </c>
+      <c r="C144" t="str">
+        <v>Despliegue v1.58 producción</v>
+      </c>
+      <c r="D144" t="str">
+        <v>Push main y vercel --prod: scroll modal detalle, conversión montos, edición matriz, bitácora con fechas congeladas; APP_VERSION 1.58.</v>
+      </c>
+      <c r="E144" t="str">
+        <v>Despliegue</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E138"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E144"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2801,7 +2903,7 @@
         <v>Moneda</v>
       </c>
       <c r="B4" t="str">
-        <v>Selector ARS / USD. Maestro caja→moneda (medio de pago) alineado a scripts/lib/fornitalia-moneda-por-medio.js en import normalizado y en esTransaccionUSD. En ARS: prioridad monto_cambio, tipo_cambio por fila y tabla tipo_de_cambio (MEP/CCL/Oficial); con MEP y datos cargados coincide con el informe PDF.</v>
+        <v>Selector ARS / USD. Maestro caja→moneda (medio de pago) alineado a scripts/lib/fornitalia-moneda-por-medio.js en import normalizado y en esTransaccionUSD. En ARS: USD con monto × tipo_cambio o cotización de tabla; movimientos en ARS usan monto (no monto_cambio si viene desalineado del extracto).</v>
       </c>
     </row>
     <row r="5">
@@ -2897,7 +2999,7 @@
         <v>Detalle transacciones (tabla)</v>
       </c>
       <c r="B16" t="str">
-        <v>En el modal mensual, al expandir una categoría/cuenta se muestra una tabla con títulos y filas de transacciones (Fecha, Tipo, Medio, Moneda, Monto, moneda vista, Descripción, Origen).</v>
+        <v>En el modal mensual, al expandir una categoría/cuenta se muestra una tabla con títulos y filas de transacciones (Fecha, Tipo, Medio, Moneda, Monto, moneda vista, Descripción, Origen). El detalle expandido tiene scroll vertical con encabezados fijos; el cuerpo del modal también desplaza cuando el contenido supera la ventana.</v>
       </c>
     </row>
     <row r="17">
@@ -3145,7 +3247,7 @@
         <v>Edición completa de registros</v>
       </c>
       <c r="B47" t="str">
-        <v>Modal de edición con todos los campos: fecha, mes, año, tipo movimiento, monto, moneda, status, medio pago, categoría, cuenta contable, costo_directo y costo_indirecto (Y/N o vacío), origen archivo, descripción, cliente, cat_desc, id_origen, id_operación. Combos para campos normalizados (valores existentes en BD). editado y editado_detalle al guardar. Tras guardar OK: recarga datos, recalcula flujo, y si el modal de detalle del mes sigue abierto se vuelve a armar ese modal para no mostrar HTML viejo.</v>
+        <v>Modal de edición con todos los campos: fecha, mes, año, tipo movimiento, monto, moneda, status, medio pago, categoría, nueva categoría (matriz), cuenta contable, nueva cuenta contable (matriz), costo_directo y costo_indirecto (Y/N o vacío), origen archivo, descripción, cliente, cat_desc, id_origen, id_operación. Combos para campos normalizados (valores existentes en BD). editado y editado_detalle al guardar. Tras guardar OK: recarga datos, recalcula flujo, y si el modal de detalle del mes sigue abierto se vuelve a armar ese modal para no mostrar HTML viejo.</v>
       </c>
     </row>
     <row r="48">
@@ -3364,7 +3466,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C43"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -3833,9 +3935,20 @@
         <v>Dashboard: Evolución y agregados con categoría/cuenta matriz (nueva_* + fallback); Configuración Inclusión por mes (meses_excluidos localStorage + Supabase, sql supabase_config_dashboard_meses_excluidos.sql); modal editar costo_directo y costo_indirecto; ayuda informe PDF tras ícono en Flujo por mes (popover template); duplicados sin filtrar por mes excluido; APP_VERSION 1.57. Despliegue producción Vercel.</v>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>1.58</v>
+      </c>
+      <c r="B43" t="str">
+        <v>13/05/2026</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Modal detalle con scroll; montoConvertido USD×TC y ARS por monto; edición nueva_categoria/nueva_cuenta_contable; bitácora conserva fechas históricas al regenerar; APP_VERSION 1.58. Despliegue producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C42"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C43"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4078,7 +4191,7 @@
         <v>Bitácora</v>
       </c>
       <c r="B6" t="str">
-        <v>Node.js + SheetJS (xlsx). Script scripts/crear-bitacora-excel.js genera Bitacora_tareas.xlsx con las solapas Log, Resumen, Ref Git y Vercel, Versiones, Presupuesto, Tecnología.</v>
+        <v>Node.js + SheetJS (xlsx). Script scripts/crear-bitacora-excel.js genera Bitacora_tareas.xlsx con las solapas Log, Resumen, Ref Git y Vercel, Versiones, Presupuesto, Tecnología. Al regenerar, conserva Fecha/Hora de filas ya presentes en Log y Versiones.</v>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
v1.59: combo Cliente en edición y columna Costo total en flujo
Quita Neto bruto de Flujo por mes y despliega APP_VERSION 1.59 con bitácora actualizada.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E144"/>
+  <dimension ref="A1:E146"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -2850,18 +2850,52 @@
         <v>13:55</v>
       </c>
       <c r="C144" t="str">
-        <v>Despliegue v1.58 producción</v>
+        <v>Modal editar: Cliente en combo</v>
       </c>
       <c r="D144" t="str">
-        <v>Push main y vercel --prod: scroll modal detalle, conversión montos, edición matriz, bitácora con fechas congeladas; APP_VERSION 1.58.</v>
+        <v>Campo Cliente pasa a select con valores existentes en la base (sin texto libre); incluye el cliente del registro si no estaba en la lista.</v>
       </c>
       <c r="E144" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="str">
+        <v>14/05/2026</v>
+      </c>
+      <c r="B145" t="str">
+        <v>11:50</v>
+      </c>
+      <c r="C145" t="str">
+        <v>Flujo por mes: Costo total / Ingreso total</v>
+      </c>
+      <c r="D145" t="str">
+        <v>Se quita columna Neto bruto; nueva columna Costo total / Ingreso total (egresos operativos ÷ ingresos operativos) tras Costo ind. / Ingresos; total y proyección alineados. Ayuda del panel actualizada.</v>
+      </c>
+      <c r="E145" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="str">
+        <v>14/05/2026</v>
+      </c>
+      <c r="B146" t="str">
+        <v>11:50</v>
+      </c>
+      <c r="C146" t="str">
+        <v>Despliegue v1.59 producción</v>
+      </c>
+      <c r="D146" t="str">
+        <v>Push main y vercel --prod: combo Cliente en edición; tabla Flujo sin Neto bruto y con Costo total / Ingreso total; APP_VERSION 1.59.</v>
+      </c>
+      <c r="E146" t="str">
         <v>Despliegue</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E144"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E146"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2887,7 +2921,7 @@
         <v>Flujo de caja por mes</v>
       </c>
       <c r="B2" t="str">
-        <v>Tabla alineada al informe financiero PDF: columnas Ingresos y Egresos = totales del libro de movimientos (incluyen traspasos entre cuentas); Neto bruto; G/P operativo sin Transferencia/Depósito ni Apertura/Cierre; ratios y columna Caución (mismo criterio que esTransaccionUSD, montos en pesos; tasas desde serie_cauciones.json o Serie_Cauciones.xlsx; normalización automática si el JSON está en escala antigua; % configurable). Proyección de caución en ARS con la misma base. Meses excluidos por Configuración → Inclusión por mes no aparecen en filas ni totales agregados. Icono de ayuda discreto sobre la tabla abre el texto detallado de alineación al PDF (popover).</v>
+        <v>Tabla alineada al informe financiero PDF: columnas Ingresos y Egresos = totales del libro de movimientos (incluyen traspasos entre cuentas); G/P operativo sin Transferencia/Depósito ni Apertura/Cierre; ratios Costo dir./ind./total sobre ingresos operativos; columna Caución (mismo criterio que esTransaccionUSD, montos en pesos; tasas desde serie_cauciones.json o Serie_Cauciones.xlsx; normalización automática si el JSON está en escala antigua; % configurable). Proyección de caución en ARS con la misma base. Meses excluidos por Configuración → Inclusión por mes no aparecen en filas ni totales agregados. Icono de ayuda discreto sobre la tabla abre el texto detallado de alineación al PDF (popover).</v>
       </c>
     </row>
     <row r="3">
@@ -3247,7 +3281,7 @@
         <v>Edición completa de registros</v>
       </c>
       <c r="B47" t="str">
-        <v>Modal de edición con todos los campos: fecha, mes, año, tipo movimiento, monto, moneda, status, medio pago, categoría, nueva categoría (matriz), cuenta contable, nueva cuenta contable (matriz), costo_directo y costo_indirecto (Y/N o vacío), origen archivo, descripción, cliente, cat_desc, id_origen, id_operación. Combos para campos normalizados (valores existentes en BD). editado y editado_detalle al guardar. Tras guardar OK: recarga datos, recalcula flujo, y si el modal de detalle del mes sigue abierto se vuelve a armar ese modal para no mostrar HTML viejo.</v>
+        <v>Modal de edición con todos los campos: fecha, mes, año, tipo movimiento, monto, moneda, status, medio pago, categoría, nueva categoría (matriz), cuenta contable, nueva cuenta contable (matriz), costo_directo y costo_indirecto (Y/N o vacío), origen archivo, descripción, cliente (combo con valores existentes en BD), cat_desc, id_origen, id_operación. Combos para campos normalizados (valores existentes en BD). editado y editado_detalle al guardar. Tras guardar OK: recarga datos, recalcula flujo, y si el modal de detalle del mes sigue abierto se vuelve a armar ese modal para no mostrar HTML viejo.</v>
       </c>
     </row>
     <row r="48">
@@ -3466,7 +3500,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C43"/>
+  <dimension ref="A1:C44"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -3946,9 +3980,20 @@
         <v>Modal detalle con scroll; montoConvertido USD×TC y ARS por monto; edición nueva_categoria/nueva_cuenta_contable; bitácora conserva fechas históricas al regenerar; APP_VERSION 1.58. Despliegue producción Vercel.</v>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>1.59</v>
+      </c>
+      <c r="B44" t="str">
+        <v>14/05/2026</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Modal editar: Cliente en combo (valores existentes). Flujo por mes: sin Neto bruto; columna Costo total / Ingreso total; ayuda y proyección alineadas. APP_VERSION 1.59. Despliegue producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C43"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C44"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.60: Cliente e icono ver transacción en detalle del modal mensual
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E146"/>
+  <dimension ref="A1:E148"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -2893,9 +2893,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="147">
+      <c r="A147" t="str">
+        <v>21/05/2026</v>
+      </c>
+      <c r="B147" t="str">
+        <v>09:33</v>
+      </c>
+      <c r="C147" t="str">
+        <v>Modal detalle mes: Cliente e icono ver transacción</v>
+      </c>
+      <c r="D147" t="str">
+        <v>Tabla expandida del modal mensual: columna Cliente; icono ojo por fila abre modal de edición (detalle completo). Ya no se abre al clic en toda la fila. APP_VERSION 1.60.</v>
+      </c>
+      <c r="E147" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="str">
+        <v>21/05/2026</v>
+      </c>
+      <c r="B148" t="str">
+        <v>09:44</v>
+      </c>
+      <c r="C148" t="str">
+        <v>Despliegue v1.60 producción</v>
+      </c>
+      <c r="D148" t="str">
+        <v>Push main y vercel --prod: modal detalle mes con columna Cliente e icono ojo para abrir edición/detalle completo. APP_VERSION 1.60.</v>
+      </c>
+      <c r="E148" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E146"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E148"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3033,7 +3067,7 @@
         <v>Detalle transacciones (tabla)</v>
       </c>
       <c r="B16" t="str">
-        <v>En el modal mensual, al expandir una categoría/cuenta se muestra una tabla con títulos y filas de transacciones (Fecha, Tipo, Medio, Moneda, Monto, moneda vista, Descripción, Origen). El detalle expandido tiene scroll vertical con encabezados fijos; el cuerpo del modal también desplaza cuando el contenido supera la ventana.</v>
+        <v>En el modal mensual, al expandir una categoría/cuenta se muestra una tabla con títulos y filas de transacciones (Fecha, Tipo, Medio, Moneda, Monto, moneda vista, TC, Cliente, Descripción, Origen). Icono ojo por fila (operadores) abre el modal de edición con el detalle completo del registro. Scroll vertical con encabezados fijos en el detalle expandido.</v>
       </c>
     </row>
     <row r="17">
@@ -3500,7 +3534,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C44"/>
+  <dimension ref="A1:C45"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -3991,9 +4025,20 @@
         <v>Modal editar: Cliente en combo (valores existentes). Flujo por mes: sin Neto bruto; columna Costo total / Ingreso total; ayuda y proyección alineadas. APP_VERSION 1.59. Despliegue producción Vercel.</v>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>1.60</v>
+      </c>
+      <c r="B45" t="str">
+        <v>21/05/2026</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Modal detalle mensual: columna Cliente en tabla expandida; icono ojo por fila abre modal de edición (detalle completo). APP_VERSION 1.60. Despliegue producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C44"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C45"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.78: EF export Excel, UI flujo sin traspasos y resumen operativo.
Estado Financiero con export estilizado (% corregidos, Notas, colores en celdas vacías); eliminada solapa Traspasos y tarjeta Neto caja; bitácora actualizada.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E148"/>
+  <dimension ref="A1:E155"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -2927,9 +2927,128 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="149">
+      <c r="A149" t="str">
+        <v>21/05/2026</v>
+      </c>
+      <c r="B149" t="str">
+        <v>10:28</v>
+      </c>
+      <c r="C149" t="str">
+        <v>Excel matriz relaciones transacciones</v>
+      </c>
+      <c r="D149" t="str">
+        <v>scripts/generar-matriz-relaciones-transacciones.js desde Transacciones_Fornitalia_Matriz_Final.xlsx: Matriz_Cat_Cuenta_Costo (4 columnas), Proveedores_Egreso y Proveedores_por_Cat_Cuenta. Salida docs/Matriz_Relaciones_Transacciones_Fornitalia.xlsx; npm run matriz-relaciones-transacciones.</v>
+      </c>
+      <c r="E149" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="str">
+        <v>28/05/2026</v>
+      </c>
+      <c r="B150" t="str">
+        <v>11:42</v>
+      </c>
+      <c r="C150" t="str">
+        <v>Matriz relaciones: exclusiones y proveedor primero</v>
+      </c>
+      <c r="D150" t="str">
+        <v>Excluye Impuestos, MP - Costo Financiero, Ventas y Comisiones Morvalab. Solapa Proveedores_por_Cat_Cuenta agrupa por Proveedor (1ª col.) con combinaciones Nueva Categoria → Cuenta elegibles.</v>
+      </c>
+      <c r="E150" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="str">
+        <v>28/05/2026</v>
+      </c>
+      <c r="B151" t="str">
+        <v>11:42</v>
+      </c>
+      <c r="C151" t="str">
+        <v>EF_Item y EF_SubItem en Supabase y upload</v>
+      </c>
+      <c r="D151" t="str">
+        <v>Columnas ef_item/ef_subitem en transacciones (migración Supabase). Import normalizado desde Base_Fornitalia_To_App (EF_Item, EF_SubItem). Export, Todas las transacciones y modal editar. APP_VERSION 1.61.</v>
+      </c>
+      <c r="E151" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="str">
+        <v>28/05/2026</v>
+      </c>
+      <c r="B152" t="str">
+        <v>13:37</v>
+      </c>
+      <c r="C152" t="str">
+        <v>Estado Financiero: ef_estructura y solapa EF</v>
+      </c>
+      <c r="D152" t="str">
+        <v>Tabla Supabase ef_estructura desde hoja EF_Estructura; upload normalizado la reemplaza. Solapa Estado Financiero (Ítem/Subítem con sangría, columnas por período). scripts/cargar-ef-estructura-desde-excel.js. APP_VERSION 1.62.</v>
+      </c>
+      <c r="E152" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="str">
+        <v>28/05/2026</v>
+      </c>
+      <c r="B153" t="str">
+        <v>14:30</v>
+      </c>
+      <c r="C153" t="str">
+        <v>Estado Financiero: UI, fórmulas y export Excel</v>
+      </c>
+      <c r="D153" t="str">
+        <v>Tabla EF horizontal (Ítem único con viñeta); subtotales y fórmulas con colores y % del Flujo Operativo; scroll anclado; ayuda en iconos; conciliación (§7) oculta en vista/export; export xlsx-js-style con montos enteros, columna Notas (análisis +/−), % como fracción 0.0%, relleno ARGB en celdas vacías. Fix fórmulas totales EF (Margen Bruto, etc.). APP_VERSION 1.74–1.77.</v>
+      </c>
+      <c r="E153" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="str">
+        <v>28/05/2026</v>
+      </c>
+      <c r="B154" t="str">
+        <v>15:00</v>
+      </c>
+      <c r="C154" t="str">
+        <v>Flujo: sin traspasos en UI; resumen operativo</v>
+      </c>
+      <c r="D154" t="str">
+        <v>Eliminada solapa Traspasos internos, tarjeta Neto caja y leyendas bruto/con traspasos. Resumen: 3 tarjetas (Ingresos, Egresos, G/P operativo). Flujo por mes usa misma base operativa en columnas y totales. APP_VERSION 1.76.</v>
+      </c>
+      <c r="E154" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="str">
+        <v>28/05/2026</v>
+      </c>
+      <c r="B155" t="str">
+        <v>15:10</v>
+      </c>
+      <c r="C155" t="str">
+        <v>Despliegue v1.78 producción</v>
+      </c>
+      <c r="D155" t="str">
+        <v>Push main y vercel --prod: Estado Financiero export Excel (%, colores fila, Notas); UI EF; flujo sin traspasos en dashboard; APP_VERSION 1.78.</v>
+      </c>
+      <c r="E155" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E148"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E155"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2955,7 +3074,7 @@
         <v>Flujo de caja por mes</v>
       </c>
       <c r="B2" t="str">
-        <v>Tabla alineada al informe financiero PDF: columnas Ingresos y Egresos = totales del libro de movimientos (incluyen traspasos entre cuentas); G/P operativo sin Transferencia/Depósito ni Apertura/Cierre; ratios Costo dir./ind./total sobre ingresos operativos; columna Caución (mismo criterio que esTransaccionUSD, montos en pesos; tasas desde serie_cauciones.json o Serie_Cauciones.xlsx; normalización automática si el JSON está en escala antigua; % configurable). Proyección de caución en ARS con la misma base. Meses excluidos por Configuración → Inclusión por mes no aparecen en filas ni totales agregados. Icono de ayuda discreto sobre la tabla abre el texto detallado de alineación al PDF (popover).</v>
+        <v>Tabla de caja operativa: columnas Ingresos, Egresos y G/P operativo (sin anulados ni apertura/cierre de caja; traspasos no incluidos en el import). Ratios Costo dir./ind./total sobre ingresos operativos; columna Caución (solo origen ARS, montos en pesos; tasas desde serie_cauciones.json o Serie_Cauciones.xlsx; % configurable). Proyección de caución en ARS. Meses excluidos por Configuración → Inclusión por mes no aparecen en filas ni totales. Icono de ayuda con criterios de la tabla.</v>
       </c>
     </row>
     <row r="3">
@@ -2963,7 +3082,7 @@
         <v>Resumen global</v>
       </c>
       <c r="B3" t="str">
-        <v>Cuatro tarjetas: Ingresos totales y Egresos totales del libro de movimientos (con traspasos), Neto caja (bruto) y G/P operativo (sin traspasos internos), en ARS o USD según selector.</v>
+        <v>Tres tarjetas: Ingresos totales, Egresos totales y G/P operativo (misma base operativa que la tabla Flujo por mes), en ARS o USD según selector.</v>
       </c>
     </row>
     <row r="4">
@@ -3107,167 +3226,167 @@
         <v>Exclusiones (flujo operativo)</v>
       </c>
       <c r="B21" t="str">
-        <v>No se incluyen en G/P operativo, Evolución ni Caución: anulados; apertura/cierre (categoría o heurística en fila); Transferencia ni Deposito/Depósito; meses desmarcados en Configuración → Inclusión por mes (meses_excluidos en Supabase/localStorage). Traspasos en solapa dedicada. Base histórica y Todas las transacciones siguen completas.</v>
+        <v>No se incluyen en G/P operativo, Evolución ni Caución: anulados; apertura/cierre (categoría o heurística en fila); Transferencia ni Deposito/Depósito si aparecieran en datos; meses desmarcados en Configuración → Inclusión por mes (meses_excluidos en Supabase/localStorage). Base histórica y Todas las transacciones siguen completas.</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Traspasos internos (solapa)</v>
+        <v>Datos</v>
       </c>
       <c r="B22" t="str">
-        <v>Listado de movimientos con categoría extracto Transferencia o Deposito/Depósito (no anulados), con monto de registro y equivalente en moneda de vista; columnas extracto y categoría/cuenta de matriz (nueva en BD o fallback).</v>
+        <v>Transacciones y tipo de cambio desde Supabase (carga paginada de a 1000 filas por request para no truncar resultados). Cotización faltante: se usa la fecha anterior disponible.</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Datos</v>
+        <v>Tablas y scroll</v>
       </c>
       <c r="B23" t="str">
-        <v>Transacciones y tipo de cambio desde Supabase (carga paginada de a 1000 filas por request para no truncar resultados). Cotización faltante: se usa la fecha anterior disponible.</v>
+        <v>Encabezados de columna anclados (sticky) al desplazarse. Flujo por mes: scroll vertical de la página (sin caja con max-height) para llegar bien al pie de la tabla; scroll horizontal en el wrap si hace falta. Otras solapas listas anchas con scroll horizontal.</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Tablas y scroll</v>
+        <v>Menú lateral</v>
       </c>
       <c r="B24" t="str">
-        <v>Encabezados de columna anclados (sticky) al desplazarse. Flujo por mes: scroll vertical de la página (sin caja con max-height) para llegar bien al pie de la tabla; scroll horizontal en el wrap si hace falta. Otras solapas listas anchas con scroll horizontal.</v>
+        <v>Sidebar izquierdo colapsable/expandible; botón toggle (▶/◀); Home, Novedades, Configuración, Seguridad (solo admin con permiso), Cerrar sesión; estado expandido en localStorage.</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Menú lateral</v>
+        <v>Seguridad y roles</v>
       </c>
       <c r="B25" t="str">
-        <v>Sidebar izquierdo colapsable/expandible; botón toggle (▶/◀); Home, Novedades, Configuración, Seguridad (solo admin con permiso), Cerrar sesión; estado expandido en localStorage.</v>
+        <v>Login con email/contraseña, registro o invitado anónimo (visor). Permisos desde Supabase: exportar_base_historica, dashboard_operador, assign_roles. Visor: solo solapa Flujo por mes y botón Exportar Base Histórica (sin edición ni solapa Errores en modal mes). Encargado/Admin: resto del dashboard. Admin: vista Seguridad (usuarios/roles y permisos por rol). La tabla de usuarios solo muestra cuentas con email (no sesiones anónimas). Sin SQL de seguridad desplegado, la app mantiene modo compatibilidad con acceso completo.</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Seguridad y roles</v>
+        <v>Registro y contraseña</v>
       </c>
       <c r="B26" t="str">
-        <v>Login con email/contraseña, registro o invitado anónimo (visor). Permisos desde Supabase: exportar_base_historica, dashboard_operador, assign_roles. Visor: solo solapa Flujo por mes y botón Exportar Base Histórica (sin edición ni solapa Errores en modal mes). Encargado/Admin: resto del dashboard. Admin: vista Seguridad (usuarios/roles y permisos por rol). La tabla de usuarios solo muestra cuentas con email (no sesiones anónimas). Sin SQL de seguridad desplegado, la app mantiene modo compatibilidad con acceso completo.</v>
+        <v>Si Supabase rechaza la contraseña (débil o en listas de filtrados), el mensaje se muestra en español en pantalla; ayuda bajo el campo y mínimo 8 caracteres en el formulario.</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Registro y contraseña</v>
+        <v>Repositorio Git (GitHub)</v>
       </c>
       <c r="B27" t="str">
-        <v>Si Supabase rechaza la contraseña (débil o en listas de filtrados), el mensaje se muestra en español en pantalla; ayuda bajo el campo y mínimo 8 caracteres en el formulario.</v>
+        <v>Repo: https://github.com/lucasbustosmartin-coder/fornitalia. Rama main. .gitignore excluye node_modules, .venv, .env. Para actualizar: git add . ; git commit -m "mensaje" ; git push origin main.</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Repositorio Git (GitHub)</v>
+        <v>App en producción (Vercel)</v>
       </c>
       <c r="B28" t="str">
-        <v>Repo: https://github.com/lucasbustosmartin-coder/fornitalia. Rama main. .gitignore excluye node_modules, .venv, .env. Para actualizar: git add . ; git commit -m "mensaje" ; git push origin main.</v>
+        <v>URL pública: https://fornitalia.vercel.app/ (vercel.json reescribe / al dashboard). Cada push a main en GitHub dispara redeploy automático en Vercel. Proyecto: fornitalia, equipo Lucas Bustos, plan Hobby.</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>App en producción (Vercel)</v>
+        <v>Exportar a Excel</v>
       </c>
       <c r="B29" t="str">
-        <v>URL pública: https://fornitalia.vercel.app/ (vercel.json reescribe / al dashboard). Cada push a main en GitHub dispara redeploy automático en Vercel. Proyecto: fornitalia, equipo Lucas Bustos, plan Hobby.</v>
+        <v>Botón en la barra de la tabla (solo icono). Exporta la tabla de transacciones tal como está en Supabase: una hoja "Transacciones" con columnas fecha, mes, anio, tipo_movimiento, monto (valor numérico para fórmulas), status, medio_pago, moneda, descripcion, cliente, categoria, cat_desc, origen_archivo, cuenta_contable, editado, editado_detalle. Export Errores: incluye categoria_matriz y cuenta_matriz (misma lógica que el dashboard); monto como número.</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Exportar a Excel</v>
+        <v>Flujo de despliegue</v>
       </c>
       <c r="B30" t="str">
-        <v>Botón en la barra de la tabla (solo icono). Exporta la tabla de transacciones tal como está en Supabase: una hoja "Transacciones" con columnas fecha, mes, anio, tipo_movimiento, monto (valor numérico para fórmulas), status, medio_pago, moneda, descripcion, cliente, categoria, cat_desc, origen_archivo, cuenta_contable, editado, editado_detalle. Export Errores: incluye categoria_matriz y cuenta_matriz (misma lógica que el dashboard); monto como número.</v>
+        <v>Al terminar cada tarea: el usuario prueba en local y confirma; recién entonces el asistente hace git add, commit y push (Vercel redepliega automático). No se despliega hasta confirmación.</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Flujo de despliegue</v>
+        <v>Versiones en bitácora</v>
       </c>
       <c r="B31" t="str">
-        <v>Al terminar cada tarea: el usuario prueba en local y confirma; recién entonces el asistente hace git add, commit y push (Vercel redepliega automático). No se despliega hasta confirmación.</v>
+        <v>Hoja "Versiones" en Bitacora_tareas.xlsx: registro incremental (1.0, 1.1, …) con fecha y descripción de cada despliegue a Git/Vercel.</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Versiones en bitácora</v>
+        <v>Campo moneda (BD)</v>
       </c>
       <c r="B32" t="str">
-        <v>Hoja "Versiones" en Bitacora_tareas.xlsx: registro incremental (1.0, 1.1, …) con fecha y descripción de cada despliegue a Git/Vercel.</v>
+        <v>Columna moneda en tabla transacciones (ARS/USD). Si está informada, el dashboard la usa salvo reglas de negocio: Mercado Pago y Transferencia Morba siempre ARS para conversión (también morva por typo). Si moneda vacía, infiere desde textos/medio (dólar → USD). Export a Excel incluye moneda.</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Campo moneda (BD)</v>
+        <v>Edición desde modal Errores</v>
       </c>
       <c r="B33" t="str">
-        <v>Columna moneda en tabla transacciones (ARS/USD). Si está informada, el dashboard la usa salvo reglas de negocio: Mercado Pago y Transferencia Morba siempre ARS para conversión (también morva por typo). Si moneda vacía, infiere desde textos/medio (dólar → USD). Export a Excel incluye moneda.</v>
+        <v>En el detalle de errores, icono de edición por registro. Abre modal para corregir: Categoría y Cuenta contable solo desde valores existentes en BD; Descripción libre. UPDATE en transacciones solo si hubo cambios respecto a la fila; si no, aviso (antes el modal cerraba sin guardar). Tras UPDATE se verifica que haya filas actualizadas; nota contextual para inconsistencia categoría/cuenta/descripción. editado y editado_detalle al guardar con cambios.</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Edición desde modal Errores</v>
+        <v>Campos editado y editado_detalle</v>
       </c>
       <c r="B34" t="str">
-        <v>En el detalle de errores, icono de edición por registro. Abre modal para corregir: Categoría y Cuenta contable solo desde valores existentes en BD; Descripción libre. UPDATE en transacciones solo si hubo cambios respecto a la fila; si no, aviso (antes el modal cerraba sin guardar). Tras UPDATE se verifica que haya filas actualizadas; nota contextual para inconsistencia categoría/cuenta/descripción. editado y editado_detalle al guardar con cambios.</v>
+        <v>En transacciones: editado (boolean) y editado_detalle (texto, ej. "Categoria, Descripcion, Cuenta Contable"). Migración supabase_transacciones_editado.sql. Export Excel los incluye.</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Campos editado y editado_detalle</v>
+        <v>Tipo de error en Errores</v>
       </c>
       <c r="B35" t="str">
-        <v>En transacciones: editado (boolean) y editado_detalle (texto, ej. "Categoria, Descripcion, Cuenta Contable"). Migración supabase_transacciones_editado.sql. Export Excel los incluye.</v>
+        <v>Tabla de errores muestra columna Tipo de error: Inconsistencia entre Categoria, Cuenta Contable y Descripcion; o Potencial registro duplicado. Excepciones explícitas cat/cuenta (Impuestos/IIBB, Logistica/Fletes, Alquileres varias cuentas, Activos/Hornos, Mantenimiento/Ferreteria, Sueldos/Comisiones Ventas y variantes, Marketing/Creación contenido, Honorarios/Honorarios Contables) no marcan inconsistencia. Export a Excel incluye tipo_error.</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Tipo de error en Errores</v>
+        <v>Detección de potencial duplicado</v>
       </c>
       <c r="B36" t="str">
-        <v>Tabla de errores muestra columna Tipo de error: Inconsistencia entre Categoria, Cuenta Contable y Descripcion; o Potencial registro duplicado. Excepciones explícitas cat/cuenta (Impuestos/IIBB, Logistica/Fletes, Alquileres varias cuentas, Activos/Hornos, Mantenimiento/Ferreteria, Sueldos/Comisiones Ventas y variantes, Marketing/Creación contenido, Honorarios/Honorarios Contables) no marcan inconsistencia. Export a Excel incluye tipo_error.</v>
+        <v>Registros con misma fecha, monto, tipo_movimiento y descripción similar se marcan como potencial duplicado. Icono Ver abre modal con comparación Este registro / Posible duplicado; acciones: Excluir de cálculos (anular) o Eliminar registro.</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Detección de potencial duplicado</v>
+        <v>Filtro por tipo de error</v>
       </c>
       <c r="B37" t="str">
-        <v>Registros con misma fecha, monto, tipo_movimiento y descripción similar se marcan como potencial duplicado. Icono Ver abre modal con comparación Este registro / Posible duplicado; acciones: Excluir de cálculos (anular) o Eliminar registro.</v>
+        <v>En la solapa Errores, selector para filtrar por tipo: Todos, Inconsistencia (categoría/cuenta/descripción), Potencial registro duplicado. La exportación a Excel exporta solo los registros visibles según el filtro.</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Filtro por tipo de error</v>
+        <v>Duplicados: condición cliente</v>
       </c>
       <c r="B38" t="str">
-        <v>En la solapa Errores, selector para filtrar por tipo: Todos, Inconsistencia (categoría/cuenta/descripción), Potencial registro duplicado. La exportación a Excel exporta solo los registros visibles según el filtro.</v>
+        <v>Dos registros son potencial duplicado solo si coinciden en fecha, monto, tipo_movimiento, descripción similar y además cliente es igual; si cliente es distinto no se marcan como duplicado. Modal de comparación muestra id_origen y Cliente.</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Duplicados: condición cliente</v>
+        <v>Regla bitácora</v>
       </c>
       <c r="B39" t="str">
-        <v>Dos registros son potencial duplicado solo si coinciden en fecha, monto, tipo_movimiento, descripción similar y además cliente es igual; si cliente es distinto no se marcan como duplicado. Modal de comparación muestra id_origen y Cliente.</v>
+        <v>Actualizar todas las solapas necesarias: Log (siempre que haya tarea), Resumen (si cambia funcionalidad), Presupuesto (si agrega o cambia entregable comercial), Versiones (en despliegue). Regenerar Excel tras editar crear-bitacora-excel.js.</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Regla bitácora</v>
+        <v>Evolución (tabla dinámica)</v>
       </c>
       <c r="B40" t="str">
-        <v>Actualizar todas las solapas necesarias: Log (siempre que haya tarea), Resumen (si cambia funcionalidad), Presupuesto (si agrega o cambia entregable comercial), Versiones (en despliegue). Regenerar Excel tras editar crear-bitacora-excel.js.</v>
+        <v>Solapa Evolución: Agrupar por = Nueva categoría (matriz) o Nueva cuenta contable (matriz) —prioriza nueva_categoria / nueva_cuenta_contable en BD y si faltan usa extracto con validación—; Período = Diario o Mensual (MM-YYYY). Columnas = períodos, celdas = neto en moneda seleccionada, columna Total.</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Evolución (tabla dinámica)</v>
+        <v>Estado Financiero (tabla dinámica)</v>
       </c>
       <c r="B41" t="str">
-        <v>Solapa Evolución: Agrupar por = Nueva categoría (matriz) o Nueva cuenta contable (matriz) —prioriza nueva_categoria / nueva_cuenta_contable en BD y si faltan usa extracto con validación—; Período = Diario o Mensual (MM-YYYY). Columnas = períodos, celdas = neto en moneda seleccionada, columna Total.</v>
+        <v>Solapa Estado Financiero: estructura desde Supabase ef_estructura (hoja EF_Estructura del extracto). Columna Ítem con viñeta en detalle; períodos en columnas horizontales; subtotales (secciones) y fórmulas (Margen Bruto, Flujo operativo, etc.) con colores distintos y % del Flujo Operativo Generado bajo montos; conciliación (§7) oculta en vista y export. Montos por ef_subitem; scroll anclado con thead sticky. Exportar EF a Excel (xlsx-js-style): montos enteros, columna Notas con análisis interpretativo (+/−), % en formato 0.0%, colores de fila también en meses sin dato.</v>
       </c>
     </row>
     <row r="42">
@@ -3315,7 +3434,7 @@
         <v>Edición completa de registros</v>
       </c>
       <c r="B47" t="str">
-        <v>Modal de edición con todos los campos: fecha, mes, año, tipo movimiento, monto, moneda, status, medio pago, categoría, nueva categoría (matriz), cuenta contable, nueva cuenta contable (matriz), costo_directo y costo_indirecto (Y/N o vacío), origen archivo, descripción, cliente (combo con valores existentes en BD), cat_desc, id_origen, id_operación. Combos para campos normalizados (valores existentes en BD). editado y editado_detalle al guardar. Tras guardar OK: recarga datos, recalcula flujo, y si el modal de detalle del mes sigue abierto se vuelve a armar ese modal para no mostrar HTML viejo.</v>
+        <v>Modal de edición con todos los campos: fecha, mes, año, tipo movimiento, monto, moneda, status, medio pago, categoría, nueva categoría (matriz), cuenta contable, nueva cuenta contable (matriz), costo_directo y costo_indirecto (Y/N o vacío), ef_item y ef_subitem (estado de flujo), origen archivo, descripción, cliente (combo con valores existentes en BD), cat_desc, id_origen, id_operación. Combos para campos normalizados (valores existentes en BD). editado y editado_detalle al guardar. Tras guardar OK: recarga datos, recalcula flujo, y si el modal de detalle del mes sigue abierto se vuelve a armar ese modal para no mostrar HTML viejo.</v>
       </c>
     </row>
     <row r="48">
@@ -3419,7 +3538,7 @@
         <v>Upload de extracto normalizado</v>
       </c>
       <c r="B60" t="str">
-        <v>Botón en la app para reemplazar transacciones desde la hoja Normalizado (generada con npm run normalizar-extracto desde Fornitalia_Movimientos), con validación previa, IDs y cat_desc persistidos cuando existen, confirmación de seguridad, id_origen técnico y carga en lotes.</v>
+        <v>Botón en la app para reemplazar transacciones desde la hoja Normalizado (p. ej. Base_Fornitalia_To_App): incluye nueva_categoria, nueva_cuenta_contable, costo_directo/indirecto y columnas EF_Item / EF_SubItem → ef_item / ef_subitem en Supabase. Validación previa, carga en lotes y log de excluidos.</v>
       </c>
     </row>
     <row r="61">
@@ -3534,7 +3653,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C45"/>
+  <dimension ref="A1:C46"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -4036,9 +4155,20 @@
         <v>Modal detalle mensual: columna Cliente en tabla expandida; icono ojo por fila abre modal de edición (detalle completo). APP_VERSION 1.60. Despliegue producción Vercel.</v>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>1.78</v>
+      </c>
+      <c r="B46" t="str">
+        <v>28/05/2026</v>
+      </c>
+      <c r="C46" t="str">
+        <v>Estado Financiero: export Excel con % corregidos, columna Notas, colores de fila en celdas vacías (xlsx-js-style); UI EF (horizontal, fórmulas, scroll, ayudas). Flujo: eliminada solapa Traspasos internos y tarjeta Neto caja; resumen 3 tarjetas operativas. APP_VERSION 1.78. Despliegue producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C45"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C46"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.96: EF gráficos y detalle, ratios alineados, fix meses_excluidos en Supabase.
Incluye trabajo desde v1.78: solapa Estado Financiero con gráficos y modal de detalle por celda, persistencia de inclusión por mes en config_dashboard y alerta si falla el guardado.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E155"/>
+  <dimension ref="A1:E166"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -3046,9 +3046,196 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="156">
+      <c r="A156" t="str">
+        <v>28/05/2026</v>
+      </c>
+      <c r="B156" t="str">
+        <v>15:52</v>
+      </c>
+      <c r="C156" t="str">
+        <v>Comisiones/Ventas % por subítems EF</v>
+      </c>
+      <c r="D156" t="str">
+        <v>Ratio Flujo por mes: numerador egresos con ef_subitem Comisiones por Ventas; denominador ingresos con ef_subitem Cobranzas por Ventas (Efectivo neto ingresado). Alias cortos normalizados (resolveEfSubitemCanon). Sin ef_subitem la fila no entra. Ayuda PDF/tooltip y fornitalia-ef-estructura.js documentados. APP_VERSION 1.82.</v>
+      </c>
+      <c r="E156" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="str">
+        <v>28/05/2026</v>
+      </c>
+      <c r="B157" t="str">
+        <v>15:59</v>
+      </c>
+      <c r="C157" t="str">
+        <v>Ratios Flujo = EF sin redondeo en %</v>
+      </c>
+      <c r="D157" t="str">
+        <v>Costo dir./ind. desde totales §2/§3 computeEfMontosPorOrden (igual EF). % con montos completos (no enteros de pantalla). EF corregido: pct sobre valor real, display entero. APP_VERSION 1.88.</v>
+      </c>
+      <c r="E157" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="str">
+        <v>30/05/2026</v>
+      </c>
+      <c r="B158" t="str">
+        <v>17:04</v>
+      </c>
+      <c r="C158" t="str">
+        <v>Estado Financiero: gráficos por fila y columna</v>
+      </c>
+      <c r="D158" t="str">
+        <v>Icono línea en cada fila (evolución mensual del rubro en modal Chart.js). Icono barras en columnas de período y Total (waterfall del Flujo Operativo Generado con líneas de Margen bruto, Utilidad operativa, Flujo neto operativo y Flujo neto del período). Ayuda del panel actualizada.</v>
+      </c>
+      <c r="E158" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="str">
+        <v>30/05/2026</v>
+      </c>
+      <c r="B159" t="str">
+        <v>17:11</v>
+      </c>
+      <c r="C159" t="str">
+        <v>EF gráficos: iconos compactos y waterfall</v>
+      </c>
+      <c r="D159" t="str">
+        <v>Iconos más pequeños; barras al lado derecho del período en cabecera. Gráfico de consumo: solo barras de tramos (flujo y costos); hitos Margen/Utilidad/Flujos netos solo como líneas punteadas horizontales.</v>
+      </c>
+      <c r="E159" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="str">
+        <v>30/05/2026</v>
+      </c>
+      <c r="B160" t="str">
+        <v>17:11</v>
+      </c>
+      <c r="C160" t="str">
+        <v>EF gráficos: línea abs, escala y % hitos</v>
+      </c>
+      <c r="D160" t="str">
+        <v>Serie línea: costos en valor absoluto y color único (azul), eje desde 0. Waterfall: escala Y con padding y zoom cuando hitos están muy juntos; líneas punteadas con monto y % del Flujo Operativo Generado.</v>
+      </c>
+      <c r="E160" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="str">
+        <v>30/05/2026</v>
+      </c>
+      <c r="B161" t="str">
+        <v>17:17</v>
+      </c>
+      <c r="C161" t="str">
+        <v>EF waterfall: solo 2 líneas de referencia</v>
+      </c>
+      <c r="D161" t="str">
+        <v>Gráfico de consumo por columna: líneas punteadas únicamente Utilidad operativa y Flujo neto del período (sin Margen bruto ni Flujo neto operativo).</v>
+      </c>
+      <c r="E161" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="str">
+        <v>30/05/2026</v>
+      </c>
+      <c r="B162" t="str">
+        <v>17:19</v>
+      </c>
+      <c r="C162" t="str">
+        <v>EF waterfall: escala y etiquetas hitos</v>
+      </c>
+      <c r="D162" t="str">
+        <v>Escala Y centrada en Utilidad operativa y Flujo neto del período (no aplasta por Flujo Op. alto). Etiquetas en dos líneas con separación mínima en px; conector si el texto se desplaza. Modal EF más alto.</v>
+      </c>
+      <c r="E162" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="str">
+        <v>30/05/2026</v>
+      </c>
+      <c r="B163" t="str">
+        <v>17:30</v>
+      </c>
+      <c r="C163" t="str">
+        <v>EF: etiqueta Anticipos de impuestos</v>
+      </c>
+      <c r="D163" t="str">
+        <v>LÍNEA B: ANTICIPOS DE IMPUESTOS → ANTICIPOS DE IMPUESTOS en Estado Financiero, export y parse EF_Estructura (efItemEtiquetaDisplay).</v>
+      </c>
+      <c r="E163" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="str">
+        <v>30/05/2026</v>
+      </c>
+      <c r="B164" t="str">
+        <v>17:37</v>
+      </c>
+      <c r="C164" t="str">
+        <v>EF: detalle al clic en importe</v>
+      </c>
+      <c r="D164" t="str">
+        <v>Clic en celda de monto abre modal con transacciones (ef_subitem) del rubro/sección/fórmula y período; suma y total de fila. Indicadores de gestión sin detalle.</v>
+      </c>
+      <c r="E164" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="str">
+        <v>30/05/2026</v>
+      </c>
+      <c r="B165" t="str">
+        <v>17:47</v>
+      </c>
+      <c r="C165" t="str">
+        <v>Fix meses_excluidos no persistía en Supabase</v>
+      </c>
+      <c r="D165" t="str">
+        <v>En producción faltaba columna config_dashboard.meses_excluidos: el upsert fallaba en silencio. Migración aplicada en proyecto Fornitalia; syncConfigToSupabase devuelve error y alerta al guardar Config si falla.</v>
+      </c>
+      <c r="E165" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="str">
+        <v>30/05/2026</v>
+      </c>
+      <c r="B166" t="str">
+        <v>17:48</v>
+      </c>
+      <c r="C166" t="str">
+        <v>Despliegue v1.96 producción</v>
+      </c>
+      <c r="D166" t="str">
+        <v>Push main y vercel --prod: EF gráficos y detalle por celda; ratios Flujo=EF; fix meses_excluidos en Supabase; APP_VERSION 1.96.</v>
+      </c>
+      <c r="E166" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E155"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E166"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3074,7 +3261,7 @@
         <v>Flujo de caja por mes</v>
       </c>
       <c r="B2" t="str">
-        <v>Tabla de caja operativa: columnas Ingresos, Egresos y G/P operativo (sin anulados ni apertura/cierre de caja; traspasos no incluidos en el import). Ratios Costo dir./ind./total sobre ingresos operativos; columna Caución (solo origen ARS, montos en pesos; tasas desde serie_cauciones.json o Serie_Cauciones.xlsx; % configurable). Proyección de caución en ARS. Meses excluidos por Configuración → Inclusión por mes no aparecen en filas ni totales. Icono de ayuda con criterios de la tabla.</v>
+        <v>Tabla de caja operativa: columnas Ingresos, Egresos y G/P operativo (sin anulados ni apertura/cierre de caja; traspasos no incluidos en el import). Comisiones/Ventas % por subítems EF; Costo dir./ind. ÷ FLUJO OPERATIVO GENERADO (§2/§3); Costo total/Ingreso total = total egresos operativos ÷ FLUJO OPERATIVO GENERADO; columna Caución (solo origen ARS). Proyección de ratios y caución en ARS. Meses excluidos por Configuración → Inclusión por mes no aparecen en filas ni totales. Icono de ayuda con criterios de la tabla.</v>
       </c>
     </row>
     <row r="3">
@@ -3106,7 +3293,7 @@
         <v>Comisiones/Ventas %</v>
       </c>
       <c r="B6" t="str">
-        <v>Columna: porcentaje comisiones (egresos comisión desde Sueldos) sobre ventas del mes. Icono de ayuda al clic: "Corresponde solo a las comisiones por venta."</v>
+        <v>Columna: egresos con ef_subitem «Comisiones por Ventas» ÷ ingresos con ef_subitem «Cobranzas por Ventas (Efectivo neto ingresado)» del mes (subítems canónicos EF; alias cortos se normalizan al import). Sin ef_subitem la fila no entra al ratio. Ayuda al clic en icono de columna e informe PDF (template-flujo-informe-pdf).</v>
       </c>
     </row>
     <row r="7">
@@ -3386,7 +3573,7 @@
         <v>Estado Financiero (tabla dinámica)</v>
       </c>
       <c r="B41" t="str">
-        <v>Solapa Estado Financiero: estructura desde Supabase ef_estructura (hoja EF_Estructura del extracto). Columna Ítem con viñeta en detalle; períodos en columnas horizontales; subtotales (secciones) y fórmulas (Margen Bruto, Flujo operativo, etc.) con colores distintos y % del Flujo Operativo Generado bajo montos; conciliación (§7) oculta en vista y export. Montos por ef_subitem; scroll anclado con thead sticky. Exportar EF a Excel (xlsx-js-style): montos enteros, columna Notas con análisis interpretativo (+/−), % en formato 0.0%, colores de fila también en meses sin dato.</v>
+        <v>Solapa Estado Financiero: estructura desde Supabase ef_estructura (hoja EF_Estructura del extracto). Columna Ítem con viñeta en detalle; períodos en columnas horizontales; subtotales y fórmulas con % del Flujo Operativo Generado. Clic en importe: modal con todas las transacciones (ef_subitem) que componen el valor del período o total. Gráficos línea (fila) y barras (columna). Exportar EF a Excel. Conciliación §7 oculta en vista y export.</v>
       </c>
     </row>
     <row r="42">
@@ -3653,7 +3840,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C46"/>
+  <dimension ref="A1:C48"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -4166,9 +4353,31 @@
         <v>Estado Financiero: export Excel con % corregidos, columna Notas, colores de fila en celdas vacías (xlsx-js-style); UI EF (horizontal, fórmulas, scroll, ayudas). Flujo: eliminada solapa Traspasos internos y tarjeta Neto caja; resumen 3 tarjetas operativas. APP_VERSION 1.78. Despliegue producción Vercel.</v>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>1.82</v>
+      </c>
+      <c r="B47" t="str">
+        <v>28/05/2026</v>
+      </c>
+      <c r="C47" t="str">
+        <v>Comisiones/Ventas %: ratio por ef_subitem (Comisiones por Ventas ÷ Cobranzas por Ventas Efectivo neto ingresado); alias en fornitalia-ef-estructura.js; ayuda PDF/tooltip y bitácora actualizados. APP_VERSION 1.82.</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>1.88</v>
+      </c>
+      <c r="B48" t="str">
+        <v>28/05/2026</v>
+      </c>
+      <c r="C48" t="str">
+        <v>Ratios costo Flujo alineados a EF: secciones §1–§3, % sin redondear montos; Costo total = egresos operativos ÷ Flujo Op. APP_VERSION 1.88.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C46"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C48"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v2.02: Reportes, matriz relaciones, Cat×cuenta Confirmado y filtro Cliente.
Menú Reportes con export Excel desde Supabase; solapa cruce cat×cuenta solo Confirmado; filtro Cliente en Todas las transacciones.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E166"/>
+  <dimension ref="A1:E172"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -3233,16 +3233,118 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="167">
+      <c r="A167" t="str">
+        <v>01/06/2026</v>
+      </c>
+      <c r="B167" t="str">
+        <v>15:16</v>
+      </c>
+      <c r="C167" t="str">
+        <v>Menú Reportes: export Matriz Relaciones desde Supabase</v>
+      </c>
+      <c r="D167" t="str">
+        <v>Nueva vista Reportes en sidebar; export Excel Matriz_Relaciones_Transacciones_Fornitalia (4 solapas) desde cacheTransacciones. Módulo compartido scripts/lib/fornitalia-matriz-relaciones-transacciones.js. Permiso exportar base o panel operador. APP_VERSION 1.97.</v>
+      </c>
+      <c r="E167" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="str">
+        <v>01/06/2026</v>
+      </c>
+      <c r="B168" t="str">
+        <v>15:19</v>
+      </c>
+      <c r="C168" t="str">
+        <v>Matriz relaciones: solapa Cat_x_Cuenta_Registros</v>
+      </c>
+      <c r="D168" t="str">
+        <v>Tabla cruzada Nueva Categoria (filas) × Cuenta Contable (columnas) con # registros por cruce y totales; en export Reportes y script generar-matriz. APP_VERSION 1.98.</v>
+      </c>
+      <c r="E168" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="str">
+        <v>01/06/2026</v>
+      </c>
+      <c r="B169" t="str">
+        <v>15:35</v>
+      </c>
+      <c r="C169" t="str">
+        <v>Matriz relaciones: solo status Confirmado</v>
+      </c>
+      <c r="D169" t="str">
+        <v>Quita exclusion por categoría (Impuestos, Ventas, etc.); todas las solapas del export Reportes filtran únicamente status Confirmado. fornitalia-matriz-relaciones-transacciones.js. APP_VERSION 1.99.</v>
+      </c>
+      <c r="E169" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="str">
+        <v>01/06/2026</v>
+      </c>
+      <c r="B170" t="str">
+        <v>15:38</v>
+      </c>
+      <c r="C170" t="str">
+        <v>Cat_x_Cuenta_Registros: filtro Confirmado aislado</v>
+      </c>
+      <c r="D170" t="str">
+        <v>Solo la solapa cruce cat×cuenta filtra status Confirmado sin exclusion por categoria; matriz costo y proveedores mantienen exclusiones de categorias. APP_VERSION 2.0.</v>
+      </c>
+      <c r="E170" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="str">
+        <v>01/06/2026</v>
+      </c>
+      <c r="B171" t="str">
+        <v>18:18</v>
+      </c>
+      <c r="C171" t="str">
+        <v>Todas las transacciones: filtro Cliente</v>
+      </c>
+      <c r="D171" t="str">
+        <v>Select Cliente en barra de filtros (valores únicos de la base); combinable con mes, categoría, cuenta, tipo e id operación. APP_VERSION 2.01.</v>
+      </c>
+      <c r="E171" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="str">
+        <v>01/06/2026</v>
+      </c>
+      <c r="B172" t="str">
+        <v>22:39</v>
+      </c>
+      <c r="C172" t="str">
+        <v>Despliegue v2.02 producción</v>
+      </c>
+      <c r="D172" t="str">
+        <v>Push main y vercel --prod: menú Reportes y export Matriz Relaciones; Cat_x_Cuenta_Registros solo Confirmado; filtro Cliente en Todas las transacciones; APP_VERSION 2.02.</v>
+      </c>
+      <c r="E172" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E166"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E172"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B62"/>
+  <dimension ref="A1:B63"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -3578,175 +3680,183 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Evolución: detalle al clic y exportar</v>
+        <v>Reportes (menú lateral)</v>
       </c>
       <c r="B42" t="str">
-        <v>Clic en un valor abre modal con detalle: Fecha, Categoría (matriz), Cuenta (matriz), Descripción, Monto. Exportar Evolución a Excel: primera columna con el mismo criterio de agrupación.</v>
+        <v>Vista Reportes: exportar Matriz de relaciones desde Supabase. Matriz costo y proveedores con exclusiones de categoría; solapa Cat_x_Cuenta_Registros solo status Confirmado (todas las categorías). Resumen antes de exportar.</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Exportaciones Excel</v>
+        <v>Evolución: detalle al clic y exportar</v>
       </c>
       <c r="B43" t="str">
-        <v>Todas las exportaciones incluyen una fila título con la moneda. Exportar Base Histórica (icono Excel) en la línea del selector de moneda; Exportar Evolución a Excel con el mismo icono.</v>
+        <v>Clic en un valor abre modal con detalle: Fecha, Categoría (matriz), Cuenta (matriz), Descripción, Monto. Exportar Evolución a Excel: primera columna con el mismo criterio de agrupación.</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Evolución: orden ingreso/egreso</v>
+        <v>Exportaciones Excel</v>
       </c>
       <c r="B44" t="str">
-        <v>En la tabla Evolución las filas se muestran primero las de ingreso (total &gt;= 0) y luego las de egreso (total &lt; 0); dentro de cada grupo orden alfabético. Aplica al agrupar por categoría o cuenta de matriz.</v>
+        <v>Todas las exportaciones incluyen una fila título con la moneda. Exportar Base Histórica (icono Excel) en la línea del selector de moneda; Exportar Evolución a Excel con el mismo icono.</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Int. por caución</v>
+        <v>Evolución: orden ingreso/egreso</v>
       </c>
       <c r="B45" t="str">
-        <v>Columna en flujo por mes: interés mensual por colocar el sobrante de caja a la tasa diaria de la serie de cauciones. Carga Serie_Cauciones.xlsx al refrescar (o serie_cauciones.json si no hay Excel). Cálculo: base = G/P acumulado a la fecha + interés acumulado; Int T = base × tasa. Clic en el valor abre modal con marcha (G/P acum, Int T-1, Base, Tasa, Int T).</v>
+        <v>En la tabla Evolución las filas se muestran primero las de ingreso (total &gt;= 0) y luego las de egreso (total &lt; 0); dentro de cada grupo orden alfabético. Aplica al agrupar por categoría o cuenta de matriz.</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Todas las transacciones</v>
+        <v>Int. por caución</v>
       </c>
       <c r="B46" t="str">
-        <v>Solapa que lista todas las transacciones con todas las columnas. Filtros por mes, categoría (matriz) y cuenta (matriz) —misma prioridad nueva_* que Evolución—, tipo (Ingreso/Egreso) e id operación (texto). Columnas principales cat/cuenta por matriz; columnas nueva_* como en BD. Botón Editar por registro abre modal de edición completa.</v>
+        <v>Columna en flujo por mes: interés mensual por colocar el sobrante de caja a la tasa diaria de la serie de cauciones. Carga Serie_Cauciones.xlsx al refrescar (o serie_cauciones.json si no hay Excel). Cálculo: base = G/P acumulado a la fecha + interés acumulado; Int T = base × tasa. Clic en el valor abre modal con marcha (G/P acum, Int T-1, Base, Tasa, Int T).</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Edición completa de registros</v>
+        <v>Todas las transacciones</v>
       </c>
       <c r="B47" t="str">
-        <v>Modal de edición con todos los campos: fecha, mes, año, tipo movimiento, monto, moneda, status, medio pago, categoría, nueva categoría (matriz), cuenta contable, nueva cuenta contable (matriz), costo_directo y costo_indirecto (Y/N o vacío), ef_item y ef_subitem (estado de flujo), origen archivo, descripción, cliente (combo con valores existentes en BD), cat_desc, id_origen, id_operación. Combos para campos normalizados (valores existentes en BD). editado y editado_detalle al guardar. Tras guardar OK: recarga datos, recalcula flujo, y si el modal de detalle del mes sigue abierto se vuelve a armar ese modal para no mostrar HTML viejo.</v>
+        <v>Solapa que lista todas las transacciones con todas las columnas. Filtros por mes, categoría (matriz), cuenta (matriz), cliente, tipo (Ingreso/Egreso) e id operación (texto). Columnas principales cat/cuenta por matriz; columnas nueva_* como en BD. Botón Editar por registro abre modal de edición completa.</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Proyección próximos 3 meses</v>
+        <v>Edición completa de registros</v>
       </c>
       <c r="B48" t="str">
-        <v>Debajo del total real en Flujo por mes: "Próximos 3 meses proyectados" con ventana rodante. Configuración (sidebar): método (Mediana/Promedio) y meses de historia (3, 6, 12, 24). Ingresos, egresos, G/P y ratios proyectados por mes.</v>
+        <v>Modal de edición con todos los campos: fecha, mes, año, tipo movimiento, monto, moneda, status, medio pago, categoría, nueva categoría (matriz), cuenta contable, nueva cuenta contable (matriz), costo_directo y costo_indirecto (Y/N o vacío), ef_item y ef_subitem (estado de flujo), origen archivo, descripción, cliente (combo con valores existentes en BD), cat_desc, id_origen, id_operación. Combos para campos normalizados (valores existentes en BD). editado y editado_detalle al guardar. Tras guardar OK: recarga datos, recalcula flujo, y si el modal de detalle del mes sigue abierto se vuelve a armar ese modal para no mostrar HTML viejo.</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Int. por caución proyectado</v>
+        <v>Proyección próximos 3 meses</v>
       </c>
       <c r="B49" t="str">
-        <v>Punto de partida = G/P Total real + interés acumulado; tasa = promedio último mes real; días naturales; Int T-1 día 1 = (Int T-1 + Int T) último día del mes anterior. G/P acum en marcha = al inicio de cada día (real y proyectado). Ventana rodante: ingresos/egresos distintos por mes.</v>
+        <v>Debajo del total real en Flujo por mes: "Próximos 3 meses proyectados" con ventana rodante. Configuración (sidebar): método (Mediana/Promedio) y meses de historia (3, 6, 12, 24). Ingresos, egresos, G/P y ratios proyectados por mes.</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Disclaimer proyección</v>
+        <v>Int. por caución proyectado</v>
       </c>
       <c r="B50" t="str">
-        <v>Debajo de las filas proyectadas, texto en letra chica y gris oscuro que explica la metodología: Mediana/Promedio de N meses, ventana rodante, y cálculo de Int. por caución proyectado.</v>
+        <v>Punto de partida = G/P Total real + interés acumulado; tasa = promedio último mes real; días naturales; Int T-1 día 1 = (Int T-1 + Int T) último día del mes anterior. G/P acum en marcha = al inicio de cada día (real y proyectado). Ventana rodante: ingresos/egresos distintos por mes.</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Botones e iconos unificados</v>
+        <v>Disclaimer proyección</v>
       </c>
       <c r="B51" t="str">
-        <v>Todos los botones con mismo estilo: icono SVG + texto. Sidebar (chevron, home, engranaje), tabs con iconos, exportar con icono descarga, modales con iconos (Guardar, Cerrar, Excluir, Eliminar). Iconos solos (cerrar, editar, alerta) en SVG.</v>
+        <v>Debajo de las filas proyectadas, texto en letra chica y gris oscuro que explica la metodología: Mediana/Promedio de N meses, ventana rodante, y cálculo de Int. por caución proyectado.</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Configuración % G/P en caución</v>
+        <v>Botones e iconos unificados</v>
       </c>
       <c r="B52" t="str">
-        <v>Combo "% G/P acum. en caución" en Configuración con escala de 5 en 5 (100, 95, 90… hasta 0). Por defecto 100 %; menor % = más liquidez (menos interés por caución).</v>
+        <v>Todos los botones con mismo estilo: icono SVG + texto. Sidebar (chevron, home, engranaje), tabs con iconos, exportar con icono descarga, modales con iconos (Guardar, Cerrar, Excluir, Eliminar). Iconos solos (cerrar, editar, alerta) en SVG.</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Etiqueta Caución (x% cash)</v>
+        <v>Configuración % G/P en caución</v>
       </c>
       <c r="B53" t="str">
-        <v>Columna en flujo por mes: cabecera "Caución (x% cash)" donde x es el valor del parámetro % G/P; sin icono % a la izquierda. Modales de marcha y disclaimer usan "Caución".</v>
+        <v>Combo "% G/P acum. en caución" en Configuración con escala de 5 en 5 (100, 95, 90… hasta 0). Por defecto 100 %; menor % = más liquidez (menos interés por caución).</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>Meses a proyectar</v>
+        <v>Etiqueta Caución (x% cash)</v>
       </c>
       <c r="B54" t="str">
-        <v>En Configuración: combo Meses a proyectar (1, 2, 3, 4, 5, 6, 12). Flujo por mes y Evolución muestran esa cantidad de columnas/filas proyectadas.</v>
+        <v>Columna en flujo por mes: cabecera "Caución (x% cash)" donde x es el valor del parámetro % G/P; sin icono % a la izquierda. Modales de marcha y disclaimer usan "Caución".</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>Config por usuario en Supabase</v>
+        <v>Meses a proyectar</v>
       </c>
       <c r="B55" t="str">
-        <v>Tabla config_dashboard (user_id, proyección, caución, alertas y meses_excluidos JSON). Con Auth anónimo se sincroniza al cargar y al guardar; la config persiste por usuario en la base. Migración: supabase_config_dashboard.sql; meses excluidos: supabase_config_dashboard_meses_excluidos.sql.</v>
+        <v>En Configuración: combo Meses a proyectar (1, 2, 3, 4, 5, 6, 12). Flujo por mes y Evolución muestran esa cantidad de columnas/filas proyectadas.</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>Recorte % (cada lado)</v>
+        <v>Config por usuario en Supabase</v>
       </c>
       <c r="B56" t="str">
-        <v>En Configuración, combo Recorte % (cada lado) (0, 5, 10, 15, 20, 25) visible solo cuando el método es Promedio recortado. Más % = más suavizado. Persistido en config_dashboard (proyeccion_recorte).</v>
+        <v>Tabla config_dashboard (user_id, proyección, caución, alertas y meses_excluidos JSON). Con Auth anónimo se sincroniza al cargar y al guardar; la config persiste por usuario en la base. Migración: supabase_config_dashboard.sql; meses excluidos: supabase_config_dashboard_meses_excluidos.sql.</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>Novedades del Negocio</v>
+        <v>Recorte % (cada lado)</v>
       </c>
       <c r="B57" t="str">
-        <v>Ítem en sidebar que abre una vista con importadores de hornos y comercios de venta de hornos en Argentina (Buenos Aires). Datos recuperados por IA (Edge Function con Gemini + google_search). Nombre, dirección, teléfono y web por contacto.</v>
+        <v>En Configuración, combo Recorte % (cada lado) (0, 5, 10, 15, 20, 25) visible solo cuando el método es Promedio recortado. Más % = más suavizado. Persistido en config_dashboard (proyeccion_recorte).</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>Normalización de extracto bancario</v>
+        <v>Novedades del Negocio</v>
       </c>
       <c r="B58" t="str">
-        <v>npm run normalizar-extracto: lee Fornitalia_Movimientos.xlsx (o Extracto legado), hoja Normalizado con fecha_iso, tipo, medio, categoría, cuenta, moneda inferida, monto_original, tipo_cambio, monto_ars, id_cierre_caja, id_comprobante_pago, id_impuesto, cat_desc cuando vienen del export.</v>
+        <v>Ítem en sidebar que abre una vista con importadores de hornos y comercios de venta de hornos en Argentina (Buenos Aires). Datos recuperados por IA (Edge Function con Gemini + google_search). Nombre, dirección, teléfono y web por contacto.</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>Informe inconsistencias datos legacy (cliente)</v>
+        <v>Normalización de extracto bancario</v>
       </c>
       <c r="B59" t="str">
-        <v>docs/ANALISIS_NORMALIZACION_DATOS_LEGACY_FORNITALIA.md alineado a Fornitalia_Movimientos.xlsx, §0 validaciones IDs/CatDesc, pipeline normalizar-extracto. Regenerar HTML+PDF: npm run informe-normalizacion (informe-normalizacion-solo-html solo si hace falta iterar sin Playwright).</v>
+        <v>npm run normalizar-extracto: lee Fornitalia_Movimientos.xlsx (o Extracto legado), hoja Normalizado con fecha_iso, tipo, medio, categoría, cuenta, moneda inferida, monto_original, tipo_cambio, monto_ars, id_cierre_caja, id_comprobante_pago, id_impuesto, cat_desc cuando vienen del export.</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>Upload de extracto normalizado</v>
+        <v>Informe inconsistencias datos legacy (cliente)</v>
       </c>
       <c r="B60" t="str">
-        <v>Botón en la app para reemplazar transacciones desde la hoja Normalizado (p. ej. Base_Fornitalia_To_App): incluye nueva_categoria, nueva_cuenta_contable, costo_directo/indirecto y columnas EF_Item / EF_SubItem → ef_item / ef_subitem en Supabase. Validación previa, carga en lotes y log de excluidos.</v>
+        <v>docs/ANALISIS_NORMALIZACION_DATOS_LEGACY_FORNITALIA.md alineado a Fornitalia_Movimientos.xlsx, §0 validaciones IDs/CatDesc, pipeline normalizar-extracto. Regenerar HTML+PDF: npm run informe-normalizacion (informe-normalizacion-solo-html solo si hace falta iterar sin Playwright).</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>Log de excluidos en upload</v>
+        <v>Upload de extracto normalizado</v>
       </c>
       <c r="B61" t="str">
-        <v>Nueva solapa Excluidos upload con registros no insertados por error o por regla de negocio (Apertura/Cierre de Caja), persistidos en Supabase para auditoría.</v>
+        <v>Botón en la app para reemplazar transacciones desde la hoja Normalizado (p. ej. Base_Fornitalia_To_App): incluye nueva_categoria, nueva_cuenta_contable, costo_directo/indirecto y columnas EF_Item / EF_SubItem → ef_item / ef_subitem en Supabase. Validación previa, carga en lotes y log de excluidos.</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
+        <v>Log de excluidos en upload</v>
+      </c>
+      <c r="B62" t="str">
+        <v>Nueva solapa Excluidos upload con registros no insertados por error o por regla de negocio (Apertura/Cierre de Caja), persistidos en Supabase para auditoría.</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
         <v>Análisis financiero extracto (PDF)</v>
       </c>
-      <c r="B62" t="str">
+      <c r="B63" t="str">
         <v>npm run analisis-financiero-pdf: métricas desde Fornitalia_Movimientos.xlsx (fallback Extracto legado); ARS vía MontoCambio/Monto en $, TC por fila o MEP; exclusiones y USD sin conversión. Sección ventas: ranking por vendedor desde Resumen_Operaciones (Tabla, Vendedor_RO) por N° operación; ranking proxy por producto (detalle hasta mes cierre feb 2026). Ver docs/ANALISIS_FINANCIERO_EXTRACTO_README.md.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B62"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B63"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3840,7 +3950,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C48"/>
+  <dimension ref="A1:C49"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -4375,9 +4485,20 @@
         <v>Ratios costo Flujo alineados a EF: secciones §1–§3, % sin redondear montos; Costo total = egresos operativos ÷ Flujo Op. APP_VERSION 1.88.</v>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>1.96</v>
+      </c>
+      <c r="B49" t="str">
+        <v>01/06/2026</v>
+      </c>
+      <c r="C49" t="str">
+        <v>Despliegue v1.96: Estado Financiero (gráficos línea/barras waterfall, detalle transacciones al clic en importe, Anticipos de impuestos); ratios Flujo alineados a EF y Comisiones/Ventas por ef_subitem; persistencia meses_excluidos en Supabase (columna migrada) y alerta si falla guardar Config. APP_VERSION 1.96. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C48"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C49"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v2.07: matriz costo ampliada, filas verde únicas y Todas transacciones extracto vs BD.
Despliegue con export matriz xlsx-js-style, columnas vieja/nueva en listado y bitácora actualizada.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E172"/>
+  <dimension ref="A1:E178"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -3335,9 +3335,111 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="173">
+      <c r="A173" t="str">
+        <v>17/06/2026</v>
+      </c>
+      <c r="B173" t="str">
+        <v>12:58</v>
+      </c>
+      <c r="C173" t="str">
+        <v>Matriz costo: cat/cuenta vieja, nueva y EF</v>
+      </c>
+      <c r="D173" t="str">
+        <v>Solapa Matriz_Cat_Cuenta_Costo: columnas categoria y cuenta extracto (vieja), nueva, EF Item, EF SubItem, costos y conteos por combinación distinta. APP_VERSION 2.03.</v>
+      </c>
+      <c r="E173" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="str">
+        <v>17/06/2026</v>
+      </c>
+      <c r="B174" t="str">
+        <v>13:06</v>
+      </c>
+      <c r="C174" t="str">
+        <v>Fix EF vacíos en Matriz_Cat_Cuenta_Costo</v>
+      </c>
+      <c r="D174" t="str">
+        <v>Lectura ef_item/ef_subitem con alias EF_Item/EF_SubItem (Excel y upload). Script generar-matriz prioriza Base_Fornitalia_To_App.xlsx. APP_VERSION 2.04.</v>
+      </c>
+      <c r="E174" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="str">
+        <v>17/06/2026</v>
+      </c>
+      <c r="B175" t="str">
+        <v>13:30</v>
+      </c>
+      <c r="C175" t="str">
+        <v>Matriz_Cat_Cuenta_Costo sin exclusiones</v>
+      </c>
+      <c r="D175" t="str">
+        <v>Solapa matriz costo usa todas las filas de origen (sin filtro por categoria); suma # Registros = total cargado. Proveedores mantienen exclusiones. APP_VERSION 2.05.</v>
+      </c>
+      <c r="E175" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="str">
+        <v>17/06/2026</v>
+      </c>
+      <c r="B176" t="str">
+        <v>15:09</v>
+      </c>
+      <c r="C176" t="str">
+        <v>Todas transacciones: extracto vs nueva BD</v>
+      </c>
+      <c r="D176" t="str">
+        <v>Columnas detalle: categoria/cuenta_contable (extracto) y nueva_* (BD) por separado; filtros solo por nueva categoría/cuenta. APP_VERSION 2.06.</v>
+      </c>
+      <c r="E176" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="str">
+        <v>18/06/2026</v>
+      </c>
+      <c r="B177" t="str">
+        <v>08:48</v>
+      </c>
+      <c r="C177" t="str">
+        <v>Matriz costo: filas verde relación única</v>
+      </c>
+      <c r="D177" t="str">
+        <v>Matriz_Cat_Cuenta_Costo: sombreado verde claro cuando cat/cuenta vieja tiene una sola fila (nueva, EF, costos). Export dashboard y script Node con xlsx-js-style. APP_VERSION 2.07.</v>
+      </c>
+      <c r="E177" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="str">
+        <v>25/06/2026</v>
+      </c>
+      <c r="B178" t="str">
+        <v>09:51</v>
+      </c>
+      <c r="C178" t="str">
+        <v>Despliegue v2.07 producción</v>
+      </c>
+      <c r="D178" t="str">
+        <v>Push main y vercel --prod: matriz costo ampliada (vieja/nueva/EF, sin exclusiones, filas verde relación única); Todas transacciones extracto vs BD; xlsx-js-style en export matriz. APP_VERSION 2.07.</v>
+      </c>
+      <c r="E178" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E172"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E178"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3683,7 +3785,7 @@
         <v>Reportes (menú lateral)</v>
       </c>
       <c r="B42" t="str">
-        <v>Vista Reportes: exportar Matriz de relaciones desde Supabase. Matriz costo y proveedores con exclusiones de categoría; solapa Cat_x_Cuenta_Registros solo status Confirmado (todas las categorías). Resumen antes de exportar.</v>
+        <v>Vista Reportes: exportar Matriz de relaciones desde Supabase. Matriz_Cat_Cuenta_Costo sin exclusiones (suma # Registros = transacciones en sesión); filas verde claro si cat/cuenta vieja tiene relación única a nueva. Cat×cuenta solo Confirmado; proveedores con exclusiones de categoría. Resumen antes de exportar.</v>
       </c>
     </row>
     <row r="43">
@@ -3723,7 +3825,7 @@
         <v>Todas las transacciones</v>
       </c>
       <c r="B47" t="str">
-        <v>Solapa que lista todas las transacciones con todas las columnas. Filtros por mes, categoría (matriz), cuenta (matriz), cliente, tipo (Ingreso/Egreso) e id operación (texto). Columnas principales cat/cuenta por matriz; columnas nueva_* como en BD. Botón Editar por registro abre modal de edición completa.</v>
+        <v>Solapa que lista todas las transacciones con todas las columnas. Filtros por mes, categoría nueva (BD), cuenta nueva (BD), cliente, tipo (Ingreso/Egreso) e id operación (texto). Tabla: categoría/cuenta del extracto (vieja) y nueva en BD en columnas separadas. Botón Editar por registro abre modal de edición completa.</v>
       </c>
     </row>
     <row r="48">
@@ -3950,7 +4052,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C49"/>
+  <dimension ref="A1:C51"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -4496,9 +4598,31 @@
         <v>Despliegue v1.96: Estado Financiero (gráficos línea/barras waterfall, detalle transacciones al clic en importe, Anticipos de impuestos); ratios Flujo alineados a EF y Comisiones/Ventas por ef_subitem; persistencia meses_excluidos en Supabase (columna migrada) y alerta si falla guardar Config. APP_VERSION 1.96. Producción Vercel.</v>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>2.02</v>
+      </c>
+      <c r="B50" t="str">
+        <v>17/06/2026</v>
+      </c>
+      <c r="C50" t="str">
+        <v>Despliegue v2.02: menú Reportes con export Matriz Relaciones desde Supabase (módulo fornitalia-matriz-relaciones-transacciones.js); solapa Cat_x_Cuenta_Registros solo Confirmado; matriz/proveedores con exclusiones de categoría; filtro Cliente en Todas las transacciones. Producción Vercel.</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>2.07</v>
+      </c>
+      <c r="B51" t="str">
+        <v>25/06/2026</v>
+      </c>
+      <c r="C51" t="str">
+        <v>Despliegue v2.07: Matriz_Cat_Cuenta_Costo ampliada (cat/cuenta vieja y nueva, EF, sin exclusiones); filas verde claro si relación extracto→nueva es única; Todas transacciones con columnas extracto vs BD y filtros por nueva; export matriz con xlsx-js-style. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C49"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C51"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v2.08: permisos granulares por solapa y fix toggles Seguridad.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E178"/>
+  <dimension ref="A1:E180"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -3422,24 +3422,58 @@
     </row>
     <row r="178">
       <c r="A178" t="str">
-        <v>25/06/2026</v>
+        <v>23/07/2026</v>
       </c>
       <c r="B178" t="str">
-        <v>09:51</v>
+        <v>09:52</v>
       </c>
       <c r="C178" t="str">
-        <v>Despliegue v2.07 producción</v>
+        <v>Permisos granulares por solapa (Visor editable)</v>
       </c>
       <c r="D178" t="str">
-        <v>Push main y vercel --prod: matriz costo ampliada (vieja/nueva/EF, sin exclusiones, filas verde relación única); Todas transacciones extracto vs BD; xlsx-js-style en export matriz. APP_VERSION 2.07.</v>
+        <v>Causa: dashboard_operador era todo-o-nada y no permitía configurar solapas sueltas para Visor. Migración sql/migracion_permisos_solapas_granulares.sql + MCP: ver_solapa_*, ver_novedades/configuracion/reportes, carga_normalizada, editar_registros. Seguridad: toggles por solapa/menú/acción con verificación .select(); RLS INSERT/DELETE reafirmado. Frontend applySecurityUI por permiso. Compatibilidad con dashboard_operador legacy.</v>
       </c>
       <c r="E178" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="str">
+        <v>23/07/2026</v>
+      </c>
+      <c r="B179" t="str">
+        <v>10:06</v>
+      </c>
+      <c r="C179" t="str">
+        <v>Fix toggle permisos Seguridad (clic on/off)</v>
+      </c>
+      <c r="D179" t="str">
+        <v>CSS del switch en Seguridad alineado a Pandi: input cubre el área (inset 0, z-index 1) y slider con pointer-events none. Antes width/height 0 impedía el clic en el interruptor (solo GET a app_role_permission, sin POST/DELETE).</v>
+      </c>
+      <c r="E179" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="str">
+        <v>23/07/2026</v>
+      </c>
+      <c r="B180" t="str">
+        <v>10:10</v>
+      </c>
+      <c r="C180" t="str">
+        <v>Despliegue v2.08 producción</v>
+      </c>
+      <c r="D180" t="str">
+        <v>Push main y vercel --prod: permisos granulares por solapa/menú/acción; toggles Seguridad clicables (estilo Pandi); migración SQL en Supabase. APP_VERSION 2.08.</v>
+      </c>
+      <c r="E180" t="str">
         <v>Despliegue</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E178"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E180"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3649,7 +3683,7 @@
         <v>Seguridad y roles</v>
       </c>
       <c r="B25" t="str">
-        <v>Login con email/contraseña, registro o invitado anónimo (visor). Permisos desde Supabase: exportar_base_historica, dashboard_operador, assign_roles. Visor: solo solapa Flujo por mes y botón Exportar Base Histórica (sin edición ni solapa Errores en modal mes). Encargado/Admin: resto del dashboard. Admin: vista Seguridad (usuarios/roles y permisos por rol). La tabla de usuarios solo muestra cuentas con email (no sesiones anónimas). Sin SQL de seguridad desplegado, la app mantiene modo compatibilidad con acceso completo.</v>
+        <v>Login con email/contraseña, registro o invitado anónimo (visor). Permisos granulares desde Supabase: ver_solapa_* (cada solapa del dashboard), ver_novedades/configuracion/reportes, exportar_base_historica, carga_normalizada, editar_registros, assign_roles. Visor por defecto: Flujo por mes + exportar/reportes; un admin puede activar solapas sueltas en Seguridad. Encargado/Admin: pack operador completo. dashboard_operador se conserva como compatibilidad legacy. Sin SQL de seguridad, modo acceso completo.</v>
       </c>
     </row>
     <row r="26">
@@ -4052,7 +4086,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C51"/>
+  <dimension ref="A1:C52"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -4620,9 +4654,20 @@
         <v>Despliegue v2.07: Matriz_Cat_Cuenta_Costo ampliada (cat/cuenta vieja y nueva, EF, sin exclusiones); filas verde claro si relación extracto→nueva es única; Todas transacciones con columnas extracto vs BD y filtros por nueva; export matriz con xlsx-js-style. Producción Vercel.</v>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>2.08</v>
+      </c>
+      <c r="B52" t="str">
+        <v>23/07/2026</v>
+      </c>
+      <c r="C52" t="str">
+        <v>Despliegue v2.08: permisos granulares por solapa/menú/acción (Visor configurable); fix toggle Seguridad on/off como Pandi; sql/migracion_permisos_solapas_granulares.sql. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C51"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C52"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4782,7 +4827,7 @@
         <v>Seguridad y roles (dashboard)</v>
       </c>
       <c r="B11" t="str">
-        <v>Autenticación email/anónimo, roles Admin/Encargado/Visor, permisos en Supabase (RPC y RLS), pantalla Seguridad para asignar roles y toggles por rol; visor restringido a Flujo por mes y exportar base histórica.</v>
+        <v>Autenticación email/anónimo, roles Admin/Encargado/Visor, permisos granulares por solapa/menú/acción en Supabase (RPC y RLS), pantalla Seguridad para asignar roles y toggles por ítem (incluido Visor).</v>
       </c>
       <c r="C11">
         <v>18</v>

</xml_diff>

<commit_message>
v2.09: Gestión de Proyectos a producción (horas, SPI, observaciones y Gantt).
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E180"/>
+  <dimension ref="A1:E201"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -3471,16 +3471,373 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="181">
+      <c r="A181" t="str">
+        <v>24/08/2026</v>
+      </c>
+      <c r="B181" t="str">
+        <v>10:45</v>
+      </c>
+      <c r="C181" t="str">
+        <v>Gestión de Proyectos (ABM plan de trabajo)</v>
+      </c>
+      <c r="D181" t="str">
+        <v>Menú Gestión de Proyectos configurable en perfiles (ver/crear/editar/eliminar). Componente scripts/lib (no ampliar main): ABM proyecto → entregables → tareas y dependencias; To-Do jerárquico expandable; Gantt one-page con % y SPI; export Excel (números) y PDF. SQL helpers_fecha_argentina + supabase_gestion_proyectos.</v>
+      </c>
+      <c r="E181" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="str">
+        <v>24/08/2026</v>
+      </c>
+      <c r="B182" t="str">
+        <v>10:50</v>
+      </c>
+      <c r="C182" t="str">
+        <v>Gestión de Proyectos: icono en cabecera</v>
+      </c>
+      <c r="D182" t="str">
+        <v>El h1 del componente usa el mismo SVG de carpeta que el ítem del menú lateral (stroke currentColor, 28px), alineado a Reportes/Novedades.</v>
+      </c>
+      <c r="E182" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="str">
+        <v>24/08/2026</v>
+      </c>
+      <c r="B183" t="str">
+        <v>10:55</v>
+      </c>
+      <c r="C183" t="str">
+        <v>Iconos de menú en cabeceras de vistas</v>
+      </c>
+      <c r="D183" t="str">
+        <v>Cada opción de menú replica su SVG en el título: Home (Flujo de caja), Gestión de Proyectos, Reportes, Novedades, Configuración (modal) y Seguridad. Clase común vista-titulo / vista-titulo-icon.</v>
+      </c>
+      <c r="E183" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="str">
+        <v>24/08/2026</v>
+      </c>
+      <c r="B184" t="str">
+        <v>10:56</v>
+      </c>
+      <c r="C184" t="str">
+        <v>Plan: nombre de entregable sin corte</v>
+      </c>
+      <c r="D184" t="str">
+        <v>Columna Plan sin max-width; el nombre va en bloque debajo de ENTREGABLE/TAREA y se muestra completo (word-break), el resto de columnas queda en una línea.</v>
+      </c>
+      <c r="E184" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="str">
+        <v>24/08/2026</v>
+      </c>
+      <c r="B185" t="str">
+        <v>11:20</v>
+      </c>
+      <c r="C185" t="str">
+        <v>Responsable: nombre de usuario (iniciales) como Everfit</v>
+      </c>
+      <c r="D185" t="str">
+        <v>user_profiles.nombre_usuario; RPCs get_my_profile, set_my_nombre_usuario, set_user_nombre_usuario; modal Mi perfil; Seguridad con campo Nombre. En Gestión de Proyectos el responsable muestra iniciales/nombre corto (email al hover), no el mail. sql/supabase_user_profiles_nombre_usuario.sql.</v>
+      </c>
+      <c r="E185" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="str">
+        <v>24/08/2026</v>
+      </c>
+      <c r="B186" t="str">
+        <v>11:35</v>
+      </c>
+      <c r="C186" t="str">
+        <v>PDF one-page sin pop-up bloqueado</v>
+      </c>
+      <c r="D186" t="str">
+        <v>Export PDF del plan imprime el one-page en el mismo documento (window.print) en lugar de window.open+fetch. Chrome ya no bloquea la vista previa; se puede Guardar como PDF.</v>
+      </c>
+      <c r="E186" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="str">
+        <v>24/08/2026</v>
+      </c>
+      <c r="B187" t="str">
+        <v>11:40</v>
+      </c>
+      <c r="C187" t="str">
+        <v>Ordenar entregables independiente de la carga</v>
+      </c>
+      <c r="D187" t="str">
+        <v>Combo Ordenar entregables (fecha inicio/fin, nombre, estado o manual). Flechas ↑↓ persisten el orden en gp_entregable.orden. Aplica a To-Do, Gantt y Excel.</v>
+      </c>
+      <c r="E187" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="str">
+        <v>24/08/2026</v>
+      </c>
+      <c r="B188" t="str">
+        <v>11:46</v>
+      </c>
+      <c r="C188" t="str">
+        <v>Fix cerrar modal Gestión de Proyectos</v>
+      </c>
+      <c r="D188" t="str">
+        <v>La X y Cancelar no cerraban (el modal está en document.body y el click se escuchaba solo en la vista). Cierre en el backdrop, Escape y botones data-gp=cerrar-modal.</v>
+      </c>
+      <c r="E188" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="str">
+        <v>24/08/2026</v>
+      </c>
+      <c r="B189" t="str">
+        <v>11:52</v>
+      </c>
+      <c r="C189" t="str">
+        <v>Horas alocadas en tareas y total en entregable</v>
+      </c>
+      <c r="D189" t="str">
+        <v>Campo horas_alocadas en gp_tarea; formulario de tarea; columna Horas en el plan (suma de tareas no canceladas en el entregable); KPI y Excel numérico. sql/supabase_gp_tarea_horas_alocadas.sql.</v>
+      </c>
+      <c r="E189" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="str">
+        <v>24/08/2026</v>
+      </c>
+      <c r="B190" t="str">
+        <v>12:25</v>
+      </c>
+      <c r="C190" t="str">
+        <v>Horas por fecha y alerta de deadline</v>
+      </c>
+      <c r="D190" t="str">
+        <v>Tabla gp_tarea_hora (tarea + fecha de negocio Argentina + horas) en lugar de un total suelto. Solapa Horas de conciliación diaria; Excel hoja Horas numérica. Alerta si la tarea o las horas superan el deadline del entregable (plan, KPI, confirm al guardar). sql/supabase_gp_tarea_hora.sql.</v>
+      </c>
+      <c r="E190" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="str">
+        <v>24/08/2026</v>
+      </c>
+      <c r="B191" t="str">
+        <v>12:30</v>
+      </c>
+      <c r="C191" t="str">
+        <v>Horas consumidas (no alocación planificada)</v>
+      </c>
+      <c r="D191" t="str">
+        <v>Leyendas de horas alocadas → horas consumidas (reales por fecha). One-page Gantt/PDF aclara que no es alocación planificada; KPI, plan, solapa, Excel y formularios alineados.</v>
+      </c>
+      <c r="E191" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="str">
+        <v>24/08/2026</v>
+      </c>
+      <c r="B192" t="str">
+        <v>12:32</v>
+      </c>
+      <c r="C192" t="str">
+        <v>Plan: entregable en negrita</v>
+      </c>
+      <c r="D192" t="str">
+        <v>Nombre del entregable en negrita (más entidad); tareas y dependencias en peso normal. Mismo criterio en Gantt/one-page y solapa Horas cons.</v>
+      </c>
+      <c r="E192" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="str">
+        <v>24/08/2026</v>
+      </c>
+      <c r="B193" t="str">
+        <v>12:45</v>
+      </c>
+      <c r="C193" t="str">
+        <v>Horas consumidas propias del entregable</v>
+      </c>
+      <c r="D193" t="str">
+        <v>Tabla gp_entregable_hora: mismas horas por fecha que en la tarea, también sin tareas. Conciliación = propias del entregable + horas de sus tareas. Formulario, KPI, Excel (columna Origen) y one-page. sql/supabase_gp_entregable_hora.sql.</v>
+      </c>
+      <c r="E193" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="str">
+        <v>24/08/2026</v>
+      </c>
+      <c r="B194" t="str">
+        <v>12:51</v>
+      </c>
+      <c r="C194" t="str">
+        <v>Excel Resumen: alcance del proyecto</v>
+      </c>
+      <c r="D194" t="str">
+        <v>La hoja Resumen del export Excel del plan incluye la fila Alcance del proyecto.</v>
+      </c>
+      <c r="E194" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="str">
+        <v>24/08/2026</v>
+      </c>
+      <c r="B195" t="str">
+        <v>12:55</v>
+      </c>
+      <c r="C195" t="str">
+        <v>Excel Gantt gráfico (sin unos) y estilos</v>
+      </c>
+      <c r="D195" t="str">
+        <v>Hoja Gantt del Excel tipo one-page/PDF: barras de color por duración (entregable/tarea/atrasado), leyenda, semana de hoy, % en la barra. Sin celdas con 1. Cabeceras y filas de entregable estiladas también en Resumen, Plan y Horas cons.</v>
+      </c>
+      <c r="E195" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="str">
+        <v>24/08/2026</v>
+      </c>
+      <c r="B196" t="str">
+        <v>14:20</v>
+      </c>
+      <c r="C196" t="str">
+        <v>Gantt: fecha fin planificada en la barra</v>
+      </c>
+      <c r="D196" t="str">
+        <v>En cada barra del Gantt (pantalla, PDF y Excel) se muestra adentro la fecha fin planificada. Excel: % al inicio de la barra y fecha al final.</v>
+      </c>
+      <c r="E196" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="str">
+        <v>24/08/2026</v>
+      </c>
+      <c r="B197" t="str">
+        <v>14:35</v>
+      </c>
+      <c r="C197" t="str">
+        <v>SPI ponderado por horas consumidas</v>
+      </c>
+      <c r="D197" t="str">
+        <v>El avance y el SPI del proyecto ponderan horas de tareas + horas propias del entregable (si no hay tareas). Un entregable hecho como Elaborar Plan (4 h) cuenta en el SPI; los que aún no empiezan no diluyen. Esperado a hoy usa el mismo peso.</v>
+      </c>
+      <c r="E197" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="str">
+        <v>25/08/2026</v>
+      </c>
+      <c r="B198" t="str">
+        <v>10:05</v>
+      </c>
+      <c r="C198" t="str">
+        <v>Fix RLS horas + Observaciones en tarea y entregable</v>
+      </c>
+      <c r="D198" t="str">
+        <v>El guardar horas de tarea fallaba (RLS en gp_tarea_hora) por el FK created_by→auth.users al insertar. Horas se guardan con RPC SECURITY DEFINER. Campo Observaciones en entregable y tarea (formulario, plan, Excel). sql/supabase_gp_observaciones_y_horas_rls.sql.</v>
+      </c>
+      <c r="E198" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="str">
+        <v>25/08/2026</v>
+      </c>
+      <c r="B199" t="str">
+        <v>11:00</v>
+      </c>
+      <c r="C199" t="str">
+        <v>Observaciones en carga de horas y scroll de modales GP</v>
+      </c>
+      <c r="D199" t="str">
+        <v>Observaciones pasa a cada fila de horas (fecha + horas + nota), en tarea y entregable. Solapa Horas cons. y Excel. Modales GP: cuerpo con scroll y pie fijo para ver Cancelar/Guardar. sql/supabase_gp_hora_observaciones.sql.</v>
+      </c>
+      <c r="E199" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="str">
+        <v>25/08/2026</v>
+      </c>
+      <c r="B200" t="str">
+        <v>13:35</v>
+      </c>
+      <c r="C200" t="str">
+        <v>Gantt: año en dos dígitos en la barra</v>
+      </c>
+      <c r="D200" t="str">
+        <v>La fecha fin planificada dentro de las barras del Gantt (pantalla, PDF y Excel) se muestra como dd/mm/aa para que entre en periodos cortos. El resto de la app sigue con año de cuatro dígitos.</v>
+      </c>
+      <c r="E200" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="str">
+        <v>25/08/2026</v>
+      </c>
+      <c r="B201" t="str">
+        <v>15:21</v>
+      </c>
+      <c r="C201" t="str">
+        <v>Despliegue v2.09 producción</v>
+      </c>
+      <c r="D201" t="str">
+        <v>Push a main y Vercel --prod: Gestión de Proyectos (horas, SPI, observaciones en carga, modales, Gantt). APP_VERSION 2.09.</v>
+      </c>
+      <c r="E201" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E180"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E201"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B63"/>
+  <dimension ref="A1:B64"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -3675,7 +4032,7 @@
         <v>Menú lateral</v>
       </c>
       <c r="B24" t="str">
-        <v>Sidebar izquierdo colapsable/expandible; botón toggle (▶/◀); Home, Novedades, Configuración, Seguridad (solo admin con permiso), Cerrar sesión; estado expandido en localStorage.</v>
+        <v>Sidebar izquierdo colapsable/expandible; botón toggle (▶/◀); Home, Gestión de Proyectos, Reportes, Novedades, Configuración, Seguridad (solo admin con permiso), Mi perfil, Cerrar sesión; estado expandido en localStorage.</v>
       </c>
     </row>
     <row r="25">
@@ -3683,7 +4040,7 @@
         <v>Seguridad y roles</v>
       </c>
       <c r="B25" t="str">
-        <v>Login con email/contraseña, registro o invitado anónimo (visor). Permisos granulares desde Supabase: ver_solapa_* (cada solapa del dashboard), ver_novedades/configuracion/reportes, exportar_base_historica, carga_normalizada, editar_registros, assign_roles. Visor por defecto: Flujo por mes + exportar/reportes; un admin puede activar solapas sueltas en Seguridad. Encargado/Admin: pack operador completo. dashboard_operador se conserva como compatibilidad legacy. Sin SQL de seguridad, modo acceso completo.</v>
+        <v>Login con email/contraseña, registro o invitado anónimo (visor). Permisos granulares desde Supabase: ver_solapa_* (cada solapa del dashboard), ver_novedades/configuracion/reportes/gestion_proyectos, crear/editar/eliminar_proyecto, exportar_base_historica, carga_normalizada, editar_registros, assign_roles. Visor por defecto: Flujo por mes + exportar/reportes; un admin puede activar solapas y menús sueltos en Seguridad. Encargado/Admin: pack operador + Gestión de Proyectos. dashboard_operador se conserva como compatibilidad legacy. Sin SQL de seguridad, modo acceso completo. Tabla Usuarios: email, nombre para mostrar (iniciales) y rol; Mi perfil para el propio usuario.</v>
       </c>
     </row>
     <row r="26">
@@ -3899,7 +4256,7 @@
         <v>Botones e iconos unificados</v>
       </c>
       <c r="B52" t="str">
-        <v>Todos los botones con mismo estilo: icono SVG + texto. Sidebar (chevron, home, engranaje), tabs con iconos, exportar con icono descarga, modales con iconos (Guardar, Cerrar, Excluir, Eliminar). Iconos solos (cerrar, editar, alerta) en SVG.</v>
+        <v>Todos los botones con mismo estilo: icono SVG + texto. Sidebar (chevron, home, engranaje, usuario), tabs con iconos, exportar con icono descarga, modales con iconos (Guardar, Cerrar, Excluir, Eliminar). Iconos solos (cerrar, editar, alerta) en SVG. Cada vista de menú muestra en la cabecera el mismo icono que el ítem del sidebar (Home, Gestión de Proyectos, Reportes, Novedades, Configuración, Seguridad, Mi perfil).</v>
       </c>
     </row>
     <row r="53">
@@ -3952,47 +4309,55 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>Normalización de extracto bancario</v>
+        <v>Gestión de Proyectos</v>
       </c>
       <c r="B59" t="str">
-        <v>npm run normalizar-extracto: lee Fornitalia_Movimientos.xlsx (o Extracto legado), hoja Normalizado con fecha_iso, tipo, medio, categoría, cuenta, moneda inferida, monto_original, tipo_cambio, monto_ars, id_cierre_caja, id_comprobante_pago, id_impuesto, cat_desc cuando vienen del export.</v>
+        <v>Menú lateral (permiso ver_gestion_proyectos). ABM de planes: Proyecto → Entregables (nombre, alcance, fechas, responsable usuario o perfil) → Tareas (misma metadata) y Dependencias (viñeta + responsable). Las horas son las realmente consumidas por fecha en el entregable (gp_entregable_hora) y/o en las tareas (gp_tarea_hora), cada fila con observaciones; el total del entregable es propias + tareas (RPC gp_guardar_horas_*). Solapa Horas cons.: conciliación diaria. Alerta si una tarea o sus horas superan el deadline del entregable. El responsable de usuario se muestra como nombre corto / iniciales (no el email; el correo va en el tooltip). Solapa To-Do: tabla jerárquica expandable o solo entregables (entregable en negrita, tareas y dependencias en peso normal), cards de pendientes/en curso/vencidas, cambio de estado. Ordenar entregables por fecha, nombre, estado o manual (flechas ↑↓ persistidas). Solapa Gantt one-page: anillo de avance, SPI ponderado por horas consumidas (tareas + horas propias del entregable si no tiene tareas) vs calendario, barras con % y horas consumidas (reales, no planificadas); export Excel (Plan/Resumen/Horas cons./Gantt gráfico con barras de color como el PDF, sin unos, importes, % y horas numéricos) y PDF (impresión en la misma pestaña, sin pop-up). Permisos crear_proyecto / editar_proyecto / eliminar_proyecto en Seguridad. Componente: scripts/lib/fornitalia-gestion-proyectos.js + .css. SQL: sql/supabase_gestion_proyectos.sql, sql/supabase_user_profiles_nombre_usuario.sql, sql/supabase_gp_tarea_horas_alocadas.sql, sql/supabase_gp_tarea_hora.sql, sql/supabase_gp_entregable_hora.sql, sql/supabase_gp_observaciones_y_horas_rls.sql y sql/supabase_gp_hora_observaciones.sql.</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>Informe inconsistencias datos legacy (cliente)</v>
+        <v>Normalización de extracto bancario</v>
       </c>
       <c r="B60" t="str">
-        <v>docs/ANALISIS_NORMALIZACION_DATOS_LEGACY_FORNITALIA.md alineado a Fornitalia_Movimientos.xlsx, §0 validaciones IDs/CatDesc, pipeline normalizar-extracto. Regenerar HTML+PDF: npm run informe-normalizacion (informe-normalizacion-solo-html solo si hace falta iterar sin Playwright).</v>
+        <v>npm run normalizar-extracto: lee Fornitalia_Movimientos.xlsx (o Extracto legado), hoja Normalizado con fecha_iso, tipo, medio, categoría, cuenta, moneda inferida, monto_original, tipo_cambio, monto_ars, id_cierre_caja, id_comprobante_pago, id_impuesto, cat_desc cuando vienen del export.</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>Upload de extracto normalizado</v>
+        <v>Informe inconsistencias datos legacy (cliente)</v>
       </c>
       <c r="B61" t="str">
-        <v>Botón en la app para reemplazar transacciones desde la hoja Normalizado (p. ej. Base_Fornitalia_To_App): incluye nueva_categoria, nueva_cuenta_contable, costo_directo/indirecto y columnas EF_Item / EF_SubItem → ef_item / ef_subitem en Supabase. Validación previa, carga en lotes y log de excluidos.</v>
+        <v>docs/ANALISIS_NORMALIZACION_DATOS_LEGACY_FORNITALIA.md alineado a Fornitalia_Movimientos.xlsx, §0 validaciones IDs/CatDesc, pipeline normalizar-extracto. Regenerar HTML+PDF: npm run informe-normalizacion (informe-normalizacion-solo-html solo si hace falta iterar sin Playwright).</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>Log de excluidos en upload</v>
+        <v>Upload de extracto normalizado</v>
       </c>
       <c r="B62" t="str">
-        <v>Nueva solapa Excluidos upload con registros no insertados por error o por regla de negocio (Apertura/Cierre de Caja), persistidos en Supabase para auditoría.</v>
+        <v>Botón en la app para reemplazar transacciones desde la hoja Normalizado (p. ej. Base_Fornitalia_To_App): incluye nueva_categoria, nueva_cuenta_contable, costo_directo/indirecto y columnas EF_Item / EF_SubItem → ef_item / ef_subitem en Supabase. Validación previa, carga en lotes y log de excluidos.</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
+        <v>Log de excluidos en upload</v>
+      </c>
+      <c r="B63" t="str">
+        <v>Nueva solapa Excluidos upload con registros no insertados por error o por regla de negocio (Apertura/Cierre de Caja), persistidos en Supabase para auditoría.</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
         <v>Análisis financiero extracto (PDF)</v>
       </c>
-      <c r="B63" t="str">
+      <c r="B64" t="str">
         <v>npm run analisis-financiero-pdf: métricas desde Fornitalia_Movimientos.xlsx (fallback Extracto legado); ARS vía MontoCambio/Monto en $, TC por fila o MEP; exclusiones y USD sin conversión. Sección ventas: ranking por vendedor desde Resumen_Operaciones (Tabla, Vendedor_RO) por N° operación; ranking proxy por producto (detalle hasta mes cierre feb 2026). Ver docs/ANALISIS_FINANCIERO_EXTRACTO_README.md.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B63"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B64"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4086,7 +4451,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C52"/>
+  <dimension ref="A1:C53"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -4665,16 +5030,27 @@
         <v>Despliegue v2.08: permisos granulares por solapa/menú/acción (Visor configurable); fix toggle Seguridad on/off como Pandi; sql/migracion_permisos_solapas_granulares.sql. Producción Vercel.</v>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>2.09</v>
+      </c>
+      <c r="B53" t="str">
+        <v>25/08/2026</v>
+      </c>
+      <c r="C53" t="str">
+        <v>Despliegue v2.09: Gestión de Proyectos (horas por fecha, SPI ponderado por horas, observaciones en cada carga, RPC RLS, scroll de modales, fecha dd/mm/aa en barras Gantt). Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C52"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C53"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D13"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="90.83203125" customWidth="1"/>
@@ -4850,9 +5226,23 @@
         <v>500</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Gestión de Proyectos</v>
+      </c>
+      <c r="B13" t="str">
+        <v>ABM de planes de trabajo (proyecto, entregables, tareas y dependencias), To-Do jerárquico, Gantt one-page con avance y SPI, export Excel/PDF, permisos por perfil.</v>
+      </c>
+      <c r="C13">
+        <v>40</v>
+      </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D13"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4878,7 +5268,7 @@
         <v>Frontend</v>
       </c>
       <c r="B2" t="str">
-        <v>Una sola página dashboard-flujo-caja.html (HTML, CSS, JavaScript en el mismo archivo). Sin framework; llamadas a Supabase desde el cliente.</v>
+        <v>Página dashboard-flujo-caja.html (HTML/CSS/JS). Gestión de Proyectos en componente aparte: scripts/lib/fornitalia-gestion-proyectos.js + .css. Sin framework; llamadas a Supabase desde el cliente.</v>
       </c>
     </row>
     <row r="3">
@@ -4886,7 +5276,7 @@
         <v>Datos</v>
       </c>
       <c r="B3" t="str">
-        <v>Supabase (PostgreSQL). Tablas: transacciones, tipo_de_cambio, config_dashboard. Scripts SQL en carpeta sql/ se ejecutan en Supabase SQL Editor.</v>
+        <v>Supabase (PostgreSQL). Tablas: transacciones, tipo_de_cambio, config_dashboard, gp_proyecto, gp_entregable, gp_entregable_hora, gp_tarea, gp_tarea_hora, gp_dependencia. Scripts SQL en carpeta sql/ se ejecutan en Supabase SQL Editor.</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
v2.10: export Excel de Flujo por mes y fechas Argentina en el plan GP.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E201"/>
+  <dimension ref="A1:E207"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -3828,9 +3828,111 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="202">
+      <c r="A202" t="str">
+        <v>25/08/2026</v>
+      </c>
+      <c r="B202" t="str">
+        <v>15:40</v>
+      </c>
+      <c r="C202" t="str">
+        <v>Excel/PDF plan: fechas calendario Argentina</v>
+      </c>
+      <c r="D202" t="str">
+        <v>El export Excel escribía Date UTC y en Argentina el día se corría. Ahora serial del YYYY-MM-DD + formato dd/mm/yyyy (Plan, Horas, Gantt). PDF/HTML formatea dd/mm/aaaa desde las partes del día, no desde Date UTC. Regla fechas-argentina-negocio y docs/FECHAS_ARGENTINA.md.</v>
+      </c>
+      <c r="E202" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="str">
+        <v>26/08/2026</v>
+      </c>
+      <c r="B203" t="str">
+        <v>09:20</v>
+      </c>
+      <c r="C203" t="str">
+        <v>Word: aportes de capital e inversiones en el EF</v>
+      </c>
+      <c r="D203" t="str">
+        <v>docs/EF_Aportes_Capital_e_Inversiones.docx: dónde van aportes de capital y colocaciones (fondos/activos) en el Estado Financiero actual vs estados argentinos estándar (RT 8/9); propuesta de partir 6.1 y agregar 6.4/6.5.</v>
+      </c>
+      <c r="E203" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="str">
+        <v>26/08/2026</v>
+      </c>
+      <c r="B204" t="str">
+        <v>09:35</v>
+      </c>
+      <c r="C204" t="str">
+        <v>Word EF: rendimiento y caución dentro del EF</v>
+      </c>
+      <c r="D204" t="str">
+        <v>Misma nota: se saca la columna Caución del flujo; capital y yield ( +/− ) visibles en el EF. Sección 6 propuesta: 6.1a/6.1b, 6.4 colocación, 6.5 rescate, 6.6 rendimiento neto (incluye interés de caución); fórmula D.</v>
+      </c>
+      <c r="E204" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="str">
+        <v>26/08/2026</v>
+      </c>
+      <c r="B205" t="str">
+        <v>10:15</v>
+      </c>
+      <c r="C205" t="str">
+        <v>Word EF: FCI práctico y caja inmovilizada</v>
+      </c>
+      <c r="D205" t="str">
+        <v>docs/EF_Aportes_Capital_e_Inversiones.docx: no forzar yield del FCI (suscripciones/rescates); 6.6 solo si el extracto lo trae (caución). Saldo parked = estrategia de tesorería a bajo riesgo alineada al flujo de pagos (flujo vs stock).</v>
+      </c>
+      <c r="E205" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="str">
+        <v>27/08/2026</v>
+      </c>
+      <c r="B206" t="str">
+        <v>09:00</v>
+      </c>
+      <c r="C206" t="str">
+        <v>Export Excel Flujo por mes</v>
+      </c>
+      <c r="D206" t="str">
+        <v>Solapa Flujo por mes: botón Exportar Flujo a Excel (mismo patrón verde + icono que Evolución/EF). Hoja con importes numéricos, % como fracción, Caución en ARS, totales, proyección y alertas. xlsx-js-style.</v>
+      </c>
+      <c r="E206" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="str">
+        <v>27/08/2026</v>
+      </c>
+      <c r="B207" t="str">
+        <v>15:10</v>
+      </c>
+      <c r="C207" t="str">
+        <v>Despliegue v2.10 producción</v>
+      </c>
+      <c r="D207" t="str">
+        <v>Push a main y Vercel --prod: export Excel Flujo por mes; fechas calendario Argentina en Excel/PDF del plan GP. APP_VERSION 2.10.</v>
+      </c>
+      <c r="E207" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E201"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E207"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3856,7 +3958,7 @@
         <v>Flujo de caja por mes</v>
       </c>
       <c r="B2" t="str">
-        <v>Tabla de caja operativa: columnas Ingresos, Egresos y G/P operativo (sin anulados ni apertura/cierre de caja; traspasos no incluidos en el import). Comisiones/Ventas % por subítems EF; Costo dir./ind. ÷ FLUJO OPERATIVO GENERADO (§2/§3); Costo total/Ingreso total = total egresos operativos ÷ FLUJO OPERATIVO GENERADO; columna Caución (solo origen ARS). Proyección de ratios y caución en ARS. Meses excluidos por Configuración → Inclusión por mes no aparecen en filas ni totales. Icono de ayuda con criterios de la tabla.</v>
+        <v>Tabla de caja operativa: columnas Ingresos, Egresos y G/P operativo (sin anulados ni apertura/cierre de caja; traspasos no incluidos en el import). Comisiones/Ventas % por subítems EF; Costo dir./ind. ÷ FLUJO OPERATIVO GENERADO (§2/§3); Costo total/Ingreso total = total egresos operativos ÷ FLUJO OPERATIVO GENERADO; columna Caución (solo origen ARS). Proyección de ratios y caución en ARS. Meses excluidos por Configuración → Inclusión por mes no aparecen en filas ni totales. Icono de ayuda con criterios de la tabla. Exportar Flujo a Excel (mismo método que Evolución/EF: xlsx-js-style, importes numéricos, % como fracción).</v>
       </c>
     </row>
     <row r="3">
@@ -4192,7 +4294,7 @@
         <v>Exportaciones Excel</v>
       </c>
       <c r="B44" t="str">
-        <v>Todas las exportaciones incluyen una fila título con la moneda. Exportar Base Histórica (icono Excel) en la línea del selector de moneda; Exportar Evolución a Excel con el mismo icono.</v>
+        <v>Todas las exportaciones incluyen una fila título con la moneda. Exportar Base Histórica (icono Excel) en la línea del selector de moneda; Exportar Flujo a Excel, Exportar Evolución a Excel y Exportar EF a Excel con el mismo icono y método (SheetJS/xlsx-js-style). Importes como número; % del Flujo y EF como fracción.</v>
       </c>
     </row>
     <row r="45">
@@ -4451,7 +4553,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C54"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -5041,9 +5143,20 @@
         <v>Despliegue v2.09: Gestión de Proyectos (horas por fecha, SPI ponderado por horas, observaciones en cada carga, RPC RLS, scroll de modales, fecha dd/mm/aa en barras Gantt). Producción Vercel.</v>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>2.10</v>
+      </c>
+      <c r="B54" t="str">
+        <v>27/08/2026</v>
+      </c>
+      <c r="C54" t="str">
+        <v>Despliegue v2.10: export Excel de Flujo por mes (importes numéricos, % como fracción, caución en ARS, totales y proyección); fechas calendario Argentina en Excel/PDF del plan de Gestión de Proyectos. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C53"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C54"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5231,7 +5344,7 @@
         <v>Gestión de Proyectos</v>
       </c>
       <c r="B13" t="str">
-        <v>ABM de planes de trabajo (proyecto, entregables, tareas y dependencias), To-Do jerárquico, Gantt one-page con avance y SPI, export Excel/PDF, permisos por perfil.</v>
+        <v>ABM de planes de trabajo (proyecto, entregables, tareas y dependencias), To-Do jerárquico, Gantt one-page con avance y SPI, horas consumidas por fecha con observaciones, export Excel/PDF, permisos por perfil.</v>
       </c>
       <c r="C13">
         <v>40</v>

</xml_diff>

<commit_message>
v2.11: horas consumidas propias del proyecto.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E207"/>
+  <dimension ref="A1:E209"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -3930,9 +3930,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="208">
+      <c r="A208" t="str">
+        <v>31/08/2026</v>
+      </c>
+      <c r="B208" t="str">
+        <v>10:31</v>
+      </c>
+      <c r="C208" t="str">
+        <v>Horas consumidas propias del proyecto</v>
+      </c>
+      <c r="D208" t="str">
+        <v>Tabla gp_proyecto_hora: mismas fecha + horas + observaciones que en entregable/tarea, cargadas en el formulario del proyecto. El total del proyecto = propias + entregables + tareas. SPI, avance, KPI, solapa Horas cons., Excel y alerta de deadline integran esas horas (RPC gp_guardar_horas_proyecto). sql/supabase_gp_proyecto_hora.sql.</v>
+      </c>
+      <c r="E208" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="str">
+        <v>31/08/2026</v>
+      </c>
+      <c r="B209" t="str">
+        <v>10:48</v>
+      </c>
+      <c r="C209" t="str">
+        <v>Despliegue v2.11 producción</v>
+      </c>
+      <c r="D209" t="str">
+        <v>Push a main y Vercel --prod: horas consumidas propias del proyecto (gp_proyecto_hora, SPI/avance/KPI/conciliación/Excel). APP_VERSION 2.11.</v>
+      </c>
+      <c r="E209" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E207"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E209"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4414,7 +4448,7 @@
         <v>Gestión de Proyectos</v>
       </c>
       <c r="B59" t="str">
-        <v>Menú lateral (permiso ver_gestion_proyectos). ABM de planes: Proyecto → Entregables (nombre, alcance, fechas, responsable usuario o perfil) → Tareas (misma metadata) y Dependencias (viñeta + responsable). Las horas son las realmente consumidas por fecha en el entregable (gp_entregable_hora) y/o en las tareas (gp_tarea_hora), cada fila con observaciones; el total del entregable es propias + tareas (RPC gp_guardar_horas_*). Solapa Horas cons.: conciliación diaria. Alerta si una tarea o sus horas superan el deadline del entregable. El responsable de usuario se muestra como nombre corto / iniciales (no el email; el correo va en el tooltip). Solapa To-Do: tabla jerárquica expandable o solo entregables (entregable en negrita, tareas y dependencias en peso normal), cards de pendientes/en curso/vencidas, cambio de estado. Ordenar entregables por fecha, nombre, estado o manual (flechas ↑↓ persistidas). Solapa Gantt one-page: anillo de avance, SPI ponderado por horas consumidas (tareas + horas propias del entregable si no tiene tareas) vs calendario, barras con % y horas consumidas (reales, no planificadas); export Excel (Plan/Resumen/Horas cons./Gantt gráfico con barras de color como el PDF, sin unos, importes, % y horas numéricos) y PDF (impresión en la misma pestaña, sin pop-up). Permisos crear_proyecto / editar_proyecto / eliminar_proyecto en Seguridad. Componente: scripts/lib/fornitalia-gestion-proyectos.js + .css. SQL: sql/supabase_gestion_proyectos.sql, sql/supabase_user_profiles_nombre_usuario.sql, sql/supabase_gp_tarea_horas_alocadas.sql, sql/supabase_gp_tarea_hora.sql, sql/supabase_gp_entregable_hora.sql, sql/supabase_gp_observaciones_y_horas_rls.sql y sql/supabase_gp_hora_observaciones.sql.</v>
+        <v>Menú lateral (permiso ver_gestion_proyectos). ABM de planes: Proyecto → Entregables (nombre, alcance, fechas, responsable usuario o perfil) → Tareas (misma metadata) y Dependencias (viñeta + responsable). Las horas son las realmente consumidas por fecha en el proyecto (gp_proyecto_hora), el entregable (gp_entregable_hora) y/o las tareas (gp_tarea_hora), cada fila con observaciones; el total del proyecto es propias + entregables + tareas (RPC gp_guardar_horas_*). Solapa Horas cons.: conciliación diaria. Alerta si una tarea o las horas superan el deadline del entregable o del proyecto. El responsable de usuario se muestra como nombre corto / iniciales (no el email; el correo va en el tooltip). Solapa To-Do: tabla jerárquica expandable o solo entregables (entregable en negrita, tareas y dependencias en peso normal), cards de pendientes/en curso/vencidas, cambio de estado. Ordenar entregables por fecha, nombre, estado o manual (flechas ↑↓ persistidas). Solapa Gantt one-page: anillo de avance, SPI ponderado por horas consumidas (propias del proyecto + entregables/tareas; sin horas no diluye) vs calendario, barras con % y horas consumidas (reales, no planificadas); export Excel (Plan/Resumen/Horas cons./Gantt gráfico con barras de color como el PDF, sin unos, importes, % y horas numéricos) y PDF (impresión en la misma pestaña, sin pop-up). Permisos crear_proyecto / editar_proyecto / eliminar_proyecto en Seguridad. Componente: scripts/lib/fornitalia-gestion-proyectos.js + .css. SQL: sql/supabase_gestion_proyectos.sql, sql/supabase_user_profiles_nombre_usuario.sql, sql/supabase_gp_tarea_horas_alocadas.sql, sql/supabase_gp_tarea_hora.sql, sql/supabase_gp_entregable_hora.sql, sql/supabase_gp_proyecto_hora.sql, sql/supabase_gp_observaciones_y_horas_rls.sql y sql/supabase_gp_hora_observaciones.sql.</v>
       </c>
     </row>
     <row r="60">
@@ -4553,7 +4587,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C54"/>
+  <dimension ref="A1:C55"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -5154,9 +5188,20 @@
         <v>Despliegue v2.10: export Excel de Flujo por mes (importes numéricos, % como fracción, caución en ARS, totales y proyección); fechas calendario Argentina en Excel/PDF del plan de Gestión de Proyectos. Producción Vercel.</v>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>2.11</v>
+      </c>
+      <c r="B55" t="str">
+        <v>31/08/2026</v>
+      </c>
+      <c r="C55" t="str">
+        <v>Despliegue v2.11: horas consumidas propias del proyecto (fecha + horas + observaciones, igual que entregable/tarea); total del proyecto = propias + entregables + tareas; SPI, avance, KPI, solapa Horas cons. y Excel integrados. sql/supabase_gp_proyecto_hora.sql. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C54"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C55"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5344,7 +5389,7 @@
         <v>Gestión de Proyectos</v>
       </c>
       <c r="B13" t="str">
-        <v>ABM de planes de trabajo (proyecto, entregables, tareas y dependencias), To-Do jerárquico, Gantt one-page con avance y SPI, horas consumidas por fecha con observaciones, export Excel/PDF, permisos por perfil.</v>
+        <v>ABM de planes de trabajo (proyecto, entregables, tareas y dependencias), To-Do jerárquico, Gantt one-page con avance y SPI, horas consumidas por fecha con observaciones (proyecto, entregable y tarea), export Excel/PDF, permisos por perfil.</v>
       </c>
       <c r="C13">
         <v>40</v>
@@ -5389,7 +5434,7 @@
         <v>Datos</v>
       </c>
       <c r="B3" t="str">
-        <v>Supabase (PostgreSQL). Tablas: transacciones, tipo_de_cambio, config_dashboard, gp_proyecto, gp_entregable, gp_entregable_hora, gp_tarea, gp_tarea_hora, gp_dependencia. Scripts SQL en carpeta sql/ se ejecutan en Supabase SQL Editor.</v>
+        <v>Supabase (PostgreSQL). Tablas: transacciones, tipo_de_cambio, config_dashboard, gp_proyecto, gp_entregable, gp_entregable_hora, gp_tarea, gp_tarea_hora, gp_proyecto_hora, gp_dependencia. Scripts SQL en carpeta sql/ se ejecutan en Supabase SQL Editor.</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
v2.12: Conciliación Bancaria (Mercado Pago y Galicia).
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E209"/>
+  <dimension ref="A1:E220"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -3964,16 +3964,203 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="210">
+      <c r="A210" t="str">
+        <v>09/09/2026</v>
+      </c>
+      <c r="B210" t="str">
+        <v>08:53</v>
+      </c>
+      <c r="C210" t="str">
+        <v>Conciliación Bancaria (Mercado Pago)</v>
+      </c>
+      <c r="D210" t="str">
+        <v>Menú Conciliación Bancaria con permisos en Seguridad. Mercado Pago: upload extracto (Número de Movimiento, sin duplicar) y tesorería sistema; sugerencias de match por importe/fecha; ojito de detalle y confirmación. Galicia queda como solapa próxima. sql/supabase_conciliacion_bancaria.sql.</v>
+      </c>
+      <c r="E210" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="str">
+        <v>09/09/2026</v>
+      </c>
+      <c r="B211" t="str">
+        <v>08:57</v>
+      </c>
+      <c r="C211" t="str">
+        <v>Fix trigger sugerencias conciliación</v>
+      </c>
+      <c r="D211" t="str">
+        <v>El upload de tesorería guardaba bien; al generar sugerencias el trigger cb_set_updated_at leía created_by en cb_match (esa tabla no lo tiene). Ahora created_by solo se setea en cb_movimiento.</v>
+      </c>
+      <c r="E211" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="str">
+        <v>09/09/2026</v>
+      </c>
+      <c r="B212" t="str">
+        <v>09:45</v>
+      </c>
+      <c r="C212" t="str">
+        <v>Conciliación Bancaria: extracto Galicia</v>
+      </c>
+      <c r="D212" t="str">
+        <v>Solapa Banco Galicia activa. Parser del extracto Galicia (Extracto_CC…, hoja Movimientos: Fecha, Descripción, Débitos, Créditos, Saldo). ID estable fecha+débito/crédito+saldo para no duplicar. Tesorería lista para hoja Transferencia Galicia. Mismo matching, ojito y confirmación que MP.</v>
+      </c>
+      <c r="E212" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="str">
+        <v>09/09/2026</v>
+      </c>
+      <c r="B213" t="str">
+        <v>09:55</v>
+      </c>
+      <c r="C213" t="str">
+        <v>Conciliación Bancaria: tesorería Galicia</v>
+      </c>
+      <c r="D213" t="str">
+        <v>Tesorería tesoreria_transferencia_galicia (hoja Transferencia Galicia: mismas columnas que Mercado Pago). Botón Cargar tesorería Galicia, detección por hoja/nombre y sugerencias contra el extracto CC. Apertura de caja se excluye del match.</v>
+      </c>
+      <c r="E213" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="str">
+        <v>09/09/2026</v>
+      </c>
+      <c r="B214" t="str">
+        <v>10:05</v>
+      </c>
+      <c r="C214" t="str">
+        <v>Filtros mes y concepto en conciliación</v>
+      </c>
+      <c r="D214" t="str">
+        <v>En Conciliación Bancaria: combos Mes (mm/aaaa) y Concepto del extracto (tipo/descripción del banco). Filtran listados y KPIs; tesorería respeta el mes. Móvil: selects a ancho completo.</v>
+      </c>
+      <c r="E214" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="str">
+        <v>09/09/2026</v>
+      </c>
+      <c r="B215" t="str">
+        <v>10:20</v>
+      </c>
+      <c r="C215" t="str">
+        <v>Orden columnas conciliación bancaria</v>
+      </c>
+      <c r="D215" t="str">
+        <v>Tablas de Conciliación Bancaria: clic en encabezado ordena asc/desc (fecha, importe, concepto, etc.). Indicador ▲/▼; toque ≥44px. Orden por listado (sugeridos, confirmados, solo banco/sistema).</v>
+      </c>
+      <c r="E215" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="str">
+        <v>09/09/2026</v>
+      </c>
+      <c r="B216" t="str">
+        <v>10:25</v>
+      </c>
+      <c r="C216" t="str">
+        <v>Sugerencias mismo importe fecha lejana</v>
+      </c>
+      <c r="D216" t="str">
+        <v>Conciliación: además de misma fecha y fecha cercana (±14 días), se sugieren parejas con el mismo importe y fecha lejana (&gt;14 días), con badge “Mismo importe, fecha lejana” (y “hay otros iguales” si el monto se repite). Recalcular sugerencias para verlas.</v>
+      </c>
+      <c r="E216" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="str">
+        <v>09/09/2026</v>
+      </c>
+      <c r="B217" t="str">
+        <v>10:35</v>
+      </c>
+      <c r="C217" t="str">
+        <v>Match MP 1.213.703,21 vs tesorería 1.213.703,20</v>
+      </c>
+      <c r="D217" t="str">
+        <v>El caso Mercado Pago (11/08 vs 08/09) no salía en sugeridos: extracto -1.213.703,21 y tesorería -1.213.703,20 (1 centavo). Ahora el match acepta hasta 1 centavo de diferencia. Recalcular sugerencias.</v>
+      </c>
+      <c r="E217" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="str">
+        <v>09/09/2026</v>
+      </c>
+      <c r="B218" t="str">
+        <v>10:50</v>
+      </c>
+      <c r="C218" t="str">
+        <v>Match por descripción para no cruzar impuestos</v>
+      </c>
+      <c r="D218" t="str">
+        <v>Con el mismo importe, el match prioriza concepto en la descripción (IVA, IIBB, SIRCREB, Ganancias, Ley 25413, etc.) y no arma la pareja si los impuestos chocan. Evita sugerencias invertidas. Recalcular sugerencias.</v>
+      </c>
+      <c r="E218" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="str">
+        <v>09/09/2026</v>
+      </c>
+      <c r="B219" t="str">
+        <v>10:55</v>
+      </c>
+      <c r="C219" t="str">
+        <v>Tolerancia de match: hasta $1</v>
+      </c>
+      <c r="D219" t="str">
+        <v>La coincidencia de importe en Conciliación Bancaria admite hasta 1 peso de diferencia (no solo 1 centavo). Recalcular sugerencias.</v>
+      </c>
+      <c r="E219" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="str">
+        <v>09/09/2026</v>
+      </c>
+      <c r="B220" t="str">
+        <v>11:05</v>
+      </c>
+      <c r="C220" t="str">
+        <v>Despliegue v2.12 producción</v>
+      </c>
+      <c r="D220" t="str">
+        <v>Push a main y Vercel --prod: Conciliación Bancaria (MP y Galicia), filtros, orden, match por concepto y tolerancia $1. APP_VERSION 2.12.</v>
+      </c>
+      <c r="E220" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E209"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E220"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B64"/>
+  <dimension ref="A1:B65"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -4453,47 +4640,55 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>Normalización de extracto bancario</v>
+        <v>Conciliación Bancaria</v>
       </c>
       <c r="B60" t="str">
-        <v>npm run normalizar-extracto: lee Fornitalia_Movimientos.xlsx (o Extracto legado), hoja Normalizado con fecha_iso, tipo, medio, categoría, cuenta, moneda inferida, monto_original, tipo_cambio, monto_ars, id_cierre_caja, id_comprobante_pago, id_impuesto, cat_desc cuando vienen del export.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto CC (fecha+débito/crédito+saldo) + tesorería tesoreria_transferencia_galicia (mismas columnas Tipo/Fecha/Crédito/Débito). Filtros de mes y de concepto del extracto (además de buscar). Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe (misma fecha, fecha cercana ±14 días o fecha lejana) y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRCREB, etc., para no cruzar impuestos); el usuario confirma o descarta. Ojito para ver el detalle de ambos lados. Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql.</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>Informe inconsistencias datos legacy (cliente)</v>
+        <v>Normalización de extracto bancario</v>
       </c>
       <c r="B61" t="str">
-        <v>docs/ANALISIS_NORMALIZACION_DATOS_LEGACY_FORNITALIA.md alineado a Fornitalia_Movimientos.xlsx, §0 validaciones IDs/CatDesc, pipeline normalizar-extracto. Regenerar HTML+PDF: npm run informe-normalizacion (informe-normalizacion-solo-html solo si hace falta iterar sin Playwright).</v>
+        <v>npm run normalizar-extracto: lee Fornitalia_Movimientos.xlsx (o Extracto legado), hoja Normalizado con fecha_iso, tipo, medio, categoría, cuenta, moneda inferida, monto_original, tipo_cambio, monto_ars, id_cierre_caja, id_comprobante_pago, id_impuesto, cat_desc cuando vienen del export.</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>Upload de extracto normalizado</v>
+        <v>Informe inconsistencias datos legacy (cliente)</v>
       </c>
       <c r="B62" t="str">
-        <v>Botón en la app para reemplazar transacciones desde la hoja Normalizado (p. ej. Base_Fornitalia_To_App): incluye nueva_categoria, nueva_cuenta_contable, costo_directo/indirecto y columnas EF_Item / EF_SubItem → ef_item / ef_subitem en Supabase. Validación previa, carga en lotes y log de excluidos.</v>
+        <v>docs/ANALISIS_NORMALIZACION_DATOS_LEGACY_FORNITALIA.md alineado a Fornitalia_Movimientos.xlsx, §0 validaciones IDs/CatDesc, pipeline normalizar-extracto. Regenerar HTML+PDF: npm run informe-normalizacion (informe-normalizacion-solo-html solo si hace falta iterar sin Playwright).</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>Log de excluidos en upload</v>
+        <v>Upload de extracto normalizado</v>
       </c>
       <c r="B63" t="str">
-        <v>Nueva solapa Excluidos upload con registros no insertados por error o por regla de negocio (Apertura/Cierre de Caja), persistidos en Supabase para auditoría.</v>
+        <v>Botón en la app para reemplazar transacciones desde la hoja Normalizado (p. ej. Base_Fornitalia_To_App): incluye nueva_categoria, nueva_cuenta_contable, costo_directo/indirecto y columnas EF_Item / EF_SubItem → ef_item / ef_subitem en Supabase. Validación previa, carga en lotes y log de excluidos.</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
+        <v>Log de excluidos en upload</v>
+      </c>
+      <c r="B64" t="str">
+        <v>Nueva solapa Excluidos upload con registros no insertados por error o por regla de negocio (Apertura/Cierre de Caja), persistidos en Supabase para auditoría.</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
         <v>Análisis financiero extracto (PDF)</v>
       </c>
-      <c r="B64" t="str">
+      <c r="B65" t="str">
         <v>npm run analisis-financiero-pdf: métricas desde Fornitalia_Movimientos.xlsx (fallback Extracto legado); ARS vía MontoCambio/Monto en $, TC por fila o MEP; exclusiones y USD sin conversión. Sección ventas: ranking por vendedor desde Resumen_Operaciones (Tabla, Vendedor_RO) por N° operación; ranking proxy por producto (detalle hasta mes cierre feb 2026). Ver docs/ANALISIS_FINANCIERO_EXTRACTO_README.md.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B64"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B65"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4587,7 +4782,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C55"/>
+  <dimension ref="A1:C56"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -5199,16 +5394,27 @@
         <v>Despliegue v2.11: horas consumidas propias del proyecto (fecha + horas + observaciones, igual que entregable/tarea); total del proyecto = propias + entregables + tareas; SPI, avance, KPI, solapa Horas cons. y Excel integrados. sql/supabase_gp_proyecto_hora.sql. Producción Vercel.</v>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>2.12</v>
+      </c>
+      <c r="B56" t="str">
+        <v>09/09/2026</v>
+      </c>
+      <c r="C56" t="str">
+        <v>Despliegue v2.12: Conciliación Bancaria (Mercado Pago y Galicia): upload extracto y tesorería, sugerencias por importe (±$1) y concepto (evitar cruzar impuestos), fecha cercana/lejana, filtros mes/concepto, orden de columnas, ojito y confirmación. Permisos en Seguridad. sql/supabase_conciliacion_bancaria.sql. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C55"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C56"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="90.83203125" customWidth="1"/>
@@ -5398,9 +5604,23 @@
         <v/>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Conciliación Bancaria</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago y Galicia). Uploads por ID sin duplicar, sugerencias de match, detalle con ojito y confirmación del usuario. Permisos en Seguridad.</v>
+      </c>
+      <c r="C14">
+        <v>24</v>
+      </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D14"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5426,7 +5646,7 @@
         <v>Frontend</v>
       </c>
       <c r="B2" t="str">
-        <v>Página dashboard-flujo-caja.html (HTML/CSS/JS). Gestión de Proyectos en componente aparte: scripts/lib/fornitalia-gestion-proyectos.js + .css. Sin framework; llamadas a Supabase desde el cliente.</v>
+        <v>Página dashboard-flujo-caja.html (HTML/CSS/JS). Gestión de Proyectos y Conciliación Bancaria en componentes aparte (scripts/lib/fornitalia-gestion-proyectos.* y fornitalia-conciliacion-bancaria.*). Sin framework; llamadas a Supabase desde el cliente.</v>
       </c>
     </row>
     <row r="3">
@@ -5434,7 +5654,7 @@
         <v>Datos</v>
       </c>
       <c r="B3" t="str">
-        <v>Supabase (PostgreSQL). Tablas: transacciones, tipo_de_cambio, config_dashboard, gp_proyecto, gp_entregable, gp_entregable_hora, gp_tarea, gp_tarea_hora, gp_proyecto_hora, gp_dependencia. Scripts SQL en carpeta sql/ se ejecutan en Supabase SQL Editor.</v>
+        <v>Supabase (PostgreSQL). Tablas: transacciones, tipo_de_cambio, config_dashboard, gp_proyecto, gp_entregable, gp_entregable_hora, gp_tarea, gp_tarea_hora, gp_proyecto_hora, gp_dependencia, cb_movimiento, cb_match. Scripts SQL en carpeta sql/ se ejecutan en Supabase SQL Editor.</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
v2.13: conciliación manual, deshacer confirmados y filtros activos.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E220"/>
+  <dimension ref="A1:E224"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -4151,9 +4151,77 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="221">
+      <c r="A221" t="str">
+        <v>09/09/2026</v>
+      </c>
+      <c r="B221" t="str">
+        <v>11:45</v>
+      </c>
+      <c r="C221" t="str">
+        <v>Conciliación manual, Excel y filtros activos</v>
+      </c>
+      <c r="D221" t="str">
+        <v>Conciliación Bancaria: pareja extracto+tesorería a mano con justificación obligatoria (queda registrada la diferencia aunque sea &gt; $1, RPC cb_confirmar_manual). Botón Excel verde del listado visible con los filtros. Mes/concepto/buscar en naranja cuando están activos. sql/supabase_conciliacion_bancaria_manual.sql.</v>
+      </c>
+      <c r="E221" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="str">
+        <v>09/09/2026</v>
+      </c>
+      <c r="B222" t="str">
+        <v>11:58</v>
+      </c>
+      <c r="C222" t="str">
+        <v>Deshacer conciliación confirmada</v>
+      </c>
+      <c r="D222" t="str">
+        <v>En Confirmados (y en el detalle): botón de acción para deshacer. La pareja vuelve a Sugeridos (no se rechaza, así se puede volver a confirmar). RPC cb_set_match_estado admite estado sugerido solo desde confirmado.</v>
+      </c>
+      <c r="E222" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="str">
+        <v>09/09/2026</v>
+      </c>
+      <c r="B223" t="str">
+        <v>12:05</v>
+      </c>
+      <c r="C223" t="str">
+        <v>Orden columnas en conciliación manual</v>
+      </c>
+      <c r="D223" t="str">
+        <v>En el modal de Conciliación manual, los encabezados de extracto y tesorería ordenan asc/desc (fecha, concepto, importe y estado sugerido), igual que el resto de las tablas.</v>
+      </c>
+      <c r="E223" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="str">
+        <v>09/09/2026</v>
+      </c>
+      <c r="B224" t="str">
+        <v>12:32</v>
+      </c>
+      <c r="C224" t="str">
+        <v>Despliegue v2.13 producción</v>
+      </c>
+      <c r="D224" t="str">
+        <v>Push a main y Vercel --prod: conciliación manual con justificación (RPC cb_confirmar_manual), deshacer confirmados (vuelve a Sugeridos), orden de columnas en el modal, Excel y filtros activos en naranja. APP_VERSION 2.13.</v>
+      </c>
+      <c r="E224" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E220"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E224"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4643,7 +4711,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto CC (fecha+débito/crédito+saldo) + tesorería tesoreria_transferencia_galicia (mismas columnas Tipo/Fecha/Crédito/Débito). Filtros de mes y de concepto del extracto (además de buscar). Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe (misma fecha, fecha cercana ±14 días o fecha lejana) y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRCREB, etc., para no cruzar impuestos); el usuario confirma o descarta. Ojito para ver el detalle de ambos lados. Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto CC (fecha+débito/crédito+saldo) + tesorería tesoreria_transferencia_galicia (mismas columnas Tipo/Fecha/Crédito/Débito). Filtros de mes y de concepto del extracto (además de buscar); el control se marca en naranja cuando hay filtro activo. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe (misma fecha, fecha cercana ±14 días o fecha lejana, tolerancia ±$1) y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRCREB, etc., para no cruzar impuestos); el usuario confirma o descarta. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se elige un movimiento de extracto y uno de tesorería (encabezados ordenan asc/desc), se justifica la diferencia (aunque sea mayor a $1) y queda registrada (justificación, diferencia, usuario y fecha). Ojito para ver el detalle de ambos lados. Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql y sql/supabase_conciliacion_bancaria_manual.sql.</v>
       </c>
     </row>
     <row r="61">
@@ -4782,7 +4850,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:C57"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -5405,9 +5473,20 @@
         <v>Despliegue v2.12: Conciliación Bancaria (Mercado Pago y Galicia): upload extracto y tesorería, sugerencias por importe (±$1) y concepto (evitar cruzar impuestos), fecha cercana/lejana, filtros mes/concepto, orden de columnas, ojito y confirmación. Permisos en Seguridad. sql/supabase_conciliacion_bancaria.sql. Producción Vercel.</v>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>2.13</v>
+      </c>
+      <c r="B57" t="str">
+        <v>09/09/2026</v>
+      </c>
+      <c r="C57" t="str">
+        <v>Despliegue v2.13: Conciliación Bancaria — pareja manual con justificación (queda registrada aunque la diferencia sea &gt; $1), deshacer confirmados (vuelve a Sugeridos), orden de columnas en el modal, Excel del listado con filtros y controles activos en naranja. sql/supabase_conciliacion_bancaria_manual.sql. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C56"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C57"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5609,7 +5688,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B14" t="str">
-        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago y Galicia). Uploads por ID sin duplicar, sugerencias de match, detalle con ojito y confirmación del usuario. Permisos en Seguridad.</v>
+        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago y Galicia). Uploads por ID sin duplicar, sugerencias de match, conciliación manual con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Permisos en Seguridad.</v>
       </c>
       <c r="C14">
         <v>24</v>

</xml_diff>

<commit_message>
v2.14: conciliación sin tope de 1000 y filtros en el modal manual.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E224"/>
+  <dimension ref="A1:E227"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -4219,9 +4219,60 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="225">
+      <c r="A225" t="str">
+        <v>09/09/2026</v>
+      </c>
+      <c r="B225" t="str">
+        <v>13:20</v>
+      </c>
+      <c r="C225" t="str">
+        <v>Fix carga conciliación: no cortar en 1000 filas</v>
+      </c>
+      <c r="D225" t="str">
+        <v>Galicia en BD tenía 700 extracto + 392 tesorería (1092) y la UI mostraba 670 + 330: PostgREST limita 1000 por request. Parecía que un extracto nuevo borraba tesorería (lado sistema en Confirmados vacío). La carga nunca DELETE movimientos: upsert por origen_id. Ahora se pagina igual que transacciones; el mensaje de upload informa nuevas vs ya existentes.</v>
+      </c>
+      <c r="E225" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="str">
+        <v>09/09/2026</v>
+      </c>
+      <c r="B226" t="str">
+        <v>13:32</v>
+      </c>
+      <c r="C226" t="str">
+        <v>Filtros Mes/Concepto en conciliación manual</v>
+      </c>
+      <c r="D226" t="str">
+        <v>El modal de Conciliación manual replica Mes y Concepto del extracto (mismos controles que la vista, naranja si están activos). Arranca con los filtros ya aplicados en la pantalla; buscar por lado se mantiene. Mes filtra extracto y tesorería; concepto solo el extracto. El movimiento elegido sigue visible aunque el filtro lo oculte.</v>
+      </c>
+      <c r="E226" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="str">
+        <v>09/09/2026</v>
+      </c>
+      <c r="B227" t="str">
+        <v>13:42</v>
+      </c>
+      <c r="C227" t="str">
+        <v>Despliegue v2.14 producción</v>
+      </c>
+      <c r="D227" t="str">
+        <v>Push a main y Vercel --prod: conciliación pagina &gt;1000 movimientos (Galicia ya no recorta tesorería); carga incremental sin borrar; filtros Mes/Concepto en conciliación manual. APP_VERSION 2.14.</v>
+      </c>
+      <c r="E227" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E224"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E227"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4711,7 +4762,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto CC (fecha+débito/crédito+saldo) + tesorería tesoreria_transferencia_galicia (mismas columnas Tipo/Fecha/Crédito/Débito). Filtros de mes y de concepto del extracto (además de buscar); el control se marca en naranja cuando hay filtro activo. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe (misma fecha, fecha cercana ±14 días o fecha lejana, tolerancia ±$1) y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRCREB, etc., para no cruzar impuestos); el usuario confirma o descarta. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se elige un movimiento de extracto y uno de tesorería (encabezados ordenan asc/desc), se justifica la diferencia (aunque sea mayor a $1) y queda registrada (justificación, diferencia, usuario y fecha). Ojito para ver el detalle de ambos lados. Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql y sql/supabase_conciliacion_bancaria_manual.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + saldo). La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto CC (fecha+débito/crédito+saldo) + tesorería tesoreria_transferencia_galicia (mismas columnas Tipo/Fecha/Crédito/Débito). Filtros de mes y de concepto del extracto (además de buscar); el control se marca en naranja cuando hay filtro activo. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe (misma fecha, fecha cercana ±14 días o fecha lejana, tolerancia ±$1) y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRCREB, etc., para no cruzar impuestos); el usuario confirma o descarta. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se elige un movimiento de extracto y uno de tesorería (mismos filtros Mes / Concepto del extracto / Buscar que la vista; si ya estaban activos, el modal los hereda; encabezados ordenan asc/desc), se justifica la diferencia (aunque sea mayor a $1) y queda registrada (justificación, diferencia, usuario y fecha). Ojito para ver el detalle de ambos lados. Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql y sql/supabase_conciliacion_bancaria_manual.sql.</v>
       </c>
     </row>
     <row r="61">
@@ -4850,7 +4901,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C57"/>
+  <dimension ref="A1:C58"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -5484,9 +5535,20 @@
         <v>Despliegue v2.13: Conciliación Bancaria — pareja manual con justificación (queda registrada aunque la diferencia sea &gt; $1), deshacer confirmados (vuelve a Sugeridos), orden de columnas en el modal, Excel del listado con filtros y controles activos en naranja. sql/supabase_conciliacion_bancaria_manual.sql. Producción Vercel.</v>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>2.14</v>
+      </c>
+      <c r="B58" t="str">
+        <v>09/09/2026</v>
+      </c>
+      <c r="C58" t="str">
+        <v>Despliegue v2.14: Conciliación Bancaria pagina movimientos/matches (deja de cortar en 1000; Galicia 700+392 visibles); carga incremental sin borrar; filtros Mes/Concepto en el modal manual (hereda los de la vista). Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C57"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C58"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v2.15: no cargar Apertura de Caja en conciliación.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E227"/>
+  <dimension ref="A1:E229"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -4270,9 +4270,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="228">
+      <c r="A228" t="str">
+        <v>09/09/2026</v>
+      </c>
+      <c r="B228" t="str">
+        <v>16:08</v>
+      </c>
+      <c r="C228" t="str">
+        <v>Conciliación: no cargar ni guardar Apertura de Caja</v>
+      </c>
+      <c r="D228" t="str">
+        <v>Tesorería MP/Galicia omite Tipo/Descripción Apertura de Caja en el upload. Borradas 4 filas ya cargadas (2 Galicia, 2 Mercado Pago; sin matches). sql/supabase_cb_borrar_apertura_caja.sql.</v>
+      </c>
+      <c r="E228" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="str">
+        <v>09/09/2026</v>
+      </c>
+      <c r="B229" t="str">
+        <v>16:08</v>
+      </c>
+      <c r="C229" t="str">
+        <v>Despliegue v2.15 producción</v>
+      </c>
+      <c r="D229" t="str">
+        <v>Push a main y Vercel --prod: tesorería de conciliación no sube Apertura de Caja; filas previas ya borradas en Supabase. APP_VERSION 2.15.</v>
+      </c>
+      <c r="E229" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E227"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E229"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4762,7 +4796,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + saldo). La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto CC (fecha+débito/crédito+saldo) + tesorería tesoreria_transferencia_galicia (mismas columnas Tipo/Fecha/Crédito/Débito). Filtros de mes y de concepto del extracto (además de buscar); el control se marca en naranja cuando hay filtro activo. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe (misma fecha, fecha cercana ±14 días o fecha lejana, tolerancia ±$1) y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRCREB, etc., para no cruzar impuestos); el usuario confirma o descarta. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se elige un movimiento de extracto y uno de tesorería (mismos filtros Mes / Concepto del extracto / Buscar que la vista; si ya estaban activos, el modal los hereda; encabezados ordenan asc/desc), se justifica la diferencia (aunque sea mayor a $1) y queda registrada (justificación, diferencia, usuario y fecha). Ojito para ver el detalle de ambos lados. Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql y sql/supabase_conciliacion_bancaria_manual.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + saldo). Apertura de Caja no se sube (tesorería). La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto CC (fecha+débito/crédito+saldo) + tesorería tesoreria_transferencia_galicia (mismas columnas Tipo/Fecha/Crédito/Débito). Filtros de mes y de concepto del extracto (además de buscar); el control se marca en naranja cuando hay filtro activo. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe (misma fecha, fecha cercana ±14 días o fecha lejana, tolerancia ±$1) y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRCREB, etc., para no cruzar impuestos); el usuario confirma o descarta. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se elige un movimiento de extracto y uno de tesorería (mismos filtros Mes / Concepto del extracto / Buscar que la vista; si ya estaban activos, el modal los hereda; encabezados ordenan asc/desc), se justifica la diferencia (aunque sea mayor a $1) y queda registrada (justificación, diferencia, usuario y fecha). Ojito para ver el detalle de ambos lados. Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql y sql/supabase_conciliacion_bancaria_manual.sql.</v>
       </c>
     </row>
     <row r="61">
@@ -4901,7 +4935,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C58"/>
+  <dimension ref="A1:C59"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -5546,9 +5580,20 @@
         <v>Despliegue v2.14: Conciliación Bancaria pagina movimientos/matches (deja de cortar en 1000; Galicia 700+392 visibles); carga incremental sin borrar; filtros Mes/Concepto en el modal manual (hereda los de la vista). Producción Vercel.</v>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>2.15</v>
+      </c>
+      <c r="B59" t="str">
+        <v>09/09/2026</v>
+      </c>
+      <c r="C59" t="str">
+        <v>Despliegue v2.15: tesorería de Conciliación Bancaria no carga Apertura de Caja; se eliminaron las 4 filas ya subidas (MP y Galicia). sql/supabase_cb_borrar_apertura_caja.sql. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C58"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C59"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v2.16: menú Saldos extractos (Galicia) con tabla, gráfico y permisos.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E229"/>
+  <dimension ref="A1:E231"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -4292,7 +4292,7 @@
         <v>09/09/2026</v>
       </c>
       <c r="B229" t="str">
-        <v>16:08</v>
+        <v>16:09</v>
       </c>
       <c r="C229" t="str">
         <v>Despliegue v2.15 producción</v>
@@ -4304,16 +4304,50 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="230">
+      <c r="A230" t="str">
+        <v>10/09/2026</v>
+      </c>
+      <c r="B230" t="str">
+        <v>09:15</v>
+      </c>
+      <c r="C230" t="str">
+        <v>Menú Saldos extractos (Galicia)</v>
+      </c>
+      <c r="D230" t="str">
+        <v>Nuevo menú con carga de PDFs de resumen de cuenta Galicia (varios a la vez, parseo de a uno, un solo guardado). Serie de saldos inicial/cierre en tabla y gráfico, filtros de período, Excel. Permisos ver/cargar/exportar en Seguridad. Tabla eb_saldo_extracto + RPC eb_guardar_saldos. Componente scripts/lib/fornitalia-saldos-extractos.js.</v>
+      </c>
+      <c r="E230" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="str">
+        <v>10/09/2026</v>
+      </c>
+      <c r="B231" t="str">
+        <v>09:40</v>
+      </c>
+      <c r="C231" t="str">
+        <v>Despliegue v2.16 producción</v>
+      </c>
+      <c r="D231" t="str">
+        <v>Push a main y Vercel --prod: menú Saldos extractos (Galicia PDF), tabla y gráfico con filtros de período, Excel y permisos en Seguridad. APP_VERSION 2.16.</v>
+      </c>
+      <c r="E231" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E229"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E231"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B65"/>
+  <dimension ref="A1:B66"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -4801,47 +4835,55 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>Normalización de extracto bancario</v>
+        <v>Saldos extractos</v>
       </c>
       <c r="B61" t="str">
-        <v>npm run normalizar-extracto: lee Fornitalia_Movimientos.xlsx (o Extracto legado), hoja Normalizado con fecha_iso, tipo, medio, categoría, cuenta, moneda inferida, monto_original, tipo_cambio, monto_ars, id_cierre_caja, id_comprobante_pago, id_impuesto, cat_desc cuando vienen del export.</v>
+        <v>Menú lateral (permiso ver_saldos_extractos). Carga de PDFs de resumen de cuenta (arranca Banco Galicia): el botón admite varios archivos, los reconoce de a uno y los guarda juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha de cierre). Muestra serie de saldo inicial y de cierre en tabla y gráfico de línea, con filtros de período (naranja si están activos). KPIs: cantidad de resúmenes, último saldo y variación del período. Excel con importes numéricos y fechas serial Argentina. Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql.</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>Informe inconsistencias datos legacy (cliente)</v>
+        <v>Normalización de extracto bancario</v>
       </c>
       <c r="B62" t="str">
-        <v>docs/ANALISIS_NORMALIZACION_DATOS_LEGACY_FORNITALIA.md alineado a Fornitalia_Movimientos.xlsx, §0 validaciones IDs/CatDesc, pipeline normalizar-extracto. Regenerar HTML+PDF: npm run informe-normalizacion (informe-normalizacion-solo-html solo si hace falta iterar sin Playwright).</v>
+        <v>npm run normalizar-extracto: lee Fornitalia_Movimientos.xlsx (o Extracto legado), hoja Normalizado con fecha_iso, tipo, medio, categoría, cuenta, moneda inferida, monto_original, tipo_cambio, monto_ars, id_cierre_caja, id_comprobante_pago, id_impuesto, cat_desc cuando vienen del export.</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>Upload de extracto normalizado</v>
+        <v>Informe inconsistencias datos legacy (cliente)</v>
       </c>
       <c r="B63" t="str">
-        <v>Botón en la app para reemplazar transacciones desde la hoja Normalizado (p. ej. Base_Fornitalia_To_App): incluye nueva_categoria, nueva_cuenta_contable, costo_directo/indirecto y columnas EF_Item / EF_SubItem → ef_item / ef_subitem en Supabase. Validación previa, carga en lotes y log de excluidos.</v>
+        <v>docs/ANALISIS_NORMALIZACION_DATOS_LEGACY_FORNITALIA.md alineado a Fornitalia_Movimientos.xlsx, §0 validaciones IDs/CatDesc, pipeline normalizar-extracto. Regenerar HTML+PDF: npm run informe-normalizacion (informe-normalizacion-solo-html solo si hace falta iterar sin Playwright).</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>Log de excluidos en upload</v>
+        <v>Upload de extracto normalizado</v>
       </c>
       <c r="B64" t="str">
-        <v>Nueva solapa Excluidos upload con registros no insertados por error o por regla de negocio (Apertura/Cierre de Caja), persistidos en Supabase para auditoría.</v>
+        <v>Botón en la app para reemplazar transacciones desde la hoja Normalizado (p. ej. Base_Fornitalia_To_App): incluye nueva_categoria, nueva_cuenta_contable, costo_directo/indirecto y columnas EF_Item / EF_SubItem → ef_item / ef_subitem en Supabase. Validación previa, carga en lotes y log de excluidos.</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
+        <v>Log de excluidos en upload</v>
+      </c>
+      <c r="B65" t="str">
+        <v>Nueva solapa Excluidos upload con registros no insertados por error o por regla de negocio (Apertura/Cierre de Caja), persistidos en Supabase para auditoría.</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
         <v>Análisis financiero extracto (PDF)</v>
       </c>
-      <c r="B65" t="str">
+      <c r="B66" t="str">
         <v>npm run analisis-financiero-pdf: métricas desde Fornitalia_Movimientos.xlsx (fallback Extracto legado); ARS vía MontoCambio/Monto en $, TC por fila o MEP; exclusiones y USD sin conversión. Sección ventas: ranking por vendedor desde Resumen_Operaciones (Tabla, Vendedor_RO) por N° operación; ranking proxy por producto (detalle hasta mes cierre feb 2026). Ver docs/ANALISIS_FINANCIERO_EXTRACTO_README.md.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B65"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B66"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4935,7 +4977,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C59"/>
+  <dimension ref="A1:C60"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -5591,16 +5633,27 @@
         <v>Despliegue v2.15: tesorería de Conciliación Bancaria no carga Apertura de Caja; se eliminaron las 4 filas ya subidas (MP y Galicia). sql/supabase_cb_borrar_apertura_caja.sql. Producción Vercel.</v>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>2.16</v>
+      </c>
+      <c r="B60" t="str">
+        <v>10/09/2026</v>
+      </c>
+      <c r="C60" t="str">
+        <v>Despliegue v2.16: menú Saldos extractos (arranca Galicia): carga de varios PDF de resumen, serie de saldos en tabla y gráfico, filtros de período, Excel y permisos ver/cargar/exportar. sql/supabase_saldos_extractos.sql. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C59"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C60"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="90.83203125" customWidth="1"/>
@@ -5804,9 +5857,23 @@
         <v/>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Saldos extractos bancarios</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Menú de resúmenes de cuenta (arranca Galicia): carga de PDFs, serie de saldos en tabla y gráfico, filtros de período, Excel y permisos en Seguridad.</v>
+      </c>
+      <c r="C15">
+        <v>12</v>
+      </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D15"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5832,7 +5899,7 @@
         <v>Frontend</v>
       </c>
       <c r="B2" t="str">
-        <v>Página dashboard-flujo-caja.html (HTML/CSS/JS). Gestión de Proyectos y Conciliación Bancaria en componentes aparte (scripts/lib/fornitalia-gestion-proyectos.* y fornitalia-conciliacion-bancaria.*). Sin framework; llamadas a Supabase desde el cliente.</v>
+        <v>Página dashboard-flujo-caja.html (HTML/CSS/JS). Gestión de Proyectos, Conciliación Bancaria y Saldos extractos en componentes aparte (scripts/lib/fornitalia-gestion-proyectos.*, fornitalia-conciliacion-bancaria.* y fornitalia-saldos-extractos.*). Sin framework; llamadas a Supabase desde el cliente. PDFs Galicia con pdf.js en el navegador.</v>
       </c>
     </row>
     <row r="3">
@@ -5840,7 +5907,7 @@
         <v>Datos</v>
       </c>
       <c r="B3" t="str">
-        <v>Supabase (PostgreSQL). Tablas: transacciones, tipo_de_cambio, config_dashboard, gp_proyecto, gp_entregable, gp_entregable_hora, gp_tarea, gp_tarea_hora, gp_proyecto_hora, gp_dependencia, cb_movimiento, cb_match. Scripts SQL en carpeta sql/ se ejecutan en Supabase SQL Editor.</v>
+        <v>Supabase (PostgreSQL). Tablas: transacciones, tipo_de_cambio, config_dashboard, gp_proyecto, gp_entregable, gp_entregable_hora, gp_tarea, gp_tarea_hora, gp_proyecto_hora, gp_dependencia, cb_movimiento, cb_match, eb_saldo_extracto. Scripts SQL en carpeta sql/ se ejecutan en Supabase SQL Editor.</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
v2.17: conciliación manual N:M, cierre de caja y columnas tesorería.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E231"/>
+  <dimension ref="A1:E237"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -4338,9 +4338,111 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="232">
+      <c r="A232" t="str">
+        <v>10/09/2026</v>
+      </c>
+      <c r="B232" t="str">
+        <v>14:05</v>
+      </c>
+      <c r="C232" t="str">
+        <v>Tesorería: reconocer Excel de cierre de caja</v>
+      </c>
+      <c r="D232" t="str">
+        <v>Conciliación Bancaria acepta cierre_CIERRE-… (Fecha, Tipo, Monto) como tesorería de MP y Galicia: Ingreso→crédito, Egreso→débito; omite aperturas, Pendiente y totales. Historial de caja ya cerrada. Si el archivo no nombra el canal, usa la solapa activa.</v>
+      </c>
+      <c r="E232" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="str">
+        <v>10/09/2026</v>
+      </c>
+      <c r="B233" t="str">
+        <v>14:20</v>
+      </c>
+      <c r="C233" t="str">
+        <v>Borrar cierre MP y deduplicar tesorería por contenido</v>
+      </c>
+      <c r="D233" t="str">
+        <v>Eliminadas de BD las 168 filas de MP_CIERRE-08092026-164141-0BD1.xlsx. Al cargar tesorería (formato viejo o cierre) no se inserta si ya hay misma fecha, monto, descripción, categoría y cliente. sql/supabase_cb_borrar_cierre_mp_20260908.sql.</v>
+      </c>
+      <c r="E233" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="str">
+        <v>10/09/2026</v>
+      </c>
+      <c r="B234" t="str">
+        <v>14:40</v>
+      </c>
+      <c r="C234" t="str">
+        <v>Borrar cierre MP mal cargado en Galicia y prefijo de archivo</v>
+      </c>
+      <c r="D234" t="str">
+        <v>Eliminadas 94 filas de MP_CIERRE-03082026-204514-5AAE.xlsx cargadas en canal Galicia. El cierre de caja exige MP_… en la solapa Mercado Pago y Galicia_… en Banco Galicia (primera palabra antes del _). sql/supabase_cb_borrar_cierre_mp_mal_galicia.sql.</v>
+      </c>
+      <c r="E234" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="str">
+        <v>10/09/2026</v>
+      </c>
+      <c r="B235" t="str">
+        <v>15:10</v>
+      </c>
+      <c r="C235" t="str">
+        <v>Conciliación manual N:M (varios extractos vs tesorería)</v>
+      </c>
+      <c r="D235" t="str">
+        <v>En Conciliación manual se pueden elegir varios movimientos del banco y uno o más de tesorería. La diferencia es suma extracto − suma tesorería; queda un solo confirmado con justificación. RPC cb_confirmar_manual_grupo. sql/supabase_conciliacion_bancaria_manual_grupo.sql.</v>
+      </c>
+      <c r="E235" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="str">
+        <v>10/09/2026</v>
+      </c>
+      <c r="B236" t="str">
+        <v>15:25</v>
+      </c>
+      <c r="C236" t="str">
+        <v>Conciliación: categoría y cuenta en tesorería</v>
+      </c>
+      <c r="D236" t="str">
+        <v>En Sugeridos y Confirmados, entre Sistema e Importe: columnas Categoría y Cuenta contable de tesorería (ordenables). El Excel del listado las incluye. Si el grupo tiene más de un valor, muestra el primero y +N.</v>
+      </c>
+      <c r="E236" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="str">
+        <v>10/09/2026</v>
+      </c>
+      <c r="B237" t="str">
+        <v>15:40</v>
+      </c>
+      <c r="C237" t="str">
+        <v>Despliegue v2.17 producción</v>
+      </c>
+      <c r="D237" t="str">
+        <v>Push a main y Vercel --prod: tesorería reconoce cierre de caja (MP_/Galicia_CIERRE), no duplica por contenido, conciliación manual N:M y columnas categoría/cuenta contable. APP_VERSION 2.17.</v>
+      </c>
+      <c r="E237" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E231"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E237"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4830,7 +4932,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + saldo). Apertura de Caja no se sube (tesorería). La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto CC (fecha+débito/crédito+saldo) + tesorería tesoreria_transferencia_galicia (mismas columnas Tipo/Fecha/Crédito/Débito). Filtros de mes y de concepto del extracto (además de buscar); el control se marca en naranja cuando hay filtro activo. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe (misma fecha, fecha cercana ±14 días o fecha lejana, tolerancia ±$1) y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRCREB, etc., para no cruzar impuestos); el usuario confirma o descarta. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se elige un movimiento de extracto y uno de tesorería (mismos filtros Mes / Concepto del extracto / Buscar que la vista; si ya estaban activos, el modal los hereda; encabezados ordenan asc/desc), se justifica la diferencia (aunque sea mayor a $1) y queda registrada (justificación, diferencia, usuario y fecha). Ojito para ver el detalle de ambos lados. Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql y sql/supabase_conciliacion_bancaria_manual.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + saldo). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto; Ingreso→crédito y Egreso→débito; historial de caja ya cerrada. El archivo debe llamarse MP_… en la solapa Mercado Pago y Galicia_… en Banco Galicia (primera palabra antes del _). Filas Pendiente y totales del pie no se cargan. Tesorería no duplica si ya existe misma fecha, monto, descripción, categoría y cliente (aunque el Excel sea de otro formato). La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto CC (fecha+débito/crédito+saldo) + tesorería tesoreria_transferencia_galicia (mismas columnas Tipo/Fecha/Crédito/Débito). Filtros de mes y de concepto del extracto (además de buscar); el control se marca en naranja cuando hay filtro activo. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe (misma fecha, fecha cercana ±14 días o fecha lejana, tolerancia ±$1) y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRCREB, etc., para no cruzar impuestos); el usuario confirma o descarta. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismos filtros Mes / Concepto del extracto / Buscar que la vista; si ya estaban activos, el modal los hereda; encabezados ordenan asc/desc). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos y Confirmados, entre Sistema e Importe aparecen Categoría y Cuenta contable de tesorería. Ojito para ver el detalle de todos los movimientos del grupo. Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql y sql/supabase_conciliacion_bancaria_manual_grupo.sql.</v>
       </c>
     </row>
     <row r="61">
@@ -4977,7 +5079,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C60"/>
+  <dimension ref="A1:C61"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -5644,9 +5746,20 @@
         <v>Despliegue v2.16: menú Saldos extractos (arranca Galicia): carga de varios PDF de resumen, serie de saldos en tabla y gráfico, filtros de período, Excel y permisos ver/cargar/exportar. sql/supabase_saldos_extractos.sql. Producción Vercel.</v>
       </c>
     </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>2.17</v>
+      </c>
+      <c r="B61" t="str">
+        <v>10/09/2026</v>
+      </c>
+      <c r="C61" t="str">
+        <v>Despliegue v2.17: Conciliación Bancaria — tesorería de cierre de caja (prefijo MP_/Galicia_), sin duplicar por fecha/monto/descripción/categoría/cliente; conciliación manual N:M (varios extractos vs una o más tesorerías); columnas Categoría y Cuenta contable en Sugeridos/Confirmados. sql/supabase_conciliacion_bancaria_manual_grupo.sql. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C60"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C61"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5848,7 +5961,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B14" t="str">
-        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago y Galicia). Uploads por ID sin duplicar, sugerencias de match, conciliación manual con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Permisos en Seguridad.</v>
+        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago y Galicia). Uploads por ID sin duplicar, sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) como tesorería histórica. Permisos en Seguridad.</v>
       </c>
       <c r="C14">
         <v>24</v>

</xml_diff>

<commit_message>
v2.18: saldos Mercado Pago, consolidado mensual y promedios.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E237"/>
+  <dimension ref="A1:E239"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -4440,9 +4440,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="238">
+      <c r="A238" t="str">
+        <v>10/09/2026</v>
+      </c>
+      <c r="B238" t="str">
+        <v>16:55</v>
+      </c>
+      <c r="C238" t="str">
+        <v>Saldos extractos: Mercado Pago y consolidado</v>
+      </c>
+      <c r="D238" t="str">
+        <v>Solapa Mercado Pago con PDF Carta de saldo (MP_Saldos_…): saldo total, disponible y a liberar. Solapa Consolidado: posición mensual Galicia + MP (arrastra el último saldo si falta un mes). Cards: promedio de saldo (cuánto queda) y promedio de variación. sql/supabase_saldos_extractos_mercadopago.sql.</v>
+      </c>
+      <c r="E238" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="str">
+        <v>10/09/2026</v>
+      </c>
+      <c r="B239" t="str">
+        <v>17:40</v>
+      </c>
+      <c r="C239" t="str">
+        <v>Despliegue v2.18 producción</v>
+      </c>
+      <c r="D239" t="str">
+        <v>Push a main y Vercel --prod: Saldos extractos con Mercado Pago (carta MP_Saldos_), posición consolidada mensual y promedios de saldo/variación. APP_VERSION 2.18.</v>
+      </c>
+      <c r="E239" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E237"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E239"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4940,7 +4974,7 @@
         <v>Saldos extractos</v>
       </c>
       <c r="B61" t="str">
-        <v>Menú lateral (permiso ver_saldos_extractos). Carga de PDFs de resumen de cuenta (arranca Banco Galicia): el botón admite varios archivos, los reconoce de a uno y los guarda juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha de cierre). Muestra serie de saldo inicial y de cierre en tabla y gráfico de línea, con filtros de período (naranja si están activos). KPIs: cantidad de resúmenes, último saldo y variación del período. Excel con importes numéricos y fechas serial Argentina. Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql.</v>
+        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago, Banco Galicia y Consolidado. MP: PDF Carta de saldo (MP_Saldos_YYYYMMDD) con saldo total, disponible y a liberar; variación vs la carta anterior. Galicia: PDF de resumen de cuenta (saldo inicial/cierre del período). Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia + MP (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período, promedio de saldo (cuánto queda en las cuentas) y promedio de variación. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql y sql/supabase_saldos_extractos_mercadopago.sql.</v>
       </c>
     </row>
     <row r="62">
@@ -5079,7 +5113,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C61"/>
+  <dimension ref="A1:C62"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -5757,9 +5791,20 @@
         <v>Despliegue v2.17: Conciliación Bancaria — tesorería de cierre de caja (prefijo MP_/Galicia_), sin duplicar por fecha/monto/descripción/categoría/cliente; conciliación manual N:M (varios extractos vs una o más tesorerías); columnas Categoría y Cuenta contable en Sugeridos/Confirmados. sql/supabase_conciliacion_bancaria_manual_grupo.sql. Producción Vercel.</v>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>2.18</v>
+      </c>
+      <c r="B62" t="str">
+        <v>10/09/2026</v>
+      </c>
+      <c r="C62" t="str">
+        <v>Despliegue v2.18: Saldos extractos — Mercado Pago (PDF Carta de saldo MP_Saldos_), posición consolidada mensual Galicia+MP, cards de promedio de saldo y de variación. sql/supabase_saldos_extractos_mercadopago.sql. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C61"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C62"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5975,7 +6020,7 @@
         <v>Saldos extractos bancarios</v>
       </c>
       <c r="B15" t="str">
-        <v>Menú de resúmenes de cuenta (arranca Galicia): carga de PDFs, serie de saldos en tabla y gráfico, filtros de período, Excel y permisos en Seguridad.</v>
+        <v>Menú de saldos de cierre: Mercado Pago (carta de saldo), Galicia (resumen PDF) y posición consolidada mensual, con promedios de saldo y variación, Excel y permisos en Seguridad.</v>
       </c>
       <c r="C15">
         <v>12</v>

</xml_diff>

<commit_message>
v2.19: eliminar tesorería desde Solo sistema.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E239"/>
+  <dimension ref="A1:E241"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -4474,9 +4474,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="240">
+      <c r="A240" t="str">
+        <v>11/09/2026</v>
+      </c>
+      <c r="B240" t="str">
+        <v>11:15</v>
+      </c>
+      <c r="C240" t="str">
+        <v>Eliminar tesorería en Solo sistema</v>
+      </c>
+      <c r="D240" t="str">
+        <v>En Conciliación Bancaria, solapa Solo sistema: icono de papelera junto al ojito para borrar un movimiento de tesorería que no esté en sugerido/confirmado (permiso cargar). Confirmación previa. RPC cb_borrar_movimiento_sistema. sql/supabase_cb_borrar_movimiento_sistema.sql.</v>
+      </c>
+      <c r="E240" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="str">
+        <v>11/09/2026</v>
+      </c>
+      <c r="B241" t="str">
+        <v>11:45</v>
+      </c>
+      <c r="C241" t="str">
+        <v>Despliegue v2.19 producción</v>
+      </c>
+      <c r="D241" t="str">
+        <v>Push a main y Vercel --prod: eliminar movimiento de tesorería desde Solo sistema (papelera junto al ojito). APP_VERSION 2.19.</v>
+      </c>
+      <c r="E241" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E239"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E241"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4966,7 +5000,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + saldo). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto; Ingreso→crédito y Egreso→débito; historial de caja ya cerrada. El archivo debe llamarse MP_… en la solapa Mercado Pago y Galicia_… en Banco Galicia (primera palabra antes del _). Filas Pendiente y totales del pie no se cargan. Tesorería no duplica si ya existe misma fecha, monto, descripción, categoría y cliente (aunque el Excel sea de otro formato). La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto CC (fecha+débito/crédito+saldo) + tesorería tesoreria_transferencia_galicia (mismas columnas Tipo/Fecha/Crédito/Débito). Filtros de mes y de concepto del extracto (además de buscar); el control se marca en naranja cuando hay filtro activo. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe (misma fecha, fecha cercana ±14 días o fecha lejana, tolerancia ±$1) y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRCREB, etc., para no cruzar impuestos); el usuario confirma o descarta. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismos filtros Mes / Concepto del extracto / Buscar que la vista; si ya estaban activos, el modal los hereda; encabezados ordenan asc/desc). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos y Confirmados, entre Sistema e Importe aparecen Categoría y Cuenta contable de tesorería. Ojito para ver el detalle de todos los movimientos del grupo. Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql y sql/supabase_conciliacion_bancaria_manual_grupo.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + saldo). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto; Ingreso→crédito y Egreso→débito; historial de caja ya cerrada. El archivo debe llamarse MP_… en la solapa Mercado Pago y Galicia_… en Banco Galicia (primera palabra antes del _). Filas Pendiente y totales del pie no se cargan. Tesorería no duplica si ya existe misma fecha, monto, descripción, categoría y cliente (aunque el Excel sea de otro formato). La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto CC (fecha+débito/crédito+saldo) + tesorería tesoreria_transferencia_galicia (mismas columnas Tipo/Fecha/Crédito/Débito). Filtros de mes y de concepto del extracto (además de buscar); el control se marca en naranja cuando hay filtro activo. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe (misma fecha, fecha cercana ±14 días o fecha lejana, tolerancia ±$1) y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRCREB, etc., para no cruzar impuestos); el usuario confirma o descarta. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismos filtros Mes / Concepto del extracto / Buscar que la vista; si ya estaban activos, el modal los hereda; encabezados ordenan asc/desc). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos y Confirmados, entre Sistema e Importe aparecen Categoría y Cuenta contable de tesorería. Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql y sql/supabase_conciliacion_bancaria_manual_grupo.sql.</v>
       </c>
     </row>
     <row r="61">
@@ -5113,7 +5147,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C62"/>
+  <dimension ref="A1:C63"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -5802,9 +5836,20 @@
         <v>Despliegue v2.18: Saldos extractos — Mercado Pago (PDF Carta de saldo MP_Saldos_), posición consolidada mensual Galicia+MP, cards de promedio de saldo y de variación. sql/supabase_saldos_extractos_mercadopago.sql. Producción Vercel.</v>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>2.19</v>
+      </c>
+      <c r="B63" t="str">
+        <v>11/09/2026</v>
+      </c>
+      <c r="C63" t="str">
+        <v>Despliegue v2.19: Conciliación Bancaria — en Solo sistema, papelera para eliminar un movimiento de tesorería no conciliado (permiso cargar). sql/supabase_cb_borrar_movimiento_sistema.sql. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C62"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C63"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v2.20: sugerencias SIRTAC/IIBB y solapa Mercado Pago Anulados.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E241"/>
+  <dimension ref="A1:E244"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -4508,9 +4508,60 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="242">
+      <c r="A242" t="str">
+        <v>11/09/2026</v>
+      </c>
+      <c r="B242" t="str">
+        <v>15:40</v>
+      </c>
+      <c r="C242" t="str">
+        <v>Sugeridos: SIRTAC/IIBB e importe único</v>
+      </c>
+      <c r="D242" t="str">
+        <v>Las conciliaciones 1:1 de hoy (retenciones SIRTAC vs Ingresos Brutos, y Ley 25.413) no aparecían en Sugeridos: SIRTAC se trataba como impuesto distinto de IIBB (score −80) y el matcher descartaba cualquier par con score negativo, aunque el importe fuera único. SIRTAC/SIRCREB cuenta como IIBB; si queda un solo candidato con el mismo importe igual se sugiere. Recalcular sugerencias para ver los pares que faltan.</v>
+      </c>
+      <c r="E242" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="str">
+        <v>11/09/2026</v>
+      </c>
+      <c r="B243" t="str">
+        <v>15:50</v>
+      </c>
+      <c r="C243" t="str">
+        <v>Mercado Pago Anulados (autoanulados)</v>
+      </c>
+      <c r="D243" t="str">
+        <v>Solapa Mercado Pago Anulados: pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación). No entran a Sugeridos, Solo banco ni conciliación manual porque tesorería no los tiene. KPI y Excel del listado.</v>
+      </c>
+      <c r="E243" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="str">
+        <v>11/09/2026</v>
+      </c>
+      <c r="B244" t="str">
+        <v>16:16</v>
+      </c>
+      <c r="C244" t="str">
+        <v>Despliegue v2.20 producción</v>
+      </c>
+      <c r="D244" t="str">
+        <v>Push a main y Vercel --prod: sugerencias SIRTAC/IIBB e importe único; solapa Mercado Pago Anulados (pares autoanulados del extracto fuera de la conciliación). APP_VERSION 2.20.</v>
+      </c>
+      <c r="E244" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E241"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E244"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5000,7 +5051,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + saldo). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto; Ingreso→crédito y Egreso→débito; historial de caja ya cerrada. El archivo debe llamarse MP_… en la solapa Mercado Pago y Galicia_… en Banco Galicia (primera palabra antes del _). Filas Pendiente y totales del pie no se cargan. Tesorería no duplica si ya existe misma fecha, monto, descripción, categoría y cliente (aunque el Excel sea de otro formato). La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto CC (fecha+débito/crédito+saldo) + tesorería tesoreria_transferencia_galicia (mismas columnas Tipo/Fecha/Crédito/Débito). Filtros de mes y de concepto del extracto (además de buscar); el control se marca en naranja cuando hay filtro activo. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe (misma fecha, fecha cercana ±14 días o fecha lejana, tolerancia ±$1) y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRCREB, etc., para no cruzar impuestos); el usuario confirma o descarta. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismos filtros Mes / Concepto del extracto / Buscar que la vista; si ya estaban activos, el modal los hereda; encabezados ordenan asc/desc). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos y Confirmados, entre Sistema e Importe aparecen Categoría y Cuenta contable de tesorería. Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql y sql/supabase_conciliacion_bancaria_manual_grupo.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + saldo). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto; Ingreso→crédito y Egreso→débito; historial de caja ya cerrada. El archivo debe llamarse MP_… en la solapa Mercado Pago y Galicia_… en Banco Galicia (primera palabra antes del _). Filas Pendiente y totales del pie no se cargan. Tesorería no duplica si ya existe misma fecha, monto, descripción, categoría y cliente (aunque el Excel sea de otro formato). La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto CC (fecha+débito/crédito+saldo) + tesorería tesoreria_transferencia_galicia (mismas columnas Tipo/Fecha/Crédito/Débito). Filtros de mes y de concepto del extracto (además de buscar); el control se marca en naranja cuando hay filtro activo. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe (misma fecha, fecha cercana ±14 días o fecha lejana, tolerancia ±$1) y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismos filtros Mes / Concepto del extracto / Buscar que la vista; si ya estaban activos, el modal los hereda; encabezados ordenan asc/desc). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos y Confirmados, entre Sistema e Importe aparecen Categoría y Cuenta contable de tesorería. Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql y sql/supabase_conciliacion_bancaria_manual_grupo.sql.</v>
       </c>
     </row>
     <row r="61">
@@ -5147,7 +5198,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C63"/>
+  <dimension ref="A1:C64"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -5847,9 +5898,20 @@
         <v>Despliegue v2.19: Conciliación Bancaria — en Solo sistema, papelera para eliminar un movimiento de tesorería no conciliado (permiso cargar). sql/supabase_cb_borrar_movimiento_sistema.sql. Producción Vercel.</v>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>2.20</v>
+      </c>
+      <c r="B64" t="str">
+        <v>11/09/2026</v>
+      </c>
+      <c r="C64" t="str">
+        <v>Despliegue v2.20: Conciliación Bancaria — SIRTAC cuenta como IIBB y el importe único se sugiere aunque el concepto impositivo no coincida; solapa Mercado Pago Anulados para pares del extracto que se autoanulan (misma operación relacionada e importes opuestos) y no entran al match. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C63"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C64"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6051,7 +6113,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B14" t="str">
-        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago y Galicia). Uploads por ID sin duplicar, sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) como tesorería histórica. Permisos en Seguridad.</v>
+        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago y Galicia). Uploads por ID sin duplicar, sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) como tesorería histórica. En Mercado Pago, pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad.</v>
       </c>
       <c r="C14">
         <v>24</v>

</xml_diff>

<commit_message>
v2.21: extracto Galicia no duplica si solo cambió el saldo.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E244"/>
+  <dimension ref="A1:E246"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -4559,9 +4559,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="245">
+      <c r="A245" t="str">
+        <v>12/09/2026</v>
+      </c>
+      <c r="B245" t="str">
+        <v>08:50</v>
+      </c>
+      <c r="C245" t="str">
+        <v>Galicia: no duplicar extracto por saldo</v>
+      </c>
+      <c r="D245" t="str">
+        <v>El último Extracto_CC… (5) reinsertó 17 movimientos del 11/09 que ya estaban: el ID incluía el saldo y Galicia lo recálcula al exportar. Se borraron esas 17 copias (quedaron 3 del 10/09 que sí eran nuevas). El upload Galicia ahora no duplica si coinciden fecha, importe y descripción.</v>
+      </c>
+      <c r="E245" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="str">
+        <v>12/09/2026</v>
+      </c>
+      <c r="B246" t="str">
+        <v>09:25</v>
+      </c>
+      <c r="C246" t="str">
+        <v>Despliegue v2.21 producción</v>
+      </c>
+      <c r="D246" t="str">
+        <v>Push a main y Vercel --prod: extracto Galicia no duplica si solo cambió el saldo (ID sin saldo; dedupe por fecha, importe y descripción). APP_VERSION 2.21.</v>
+      </c>
+      <c r="E246" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E244"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E246"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5051,7 +5085,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + saldo). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto; Ingreso→crédito y Egreso→débito; historial de caja ya cerrada. El archivo debe llamarse MP_… en la solapa Mercado Pago y Galicia_… en Banco Galicia (primera palabra antes del _). Filas Pendiente y totales del pie no se cargan. Tesorería no duplica si ya existe misma fecha, monto, descripción, categoría y cliente (aunque el Excel sea de otro formato). La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto CC (fecha+débito/crédito+saldo) + tesorería tesoreria_transferencia_galicia (mismas columnas Tipo/Fecha/Crédito/Débito). Filtros de mes y de concepto del extracto (además de buscar); el control se marca en naranja cuando hay filtro activo. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe (misma fecha, fecha cercana ±14 días o fecha lejana, tolerancia ±$1) y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismos filtros Mes / Concepto del extracto / Buscar que la vista; si ya estaban activos, el modal los hereda; encabezados ordenan asc/desc). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos y Confirmados, entre Sistema e Importe aparecen Categoría y Cuenta contable de tesorería. Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql y sql/supabase_conciliacion_bancaria_manual_grupo.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto; Ingreso→crédito y Egreso→débito; historial de caja ya cerrada. El archivo debe llamarse MP_… en la solapa Mercado Pago y Galicia_… en Banco Galicia (primera palabra antes del _). Filas Pendiente y totales del pie no se cargan. Tesorería no duplica si ya existe misma fecha, monto, descripción, categoría y cliente (aunque el Excel sea de otro formato). La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto CC (fecha+débito/crédito+descripción; no duplica si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (mismas columnas Tipo/Fecha/Crédito/Débito). Filtros de mes y de concepto del extracto (además de buscar); el control se marca en naranja cuando hay filtro activo. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe (misma fecha, fecha cercana ±14 días o fecha lejana, tolerancia ±$1) y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismos filtros Mes / Concepto del extracto / Buscar que la vista; si ya estaban activos, el modal los hereda; encabezados ordenan asc/desc). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos y Confirmados, entre Sistema e Importe aparecen Categoría y Cuenta contable de tesorería. Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql y sql/supabase_conciliacion_bancaria_manual_grupo.sql.</v>
       </c>
     </row>
     <row r="61">
@@ -5198,7 +5232,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C64"/>
+  <dimension ref="A1:C65"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -5909,9 +5943,20 @@
         <v>Despliegue v2.20: Conciliación Bancaria — SIRTAC cuenta como IIBB y el importe único se sugiere aunque el concepto impositivo no coincida; solapa Mercado Pago Anulados para pares del extracto que se autoanulan (misma operación relacionada e importes opuestos) y no entran al match. Producción Vercel.</v>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>2.21</v>
+      </c>
+      <c r="B65" t="str">
+        <v>12/09/2026</v>
+      </c>
+      <c r="C65" t="str">
+        <v>Despliegue v2.21: Conciliación Bancaria — extracto Galicia ya no incluye el saldo en el ID; un reexport del banco con saldo corrido no duplica movimientos (dedupe por fecha, importe y descripción). Se eliminaron 17 copias del último upload. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C64"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C65"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>